<commit_message>
Add print-and-fill organizer for all filing types with more expense rows
Adds a 7-page handwriting edition (start-here guide, filing-type checklist,
expanded general/trucking/repair expense rows), 10 new general expense
lines across all organizer versions, and regenerated Scan Reader fields.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012ebqUPkXNMCm1mSUdBK3xi
</commit_message>
<xml_diff>
--- a/tax-prep/downloads/falcon-tax-organizer-2026.xlsx
+++ b/tax-prep/downloads/falcon-tax-organizer-2026.xlsx
@@ -50,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="433" uniqueCount="376">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="459" uniqueCount="391">
   <si>
     <t xml:space="preserve">Falcon Tax Solutions · 2026 Tax Organizer</t>
   </si>
@@ -406,6 +406,60 @@
     <t xml:space="preserve">27a</t>
   </si>
   <si>
+    <t xml:space="preserve">Materials &amp; supplies used for jobs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">22</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Parts and materials you buy for customers' jobs.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tools &amp; equipment (under $2,500 each)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Larger items may need depreciation.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Equipment rental</t>
+  </si>
+  <si>
+    <t xml:space="preserve">20a</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Repairs (business equipment, non-vehicle)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">21</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Uniforms &amp; safety gear</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Only clothing not suitable for everyday wear.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Postage &amp; shipping</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Utilities (business location)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Training, courses &amp; licenses for your trade</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Business gifts (up to $25 per person)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Home office (we calculate the deductible part)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">30</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Enter total rent/utilities for the home; we figure the business share (Form 8829).</t>
+  </si>
+  <si>
     <t xml:space="preserve">TRUCKING</t>
   </si>
   <si>
@@ -442,9 +496,6 @@
     <t xml:space="preserve">Truck or trailer lease / rent</t>
   </si>
   <si>
-    <t xml:space="preserve">20a</t>
-  </si>
-  <si>
     <t xml:space="preserve">Truck loan interest</t>
   </si>
   <si>
@@ -478,9 +529,6 @@
     <t xml:space="preserve">Electronics (tablet, dash cam, GPS, ELD device)</t>
   </si>
   <si>
-    <t xml:space="preserve">22</t>
-  </si>
-  <si>
     <t xml:space="preserve">Items over $2,500 each may need depreciation.</t>
   </si>
   <si>
@@ -491,9 +539,6 @@
   </si>
   <si>
     <t xml:space="preserve">Preventive maintenance (PM) service</t>
-  </si>
-  <si>
-    <t xml:space="preserve">21</t>
   </si>
   <si>
     <t xml:space="preserve">Oil &amp; filter change</t>
@@ -2590,7 +2635,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:F70"/>
+  <dimension ref="A1:F82"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="46"/>
@@ -2891,16 +2936,30 @@
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="23" t="s">
+      <c r="A21" s="6" t="s">
         <v>118</v>
+      </c>
+      <c r="B21" s="21" t="s">
+        <v>119</v>
+      </c>
+      <c r="C21" s="19"/>
+      <c r="D21" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="E21" s="25" t="n">
+        <f aca="false">C21*D21</f>
+        <v>0</v>
+      </c>
+      <c r="F21" s="11" t="s">
+        <v>120</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="6" t="s">
+        <v>121</v>
+      </c>
+      <c r="B22" s="21" t="s">
         <v>119</v>
-      </c>
-      <c r="B22" s="21" t="s">
-        <v>85</v>
       </c>
       <c r="C22" s="19"/>
       <c r="D22" s="24" t="n">
@@ -2910,13 +2969,16 @@
         <f aca="false">C22*D22</f>
         <v>0</v>
       </c>
+      <c r="F22" s="11" t="s">
+        <v>122</v>
+      </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="6" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="B23" s="21" t="s">
-        <v>85</v>
+        <v>124</v>
       </c>
       <c r="C23" s="19"/>
       <c r="D23" s="24" t="n">
@@ -2929,10 +2991,10 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="6" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="B24" s="21" t="s">
-        <v>107</v>
+        <v>126</v>
       </c>
       <c r="C24" s="19"/>
       <c r="D24" s="24" t="n">
@@ -2945,10 +3007,10 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="6" t="s">
-        <v>122</v>
+        <v>127</v>
       </c>
       <c r="B25" s="21" t="s">
-        <v>107</v>
+        <v>117</v>
       </c>
       <c r="C25" s="19"/>
       <c r="D25" s="24" t="n">
@@ -2958,13 +3020,16 @@
         <f aca="false">C25*D25</f>
         <v>0</v>
       </c>
+      <c r="F25" s="11" t="s">
+        <v>128</v>
+      </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="6" t="s">
-        <v>123</v>
+        <v>129</v>
       </c>
       <c r="B26" s="21" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="C26" s="19"/>
       <c r="D26" s="24" t="n">
@@ -2977,10 +3042,10 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="6" t="s">
-        <v>124</v>
+        <v>130</v>
       </c>
       <c r="B27" s="21" t="s">
-        <v>107</v>
+        <v>114</v>
       </c>
       <c r="C27" s="19"/>
       <c r="D27" s="24" t="n">
@@ -2993,10 +3058,10 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="6" t="s">
-        <v>125</v>
+        <v>131</v>
       </c>
       <c r="B28" s="21" t="s">
-        <v>107</v>
+        <v>117</v>
       </c>
       <c r="C28" s="19"/>
       <c r="D28" s="24" t="n">
@@ -3009,10 +3074,10 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="6" t="s">
-        <v>126</v>
+        <v>132</v>
       </c>
       <c r="B29" s="21" t="s">
-        <v>107</v>
+        <v>117</v>
       </c>
       <c r="C29" s="19"/>
       <c r="D29" s="24" t="n">
@@ -3023,44 +3088,36 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="30" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="6" t="s">
-        <v>127</v>
+        <v>133</v>
       </c>
       <c r="B30" s="21" t="s">
-        <v>107</v>
+        <v>134</v>
       </c>
       <c r="C30" s="19"/>
       <c r="D30" s="24" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E30" s="25" t="n">
         <f aca="false">C30*D30</f>
         <v>0</v>
       </c>
+      <c r="F30" s="11" t="s">
+        <v>135</v>
+      </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="6" t="s">
-        <v>128</v>
-      </c>
-      <c r="B31" s="21" t="s">
-        <v>97</v>
-      </c>
-      <c r="C31" s="19"/>
-      <c r="D31" s="24" t="n">
-        <v>1</v>
-      </c>
-      <c r="E31" s="25" t="n">
-        <f aca="false">C31*D31</f>
-        <v>0</v>
+      <c r="A31" s="23" t="s">
+        <v>136</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="6" t="s">
-        <v>129</v>
+        <v>137</v>
       </c>
       <c r="B32" s="21" t="s">
-        <v>130</v>
+        <v>85</v>
       </c>
       <c r="C32" s="19"/>
       <c r="D32" s="24" t="n">
@@ -3073,10 +3130,10 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="6" t="s">
-        <v>131</v>
+        <v>138</v>
       </c>
       <c r="B33" s="21" t="s">
-        <v>99</v>
+        <v>85</v>
       </c>
       <c r="C33" s="19"/>
       <c r="D33" s="24" t="n">
@@ -3089,10 +3146,10 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="6" t="s">
-        <v>132</v>
+        <v>139</v>
       </c>
       <c r="B34" s="21" t="s">
-        <v>117</v>
+        <v>107</v>
       </c>
       <c r="C34" s="19"/>
       <c r="D34" s="24" t="n">
@@ -3105,10 +3162,10 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="6" t="s">
-        <v>133</v>
+        <v>140</v>
       </c>
       <c r="B35" s="21" t="s">
-        <v>117</v>
+        <v>107</v>
       </c>
       <c r="C35" s="19"/>
       <c r="D35" s="24" t="n">
@@ -3121,10 +3178,10 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="6" t="s">
-        <v>134</v>
+        <v>141</v>
       </c>
       <c r="B36" s="21" t="s">
-        <v>117</v>
+        <v>107</v>
       </c>
       <c r="C36" s="19"/>
       <c r="D36" s="24" t="n">
@@ -3137,10 +3194,10 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="6" t="s">
-        <v>135</v>
+        <v>142</v>
       </c>
       <c r="B37" s="21" t="s">
-        <v>92</v>
+        <v>107</v>
       </c>
       <c r="C37" s="19"/>
       <c r="D37" s="24" t="n">
@@ -3153,10 +3210,10 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="6" t="s">
-        <v>136</v>
+        <v>143</v>
       </c>
       <c r="B38" s="21" t="s">
-        <v>137</v>
+        <v>107</v>
       </c>
       <c r="C38" s="19"/>
       <c r="D38" s="24" t="n">
@@ -3169,10 +3226,10 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="6" t="s">
-        <v>138</v>
+        <v>144</v>
       </c>
       <c r="B39" s="21" t="s">
-        <v>94</v>
+        <v>107</v>
       </c>
       <c r="C39" s="19"/>
       <c r="D39" s="24" t="n">
@@ -3185,10 +3242,10 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="6" t="s">
-        <v>139</v>
+        <v>145</v>
       </c>
       <c r="B40" s="21" t="s">
-        <v>117</v>
+        <v>107</v>
       </c>
       <c r="C40" s="19"/>
       <c r="D40" s="24" t="n">
@@ -3201,10 +3258,10 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="6" t="s">
-        <v>140</v>
+        <v>146</v>
       </c>
       <c r="B41" s="21" t="s">
-        <v>117</v>
+        <v>97</v>
       </c>
       <c r="C41" s="19"/>
       <c r="D41" s="24" t="n">
@@ -3217,10 +3274,10 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="6" t="s">
-        <v>141</v>
+        <v>147</v>
       </c>
       <c r="B42" s="21" t="s">
-        <v>142</v>
+        <v>124</v>
       </c>
       <c r="C42" s="19"/>
       <c r="D42" s="24" t="n">
@@ -3230,16 +3287,13 @@
         <f aca="false">C42*D42</f>
         <v>0</v>
       </c>
-      <c r="F42" s="11" t="s">
-        <v>143</v>
-      </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="6" t="s">
-        <v>144</v>
+        <v>148</v>
       </c>
       <c r="B43" s="21" t="s">
-        <v>117</v>
+        <v>99</v>
       </c>
       <c r="C43" s="19"/>
       <c r="D43" s="24" t="n">
@@ -3249,21 +3303,29 @@
         <f aca="false">C43*D43</f>
         <v>0</v>
       </c>
-      <c r="F43" s="11" t="s">
-        <v>143</v>
-      </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="23" t="s">
-        <v>145</v>
+      <c r="A44" s="6" t="s">
+        <v>149</v>
+      </c>
+      <c r="B44" s="21" t="s">
+        <v>117</v>
+      </c>
+      <c r="C44" s="19"/>
+      <c r="D44" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="E44" s="25" t="n">
+        <f aca="false">C44*D44</f>
+        <v>0</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="6" t="s">
-        <v>146</v>
+        <v>150</v>
       </c>
       <c r="B45" s="21" t="s">
-        <v>147</v>
+        <v>117</v>
       </c>
       <c r="C45" s="19"/>
       <c r="D45" s="24" t="n">
@@ -3276,10 +3338,10 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="6" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="B46" s="21" t="s">
-        <v>147</v>
+        <v>117</v>
       </c>
       <c r="C46" s="19"/>
       <c r="D46" s="24" t="n">
@@ -3292,10 +3354,10 @@
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="6" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="B47" s="21" t="s">
-        <v>147</v>
+        <v>92</v>
       </c>
       <c r="C47" s="19"/>
       <c r="D47" s="24" t="n">
@@ -3308,10 +3370,10 @@
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="6" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="B48" s="21" t="s">
-        <v>147</v>
+        <v>154</v>
       </c>
       <c r="C48" s="19"/>
       <c r="D48" s="24" t="n">
@@ -3324,10 +3386,10 @@
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="6" t="s">
-        <v>151</v>
+        <v>155</v>
       </c>
       <c r="B49" s="21" t="s">
-        <v>147</v>
+        <v>94</v>
       </c>
       <c r="C49" s="19"/>
       <c r="D49" s="24" t="n">
@@ -3340,10 +3402,10 @@
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="6" t="s">
-        <v>152</v>
+        <v>156</v>
       </c>
       <c r="B50" s="21" t="s">
-        <v>147</v>
+        <v>117</v>
       </c>
       <c r="C50" s="19"/>
       <c r="D50" s="24" t="n">
@@ -3356,10 +3418,10 @@
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="6" t="s">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="B51" s="21" t="s">
-        <v>147</v>
+        <v>117</v>
       </c>
       <c r="C51" s="19"/>
       <c r="D51" s="24" t="n">
@@ -3372,10 +3434,10 @@
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="6" t="s">
-        <v>154</v>
+        <v>158</v>
       </c>
       <c r="B52" s="21" t="s">
-        <v>147</v>
+        <v>119</v>
       </c>
       <c r="C52" s="19"/>
       <c r="D52" s="24" t="n">
@@ -3385,13 +3447,16 @@
         <f aca="false">C52*D52</f>
         <v>0</v>
       </c>
+      <c r="F52" s="11" t="s">
+        <v>159</v>
+      </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="6" t="s">
-        <v>155</v>
+        <v>160</v>
       </c>
       <c r="B53" s="21" t="s">
-        <v>147</v>
+        <v>117</v>
       </c>
       <c r="C53" s="19"/>
       <c r="D53" s="24" t="n">
@@ -3401,29 +3466,21 @@
         <f aca="false">C53*D53</f>
         <v>0</v>
       </c>
+      <c r="F53" s="11" t="s">
+        <v>159</v>
+      </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A54" s="6" t="s">
-        <v>156</v>
-      </c>
-      <c r="B54" s="21" t="s">
-        <v>147</v>
-      </c>
-      <c r="C54" s="19"/>
-      <c r="D54" s="24" t="n">
-        <v>1</v>
-      </c>
-      <c r="E54" s="25" t="n">
-        <f aca="false">C54*D54</f>
-        <v>0</v>
+      <c r="A54" s="23" t="s">
+        <v>161</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="6" t="s">
-        <v>157</v>
+        <v>162</v>
       </c>
       <c r="B55" s="21" t="s">
-        <v>147</v>
+        <v>126</v>
       </c>
       <c r="C55" s="19"/>
       <c r="D55" s="24" t="n">
@@ -3436,10 +3493,10 @@
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="6" t="s">
-        <v>158</v>
+        <v>163</v>
       </c>
       <c r="B56" s="21" t="s">
-        <v>147</v>
+        <v>126</v>
       </c>
       <c r="C56" s="19"/>
       <c r="D56" s="24" t="n">
@@ -3452,10 +3509,10 @@
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="6" t="s">
-        <v>159</v>
+        <v>164</v>
       </c>
       <c r="B57" s="21" t="s">
-        <v>147</v>
+        <v>126</v>
       </c>
       <c r="C57" s="19"/>
       <c r="D57" s="24" t="n">
@@ -3468,10 +3525,10 @@
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="6" t="s">
-        <v>160</v>
+        <v>165</v>
       </c>
       <c r="B58" s="21" t="s">
-        <v>147</v>
+        <v>126</v>
       </c>
       <c r="C58" s="19"/>
       <c r="D58" s="24" t="n">
@@ -3484,10 +3541,10 @@
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="6" t="s">
-        <v>161</v>
+        <v>166</v>
       </c>
       <c r="B59" s="21" t="s">
-        <v>147</v>
+        <v>126</v>
       </c>
       <c r="C59" s="19"/>
       <c r="D59" s="24" t="n">
@@ -3500,10 +3557,10 @@
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="6" t="s">
-        <v>162</v>
+        <v>167</v>
       </c>
       <c r="B60" s="21" t="s">
-        <v>147</v>
+        <v>126</v>
       </c>
       <c r="C60" s="19"/>
       <c r="D60" s="24" t="n">
@@ -3516,10 +3573,10 @@
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="6" t="s">
-        <v>163</v>
+        <v>168</v>
       </c>
       <c r="B61" s="21" t="s">
-        <v>147</v>
+        <v>126</v>
       </c>
       <c r="C61" s="19"/>
       <c r="D61" s="24" t="n">
@@ -3532,10 +3589,10 @@
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="6" t="s">
-        <v>164</v>
+        <v>169</v>
       </c>
       <c r="B62" s="21" t="s">
-        <v>147</v>
+        <v>126</v>
       </c>
       <c r="C62" s="19"/>
       <c r="D62" s="24" t="n">
@@ -3547,14 +3604,27 @@
       </c>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A63" s="23" t="s">
-        <v>165</v>
+      <c r="A63" s="6" t="s">
+        <v>170</v>
+      </c>
+      <c r="B63" s="21" t="s">
+        <v>126</v>
+      </c>
+      <c r="C63" s="19"/>
+      <c r="D63" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="E63" s="25" t="n">
+        <f aca="false">C63*D63</f>
+        <v>0</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A64" s="10"/>
+      <c r="A64" s="6" t="s">
+        <v>171</v>
+      </c>
       <c r="B64" s="21" t="s">
-        <v>117</v>
+        <v>126</v>
       </c>
       <c r="C64" s="19"/>
       <c r="D64" s="24" t="n">
@@ -3566,9 +3636,11 @@
       </c>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A65" s="10"/>
+      <c r="A65" s="6" t="s">
+        <v>172</v>
+      </c>
       <c r="B65" s="21" t="s">
-        <v>117</v>
+        <v>126</v>
       </c>
       <c r="C65" s="19"/>
       <c r="D65" s="24" t="n">
@@ -3580,9 +3652,11 @@
       </c>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A66" s="10"/>
+      <c r="A66" s="6" t="s">
+        <v>173</v>
+      </c>
       <c r="B66" s="21" t="s">
-        <v>117</v>
+        <v>126</v>
       </c>
       <c r="C66" s="19"/>
       <c r="D66" s="24" t="n">
@@ -3594,40 +3668,211 @@
       </c>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A67" s="9" t="s">
-        <v>166</v>
-      </c>
-      <c r="C67" s="20" t="n">
-        <f aca="false">SUM(C6:C66)</f>
-        <v>0</v>
-      </c>
-      <c r="E67" s="20" t="n">
-        <f aca="false">SUM(E6:E66)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="69" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A69" s="17" t="s">
-        <v>167</v>
-      </c>
-      <c r="B69" s="17"/>
-      <c r="C69" s="17"/>
-      <c r="D69" s="17"/>
-      <c r="E69" s="17"/>
-      <c r="F69" s="17"/>
+      <c r="A67" s="6" t="s">
+        <v>174</v>
+      </c>
+      <c r="B67" s="21" t="s">
+        <v>126</v>
+      </c>
+      <c r="C67" s="19"/>
+      <c r="D67" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="E67" s="25" t="n">
+        <f aca="false">C67*D67</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A68" s="6" t="s">
+        <v>175</v>
+      </c>
+      <c r="B68" s="21" t="s">
+        <v>126</v>
+      </c>
+      <c r="C68" s="19"/>
+      <c r="D68" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="E68" s="25" t="n">
+        <f aca="false">C68*D68</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A69" s="6" t="s">
+        <v>176</v>
+      </c>
+      <c r="B69" s="21" t="s">
+        <v>126</v>
+      </c>
+      <c r="C69" s="19"/>
+      <c r="D69" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="E69" s="25" t="n">
+        <f aca="false">C69*D69</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A70" s="17"/>
-      <c r="B70" s="17"/>
-      <c r="C70" s="17"/>
-      <c r="D70" s="17"/>
-      <c r="E70" s="17"/>
-      <c r="F70" s="17"/>
+      <c r="A70" s="6" t="s">
+        <v>177</v>
+      </c>
+      <c r="B70" s="21" t="s">
+        <v>126</v>
+      </c>
+      <c r="C70" s="19"/>
+      <c r="D70" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="E70" s="25" t="n">
+        <f aca="false">C70*D70</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A71" s="6" t="s">
+        <v>178</v>
+      </c>
+      <c r="B71" s="21" t="s">
+        <v>126</v>
+      </c>
+      <c r="C71" s="19"/>
+      <c r="D71" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="E71" s="25" t="n">
+        <f aca="false">C71*D71</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A72" s="6" t="s">
+        <v>179</v>
+      </c>
+      <c r="B72" s="21" t="s">
+        <v>126</v>
+      </c>
+      <c r="C72" s="19"/>
+      <c r="D72" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="E72" s="25" t="n">
+        <f aca="false">C72*D72</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A73" s="23" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A74" s="10"/>
+      <c r="B74" s="21" t="s">
+        <v>117</v>
+      </c>
+      <c r="C74" s="19"/>
+      <c r="D74" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="E74" s="25" t="n">
+        <f aca="false">C74*D74</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A75" s="10"/>
+      <c r="B75" s="21" t="s">
+        <v>117</v>
+      </c>
+      <c r="C75" s="19"/>
+      <c r="D75" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="E75" s="25" t="n">
+        <f aca="false">C75*D75</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A76" s="10"/>
+      <c r="B76" s="21" t="s">
+        <v>117</v>
+      </c>
+      <c r="C76" s="19"/>
+      <c r="D76" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="E76" s="25" t="n">
+        <f aca="false">C76*D76</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A77" s="10"/>
+      <c r="B77" s="21" t="s">
+        <v>117</v>
+      </c>
+      <c r="C77" s="19"/>
+      <c r="D77" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="E77" s="25" t="n">
+        <f aca="false">C77*D77</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A78" s="10"/>
+      <c r="B78" s="21" t="s">
+        <v>117</v>
+      </c>
+      <c r="C78" s="19"/>
+      <c r="D78" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="E78" s="25" t="n">
+        <f aca="false">C78*D78</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A79" s="9" t="s">
+        <v>181</v>
+      </c>
+      <c r="C79" s="20" t="n">
+        <f aca="false">SUM(C6:C78)</f>
+        <v>0</v>
+      </c>
+      <c r="E79" s="20" t="n">
+        <f aca="false">SUM(E6:E78)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="81" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A81" s="17" t="s">
+        <v>182</v>
+      </c>
+      <c r="B81" s="17"/>
+      <c r="C81" s="17"/>
+      <c r="D81" s="17"/>
+      <c r="E81" s="17"/>
+      <c r="F81" s="17"/>
+    </row>
+    <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A82" s="17"/>
+      <c r="B82" s="17"/>
+      <c r="C82" s="17"/>
+      <c r="D82" s="17"/>
+      <c r="E82" s="17"/>
+      <c r="F82" s="17"/>
     </row>
   </sheetData>
   <sheetProtection sheet="true" formatColumns="false" formatRows="false"/>
   <mergeCells count="1">
-    <mergeCell ref="A69:F70"/>
+    <mergeCell ref="A81:F82"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="true" verticalCentered="false"/>
   <pageMargins left="0.4" right="0.4" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -3653,40 +3898,40 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>168</v>
+        <v>183</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>169</v>
+        <v>184</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="14" t="s">
-        <v>170</v>
+        <v>185</v>
       </c>
       <c r="B4" s="14" t="s">
-        <v>171</v>
+        <v>186</v>
       </c>
       <c r="C4" s="14" t="s">
-        <v>172</v>
+        <v>187</v>
       </c>
       <c r="D4" s="14" t="s">
-        <v>173</v>
+        <v>188</v>
       </c>
       <c r="E4" s="14" t="s">
-        <v>174</v>
+        <v>189</v>
       </c>
       <c r="F4" s="14" t="s">
-        <v>175</v>
+        <v>190</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="15" t="s">
-        <v>176</v>
+        <v>191</v>
       </c>
       <c r="B5" s="15" t="s">
-        <v>177</v>
+        <v>192</v>
       </c>
       <c r="C5" s="15" t="n">
         <v>0</v>
@@ -4234,7 +4479,7 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E37" s="9" t="s">
-        <v>178</v>
+        <v>193</v>
       </c>
       <c r="F37" s="29" t="n">
         <f aca="false">F36*Data!$C$43</f>
@@ -4243,7 +4488,7 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="17" t="s">
-        <v>179</v>
+        <v>194</v>
       </c>
       <c r="B39" s="17"/>
       <c r="C39" s="17"/>
@@ -4296,34 +4541,34 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>180</v>
+        <v>195</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>181</v>
+        <v>196</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="14" t="s">
-        <v>182</v>
+        <v>197</v>
       </c>
       <c r="B4" s="14" t="s">
-        <v>183</v>
+        <v>198</v>
       </c>
       <c r="C4" s="14" t="s">
-        <v>184</v>
+        <v>199</v>
       </c>
       <c r="D4" s="14" t="s">
-        <v>185</v>
+        <v>200</v>
       </c>
       <c r="E4" s="14" t="s">
-        <v>184</v>
+        <v>199</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
-        <v>186</v>
+        <v>201</v>
       </c>
       <c r="B5" s="19"/>
       <c r="C5" s="26"/>
@@ -4332,7 +4577,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>187</v>
+        <v>202</v>
       </c>
       <c r="B6" s="19"/>
       <c r="C6" s="26"/>
@@ -4341,7 +4586,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>188</v>
+        <v>203</v>
       </c>
       <c r="B7" s="19"/>
       <c r="C7" s="26"/>
@@ -4350,7 +4595,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>189</v>
+        <v>204</v>
       </c>
       <c r="B8" s="19"/>
       <c r="C8" s="26"/>
@@ -4396,53 +4641,53 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>190</v>
+        <v>205</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>191</v>
+        <v>206</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>192</v>
+        <v>207</v>
       </c>
       <c r="B4" s="10"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
-        <v>193</v>
+        <v>208</v>
       </c>
       <c r="B5" s="10"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>194</v>
+        <v>209</v>
       </c>
       <c r="B6" s="10"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>195</v>
+        <v>210</v>
       </c>
       <c r="B7" s="10"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>196</v>
+        <v>211</v>
       </c>
       <c r="B8" s="10"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="s">
-        <v>197</v>
+        <v>212</v>
       </c>
       <c r="B9" s="10"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="6" t="s">
-        <v>198</v>
+        <v>213</v>
       </c>
       <c r="B10" s="10"/>
     </row>
@@ -4485,454 +4730,454 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>199</v>
+        <v>214</v>
       </c>
       <c r="E1" s="30" t="s">
         <v>22</v>
       </c>
       <c r="F1" s="30" t="s">
-        <v>200</v>
+        <v>215</v>
       </c>
       <c r="H1" s="30" t="s">
-        <v>201</v>
+        <v>216</v>
       </c>
       <c r="I1" s="30" t="s">
-        <v>200</v>
+        <v>215</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>202</v>
+        <v>217</v>
       </c>
       <c r="E2" s="30" t="s">
-        <v>203</v>
+        <v>218</v>
       </c>
       <c r="F2" s="30" t="s">
-        <v>204</v>
+        <v>219</v>
       </c>
       <c r="H2" s="30" t="s">
-        <v>205</v>
+        <v>220</v>
       </c>
       <c r="I2" s="30" t="s">
-        <v>206</v>
+        <v>221</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="31" t="s">
-        <v>207</v>
+        <v>222</v>
       </c>
       <c r="B3" s="31" t="s">
-        <v>208</v>
+        <v>223</v>
       </c>
       <c r="C3" s="31" t="s">
-        <v>209</v>
+        <v>224</v>
       </c>
       <c r="E3" s="30" t="s">
-        <v>210</v>
+        <v>225</v>
       </c>
       <c r="F3" s="30" t="s">
-        <v>211</v>
+        <v>226</v>
       </c>
       <c r="H3" s="30" t="s">
-        <v>212</v>
+        <v>227</v>
       </c>
       <c r="I3" s="30" t="s">
-        <v>213</v>
+        <v>228</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="9" t="s">
-        <v>214</v>
+        <v>229</v>
       </c>
       <c r="B4" s="21" t="s">
-        <v>215</v>
+        <v>230</v>
       </c>
       <c r="C4" s="6" t="str">
         <f aca="false">"falcon-organizer-2026"</f>
         <v>falcon-organizer-2026</v>
       </c>
       <c r="E4" s="30" t="s">
-        <v>216</v>
+        <v>231</v>
       </c>
       <c r="F4" s="30" t="s">
-        <v>217</v>
+        <v>232</v>
       </c>
       <c r="H4" s="30" t="s">
-        <v>218</v>
+        <v>233</v>
       </c>
       <c r="I4" s="30" t="s">
-        <v>219</v>
+        <v>234</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="9" t="s">
-        <v>220</v>
+        <v>235</v>
       </c>
       <c r="B5" s="21" t="s">
-        <v>221</v>
+        <v>236</v>
       </c>
       <c r="C5" s="6" t="str">
         <f aca="false">IFERROR(INDEX($F$2:$F$5,MATCH(Household!B4,$E$2:$E$5,0)),"single")</f>
         <v>single</v>
       </c>
       <c r="E5" s="30" t="s">
-        <v>222</v>
+        <v>237</v>
       </c>
       <c r="F5" s="30" t="s">
-        <v>223</v>
+        <v>238</v>
       </c>
       <c r="H5" s="30" t="s">
-        <v>224</v>
+        <v>239</v>
       </c>
       <c r="I5" s="30" t="s">
-        <v>225</v>
+        <v>240</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="9" t="s">
-        <v>226</v>
+        <v>241</v>
       </c>
       <c r="B6" s="21" t="s">
-        <v>227</v>
+        <v>242</v>
       </c>
       <c r="C6" s="6" t="str">
         <f aca="false">IFERROR(INDEX($I$2:$I$52,MATCH(Household!B5,$H$2:$H$52,0)),"")</f>
         <v/>
       </c>
       <c r="H6" s="30" t="s">
-        <v>228</v>
+        <v>243</v>
       </c>
       <c r="I6" s="30" t="s">
-        <v>229</v>
+        <v>244</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="9" t="s">
-        <v>230</v>
+        <v>245</v>
       </c>
       <c r="B7" s="21" t="s">
-        <v>231</v>
+        <v>246</v>
       </c>
       <c r="C7" s="6" t="n">
         <f aca="false">IF(AND(ISNUMBER(Household!B6),Household!B6&gt;0,Household!B6&lt;=1961),1,0)</f>
         <v>0</v>
       </c>
       <c r="H7" s="30" t="s">
-        <v>232</v>
+        <v>247</v>
       </c>
       <c r="I7" s="30" t="s">
-        <v>233</v>
+        <v>248</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="9" t="s">
-        <v>234</v>
+        <v>249</v>
       </c>
       <c r="B8" s="21" t="s">
-        <v>235</v>
+        <v>250</v>
       </c>
       <c r="C8" s="6" t="n">
         <f aca="false">IF(AND(C5="mfj",ISNUMBER(Household!B7),Household!B7&gt;0,Household!B7&lt;=1961),1,0)</f>
         <v>0</v>
       </c>
       <c r="H8" s="30" t="s">
-        <v>236</v>
+        <v>251</v>
       </c>
       <c r="I8" s="30" t="s">
-        <v>237</v>
+        <v>252</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="9" t="s">
-        <v>238</v>
+        <v>253</v>
       </c>
       <c r="B9" s="21" t="s">
-        <v>239</v>
+        <v>254</v>
       </c>
       <c r="C9" s="6" t="n">
         <f aca="false">COUNTIFS(Household!A14:A23,"?*",Household!C14:C23,"&gt;=2010")</f>
         <v>0</v>
       </c>
       <c r="H9" s="30" t="s">
-        <v>240</v>
+        <v>255</v>
       </c>
       <c r="I9" s="30" t="s">
-        <v>241</v>
+        <v>256</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="9" t="s">
-        <v>242</v>
+        <v>257</v>
       </c>
       <c r="B10" s="21" t="s">
-        <v>243</v>
+        <v>258</v>
       </c>
       <c r="C10" s="6" t="n">
         <f aca="false">COUNTIF(Household!A14:A23,"?*")-C9</f>
         <v>0</v>
       </c>
       <c r="H10" s="30" t="s">
-        <v>244</v>
+        <v>259</v>
       </c>
       <c r="I10" s="30" t="s">
-        <v>245</v>
+        <v>260</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="9" t="s">
-        <v>246</v>
+        <v>261</v>
       </c>
       <c r="B11" s="21" t="s">
-        <v>247</v>
+        <v>262</v>
       </c>
       <c r="C11" s="6" t="str">
         <f aca="false">IF(C9+C10&gt;0,"yes","no")</f>
         <v>no</v>
       </c>
       <c r="H11" s="30" t="s">
-        <v>248</v>
+        <v>263</v>
       </c>
       <c r="I11" s="30" t="s">
-        <v>249</v>
+        <v>264</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="9" t="s">
-        <v>250</v>
+        <v>265</v>
       </c>
       <c r="B12" s="21" t="s">
-        <v>251</v>
+        <v>266</v>
       </c>
       <c r="C12" s="6" t="n">
         <f aca="false">IF(TRIM(Household!B8)="Yes",1,0)</f>
         <v>0</v>
       </c>
       <c r="H12" s="30" t="s">
-        <v>252</v>
+        <v>267</v>
       </c>
       <c r="I12" s="30" t="s">
-        <v>253</v>
+        <v>268</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="9" t="s">
-        <v>254</v>
+        <v>269</v>
       </c>
       <c r="B13" s="21" t="s">
-        <v>255</v>
+        <v>270</v>
       </c>
       <c r="C13" s="6" t="n">
         <f aca="false">Jobs!C16+Income!C24</f>
         <v>0</v>
       </c>
       <c r="H13" s="30" t="s">
-        <v>256</v>
+        <v>271</v>
       </c>
       <c r="I13" s="30" t="s">
-        <v>257</v>
+        <v>272</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="9" t="s">
-        <v>258</v>
+        <v>273</v>
       </c>
       <c r="B14" s="21" t="s">
-        <v>259</v>
+        <v>274</v>
       </c>
       <c r="C14" s="32" t="n">
         <f aca="false">Jobs!D16</f>
         <v>0</v>
       </c>
       <c r="H14" s="30" t="s">
-        <v>260</v>
+        <v>275</v>
       </c>
       <c r="I14" s="30" t="s">
-        <v>261</v>
+        <v>276</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="9" t="s">
-        <v>262</v>
+        <v>277</v>
       </c>
       <c r="B15" s="21" t="s">
-        <v>263</v>
+        <v>278</v>
       </c>
       <c r="C15" s="32" t="n">
         <f aca="false">Jobs!E16</f>
         <v>0</v>
       </c>
       <c r="H15" s="30" t="s">
-        <v>264</v>
+        <v>279</v>
       </c>
       <c r="I15" s="30" t="s">
-        <v>265</v>
+        <v>280</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="9" t="s">
-        <v>266</v>
+        <v>281</v>
       </c>
       <c r="B16" s="21" t="s">
-        <v>267</v>
+        <v>282</v>
       </c>
       <c r="C16" s="6" t="n">
         <f aca="false">Jobs!F16+Income!C24</f>
         <v>0</v>
       </c>
       <c r="H16" s="30" t="s">
-        <v>268</v>
+        <v>283</v>
       </c>
       <c r="I16" s="30" t="s">
-        <v>269</v>
+        <v>284</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="9" t="s">
-        <v>270</v>
+        <v>285</v>
       </c>
       <c r="B17" s="21" t="s">
-        <v>271</v>
+        <v>286</v>
       </c>
       <c r="C17" s="32" t="n">
         <f aca="false">Jobs!G16</f>
         <v>0</v>
       </c>
       <c r="H17" s="30" t="s">
-        <v>272</v>
+        <v>287</v>
       </c>
       <c r="I17" s="30" t="s">
-        <v>273</v>
+        <v>288</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="9" t="s">
-        <v>274</v>
+        <v>289</v>
       </c>
       <c r="B18" s="21" t="s">
-        <v>275</v>
+        <v>290</v>
       </c>
       <c r="C18" s="32" t="n">
         <f aca="false">Income!C19</f>
         <v>0</v>
       </c>
       <c r="H18" s="30" t="s">
-        <v>276</v>
+        <v>291</v>
       </c>
       <c r="I18" s="30" t="s">
-        <v>277</v>
+        <v>292</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="9" t="s">
-        <v>278</v>
+        <v>293</v>
       </c>
       <c r="B19" s="21" t="s">
-        <v>279</v>
+        <v>294</v>
       </c>
       <c r="C19" s="32" t="n">
-        <f aca="false">Expenses!E67</f>
+        <f aca="false">Expenses!E79</f>
         <v>0</v>
       </c>
       <c r="H19" s="30" t="s">
-        <v>280</v>
+        <v>295</v>
       </c>
       <c r="I19" s="30" t="s">
-        <v>281</v>
+        <v>296</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="9" t="s">
-        <v>282</v>
+        <v>297</v>
       </c>
       <c r="B20" s="21" t="s">
-        <v>283</v>
+        <v>298</v>
       </c>
       <c r="C20" s="32" t="n">
         <f aca="false">Payments!B9</f>
         <v>0</v>
       </c>
       <c r="H20" s="30" t="s">
-        <v>284</v>
+        <v>299</v>
       </c>
       <c r="I20" s="30" t="s">
-        <v>285</v>
+        <v>300</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="9" t="s">
-        <v>286</v>
+        <v>301</v>
       </c>
       <c r="B21" s="21" t="s">
-        <v>287</v>
+        <v>302</v>
       </c>
       <c r="C21" s="32" t="n">
         <f aca="false">Payments!D9</f>
         <v>0</v>
       </c>
       <c r="H21" s="30" t="s">
-        <v>288</v>
+        <v>303</v>
       </c>
       <c r="I21" s="30" t="s">
-        <v>289</v>
+        <v>304</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="9" t="s">
-        <v>290</v>
+        <v>305</v>
       </c>
       <c r="B22" s="21" t="s">
-        <v>291</v>
+        <v>306</v>
       </c>
       <c r="C22" s="6" t="n">
         <f aca="false">IF(Trips!D36+Trips!E36&gt;0,1,0)</f>
         <v>0</v>
       </c>
       <c r="H22" s="30" t="s">
-        <v>292</v>
+        <v>307</v>
       </c>
       <c r="I22" s="30" t="s">
-        <v>293</v>
+        <v>308</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="9" t="s">
-        <v>294</v>
+        <v>309</v>
       </c>
       <c r="B23" s="21" t="s">
-        <v>295</v>
+        <v>310</v>
       </c>
       <c r="C23" s="6" t="n">
         <f aca="false">ROUND(Trips!D36-Trips!C36+Trips!C36*C41/C40,2)</f>
         <v>0</v>
       </c>
       <c r="H23" s="30" t="s">
-        <v>296</v>
+        <v>311</v>
       </c>
       <c r="I23" s="30" t="s">
-        <v>297</v>
+        <v>312</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="9" t="s">
-        <v>298</v>
+        <v>313</v>
       </c>
       <c r="B24" s="21" t="s">
-        <v>174</v>
+        <v>189</v>
       </c>
       <c r="C24" s="33" t="n">
         <f aca="false">Trips!E36</f>
         <v>0</v>
       </c>
       <c r="H24" s="30" t="s">
-        <v>299</v>
+        <v>314</v>
       </c>
       <c r="I24" s="30" t="s">
-        <v>300</v>
+        <v>315</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="9" t="s">
-        <v>301</v>
+        <v>316</v>
       </c>
       <c r="B25" s="21" t="s">
         <v>69</v>
@@ -4942,353 +5187,353 @@
         <v>0</v>
       </c>
       <c r="H25" s="30" t="s">
-        <v>302</v>
+        <v>317</v>
       </c>
       <c r="I25" s="30" t="s">
-        <v>303</v>
+        <v>318</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="9" t="s">
-        <v>304</v>
+        <v>319</v>
       </c>
       <c r="B26" s="21" t="s">
-        <v>305</v>
+        <v>320</v>
       </c>
       <c r="C26" s="32" t="n">
         <f aca="false">Income!C26</f>
         <v>0</v>
       </c>
       <c r="H26" s="30" t="s">
-        <v>306</v>
+        <v>321</v>
       </c>
       <c r="I26" s="30" t="s">
-        <v>307</v>
+        <v>322</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="9" t="s">
-        <v>308</v>
+        <v>323</v>
       </c>
       <c r="B27" s="21" t="s">
-        <v>309</v>
+        <v>324</v>
       </c>
       <c r="C27" s="6" t="n">
         <f aca="false">Income!C27+Income!C28</f>
         <v>0</v>
       </c>
       <c r="H27" s="30" t="s">
-        <v>310</v>
+        <v>325</v>
       </c>
       <c r="I27" s="30" t="s">
-        <v>311</v>
+        <v>326</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="9" t="s">
-        <v>312</v>
+        <v>327</v>
       </c>
       <c r="B28" s="21" t="s">
-        <v>313</v>
+        <v>328</v>
       </c>
       <c r="C28" s="6" t="n">
         <f aca="false">IF(Income!C27&gt;0,1,0)</f>
         <v>0</v>
       </c>
       <c r="H28" s="30" t="s">
-        <v>314</v>
+        <v>329</v>
       </c>
       <c r="I28" s="30" t="s">
-        <v>315</v>
+        <v>330</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="9" t="s">
-        <v>316</v>
+        <v>331</v>
       </c>
       <c r="B29" s="21" t="s">
-        <v>192</v>
+        <v>207</v>
       </c>
       <c r="C29" s="6" t="n">
         <f aca="false">IF(TRIM(Checklist!B4)="Yes",1,0)</f>
         <v>0</v>
       </c>
       <c r="H29" s="30" t="s">
-        <v>317</v>
+        <v>332</v>
       </c>
       <c r="I29" s="30" t="s">
-        <v>318</v>
+        <v>333</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="9" t="s">
-        <v>319</v>
+        <v>334</v>
       </c>
       <c r="B30" s="21" t="s">
-        <v>193</v>
+        <v>208</v>
       </c>
       <c r="C30" s="6" t="n">
         <f aca="false">IF(TRIM(Checklist!B5)="Yes",1,0)</f>
         <v>0</v>
       </c>
       <c r="H30" s="30" t="s">
-        <v>320</v>
+        <v>335</v>
       </c>
       <c r="I30" s="30" t="s">
-        <v>321</v>
+        <v>336</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="9" t="s">
-        <v>322</v>
+        <v>337</v>
       </c>
       <c r="B31" s="21" t="s">
-        <v>194</v>
+        <v>209</v>
       </c>
       <c r="C31" s="6" t="n">
         <f aca="false">IF(TRIM(Checklist!B6)="Yes",1,0)</f>
         <v>0</v>
       </c>
       <c r="H31" s="30" t="s">
-        <v>323</v>
+        <v>338</v>
       </c>
       <c r="I31" s="30" t="s">
-        <v>324</v>
+        <v>339</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="9" t="s">
-        <v>325</v>
+        <v>340</v>
       </c>
       <c r="B32" s="21" t="s">
-        <v>195</v>
+        <v>210</v>
       </c>
       <c r="C32" s="6" t="n">
         <f aca="false">IF(TRIM(Checklist!B7)="Yes",1,0)</f>
         <v>0</v>
       </c>
       <c r="H32" s="30" t="s">
-        <v>326</v>
+        <v>341</v>
       </c>
       <c r="I32" s="30" t="s">
-        <v>327</v>
+        <v>342</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="9" t="s">
-        <v>328</v>
+        <v>343</v>
       </c>
       <c r="B33" s="21" t="s">
-        <v>196</v>
+        <v>211</v>
       </c>
       <c r="C33" s="6" t="n">
         <f aca="false">IF(TRIM(Checklist!B8)="Yes",1,0)</f>
         <v>0</v>
       </c>
       <c r="H33" s="30" t="s">
-        <v>329</v>
+        <v>344</v>
       </c>
       <c r="I33" s="30" t="s">
-        <v>330</v>
+        <v>345</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="9" t="s">
-        <v>331</v>
+        <v>346</v>
       </c>
       <c r="B34" s="21" t="s">
-        <v>197</v>
+        <v>212</v>
       </c>
       <c r="C34" s="6" t="n">
         <f aca="false">IF(TRIM(Checklist!B9)="Yes",1,0)</f>
         <v>0</v>
       </c>
       <c r="H34" s="30" t="s">
-        <v>332</v>
+        <v>347</v>
       </c>
       <c r="I34" s="30" t="s">
-        <v>333</v>
+        <v>348</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="9" t="s">
-        <v>334</v>
+        <v>349</v>
       </c>
       <c r="B35" s="21" t="s">
-        <v>198</v>
+        <v>213</v>
       </c>
       <c r="C35" s="6" t="n">
         <f aca="false">IF(TRIM(Checklist!B10)="Yes",1,0)</f>
         <v>0</v>
       </c>
       <c r="H35" s="30" t="s">
-        <v>335</v>
+        <v>350</v>
       </c>
       <c r="I35" s="30" t="s">
-        <v>336</v>
+        <v>351</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H36" s="0" t="s">
-        <v>337</v>
+        <v>352</v>
       </c>
       <c r="I36" s="0" t="s">
-        <v>338</v>
+        <v>353</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H37" s="0" t="s">
-        <v>339</v>
+        <v>354</v>
       </c>
       <c r="I37" s="0" t="s">
-        <v>340</v>
+        <v>355</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H38" s="0" t="s">
-        <v>341</v>
+        <v>356</v>
       </c>
       <c r="I38" s="0" t="s">
-        <v>342</v>
+        <v>357</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="34" t="s">
-        <v>343</v>
+        <v>358</v>
       </c>
       <c r="H39" s="30" t="s">
-        <v>344</v>
+        <v>359</v>
       </c>
       <c r="I39" s="30" t="s">
-        <v>345</v>
+        <v>360</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B40" s="6" t="s">
-        <v>346</v>
+        <v>361</v>
       </c>
       <c r="C40" s="35" t="n">
         <v>80</v>
       </c>
       <c r="H40" s="30" t="s">
-        <v>347</v>
+        <v>362</v>
       </c>
       <c r="I40" s="30" t="s">
-        <v>348</v>
+        <v>363</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B41" s="6" t="s">
-        <v>349</v>
+        <v>364</v>
       </c>
       <c r="C41" s="35" t="n">
         <v>86</v>
       </c>
       <c r="H41" s="30" t="s">
-        <v>350</v>
+        <v>365</v>
       </c>
       <c r="I41" s="30" t="s">
-        <v>351</v>
+        <v>366</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B42" s="6" t="s">
-        <v>352</v>
+        <v>367</v>
       </c>
       <c r="C42" s="36" t="n">
         <v>0.75</v>
       </c>
       <c r="H42" s="30" t="s">
-        <v>353</v>
+        <v>368</v>
       </c>
       <c r="I42" s="30" t="s">
-        <v>354</v>
+        <v>369</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B43" s="6" t="s">
-        <v>355</v>
+        <v>370</v>
       </c>
       <c r="C43" s="36" t="n">
         <v>0.8</v>
       </c>
       <c r="H43" s="30" t="s">
-        <v>356</v>
+        <v>371</v>
       </c>
       <c r="I43" s="30" t="s">
-        <v>357</v>
+        <v>372</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H44" s="0" t="s">
-        <v>358</v>
+        <v>373</v>
       </c>
       <c r="I44" s="0" t="s">
-        <v>359</v>
+        <v>374</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H45" s="0" t="s">
-        <v>360</v>
+        <v>375</v>
       </c>
       <c r="I45" s="0" t="s">
-        <v>361</v>
+        <v>376</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H46" s="0" t="s">
-        <v>362</v>
+        <v>377</v>
       </c>
       <c r="I46" s="0" t="s">
-        <v>363</v>
+        <v>378</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H47" s="0" t="s">
-        <v>364</v>
+        <v>379</v>
       </c>
       <c r="I47" s="0" t="s">
-        <v>365</v>
+        <v>380</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H48" s="0" t="s">
-        <v>366</v>
+        <v>381</v>
       </c>
       <c r="I48" s="0" t="s">
-        <v>367</v>
+        <v>382</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H49" s="0" t="s">
-        <v>368</v>
+        <v>383</v>
       </c>
       <c r="I49" s="0" t="s">
-        <v>369</v>
+        <v>384</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H50" s="0" t="s">
-        <v>370</v>
+        <v>385</v>
       </c>
       <c r="I50" s="0" t="s">
-        <v>371</v>
+        <v>386</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H51" s="0" t="s">
-        <v>372</v>
+        <v>387</v>
       </c>
       <c r="I51" s="0" t="s">
-        <v>373</v>
+        <v>388</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H52" s="0" t="s">
-        <v>374</v>
+        <v>389</v>
       </c>
       <c r="I52" s="0" t="s">
-        <v>375</v>
+        <v>390</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fix per diem, QBI and estimator issues found by QA and design review
- Per diem: only 2026 days count, overlapping trips merged, capped at a year
- QBI: 2026 thresholds with gradual phase-down instead of a cliff
- HoH bracket, SE tax $400 test, SE losses, amount caps
- Estimator: cents allowed, Edit my answers on results, totals row,
  per diem shown as info, collapsed organizer box, steadier step label,
  corrected disclaimer
- Organizers: dependent SSN is a tick box / Yes-No only; print sheets
  show SHEET n OF 7 and ask for all sheets

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012ebqUPkXNMCm1mSUdBK3xi
</commit_message>
<xml_diff>
--- a/tax-prep/downloads/falcon-tax-organizer-2026.xlsx
+++ b/tax-prep/downloads/falcon-tax-organizer-2026.xlsx
@@ -634,7 +634,7 @@
     <t xml:space="preserve">Deductible (80%)</t>
   </si>
   <si>
-    <t xml:space="preserve">IRS transportation per diem (Notice 2026-60): $80/day in the U.S., $86 in Canada. The day you leave and the day you return count at 75%. Drivers under DOT hours-of-service rules deduct 80%. Employee (W-2) drivers can't deduct this on their federal return. Keep your logbook or ELD records.</t>
+    <t xml:space="preserve">IRS transportation per diem (Notice 2026-60): $80/day in the U.S., $86 in Canada. The day you leave and the day you return count at 75%. Only 2026 days count; don't list the same day on two trips. Drivers under DOT hours-of-service rules deduct 80%. Employee (W-2) drivers can't deduct this on their federal return. Keep your logbook or ELD records.</t>
   </si>
   <si>
     <t xml:space="preserve">Estimated tax payments</t>
@@ -2188,7 +2188,7 @@
       <formula1>"Yes,No"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="E14:E23" type="list">
+    <dataValidation allowBlank="true" error="Choose Yes or No. Never type a Social Security number here." errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="E14:E23" type="list">
       <formula1>"Yes,No"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -3951,11 +3951,11 @@
       <c r="B6" s="26"/>
       <c r="C6" s="12"/>
       <c r="D6" s="27" t="n">
-        <f aca="false">IF(AND(ISNUMBER(A6),ISNUMBER(B6),B6&gt;A6),B6-A6-1,0)</f>
+        <f aca="false">IF(AND(ISNUMBER(A6),ISNUMBER(B6),B6&gt;A6),MAX(0,MIN(B6-1,DATE(2026,12,31))-MAX(A6+1,DATE(2026,1,1))+1),0)</f>
         <v>0</v>
       </c>
       <c r="E6" s="27" t="n">
-        <f aca="false">IF(AND(ISNUMBER(A6),ISNUMBER(B6),B6&gt;A6),2,0)</f>
+        <f aca="false">IF(AND(ISNUMBER(A6),ISNUMBER(B6),B6&gt;A6),AND(A6&gt;=DATE(2026,1,1),A6&lt;=DATE(2026,12,31))*1+AND(B6&gt;=DATE(2026,1,1),B6&lt;=DATE(2026,12,31))*1,0)</f>
         <v>0</v>
       </c>
       <c r="F6" s="25" t="n">
@@ -3968,11 +3968,11 @@
       <c r="B7" s="26"/>
       <c r="C7" s="12"/>
       <c r="D7" s="27" t="n">
-        <f aca="false">IF(AND(ISNUMBER(A7),ISNUMBER(B7),B7&gt;A7),B7-A7-1,0)</f>
+        <f aca="false">IF(AND(ISNUMBER(A7),ISNUMBER(B7),B7&gt;A7),MAX(0,MIN(B7-1,DATE(2026,12,31))-MAX(A7+1,DATE(2026,1,1))+1),0)</f>
         <v>0</v>
       </c>
       <c r="E7" s="27" t="n">
-        <f aca="false">IF(AND(ISNUMBER(A7),ISNUMBER(B7),B7&gt;A7),2,0)</f>
+        <f aca="false">IF(AND(ISNUMBER(A7),ISNUMBER(B7),B7&gt;A7),AND(A7&gt;=DATE(2026,1,1),A7&lt;=DATE(2026,12,31))*1+AND(B7&gt;=DATE(2026,1,1),B7&lt;=DATE(2026,12,31))*1,0)</f>
         <v>0</v>
       </c>
       <c r="F7" s="25" t="n">
@@ -3985,11 +3985,11 @@
       <c r="B8" s="26"/>
       <c r="C8" s="12"/>
       <c r="D8" s="27" t="n">
-        <f aca="false">IF(AND(ISNUMBER(A8),ISNUMBER(B8),B8&gt;A8),B8-A8-1,0)</f>
+        <f aca="false">IF(AND(ISNUMBER(A8),ISNUMBER(B8),B8&gt;A8),MAX(0,MIN(B8-1,DATE(2026,12,31))-MAX(A8+1,DATE(2026,1,1))+1),0)</f>
         <v>0</v>
       </c>
       <c r="E8" s="27" t="n">
-        <f aca="false">IF(AND(ISNUMBER(A8),ISNUMBER(B8),B8&gt;A8),2,0)</f>
+        <f aca="false">IF(AND(ISNUMBER(A8),ISNUMBER(B8),B8&gt;A8),AND(A8&gt;=DATE(2026,1,1),A8&lt;=DATE(2026,12,31))*1+AND(B8&gt;=DATE(2026,1,1),B8&lt;=DATE(2026,12,31))*1,0)</f>
         <v>0</v>
       </c>
       <c r="F8" s="25" t="n">
@@ -4002,11 +4002,11 @@
       <c r="B9" s="26"/>
       <c r="C9" s="12"/>
       <c r="D9" s="27" t="n">
-        <f aca="false">IF(AND(ISNUMBER(A9),ISNUMBER(B9),B9&gt;A9),B9-A9-1,0)</f>
+        <f aca="false">IF(AND(ISNUMBER(A9),ISNUMBER(B9),B9&gt;A9),MAX(0,MIN(B9-1,DATE(2026,12,31))-MAX(A9+1,DATE(2026,1,1))+1),0)</f>
         <v>0</v>
       </c>
       <c r="E9" s="27" t="n">
-        <f aca="false">IF(AND(ISNUMBER(A9),ISNUMBER(B9),B9&gt;A9),2,0)</f>
+        <f aca="false">IF(AND(ISNUMBER(A9),ISNUMBER(B9),B9&gt;A9),AND(A9&gt;=DATE(2026,1,1),A9&lt;=DATE(2026,12,31))*1+AND(B9&gt;=DATE(2026,1,1),B9&lt;=DATE(2026,12,31))*1,0)</f>
         <v>0</v>
       </c>
       <c r="F9" s="25" t="n">
@@ -4019,11 +4019,11 @@
       <c r="B10" s="26"/>
       <c r="C10" s="12"/>
       <c r="D10" s="27" t="n">
-        <f aca="false">IF(AND(ISNUMBER(A10),ISNUMBER(B10),B10&gt;A10),B10-A10-1,0)</f>
+        <f aca="false">IF(AND(ISNUMBER(A10),ISNUMBER(B10),B10&gt;A10),MAX(0,MIN(B10-1,DATE(2026,12,31))-MAX(A10+1,DATE(2026,1,1))+1),0)</f>
         <v>0</v>
       </c>
       <c r="E10" s="27" t="n">
-        <f aca="false">IF(AND(ISNUMBER(A10),ISNUMBER(B10),B10&gt;A10),2,0)</f>
+        <f aca="false">IF(AND(ISNUMBER(A10),ISNUMBER(B10),B10&gt;A10),AND(A10&gt;=DATE(2026,1,1),A10&lt;=DATE(2026,12,31))*1+AND(B10&gt;=DATE(2026,1,1),B10&lt;=DATE(2026,12,31))*1,0)</f>
         <v>0</v>
       </c>
       <c r="F10" s="25" t="n">
@@ -4036,11 +4036,11 @@
       <c r="B11" s="26"/>
       <c r="C11" s="12"/>
       <c r="D11" s="27" t="n">
-        <f aca="false">IF(AND(ISNUMBER(A11),ISNUMBER(B11),B11&gt;A11),B11-A11-1,0)</f>
+        <f aca="false">IF(AND(ISNUMBER(A11),ISNUMBER(B11),B11&gt;A11),MAX(0,MIN(B11-1,DATE(2026,12,31))-MAX(A11+1,DATE(2026,1,1))+1),0)</f>
         <v>0</v>
       </c>
       <c r="E11" s="27" t="n">
-        <f aca="false">IF(AND(ISNUMBER(A11),ISNUMBER(B11),B11&gt;A11),2,0)</f>
+        <f aca="false">IF(AND(ISNUMBER(A11),ISNUMBER(B11),B11&gt;A11),AND(A11&gt;=DATE(2026,1,1),A11&lt;=DATE(2026,12,31))*1+AND(B11&gt;=DATE(2026,1,1),B11&lt;=DATE(2026,12,31))*1,0)</f>
         <v>0</v>
       </c>
       <c r="F11" s="25" t="n">
@@ -4053,11 +4053,11 @@
       <c r="B12" s="26"/>
       <c r="C12" s="12"/>
       <c r="D12" s="27" t="n">
-        <f aca="false">IF(AND(ISNUMBER(A12),ISNUMBER(B12),B12&gt;A12),B12-A12-1,0)</f>
+        <f aca="false">IF(AND(ISNUMBER(A12),ISNUMBER(B12),B12&gt;A12),MAX(0,MIN(B12-1,DATE(2026,12,31))-MAX(A12+1,DATE(2026,1,1))+1),0)</f>
         <v>0</v>
       </c>
       <c r="E12" s="27" t="n">
-        <f aca="false">IF(AND(ISNUMBER(A12),ISNUMBER(B12),B12&gt;A12),2,0)</f>
+        <f aca="false">IF(AND(ISNUMBER(A12),ISNUMBER(B12),B12&gt;A12),AND(A12&gt;=DATE(2026,1,1),A12&lt;=DATE(2026,12,31))*1+AND(B12&gt;=DATE(2026,1,1),B12&lt;=DATE(2026,12,31))*1,0)</f>
         <v>0</v>
       </c>
       <c r="F12" s="25" t="n">
@@ -4070,11 +4070,11 @@
       <c r="B13" s="26"/>
       <c r="C13" s="12"/>
       <c r="D13" s="27" t="n">
-        <f aca="false">IF(AND(ISNUMBER(A13),ISNUMBER(B13),B13&gt;A13),B13-A13-1,0)</f>
+        <f aca="false">IF(AND(ISNUMBER(A13),ISNUMBER(B13),B13&gt;A13),MAX(0,MIN(B13-1,DATE(2026,12,31))-MAX(A13+1,DATE(2026,1,1))+1),0)</f>
         <v>0</v>
       </c>
       <c r="E13" s="27" t="n">
-        <f aca="false">IF(AND(ISNUMBER(A13),ISNUMBER(B13),B13&gt;A13),2,0)</f>
+        <f aca="false">IF(AND(ISNUMBER(A13),ISNUMBER(B13),B13&gt;A13),AND(A13&gt;=DATE(2026,1,1),A13&lt;=DATE(2026,12,31))*1+AND(B13&gt;=DATE(2026,1,1),B13&lt;=DATE(2026,12,31))*1,0)</f>
         <v>0</v>
       </c>
       <c r="F13" s="25" t="n">
@@ -4087,11 +4087,11 @@
       <c r="B14" s="26"/>
       <c r="C14" s="12"/>
       <c r="D14" s="27" t="n">
-        <f aca="false">IF(AND(ISNUMBER(A14),ISNUMBER(B14),B14&gt;A14),B14-A14-1,0)</f>
+        <f aca="false">IF(AND(ISNUMBER(A14),ISNUMBER(B14),B14&gt;A14),MAX(0,MIN(B14-1,DATE(2026,12,31))-MAX(A14+1,DATE(2026,1,1))+1),0)</f>
         <v>0</v>
       </c>
       <c r="E14" s="27" t="n">
-        <f aca="false">IF(AND(ISNUMBER(A14),ISNUMBER(B14),B14&gt;A14),2,0)</f>
+        <f aca="false">IF(AND(ISNUMBER(A14),ISNUMBER(B14),B14&gt;A14),AND(A14&gt;=DATE(2026,1,1),A14&lt;=DATE(2026,12,31))*1+AND(B14&gt;=DATE(2026,1,1),B14&lt;=DATE(2026,12,31))*1,0)</f>
         <v>0</v>
       </c>
       <c r="F14" s="25" t="n">
@@ -4104,11 +4104,11 @@
       <c r="B15" s="26"/>
       <c r="C15" s="12"/>
       <c r="D15" s="27" t="n">
-        <f aca="false">IF(AND(ISNUMBER(A15),ISNUMBER(B15),B15&gt;A15),B15-A15-1,0)</f>
+        <f aca="false">IF(AND(ISNUMBER(A15),ISNUMBER(B15),B15&gt;A15),MAX(0,MIN(B15-1,DATE(2026,12,31))-MAX(A15+1,DATE(2026,1,1))+1),0)</f>
         <v>0</v>
       </c>
       <c r="E15" s="27" t="n">
-        <f aca="false">IF(AND(ISNUMBER(A15),ISNUMBER(B15),B15&gt;A15),2,0)</f>
+        <f aca="false">IF(AND(ISNUMBER(A15),ISNUMBER(B15),B15&gt;A15),AND(A15&gt;=DATE(2026,1,1),A15&lt;=DATE(2026,12,31))*1+AND(B15&gt;=DATE(2026,1,1),B15&lt;=DATE(2026,12,31))*1,0)</f>
         <v>0</v>
       </c>
       <c r="F15" s="25" t="n">
@@ -4121,11 +4121,11 @@
       <c r="B16" s="26"/>
       <c r="C16" s="12"/>
       <c r="D16" s="27" t="n">
-        <f aca="false">IF(AND(ISNUMBER(A16),ISNUMBER(B16),B16&gt;A16),B16-A16-1,0)</f>
+        <f aca="false">IF(AND(ISNUMBER(A16),ISNUMBER(B16),B16&gt;A16),MAX(0,MIN(B16-1,DATE(2026,12,31))-MAX(A16+1,DATE(2026,1,1))+1),0)</f>
         <v>0</v>
       </c>
       <c r="E16" s="27" t="n">
-        <f aca="false">IF(AND(ISNUMBER(A16),ISNUMBER(B16),B16&gt;A16),2,0)</f>
+        <f aca="false">IF(AND(ISNUMBER(A16),ISNUMBER(B16),B16&gt;A16),AND(A16&gt;=DATE(2026,1,1),A16&lt;=DATE(2026,12,31))*1+AND(B16&gt;=DATE(2026,1,1),B16&lt;=DATE(2026,12,31))*1,0)</f>
         <v>0</v>
       </c>
       <c r="F16" s="25" t="n">
@@ -4138,11 +4138,11 @@
       <c r="B17" s="26"/>
       <c r="C17" s="12"/>
       <c r="D17" s="27" t="n">
-        <f aca="false">IF(AND(ISNUMBER(A17),ISNUMBER(B17),B17&gt;A17),B17-A17-1,0)</f>
+        <f aca="false">IF(AND(ISNUMBER(A17),ISNUMBER(B17),B17&gt;A17),MAX(0,MIN(B17-1,DATE(2026,12,31))-MAX(A17+1,DATE(2026,1,1))+1),0)</f>
         <v>0</v>
       </c>
       <c r="E17" s="27" t="n">
-        <f aca="false">IF(AND(ISNUMBER(A17),ISNUMBER(B17),B17&gt;A17),2,0)</f>
+        <f aca="false">IF(AND(ISNUMBER(A17),ISNUMBER(B17),B17&gt;A17),AND(A17&gt;=DATE(2026,1,1),A17&lt;=DATE(2026,12,31))*1+AND(B17&gt;=DATE(2026,1,1),B17&lt;=DATE(2026,12,31))*1,0)</f>
         <v>0</v>
       </c>
       <c r="F17" s="25" t="n">
@@ -4155,11 +4155,11 @@
       <c r="B18" s="26"/>
       <c r="C18" s="12"/>
       <c r="D18" s="27" t="n">
-        <f aca="false">IF(AND(ISNUMBER(A18),ISNUMBER(B18),B18&gt;A18),B18-A18-1,0)</f>
+        <f aca="false">IF(AND(ISNUMBER(A18),ISNUMBER(B18),B18&gt;A18),MAX(0,MIN(B18-1,DATE(2026,12,31))-MAX(A18+1,DATE(2026,1,1))+1),0)</f>
         <v>0</v>
       </c>
       <c r="E18" s="27" t="n">
-        <f aca="false">IF(AND(ISNUMBER(A18),ISNUMBER(B18),B18&gt;A18),2,0)</f>
+        <f aca="false">IF(AND(ISNUMBER(A18),ISNUMBER(B18),B18&gt;A18),AND(A18&gt;=DATE(2026,1,1),A18&lt;=DATE(2026,12,31))*1+AND(B18&gt;=DATE(2026,1,1),B18&lt;=DATE(2026,12,31))*1,0)</f>
         <v>0</v>
       </c>
       <c r="F18" s="25" t="n">
@@ -4172,11 +4172,11 @@
       <c r="B19" s="26"/>
       <c r="C19" s="12"/>
       <c r="D19" s="27" t="n">
-        <f aca="false">IF(AND(ISNUMBER(A19),ISNUMBER(B19),B19&gt;A19),B19-A19-1,0)</f>
+        <f aca="false">IF(AND(ISNUMBER(A19),ISNUMBER(B19),B19&gt;A19),MAX(0,MIN(B19-1,DATE(2026,12,31))-MAX(A19+1,DATE(2026,1,1))+1),0)</f>
         <v>0</v>
       </c>
       <c r="E19" s="27" t="n">
-        <f aca="false">IF(AND(ISNUMBER(A19),ISNUMBER(B19),B19&gt;A19),2,0)</f>
+        <f aca="false">IF(AND(ISNUMBER(A19),ISNUMBER(B19),B19&gt;A19),AND(A19&gt;=DATE(2026,1,1),A19&lt;=DATE(2026,12,31))*1+AND(B19&gt;=DATE(2026,1,1),B19&lt;=DATE(2026,12,31))*1,0)</f>
         <v>0</v>
       </c>
       <c r="F19" s="25" t="n">
@@ -4189,11 +4189,11 @@
       <c r="B20" s="26"/>
       <c r="C20" s="12"/>
       <c r="D20" s="27" t="n">
-        <f aca="false">IF(AND(ISNUMBER(A20),ISNUMBER(B20),B20&gt;A20),B20-A20-1,0)</f>
+        <f aca="false">IF(AND(ISNUMBER(A20),ISNUMBER(B20),B20&gt;A20),MAX(0,MIN(B20-1,DATE(2026,12,31))-MAX(A20+1,DATE(2026,1,1))+1),0)</f>
         <v>0</v>
       </c>
       <c r="E20" s="27" t="n">
-        <f aca="false">IF(AND(ISNUMBER(A20),ISNUMBER(B20),B20&gt;A20),2,0)</f>
+        <f aca="false">IF(AND(ISNUMBER(A20),ISNUMBER(B20),B20&gt;A20),AND(A20&gt;=DATE(2026,1,1),A20&lt;=DATE(2026,12,31))*1+AND(B20&gt;=DATE(2026,1,1),B20&lt;=DATE(2026,12,31))*1,0)</f>
         <v>0</v>
       </c>
       <c r="F20" s="25" t="n">
@@ -4206,11 +4206,11 @@
       <c r="B21" s="26"/>
       <c r="C21" s="12"/>
       <c r="D21" s="27" t="n">
-        <f aca="false">IF(AND(ISNUMBER(A21),ISNUMBER(B21),B21&gt;A21),B21-A21-1,0)</f>
+        <f aca="false">IF(AND(ISNUMBER(A21),ISNUMBER(B21),B21&gt;A21),MAX(0,MIN(B21-1,DATE(2026,12,31))-MAX(A21+1,DATE(2026,1,1))+1),0)</f>
         <v>0</v>
       </c>
       <c r="E21" s="27" t="n">
-        <f aca="false">IF(AND(ISNUMBER(A21),ISNUMBER(B21),B21&gt;A21),2,0)</f>
+        <f aca="false">IF(AND(ISNUMBER(A21),ISNUMBER(B21),B21&gt;A21),AND(A21&gt;=DATE(2026,1,1),A21&lt;=DATE(2026,12,31))*1+AND(B21&gt;=DATE(2026,1,1),B21&lt;=DATE(2026,12,31))*1,0)</f>
         <v>0</v>
       </c>
       <c r="F21" s="25" t="n">
@@ -4223,11 +4223,11 @@
       <c r="B22" s="26"/>
       <c r="C22" s="12"/>
       <c r="D22" s="27" t="n">
-        <f aca="false">IF(AND(ISNUMBER(A22),ISNUMBER(B22),B22&gt;A22),B22-A22-1,0)</f>
+        <f aca="false">IF(AND(ISNUMBER(A22),ISNUMBER(B22),B22&gt;A22),MAX(0,MIN(B22-1,DATE(2026,12,31))-MAX(A22+1,DATE(2026,1,1))+1),0)</f>
         <v>0</v>
       </c>
       <c r="E22" s="27" t="n">
-        <f aca="false">IF(AND(ISNUMBER(A22),ISNUMBER(B22),B22&gt;A22),2,0)</f>
+        <f aca="false">IF(AND(ISNUMBER(A22),ISNUMBER(B22),B22&gt;A22),AND(A22&gt;=DATE(2026,1,1),A22&lt;=DATE(2026,12,31))*1+AND(B22&gt;=DATE(2026,1,1),B22&lt;=DATE(2026,12,31))*1,0)</f>
         <v>0</v>
       </c>
       <c r="F22" s="25" t="n">
@@ -4240,11 +4240,11 @@
       <c r="B23" s="26"/>
       <c r="C23" s="12"/>
       <c r="D23" s="27" t="n">
-        <f aca="false">IF(AND(ISNUMBER(A23),ISNUMBER(B23),B23&gt;A23),B23-A23-1,0)</f>
+        <f aca="false">IF(AND(ISNUMBER(A23),ISNUMBER(B23),B23&gt;A23),MAX(0,MIN(B23-1,DATE(2026,12,31))-MAX(A23+1,DATE(2026,1,1))+1),0)</f>
         <v>0</v>
       </c>
       <c r="E23" s="27" t="n">
-        <f aca="false">IF(AND(ISNUMBER(A23),ISNUMBER(B23),B23&gt;A23),2,0)</f>
+        <f aca="false">IF(AND(ISNUMBER(A23),ISNUMBER(B23),B23&gt;A23),AND(A23&gt;=DATE(2026,1,1),A23&lt;=DATE(2026,12,31))*1+AND(B23&gt;=DATE(2026,1,1),B23&lt;=DATE(2026,12,31))*1,0)</f>
         <v>0</v>
       </c>
       <c r="F23" s="25" t="n">
@@ -4257,11 +4257,11 @@
       <c r="B24" s="26"/>
       <c r="C24" s="12"/>
       <c r="D24" s="27" t="n">
-        <f aca="false">IF(AND(ISNUMBER(A24),ISNUMBER(B24),B24&gt;A24),B24-A24-1,0)</f>
+        <f aca="false">IF(AND(ISNUMBER(A24),ISNUMBER(B24),B24&gt;A24),MAX(0,MIN(B24-1,DATE(2026,12,31))-MAX(A24+1,DATE(2026,1,1))+1),0)</f>
         <v>0</v>
       </c>
       <c r="E24" s="27" t="n">
-        <f aca="false">IF(AND(ISNUMBER(A24),ISNUMBER(B24),B24&gt;A24),2,0)</f>
+        <f aca="false">IF(AND(ISNUMBER(A24),ISNUMBER(B24),B24&gt;A24),AND(A24&gt;=DATE(2026,1,1),A24&lt;=DATE(2026,12,31))*1+AND(B24&gt;=DATE(2026,1,1),B24&lt;=DATE(2026,12,31))*1,0)</f>
         <v>0</v>
       </c>
       <c r="F24" s="25" t="n">
@@ -4274,11 +4274,11 @@
       <c r="B25" s="26"/>
       <c r="C25" s="12"/>
       <c r="D25" s="27" t="n">
-        <f aca="false">IF(AND(ISNUMBER(A25),ISNUMBER(B25),B25&gt;A25),B25-A25-1,0)</f>
+        <f aca="false">IF(AND(ISNUMBER(A25),ISNUMBER(B25),B25&gt;A25),MAX(0,MIN(B25-1,DATE(2026,12,31))-MAX(A25+1,DATE(2026,1,1))+1),0)</f>
         <v>0</v>
       </c>
       <c r="E25" s="27" t="n">
-        <f aca="false">IF(AND(ISNUMBER(A25),ISNUMBER(B25),B25&gt;A25),2,0)</f>
+        <f aca="false">IF(AND(ISNUMBER(A25),ISNUMBER(B25),B25&gt;A25),AND(A25&gt;=DATE(2026,1,1),A25&lt;=DATE(2026,12,31))*1+AND(B25&gt;=DATE(2026,1,1),B25&lt;=DATE(2026,12,31))*1,0)</f>
         <v>0</v>
       </c>
       <c r="F25" s="25" t="n">
@@ -4291,11 +4291,11 @@
       <c r="B26" s="26"/>
       <c r="C26" s="12"/>
       <c r="D26" s="27" t="n">
-        <f aca="false">IF(AND(ISNUMBER(A26),ISNUMBER(B26),B26&gt;A26),B26-A26-1,0)</f>
+        <f aca="false">IF(AND(ISNUMBER(A26),ISNUMBER(B26),B26&gt;A26),MAX(0,MIN(B26-1,DATE(2026,12,31))-MAX(A26+1,DATE(2026,1,1))+1),0)</f>
         <v>0</v>
       </c>
       <c r="E26" s="27" t="n">
-        <f aca="false">IF(AND(ISNUMBER(A26),ISNUMBER(B26),B26&gt;A26),2,0)</f>
+        <f aca="false">IF(AND(ISNUMBER(A26),ISNUMBER(B26),B26&gt;A26),AND(A26&gt;=DATE(2026,1,1),A26&lt;=DATE(2026,12,31))*1+AND(B26&gt;=DATE(2026,1,1),B26&lt;=DATE(2026,12,31))*1,0)</f>
         <v>0</v>
       </c>
       <c r="F26" s="25" t="n">
@@ -4308,11 +4308,11 @@
       <c r="B27" s="26"/>
       <c r="C27" s="12"/>
       <c r="D27" s="27" t="n">
-        <f aca="false">IF(AND(ISNUMBER(A27),ISNUMBER(B27),B27&gt;A27),B27-A27-1,0)</f>
+        <f aca="false">IF(AND(ISNUMBER(A27),ISNUMBER(B27),B27&gt;A27),MAX(0,MIN(B27-1,DATE(2026,12,31))-MAX(A27+1,DATE(2026,1,1))+1),0)</f>
         <v>0</v>
       </c>
       <c r="E27" s="27" t="n">
-        <f aca="false">IF(AND(ISNUMBER(A27),ISNUMBER(B27),B27&gt;A27),2,0)</f>
+        <f aca="false">IF(AND(ISNUMBER(A27),ISNUMBER(B27),B27&gt;A27),AND(A27&gt;=DATE(2026,1,1),A27&lt;=DATE(2026,12,31))*1+AND(B27&gt;=DATE(2026,1,1),B27&lt;=DATE(2026,12,31))*1,0)</f>
         <v>0</v>
       </c>
       <c r="F27" s="25" t="n">
@@ -4325,11 +4325,11 @@
       <c r="B28" s="26"/>
       <c r="C28" s="12"/>
       <c r="D28" s="27" t="n">
-        <f aca="false">IF(AND(ISNUMBER(A28),ISNUMBER(B28),B28&gt;A28),B28-A28-1,0)</f>
+        <f aca="false">IF(AND(ISNUMBER(A28),ISNUMBER(B28),B28&gt;A28),MAX(0,MIN(B28-1,DATE(2026,12,31))-MAX(A28+1,DATE(2026,1,1))+1),0)</f>
         <v>0</v>
       </c>
       <c r="E28" s="27" t="n">
-        <f aca="false">IF(AND(ISNUMBER(A28),ISNUMBER(B28),B28&gt;A28),2,0)</f>
+        <f aca="false">IF(AND(ISNUMBER(A28),ISNUMBER(B28),B28&gt;A28),AND(A28&gt;=DATE(2026,1,1),A28&lt;=DATE(2026,12,31))*1+AND(B28&gt;=DATE(2026,1,1),B28&lt;=DATE(2026,12,31))*1,0)</f>
         <v>0</v>
       </c>
       <c r="F28" s="25" t="n">
@@ -4342,11 +4342,11 @@
       <c r="B29" s="26"/>
       <c r="C29" s="12"/>
       <c r="D29" s="27" t="n">
-        <f aca="false">IF(AND(ISNUMBER(A29),ISNUMBER(B29),B29&gt;A29),B29-A29-1,0)</f>
+        <f aca="false">IF(AND(ISNUMBER(A29),ISNUMBER(B29),B29&gt;A29),MAX(0,MIN(B29-1,DATE(2026,12,31))-MAX(A29+1,DATE(2026,1,1))+1),0)</f>
         <v>0</v>
       </c>
       <c r="E29" s="27" t="n">
-        <f aca="false">IF(AND(ISNUMBER(A29),ISNUMBER(B29),B29&gt;A29),2,0)</f>
+        <f aca="false">IF(AND(ISNUMBER(A29),ISNUMBER(B29),B29&gt;A29),AND(A29&gt;=DATE(2026,1,1),A29&lt;=DATE(2026,12,31))*1+AND(B29&gt;=DATE(2026,1,1),B29&lt;=DATE(2026,12,31))*1,0)</f>
         <v>0</v>
       </c>
       <c r="F29" s="25" t="n">
@@ -4359,11 +4359,11 @@
       <c r="B30" s="26"/>
       <c r="C30" s="12"/>
       <c r="D30" s="27" t="n">
-        <f aca="false">IF(AND(ISNUMBER(A30),ISNUMBER(B30),B30&gt;A30),B30-A30-1,0)</f>
+        <f aca="false">IF(AND(ISNUMBER(A30),ISNUMBER(B30),B30&gt;A30),MAX(0,MIN(B30-1,DATE(2026,12,31))-MAX(A30+1,DATE(2026,1,1))+1),0)</f>
         <v>0</v>
       </c>
       <c r="E30" s="27" t="n">
-        <f aca="false">IF(AND(ISNUMBER(A30),ISNUMBER(B30),B30&gt;A30),2,0)</f>
+        <f aca="false">IF(AND(ISNUMBER(A30),ISNUMBER(B30),B30&gt;A30),AND(A30&gt;=DATE(2026,1,1),A30&lt;=DATE(2026,12,31))*1+AND(B30&gt;=DATE(2026,1,1),B30&lt;=DATE(2026,12,31))*1,0)</f>
         <v>0</v>
       </c>
       <c r="F30" s="25" t="n">
@@ -4376,11 +4376,11 @@
       <c r="B31" s="26"/>
       <c r="C31" s="12"/>
       <c r="D31" s="27" t="n">
-        <f aca="false">IF(AND(ISNUMBER(A31),ISNUMBER(B31),B31&gt;A31),B31-A31-1,0)</f>
+        <f aca="false">IF(AND(ISNUMBER(A31),ISNUMBER(B31),B31&gt;A31),MAX(0,MIN(B31-1,DATE(2026,12,31))-MAX(A31+1,DATE(2026,1,1))+1),0)</f>
         <v>0</v>
       </c>
       <c r="E31" s="27" t="n">
-        <f aca="false">IF(AND(ISNUMBER(A31),ISNUMBER(B31),B31&gt;A31),2,0)</f>
+        <f aca="false">IF(AND(ISNUMBER(A31),ISNUMBER(B31),B31&gt;A31),AND(A31&gt;=DATE(2026,1,1),A31&lt;=DATE(2026,12,31))*1+AND(B31&gt;=DATE(2026,1,1),B31&lt;=DATE(2026,12,31))*1,0)</f>
         <v>0</v>
       </c>
       <c r="F31" s="25" t="n">
@@ -4393,11 +4393,11 @@
       <c r="B32" s="26"/>
       <c r="C32" s="12"/>
       <c r="D32" s="27" t="n">
-        <f aca="false">IF(AND(ISNUMBER(A32),ISNUMBER(B32),B32&gt;A32),B32-A32-1,0)</f>
+        <f aca="false">IF(AND(ISNUMBER(A32),ISNUMBER(B32),B32&gt;A32),MAX(0,MIN(B32-1,DATE(2026,12,31))-MAX(A32+1,DATE(2026,1,1))+1),0)</f>
         <v>0</v>
       </c>
       <c r="E32" s="27" t="n">
-        <f aca="false">IF(AND(ISNUMBER(A32),ISNUMBER(B32),B32&gt;A32),2,0)</f>
+        <f aca="false">IF(AND(ISNUMBER(A32),ISNUMBER(B32),B32&gt;A32),AND(A32&gt;=DATE(2026,1,1),A32&lt;=DATE(2026,12,31))*1+AND(B32&gt;=DATE(2026,1,1),B32&lt;=DATE(2026,12,31))*1,0)</f>
         <v>0</v>
       </c>
       <c r="F32" s="25" t="n">
@@ -4410,11 +4410,11 @@
       <c r="B33" s="26"/>
       <c r="C33" s="12"/>
       <c r="D33" s="27" t="n">
-        <f aca="false">IF(AND(ISNUMBER(A33),ISNUMBER(B33),B33&gt;A33),B33-A33-1,0)</f>
+        <f aca="false">IF(AND(ISNUMBER(A33),ISNUMBER(B33),B33&gt;A33),MAX(0,MIN(B33-1,DATE(2026,12,31))-MAX(A33+1,DATE(2026,1,1))+1),0)</f>
         <v>0</v>
       </c>
       <c r="E33" s="27" t="n">
-        <f aca="false">IF(AND(ISNUMBER(A33),ISNUMBER(B33),B33&gt;A33),2,0)</f>
+        <f aca="false">IF(AND(ISNUMBER(A33),ISNUMBER(B33),B33&gt;A33),AND(A33&gt;=DATE(2026,1,1),A33&lt;=DATE(2026,12,31))*1+AND(B33&gt;=DATE(2026,1,1),B33&lt;=DATE(2026,12,31))*1,0)</f>
         <v>0</v>
       </c>
       <c r="F33" s="25" t="n">
@@ -4427,11 +4427,11 @@
       <c r="B34" s="26"/>
       <c r="C34" s="12"/>
       <c r="D34" s="27" t="n">
-        <f aca="false">IF(AND(ISNUMBER(A34),ISNUMBER(B34),B34&gt;A34),B34-A34-1,0)</f>
+        <f aca="false">IF(AND(ISNUMBER(A34),ISNUMBER(B34),B34&gt;A34),MAX(0,MIN(B34-1,DATE(2026,12,31))-MAX(A34+1,DATE(2026,1,1))+1),0)</f>
         <v>0</v>
       </c>
       <c r="E34" s="27" t="n">
-        <f aca="false">IF(AND(ISNUMBER(A34),ISNUMBER(B34),B34&gt;A34),2,0)</f>
+        <f aca="false">IF(AND(ISNUMBER(A34),ISNUMBER(B34),B34&gt;A34),AND(A34&gt;=DATE(2026,1,1),A34&lt;=DATE(2026,12,31))*1+AND(B34&gt;=DATE(2026,1,1),B34&lt;=DATE(2026,12,31))*1,0)</f>
         <v>0</v>
       </c>
       <c r="F34" s="25" t="n">
@@ -4444,11 +4444,11 @@
       <c r="B35" s="26"/>
       <c r="C35" s="12"/>
       <c r="D35" s="27" t="n">
-        <f aca="false">IF(AND(ISNUMBER(A35),ISNUMBER(B35),B35&gt;A35),B35-A35-1,0)</f>
+        <f aca="false">IF(AND(ISNUMBER(A35),ISNUMBER(B35),B35&gt;A35),MAX(0,MIN(B35-1,DATE(2026,12,31))-MAX(A35+1,DATE(2026,1,1))+1),0)</f>
         <v>0</v>
       </c>
       <c r="E35" s="27" t="n">
-        <f aca="false">IF(AND(ISNUMBER(A35),ISNUMBER(B35),B35&gt;A35),2,0)</f>
+        <f aca="false">IF(AND(ISNUMBER(A35),ISNUMBER(B35),B35&gt;A35),AND(A35&gt;=DATE(2026,1,1),A35&lt;=DATE(2026,12,31))*1+AND(B35&gt;=DATE(2026,1,1),B35&lt;=DATE(2026,12,31))*1,0)</f>
         <v>0</v>
       </c>
       <c r="F35" s="25" t="n">
@@ -5147,7 +5147,7 @@
         <v>310</v>
       </c>
       <c r="C23" s="6" t="n">
-        <f aca="false">ROUND(Trips!D36-Trips!C36+Trips!C36*C41/C40,2)</f>
+        <f aca="false">ROUND(MIN(365,Trips!D36+SUMPRODUCT((Trips!C6:C35&lt;Trips!D6:D35)*Trips!C6:C35+(Trips!C6:C35&gt;=Trips!D6:D35)*Trips!D6:D35)*(C41/C40-1)),2)</f>
         <v>0</v>
       </c>
       <c r="H23" s="30" t="s">

</xml_diff>

<commit_message>
Carry Canada per diem days separately; same trip counts for Excel and PDF
- Engine takes perDiemCanada ($86) so the 365-day cap keeps the Canada rate
- Estimator: Canada days field; organizer uploads no longer leave
  fractional days that block Edit my answers
- Excel upload counts trips from the Trips tab with the PDF logic
  (2026 only, overlaps merged); Trips tab flags overlapping rows

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012ebqUPkXNMCm1mSUdBK3xi
</commit_message>
<xml_diff>
--- a/tax-prep/downloads/falcon-tax-organizer-2026.xlsx
+++ b/tax-prep/downloads/falcon-tax-organizer-2026.xlsx
@@ -50,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="459" uniqueCount="391">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="462" uniqueCount="394">
   <si>
     <t xml:space="preserve">Falcon Tax Solutions · 2026 Tax Organizer</t>
   </si>
@@ -625,6 +625,9 @@
     <t xml:space="preserve">Per diem</t>
   </si>
   <si>
+    <t xml:space="preserve">Check</t>
+  </si>
+  <si>
     <t xml:space="preserve">2026-03-02</t>
   </si>
   <si>
@@ -982,7 +985,7 @@
     <t xml:space="preserve">perDiemFull</t>
   </si>
   <si>
-    <t xml:space="preserve">Full days away (Canada days converted to $80 days)</t>
+    <t xml:space="preserve">Full days away (U.S. and Canada)</t>
   </si>
   <si>
     <t xml:space="preserve">Massachusetts</t>
@@ -991,22 +994,34 @@
     <t xml:space="preserve">MA</t>
   </si>
   <si>
+    <t xml:space="preserve">perDiemCanada</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Of those, full days in Canada</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Michigan</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MI</t>
+  </si>
+  <si>
     <t xml:space="preserve">perDiemPartial</t>
   </si>
   <si>
-    <t xml:space="preserve">Michigan</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MI</t>
+    <t xml:space="preserve">Minnesota</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MN</t>
   </si>
   <si>
     <t xml:space="preserve">interest</t>
   </si>
   <si>
-    <t xml:space="preserve">Minnesota</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MN</t>
+    <t xml:space="preserve">Mississippi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MS</t>
   </si>
   <si>
     <t xml:space="preserve">unemployment</t>
@@ -1015,10 +1030,10 @@
     <t xml:space="preserve">Unemployment</t>
   </si>
   <si>
-    <t xml:space="preserve">Mississippi</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MS</t>
+    <t xml:space="preserve">Missouri</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MO</t>
   </si>
   <si>
     <t xml:space="preserve">otherIncome</t>
@@ -1027,10 +1042,10 @@
     <t xml:space="preserve">Retirement withdrawals and other income</t>
   </si>
   <si>
-    <t xml:space="preserve">Missouri</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MO</t>
+    <t xml:space="preserve">Montana</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MT</t>
   </si>
   <si>
     <t xml:space="preserve">retirement</t>
@@ -1039,73 +1054,67 @@
     <t xml:space="preserve">Has retirement withdrawals</t>
   </si>
   <si>
-    <t xml:space="preserve">Montana</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MT</t>
+    <t xml:space="preserve">Nebraska</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NE</t>
   </si>
   <si>
     <t xml:space="preserve">hasInvestments</t>
   </si>
   <si>
-    <t xml:space="preserve">Nebraska</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NE</t>
+    <t xml:space="preserve">Nevada</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NV</t>
   </si>
   <si>
     <t xml:space="preserve">mortgage</t>
   </si>
   <si>
-    <t xml:space="preserve">Nevada</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NV</t>
+    <t xml:space="preserve">New Hampshire</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NH</t>
   </si>
   <si>
     <t xml:space="preserve">studentLoan</t>
   </si>
   <si>
-    <t xml:space="preserve">New Hampshire</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NH</t>
+    <t xml:space="preserve">New Jersey</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NJ</t>
   </si>
   <si>
     <t xml:space="preserve">college</t>
   </si>
   <si>
-    <t xml:space="preserve">New Jersey</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NJ</t>
+    <t xml:space="preserve">New Mexico</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NM</t>
   </si>
   <si>
     <t xml:space="preserve">marketplace</t>
   </si>
   <si>
-    <t xml:space="preserve">New Mexico</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NM</t>
+    <t xml:space="preserve">New York</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NY</t>
   </si>
   <si>
     <t xml:space="preserve">noSsn</t>
   </si>
   <si>
-    <t xml:space="preserve">New York</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NY</t>
+    <t xml:space="preserve">North Carolina</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NC</t>
   </si>
   <si>
     <t xml:space="preserve">irsLetter</t>
-  </si>
-  <si>
-    <t xml:space="preserve">North Carolina</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NC</t>
   </si>
   <si>
     <t xml:space="preserve">North Dakota</t>
@@ -1236,7 +1245,7 @@
     <numFmt numFmtId="167" formatCode="0%"/>
     <numFmt numFmtId="168" formatCode="yyyy\-mm\-dd"/>
   </numFmts>
-  <fonts count="18">
+  <fonts count="19">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1352,6 +1361,14 @@
     <font>
       <b val="true"/>
       <sz val="10"/>
+      <color rgb="FFA3472B"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="10"/>
       <color rgb="FF1D3557"/>
       <name val="Arial"/>
       <family val="0"/>
@@ -1444,7 +1461,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="38">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1557,6 +1574,10 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="165" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1581,7 +1602,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1656,7 +1677,7 @@
       <rgbColor rgb="FF339966"/>
       <rgbColor rgb="FF003300"/>
       <rgbColor rgb="FF333300"/>
-      <rgbColor rgb="FF993300"/>
+      <rgbColor rgb="FFA3472B"/>
       <rgbColor rgb="FF993366"/>
       <rgbColor rgb="FF333399"/>
       <rgbColor rgb="FF1B2230"/>
@@ -3889,11 +3910,12 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:F41"/>
+  <dimension ref="A1:G41"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="1" style="0" width="18"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="3" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="24"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3925,13 +3947,16 @@
       <c r="F4" s="14" t="s">
         <v>190</v>
       </c>
+      <c r="G4" s="14" t="s">
+        <v>191</v>
+      </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="15" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="B5" s="15" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="C5" s="15" t="n">
         <v>0</v>
@@ -3962,6 +3987,10 @@
         <f aca="false">(D6-MIN(C6,D6))*Data!$C$40+MIN(C6,D6)*Data!$C$41+E6*Data!$C$40*Data!$C$42</f>
         <v>0</v>
       </c>
+      <c r="G6" s="28" t="str">
+        <f aca="false">IF(AND(AND(ISNUMBER(A6),ISNUMBER(B6),B6&gt;A6),SUMPRODUCT(ISNUMBER($A$6:$A$35)*ISNUMBER($B$6:$B$35)*($A$6:$A$35&lt;B6)*($B$6:$B$35&gt;A6))&gt;1),"Overlaps another trip","")</f>
+        <v/>
+      </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="26"/>
@@ -3979,6 +4008,10 @@
         <f aca="false">(D7-MIN(C7,D7))*Data!$C$40+MIN(C7,D7)*Data!$C$41+E7*Data!$C$40*Data!$C$42</f>
         <v>0</v>
       </c>
+      <c r="G7" s="28" t="str">
+        <f aca="false">IF(AND(AND(ISNUMBER(A7),ISNUMBER(B7),B7&gt;A7),SUMPRODUCT(ISNUMBER($A$6:$A$35)*ISNUMBER($B$6:$B$35)*($A$6:$A$35&lt;B7)*($B$6:$B$35&gt;A7))&gt;1),"Overlaps another trip","")</f>
+        <v/>
+      </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="26"/>
@@ -3996,6 +4029,10 @@
         <f aca="false">(D8-MIN(C8,D8))*Data!$C$40+MIN(C8,D8)*Data!$C$41+E8*Data!$C$40*Data!$C$42</f>
         <v>0</v>
       </c>
+      <c r="G8" s="28" t="str">
+        <f aca="false">IF(AND(AND(ISNUMBER(A8),ISNUMBER(B8),B8&gt;A8),SUMPRODUCT(ISNUMBER($A$6:$A$35)*ISNUMBER($B$6:$B$35)*($A$6:$A$35&lt;B8)*($B$6:$B$35&gt;A8))&gt;1),"Overlaps another trip","")</f>
+        <v/>
+      </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="26"/>
@@ -4013,6 +4050,10 @@
         <f aca="false">(D9-MIN(C9,D9))*Data!$C$40+MIN(C9,D9)*Data!$C$41+E9*Data!$C$40*Data!$C$42</f>
         <v>0</v>
       </c>
+      <c r="G9" s="28" t="str">
+        <f aca="false">IF(AND(AND(ISNUMBER(A9),ISNUMBER(B9),B9&gt;A9),SUMPRODUCT(ISNUMBER($A$6:$A$35)*ISNUMBER($B$6:$B$35)*($A$6:$A$35&lt;B9)*($B$6:$B$35&gt;A9))&gt;1),"Overlaps another trip","")</f>
+        <v/>
+      </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="26"/>
@@ -4030,6 +4071,10 @@
         <f aca="false">(D10-MIN(C10,D10))*Data!$C$40+MIN(C10,D10)*Data!$C$41+E10*Data!$C$40*Data!$C$42</f>
         <v>0</v>
       </c>
+      <c r="G10" s="28" t="str">
+        <f aca="false">IF(AND(AND(ISNUMBER(A10),ISNUMBER(B10),B10&gt;A10),SUMPRODUCT(ISNUMBER($A$6:$A$35)*ISNUMBER($B$6:$B$35)*($A$6:$A$35&lt;B10)*($B$6:$B$35&gt;A10))&gt;1),"Overlaps another trip","")</f>
+        <v/>
+      </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="26"/>
@@ -4047,6 +4092,10 @@
         <f aca="false">(D11-MIN(C11,D11))*Data!$C$40+MIN(C11,D11)*Data!$C$41+E11*Data!$C$40*Data!$C$42</f>
         <v>0</v>
       </c>
+      <c r="G11" s="28" t="str">
+        <f aca="false">IF(AND(AND(ISNUMBER(A11),ISNUMBER(B11),B11&gt;A11),SUMPRODUCT(ISNUMBER($A$6:$A$35)*ISNUMBER($B$6:$B$35)*($A$6:$A$35&lt;B11)*($B$6:$B$35&gt;A11))&gt;1),"Overlaps another trip","")</f>
+        <v/>
+      </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="26"/>
@@ -4064,6 +4113,10 @@
         <f aca="false">(D12-MIN(C12,D12))*Data!$C$40+MIN(C12,D12)*Data!$C$41+E12*Data!$C$40*Data!$C$42</f>
         <v>0</v>
       </c>
+      <c r="G12" s="28" t="str">
+        <f aca="false">IF(AND(AND(ISNUMBER(A12),ISNUMBER(B12),B12&gt;A12),SUMPRODUCT(ISNUMBER($A$6:$A$35)*ISNUMBER($B$6:$B$35)*($A$6:$A$35&lt;B12)*($B$6:$B$35&gt;A12))&gt;1),"Overlaps another trip","")</f>
+        <v/>
+      </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="26"/>
@@ -4081,6 +4134,10 @@
         <f aca="false">(D13-MIN(C13,D13))*Data!$C$40+MIN(C13,D13)*Data!$C$41+E13*Data!$C$40*Data!$C$42</f>
         <v>0</v>
       </c>
+      <c r="G13" s="28" t="str">
+        <f aca="false">IF(AND(AND(ISNUMBER(A13),ISNUMBER(B13),B13&gt;A13),SUMPRODUCT(ISNUMBER($A$6:$A$35)*ISNUMBER($B$6:$B$35)*($A$6:$A$35&lt;B13)*($B$6:$B$35&gt;A13))&gt;1),"Overlaps another trip","")</f>
+        <v/>
+      </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="26"/>
@@ -4098,6 +4155,10 @@
         <f aca="false">(D14-MIN(C14,D14))*Data!$C$40+MIN(C14,D14)*Data!$C$41+E14*Data!$C$40*Data!$C$42</f>
         <v>0</v>
       </c>
+      <c r="G14" s="28" t="str">
+        <f aca="false">IF(AND(AND(ISNUMBER(A14),ISNUMBER(B14),B14&gt;A14),SUMPRODUCT(ISNUMBER($A$6:$A$35)*ISNUMBER($B$6:$B$35)*($A$6:$A$35&lt;B14)*($B$6:$B$35&gt;A14))&gt;1),"Overlaps another trip","")</f>
+        <v/>
+      </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="26"/>
@@ -4115,6 +4176,10 @@
         <f aca="false">(D15-MIN(C15,D15))*Data!$C$40+MIN(C15,D15)*Data!$C$41+E15*Data!$C$40*Data!$C$42</f>
         <v>0</v>
       </c>
+      <c r="G15" s="28" t="str">
+        <f aca="false">IF(AND(AND(ISNUMBER(A15),ISNUMBER(B15),B15&gt;A15),SUMPRODUCT(ISNUMBER($A$6:$A$35)*ISNUMBER($B$6:$B$35)*($A$6:$A$35&lt;B15)*($B$6:$B$35&gt;A15))&gt;1),"Overlaps another trip","")</f>
+        <v/>
+      </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="26"/>
@@ -4132,6 +4197,10 @@
         <f aca="false">(D16-MIN(C16,D16))*Data!$C$40+MIN(C16,D16)*Data!$C$41+E16*Data!$C$40*Data!$C$42</f>
         <v>0</v>
       </c>
+      <c r="G16" s="28" t="str">
+        <f aca="false">IF(AND(AND(ISNUMBER(A16),ISNUMBER(B16),B16&gt;A16),SUMPRODUCT(ISNUMBER($A$6:$A$35)*ISNUMBER($B$6:$B$35)*($A$6:$A$35&lt;B16)*($B$6:$B$35&gt;A16))&gt;1),"Overlaps another trip","")</f>
+        <v/>
+      </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="26"/>
@@ -4149,6 +4218,10 @@
         <f aca="false">(D17-MIN(C17,D17))*Data!$C$40+MIN(C17,D17)*Data!$C$41+E17*Data!$C$40*Data!$C$42</f>
         <v>0</v>
       </c>
+      <c r="G17" s="28" t="str">
+        <f aca="false">IF(AND(AND(ISNUMBER(A17),ISNUMBER(B17),B17&gt;A17),SUMPRODUCT(ISNUMBER($A$6:$A$35)*ISNUMBER($B$6:$B$35)*($A$6:$A$35&lt;B17)*($B$6:$B$35&gt;A17))&gt;1),"Overlaps another trip","")</f>
+        <v/>
+      </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="26"/>
@@ -4166,6 +4239,10 @@
         <f aca="false">(D18-MIN(C18,D18))*Data!$C$40+MIN(C18,D18)*Data!$C$41+E18*Data!$C$40*Data!$C$42</f>
         <v>0</v>
       </c>
+      <c r="G18" s="28" t="str">
+        <f aca="false">IF(AND(AND(ISNUMBER(A18),ISNUMBER(B18),B18&gt;A18),SUMPRODUCT(ISNUMBER($A$6:$A$35)*ISNUMBER($B$6:$B$35)*($A$6:$A$35&lt;B18)*($B$6:$B$35&gt;A18))&gt;1),"Overlaps another trip","")</f>
+        <v/>
+      </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="26"/>
@@ -4183,6 +4260,10 @@
         <f aca="false">(D19-MIN(C19,D19))*Data!$C$40+MIN(C19,D19)*Data!$C$41+E19*Data!$C$40*Data!$C$42</f>
         <v>0</v>
       </c>
+      <c r="G19" s="28" t="str">
+        <f aca="false">IF(AND(AND(ISNUMBER(A19),ISNUMBER(B19),B19&gt;A19),SUMPRODUCT(ISNUMBER($A$6:$A$35)*ISNUMBER($B$6:$B$35)*($A$6:$A$35&lt;B19)*($B$6:$B$35&gt;A19))&gt;1),"Overlaps another trip","")</f>
+        <v/>
+      </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="26"/>
@@ -4200,6 +4281,10 @@
         <f aca="false">(D20-MIN(C20,D20))*Data!$C$40+MIN(C20,D20)*Data!$C$41+E20*Data!$C$40*Data!$C$42</f>
         <v>0</v>
       </c>
+      <c r="G20" s="28" t="str">
+        <f aca="false">IF(AND(AND(ISNUMBER(A20),ISNUMBER(B20),B20&gt;A20),SUMPRODUCT(ISNUMBER($A$6:$A$35)*ISNUMBER($B$6:$B$35)*($A$6:$A$35&lt;B20)*($B$6:$B$35&gt;A20))&gt;1),"Overlaps another trip","")</f>
+        <v/>
+      </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="26"/>
@@ -4217,6 +4302,10 @@
         <f aca="false">(D21-MIN(C21,D21))*Data!$C$40+MIN(C21,D21)*Data!$C$41+E21*Data!$C$40*Data!$C$42</f>
         <v>0</v>
       </c>
+      <c r="G21" s="28" t="str">
+        <f aca="false">IF(AND(AND(ISNUMBER(A21),ISNUMBER(B21),B21&gt;A21),SUMPRODUCT(ISNUMBER($A$6:$A$35)*ISNUMBER($B$6:$B$35)*($A$6:$A$35&lt;B21)*($B$6:$B$35&gt;A21))&gt;1),"Overlaps another trip","")</f>
+        <v/>
+      </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="26"/>
@@ -4234,6 +4323,10 @@
         <f aca="false">(D22-MIN(C22,D22))*Data!$C$40+MIN(C22,D22)*Data!$C$41+E22*Data!$C$40*Data!$C$42</f>
         <v>0</v>
       </c>
+      <c r="G22" s="28" t="str">
+        <f aca="false">IF(AND(AND(ISNUMBER(A22),ISNUMBER(B22),B22&gt;A22),SUMPRODUCT(ISNUMBER($A$6:$A$35)*ISNUMBER($B$6:$B$35)*($A$6:$A$35&lt;B22)*($B$6:$B$35&gt;A22))&gt;1),"Overlaps another trip","")</f>
+        <v/>
+      </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="26"/>
@@ -4251,6 +4344,10 @@
         <f aca="false">(D23-MIN(C23,D23))*Data!$C$40+MIN(C23,D23)*Data!$C$41+E23*Data!$C$40*Data!$C$42</f>
         <v>0</v>
       </c>
+      <c r="G23" s="28" t="str">
+        <f aca="false">IF(AND(AND(ISNUMBER(A23),ISNUMBER(B23),B23&gt;A23),SUMPRODUCT(ISNUMBER($A$6:$A$35)*ISNUMBER($B$6:$B$35)*($A$6:$A$35&lt;B23)*($B$6:$B$35&gt;A23))&gt;1),"Overlaps another trip","")</f>
+        <v/>
+      </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="26"/>
@@ -4268,6 +4365,10 @@
         <f aca="false">(D24-MIN(C24,D24))*Data!$C$40+MIN(C24,D24)*Data!$C$41+E24*Data!$C$40*Data!$C$42</f>
         <v>0</v>
       </c>
+      <c r="G24" s="28" t="str">
+        <f aca="false">IF(AND(AND(ISNUMBER(A24),ISNUMBER(B24),B24&gt;A24),SUMPRODUCT(ISNUMBER($A$6:$A$35)*ISNUMBER($B$6:$B$35)*($A$6:$A$35&lt;B24)*($B$6:$B$35&gt;A24))&gt;1),"Overlaps another trip","")</f>
+        <v/>
+      </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="26"/>
@@ -4285,6 +4386,10 @@
         <f aca="false">(D25-MIN(C25,D25))*Data!$C$40+MIN(C25,D25)*Data!$C$41+E25*Data!$C$40*Data!$C$42</f>
         <v>0</v>
       </c>
+      <c r="G25" s="28" t="str">
+        <f aca="false">IF(AND(AND(ISNUMBER(A25),ISNUMBER(B25),B25&gt;A25),SUMPRODUCT(ISNUMBER($A$6:$A$35)*ISNUMBER($B$6:$B$35)*($A$6:$A$35&lt;B25)*($B$6:$B$35&gt;A25))&gt;1),"Overlaps another trip","")</f>
+        <v/>
+      </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="26"/>
@@ -4302,6 +4407,10 @@
         <f aca="false">(D26-MIN(C26,D26))*Data!$C$40+MIN(C26,D26)*Data!$C$41+E26*Data!$C$40*Data!$C$42</f>
         <v>0</v>
       </c>
+      <c r="G26" s="28" t="str">
+        <f aca="false">IF(AND(AND(ISNUMBER(A26),ISNUMBER(B26),B26&gt;A26),SUMPRODUCT(ISNUMBER($A$6:$A$35)*ISNUMBER($B$6:$B$35)*($A$6:$A$35&lt;B26)*($B$6:$B$35&gt;A26))&gt;1),"Overlaps another trip","")</f>
+        <v/>
+      </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="26"/>
@@ -4319,6 +4428,10 @@
         <f aca="false">(D27-MIN(C27,D27))*Data!$C$40+MIN(C27,D27)*Data!$C$41+E27*Data!$C$40*Data!$C$42</f>
         <v>0</v>
       </c>
+      <c r="G27" s="28" t="str">
+        <f aca="false">IF(AND(AND(ISNUMBER(A27),ISNUMBER(B27),B27&gt;A27),SUMPRODUCT(ISNUMBER($A$6:$A$35)*ISNUMBER($B$6:$B$35)*($A$6:$A$35&lt;B27)*($B$6:$B$35&gt;A27))&gt;1),"Overlaps another trip","")</f>
+        <v/>
+      </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="26"/>
@@ -4336,6 +4449,10 @@
         <f aca="false">(D28-MIN(C28,D28))*Data!$C$40+MIN(C28,D28)*Data!$C$41+E28*Data!$C$40*Data!$C$42</f>
         <v>0</v>
       </c>
+      <c r="G28" s="28" t="str">
+        <f aca="false">IF(AND(AND(ISNUMBER(A28),ISNUMBER(B28),B28&gt;A28),SUMPRODUCT(ISNUMBER($A$6:$A$35)*ISNUMBER($B$6:$B$35)*($A$6:$A$35&lt;B28)*($B$6:$B$35&gt;A28))&gt;1),"Overlaps another trip","")</f>
+        <v/>
+      </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="26"/>
@@ -4353,6 +4470,10 @@
         <f aca="false">(D29-MIN(C29,D29))*Data!$C$40+MIN(C29,D29)*Data!$C$41+E29*Data!$C$40*Data!$C$42</f>
         <v>0</v>
       </c>
+      <c r="G29" s="28" t="str">
+        <f aca="false">IF(AND(AND(ISNUMBER(A29),ISNUMBER(B29),B29&gt;A29),SUMPRODUCT(ISNUMBER($A$6:$A$35)*ISNUMBER($B$6:$B$35)*($A$6:$A$35&lt;B29)*($B$6:$B$35&gt;A29))&gt;1),"Overlaps another trip","")</f>
+        <v/>
+      </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="26"/>
@@ -4370,6 +4491,10 @@
         <f aca="false">(D30-MIN(C30,D30))*Data!$C$40+MIN(C30,D30)*Data!$C$41+E30*Data!$C$40*Data!$C$42</f>
         <v>0</v>
       </c>
+      <c r="G30" s="28" t="str">
+        <f aca="false">IF(AND(AND(ISNUMBER(A30),ISNUMBER(B30),B30&gt;A30),SUMPRODUCT(ISNUMBER($A$6:$A$35)*ISNUMBER($B$6:$B$35)*($A$6:$A$35&lt;B30)*($B$6:$B$35&gt;A30))&gt;1),"Overlaps another trip","")</f>
+        <v/>
+      </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="26"/>
@@ -4387,6 +4512,10 @@
         <f aca="false">(D31-MIN(C31,D31))*Data!$C$40+MIN(C31,D31)*Data!$C$41+E31*Data!$C$40*Data!$C$42</f>
         <v>0</v>
       </c>
+      <c r="G31" s="28" t="str">
+        <f aca="false">IF(AND(AND(ISNUMBER(A31),ISNUMBER(B31),B31&gt;A31),SUMPRODUCT(ISNUMBER($A$6:$A$35)*ISNUMBER($B$6:$B$35)*($A$6:$A$35&lt;B31)*($B$6:$B$35&gt;A31))&gt;1),"Overlaps another trip","")</f>
+        <v/>
+      </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="26"/>
@@ -4404,6 +4533,10 @@
         <f aca="false">(D32-MIN(C32,D32))*Data!$C$40+MIN(C32,D32)*Data!$C$41+E32*Data!$C$40*Data!$C$42</f>
         <v>0</v>
       </c>
+      <c r="G32" s="28" t="str">
+        <f aca="false">IF(AND(AND(ISNUMBER(A32),ISNUMBER(B32),B32&gt;A32),SUMPRODUCT(ISNUMBER($A$6:$A$35)*ISNUMBER($B$6:$B$35)*($A$6:$A$35&lt;B32)*($B$6:$B$35&gt;A32))&gt;1),"Overlaps another trip","")</f>
+        <v/>
+      </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="26"/>
@@ -4421,6 +4554,10 @@
         <f aca="false">(D33-MIN(C33,D33))*Data!$C$40+MIN(C33,D33)*Data!$C$41+E33*Data!$C$40*Data!$C$42</f>
         <v>0</v>
       </c>
+      <c r="G33" s="28" t="str">
+        <f aca="false">IF(AND(AND(ISNUMBER(A33),ISNUMBER(B33),B33&gt;A33),SUMPRODUCT(ISNUMBER($A$6:$A$35)*ISNUMBER($B$6:$B$35)*($A$6:$A$35&lt;B33)*($B$6:$B$35&gt;A33))&gt;1),"Overlaps another trip","")</f>
+        <v/>
+      </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="26"/>
@@ -4438,6 +4575,10 @@
         <f aca="false">(D34-MIN(C34,D34))*Data!$C$40+MIN(C34,D34)*Data!$C$41+E34*Data!$C$40*Data!$C$42</f>
         <v>0</v>
       </c>
+      <c r="G34" s="28" t="str">
+        <f aca="false">IF(AND(AND(ISNUMBER(A34),ISNUMBER(B34),B34&gt;A34),SUMPRODUCT(ISNUMBER($A$6:$A$35)*ISNUMBER($B$6:$B$35)*($A$6:$A$35&lt;B34)*($B$6:$B$35&gt;A34))&gt;1),"Overlaps another trip","")</f>
+        <v/>
+      </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="26"/>
@@ -4455,20 +4596,24 @@
         <f aca="false">(D35-MIN(C35,D35))*Data!$C$40+MIN(C35,D35)*Data!$C$41+E35*Data!$C$40*Data!$C$42</f>
         <v>0</v>
       </c>
+      <c r="G35" s="28" t="str">
+        <f aca="false">IF(AND(AND(ISNUMBER(A35),ISNUMBER(B35),B35&gt;A35),SUMPRODUCT(ISNUMBER($A$6:$A$35)*ISNUMBER($B$6:$B$35)*($A$6:$A$35&lt;B35)*($B$6:$B$35&gt;A35))&gt;1),"Overlaps another trip","")</f>
+        <v/>
+      </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="9" t="s">
         <v>52</v>
       </c>
-      <c r="C36" s="28" t="n">
+      <c r="C36" s="29" t="n">
         <f aca="false">SUM(C6:C35)</f>
         <v>0</v>
       </c>
-      <c r="D36" s="28" t="n">
+      <c r="D36" s="29" t="n">
         <f aca="false">SUM(D6:D35)</f>
         <v>0</v>
       </c>
-      <c r="E36" s="28" t="n">
+      <c r="E36" s="29" t="n">
         <f aca="false">SUM(E6:E35)</f>
         <v>0</v>
       </c>
@@ -4479,16 +4624,16 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E37" s="9" t="s">
-        <v>193</v>
-      </c>
-      <c r="F37" s="29" t="n">
+        <v>194</v>
+      </c>
+      <c r="F37" s="30" t="n">
         <f aca="false">F36*Data!$C$43</f>
         <v>0</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="17" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="B39" s="17"/>
       <c r="C39" s="17"/>
@@ -4541,34 +4686,34 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="14" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="B4" s="14" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="C4" s="14" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="D4" s="14" t="s">
+        <v>201</v>
+      </c>
+      <c r="E4" s="14" t="s">
         <v>200</v>
-      </c>
-      <c r="E4" s="14" t="s">
-        <v>199</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="B5" s="19"/>
       <c r="C5" s="26"/>
@@ -4577,7 +4722,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="B6" s="19"/>
       <c r="C6" s="26"/>
@@ -4586,7 +4731,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="B7" s="19"/>
       <c r="C7" s="26"/>
@@ -4595,7 +4740,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="B8" s="19"/>
       <c r="C8" s="26"/>
@@ -4641,53 +4786,53 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="B4" s="10"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="B5" s="10"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="B6" s="10"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="B7" s="10"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="B8" s="10"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="B9" s="10"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="6" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="B10" s="10"/>
     </row>
@@ -4730,810 +4875,820 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>214</v>
-      </c>
-      <c r="E1" s="30" t="s">
+        <v>215</v>
+      </c>
+      <c r="E1" s="31" t="s">
         <v>22</v>
       </c>
-      <c r="F1" s="30" t="s">
-        <v>215</v>
-      </c>
-      <c r="H1" s="30" t="s">
+      <c r="F1" s="31" t="s">
         <v>216</v>
       </c>
-      <c r="I1" s="30" t="s">
-        <v>215</v>
+      <c r="H1" s="31" t="s">
+        <v>217</v>
+      </c>
+      <c r="I1" s="31" t="s">
+        <v>216</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>217</v>
-      </c>
-      <c r="E2" s="30" t="s">
         <v>218</v>
       </c>
-      <c r="F2" s="30" t="s">
+      <c r="E2" s="31" t="s">
         <v>219</v>
       </c>
-      <c r="H2" s="30" t="s">
+      <c r="F2" s="31" t="s">
         <v>220</v>
       </c>
-      <c r="I2" s="30" t="s">
+      <c r="H2" s="31" t="s">
         <v>221</v>
       </c>
+      <c r="I2" s="31" t="s">
+        <v>222</v>
+      </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="31" t="s">
-        <v>222</v>
-      </c>
-      <c r="B3" s="31" t="s">
+      <c r="A3" s="32" t="s">
         <v>223</v>
       </c>
-      <c r="C3" s="31" t="s">
+      <c r="B3" s="32" t="s">
         <v>224</v>
       </c>
-      <c r="E3" s="30" t="s">
+      <c r="C3" s="32" t="s">
         <v>225</v>
       </c>
-      <c r="F3" s="30" t="s">
+      <c r="E3" s="31" t="s">
         <v>226</v>
       </c>
-      <c r="H3" s="30" t="s">
+      <c r="F3" s="31" t="s">
         <v>227</v>
       </c>
-      <c r="I3" s="30" t="s">
+      <c r="H3" s="31" t="s">
         <v>228</v>
+      </c>
+      <c r="I3" s="31" t="s">
+        <v>229</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="9" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="B4" s="21" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="C4" s="6" t="str">
         <f aca="false">"falcon-organizer-2026"</f>
         <v>falcon-organizer-2026</v>
       </c>
-      <c r="E4" s="30" t="s">
-        <v>231</v>
-      </c>
-      <c r="F4" s="30" t="s">
+      <c r="E4" s="31" t="s">
         <v>232</v>
       </c>
-      <c r="H4" s="30" t="s">
+      <c r="F4" s="31" t="s">
         <v>233</v>
       </c>
-      <c r="I4" s="30" t="s">
+      <c r="H4" s="31" t="s">
         <v>234</v>
+      </c>
+      <c r="I4" s="31" t="s">
+        <v>235</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="9" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="B5" s="21" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="C5" s="6" t="str">
         <f aca="false">IFERROR(INDEX($F$2:$F$5,MATCH(Household!B4,$E$2:$E$5,0)),"single")</f>
         <v>single</v>
       </c>
-      <c r="E5" s="30" t="s">
-        <v>237</v>
-      </c>
-      <c r="F5" s="30" t="s">
+      <c r="E5" s="31" t="s">
         <v>238</v>
       </c>
-      <c r="H5" s="30" t="s">
+      <c r="F5" s="31" t="s">
         <v>239</v>
       </c>
-      <c r="I5" s="30" t="s">
+      <c r="H5" s="31" t="s">
         <v>240</v>
+      </c>
+      <c r="I5" s="31" t="s">
+        <v>241</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="9" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="B6" s="21" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="C6" s="6" t="str">
         <f aca="false">IFERROR(INDEX($I$2:$I$52,MATCH(Household!B5,$H$2:$H$52,0)),"")</f>
         <v/>
       </c>
-      <c r="H6" s="30" t="s">
-        <v>243</v>
-      </c>
-      <c r="I6" s="30" t="s">
+      <c r="H6" s="31" t="s">
         <v>244</v>
+      </c>
+      <c r="I6" s="31" t="s">
+        <v>245</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="9" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="B7" s="21" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="C7" s="6" t="n">
         <f aca="false">IF(AND(ISNUMBER(Household!B6),Household!B6&gt;0,Household!B6&lt;=1961),1,0)</f>
         <v>0</v>
       </c>
-      <c r="H7" s="30" t="s">
-        <v>247</v>
-      </c>
-      <c r="I7" s="30" t="s">
+      <c r="H7" s="31" t="s">
         <v>248</v>
+      </c>
+      <c r="I7" s="31" t="s">
+        <v>249</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="9" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="B8" s="21" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="C8" s="6" t="n">
         <f aca="false">IF(AND(C5="mfj",ISNUMBER(Household!B7),Household!B7&gt;0,Household!B7&lt;=1961),1,0)</f>
         <v>0</v>
       </c>
-      <c r="H8" s="30" t="s">
-        <v>251</v>
-      </c>
-      <c r="I8" s="30" t="s">
+      <c r="H8" s="31" t="s">
         <v>252</v>
+      </c>
+      <c r="I8" s="31" t="s">
+        <v>253</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="9" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="B9" s="21" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="C9" s="6" t="n">
         <f aca="false">COUNTIFS(Household!A14:A23,"?*",Household!C14:C23,"&gt;=2010")</f>
         <v>0</v>
       </c>
-      <c r="H9" s="30" t="s">
-        <v>255</v>
-      </c>
-      <c r="I9" s="30" t="s">
+      <c r="H9" s="31" t="s">
         <v>256</v>
+      </c>
+      <c r="I9" s="31" t="s">
+        <v>257</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="9" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="B10" s="21" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="C10" s="6" t="n">
         <f aca="false">COUNTIF(Household!A14:A23,"?*")-C9</f>
         <v>0</v>
       </c>
-      <c r="H10" s="30" t="s">
-        <v>259</v>
-      </c>
-      <c r="I10" s="30" t="s">
+      <c r="H10" s="31" t="s">
         <v>260</v>
+      </c>
+      <c r="I10" s="31" t="s">
+        <v>261</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="9" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="B11" s="21" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="C11" s="6" t="str">
         <f aca="false">IF(C9+C10&gt;0,"yes","no")</f>
         <v>no</v>
       </c>
-      <c r="H11" s="30" t="s">
-        <v>263</v>
-      </c>
-      <c r="I11" s="30" t="s">
+      <c r="H11" s="31" t="s">
         <v>264</v>
+      </c>
+      <c r="I11" s="31" t="s">
+        <v>265</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="9" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="B12" s="21" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="C12" s="6" t="n">
         <f aca="false">IF(TRIM(Household!B8)="Yes",1,0)</f>
         <v>0</v>
       </c>
-      <c r="H12" s="30" t="s">
-        <v>267</v>
-      </c>
-      <c r="I12" s="30" t="s">
+      <c r="H12" s="31" t="s">
         <v>268</v>
+      </c>
+      <c r="I12" s="31" t="s">
+        <v>269</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="9" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="B13" s="21" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="C13" s="6" t="n">
         <f aca="false">Jobs!C16+Income!C24</f>
         <v>0</v>
       </c>
-      <c r="H13" s="30" t="s">
-        <v>271</v>
-      </c>
-      <c r="I13" s="30" t="s">
+      <c r="H13" s="31" t="s">
         <v>272</v>
+      </c>
+      <c r="I13" s="31" t="s">
+        <v>273</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="9" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="B14" s="21" t="s">
-        <v>274</v>
-      </c>
-      <c r="C14" s="32" t="n">
+        <v>275</v>
+      </c>
+      <c r="C14" s="33" t="n">
         <f aca="false">Jobs!D16</f>
         <v>0</v>
       </c>
-      <c r="H14" s="30" t="s">
-        <v>275</v>
-      </c>
-      <c r="I14" s="30" t="s">
+      <c r="H14" s="31" t="s">
         <v>276</v>
+      </c>
+      <c r="I14" s="31" t="s">
+        <v>277</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="9" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="B15" s="21" t="s">
-        <v>278</v>
-      </c>
-      <c r="C15" s="32" t="n">
+        <v>279</v>
+      </c>
+      <c r="C15" s="33" t="n">
         <f aca="false">Jobs!E16</f>
         <v>0</v>
       </c>
-      <c r="H15" s="30" t="s">
-        <v>279</v>
-      </c>
-      <c r="I15" s="30" t="s">
+      <c r="H15" s="31" t="s">
         <v>280</v>
+      </c>
+      <c r="I15" s="31" t="s">
+        <v>281</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="9" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="B16" s="21" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="C16" s="6" t="n">
         <f aca="false">Jobs!F16+Income!C24</f>
         <v>0</v>
       </c>
-      <c r="H16" s="30" t="s">
-        <v>283</v>
-      </c>
-      <c r="I16" s="30" t="s">
+      <c r="H16" s="31" t="s">
         <v>284</v>
+      </c>
+      <c r="I16" s="31" t="s">
+        <v>285</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="9" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="B17" s="21" t="s">
-        <v>286</v>
-      </c>
-      <c r="C17" s="32" t="n">
+        <v>287</v>
+      </c>
+      <c r="C17" s="33" t="n">
         <f aca="false">Jobs!G16</f>
         <v>0</v>
       </c>
-      <c r="H17" s="30" t="s">
-        <v>287</v>
-      </c>
-      <c r="I17" s="30" t="s">
+      <c r="H17" s="31" t="s">
         <v>288</v>
+      </c>
+      <c r="I17" s="31" t="s">
+        <v>289</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="9" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="B18" s="21" t="s">
-        <v>290</v>
-      </c>
-      <c r="C18" s="32" t="n">
+        <v>291</v>
+      </c>
+      <c r="C18" s="33" t="n">
         <f aca="false">Income!C19</f>
         <v>0</v>
       </c>
-      <c r="H18" s="30" t="s">
-        <v>291</v>
-      </c>
-      <c r="I18" s="30" t="s">
+      <c r="H18" s="31" t="s">
         <v>292</v>
+      </c>
+      <c r="I18" s="31" t="s">
+        <v>293</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="9" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="B19" s="21" t="s">
-        <v>294</v>
-      </c>
-      <c r="C19" s="32" t="n">
+        <v>295</v>
+      </c>
+      <c r="C19" s="33" t="n">
         <f aca="false">Expenses!E79</f>
         <v>0</v>
       </c>
-      <c r="H19" s="30" t="s">
-        <v>295</v>
-      </c>
-      <c r="I19" s="30" t="s">
+      <c r="H19" s="31" t="s">
         <v>296</v>
+      </c>
+      <c r="I19" s="31" t="s">
+        <v>297</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="9" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="B20" s="21" t="s">
-        <v>298</v>
-      </c>
-      <c r="C20" s="32" t="n">
+        <v>299</v>
+      </c>
+      <c r="C20" s="33" t="n">
         <f aca="false">Payments!B9</f>
         <v>0</v>
       </c>
-      <c r="H20" s="30" t="s">
-        <v>299</v>
-      </c>
-      <c r="I20" s="30" t="s">
+      <c r="H20" s="31" t="s">
         <v>300</v>
+      </c>
+      <c r="I20" s="31" t="s">
+        <v>301</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="9" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="B21" s="21" t="s">
-        <v>302</v>
-      </c>
-      <c r="C21" s="32" t="n">
+        <v>303</v>
+      </c>
+      <c r="C21" s="33" t="n">
         <f aca="false">Payments!D9</f>
         <v>0</v>
       </c>
-      <c r="H21" s="30" t="s">
-        <v>303</v>
-      </c>
-      <c r="I21" s="30" t="s">
+      <c r="H21" s="31" t="s">
         <v>304</v>
+      </c>
+      <c r="I21" s="31" t="s">
+        <v>305</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="9" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="B22" s="21" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="C22" s="6" t="n">
         <f aca="false">IF(Trips!D36+Trips!E36&gt;0,1,0)</f>
         <v>0</v>
       </c>
-      <c r="H22" s="30" t="s">
-        <v>307</v>
-      </c>
-      <c r="I22" s="30" t="s">
+      <c r="H22" s="31" t="s">
         <v>308</v>
+      </c>
+      <c r="I22" s="31" t="s">
+        <v>309</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="9" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="B23" s="21" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="C23" s="6" t="n">
-        <f aca="false">ROUND(MIN(365,Trips!D36+SUMPRODUCT((Trips!C6:C35&lt;Trips!D6:D35)*Trips!C6:C35+(Trips!C6:C35&gt;=Trips!D6:D35)*Trips!D6:D35)*(C41/C40-1)),2)</f>
-        <v>0</v>
-      </c>
-      <c r="H23" s="30" t="s">
-        <v>311</v>
-      </c>
-      <c r="I23" s="30" t="s">
+        <f aca="false">MIN(365,Trips!D36)</f>
+        <v>0</v>
+      </c>
+      <c r="H23" s="31" t="s">
         <v>312</v>
+      </c>
+      <c r="I23" s="31" t="s">
+        <v>313</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="9" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="B24" s="21" t="s">
-        <v>189</v>
-      </c>
-      <c r="C24" s="33" t="n">
-        <f aca="false">Trips!E36</f>
-        <v>0</v>
-      </c>
-      <c r="H24" s="30" t="s">
-        <v>314</v>
-      </c>
-      <c r="I24" s="30" t="s">
         <v>315</v>
+      </c>
+      <c r="C24" s="6" t="n">
+        <f aca="false">MIN(C23,SUMPRODUCT((Trips!C6:C35&lt;Trips!D6:D35)*Trips!C6:C35+(Trips!C6:C35&gt;=Trips!D6:D35)*Trips!D6:D35))</f>
+        <v>0</v>
+      </c>
+      <c r="H24" s="31" t="s">
+        <v>316</v>
+      </c>
+      <c r="I24" s="31" t="s">
+        <v>317</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="9" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="B25" s="21" t="s">
-        <v>69</v>
-      </c>
-      <c r="C25" s="32" t="n">
-        <f aca="false">Income!C25</f>
-        <v>0</v>
-      </c>
-      <c r="H25" s="30" t="s">
-        <v>317</v>
-      </c>
-      <c r="I25" s="30" t="s">
-        <v>318</v>
+        <v>189</v>
+      </c>
+      <c r="C25" s="34" t="n">
+        <f aca="false">Trips!E36</f>
+        <v>0</v>
+      </c>
+      <c r="H25" s="31" t="s">
+        <v>319</v>
+      </c>
+      <c r="I25" s="31" t="s">
+        <v>320</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="9" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
       <c r="B26" s="21" t="s">
-        <v>320</v>
-      </c>
-      <c r="C26" s="32" t="n">
-        <f aca="false">Income!C26</f>
-        <v>0</v>
-      </c>
-      <c r="H26" s="30" t="s">
-        <v>321</v>
-      </c>
-      <c r="I26" s="30" t="s">
+        <v>69</v>
+      </c>
+      <c r="C26" s="33" t="n">
+        <f aca="false">Income!C25</f>
+        <v>0</v>
+      </c>
+      <c r="H26" s="31" t="s">
         <v>322</v>
+      </c>
+      <c r="I26" s="31" t="s">
+        <v>323</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="9" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="B27" s="21" t="s">
-        <v>324</v>
-      </c>
-      <c r="C27" s="6" t="n">
-        <f aca="false">Income!C27+Income!C28</f>
-        <v>0</v>
-      </c>
-      <c r="H27" s="30" t="s">
         <v>325</v>
       </c>
-      <c r="I27" s="30" t="s">
+      <c r="C27" s="33" t="n">
+        <f aca="false">Income!C26</f>
+        <v>0</v>
+      </c>
+      <c r="H27" s="31" t="s">
         <v>326</v>
+      </c>
+      <c r="I27" s="31" t="s">
+        <v>327</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="9" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="B28" s="21" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="C28" s="6" t="n">
-        <f aca="false">IF(Income!C27&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-      <c r="H28" s="30" t="s">
-        <v>329</v>
-      </c>
-      <c r="I28" s="30" t="s">
+        <f aca="false">Income!C27+Income!C28</f>
+        <v>0</v>
+      </c>
+      <c r="H28" s="31" t="s">
         <v>330</v>
+      </c>
+      <c r="I28" s="31" t="s">
+        <v>331</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="9" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="B29" s="21" t="s">
-        <v>207</v>
+        <v>333</v>
       </c>
       <c r="C29" s="6" t="n">
-        <f aca="false">IF(TRIM(Checklist!B4)="Yes",1,0)</f>
-        <v>0</v>
-      </c>
-      <c r="H29" s="30" t="s">
-        <v>332</v>
-      </c>
-      <c r="I29" s="30" t="s">
-        <v>333</v>
+        <f aca="false">IF(Income!C27&gt;0,1,0)</f>
+        <v>0</v>
+      </c>
+      <c r="H29" s="31" t="s">
+        <v>334</v>
+      </c>
+      <c r="I29" s="31" t="s">
+        <v>335</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="9" t="s">
-        <v>334</v>
+        <v>336</v>
       </c>
       <c r="B30" s="21" t="s">
         <v>208</v>
       </c>
       <c r="C30" s="6" t="n">
-        <f aca="false">IF(TRIM(Checklist!B5)="Yes",1,0)</f>
-        <v>0</v>
-      </c>
-      <c r="H30" s="30" t="s">
-        <v>335</v>
-      </c>
-      <c r="I30" s="30" t="s">
-        <v>336</v>
+        <f aca="false">IF(TRIM(Checklist!B4)="Yes",1,0)</f>
+        <v>0</v>
+      </c>
+      <c r="H30" s="31" t="s">
+        <v>337</v>
+      </c>
+      <c r="I30" s="31" t="s">
+        <v>338</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="9" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="B31" s="21" t="s">
         <v>209</v>
       </c>
       <c r="C31" s="6" t="n">
-        <f aca="false">IF(TRIM(Checklist!B6)="Yes",1,0)</f>
-        <v>0</v>
-      </c>
-      <c r="H31" s="30" t="s">
-        <v>338</v>
-      </c>
-      <c r="I31" s="30" t="s">
-        <v>339</v>
+        <f aca="false">IF(TRIM(Checklist!B5)="Yes",1,0)</f>
+        <v>0</v>
+      </c>
+      <c r="H31" s="31" t="s">
+        <v>340</v>
+      </c>
+      <c r="I31" s="31" t="s">
+        <v>341</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="9" t="s">
-        <v>340</v>
+        <v>342</v>
       </c>
       <c r="B32" s="21" t="s">
         <v>210</v>
       </c>
       <c r="C32" s="6" t="n">
-        <f aca="false">IF(TRIM(Checklist!B7)="Yes",1,0)</f>
-        <v>0</v>
-      </c>
-      <c r="H32" s="30" t="s">
-        <v>341</v>
-      </c>
-      <c r="I32" s="30" t="s">
-        <v>342</v>
+        <f aca="false">IF(TRIM(Checklist!B6)="Yes",1,0)</f>
+        <v>0</v>
+      </c>
+      <c r="H32" s="31" t="s">
+        <v>343</v>
+      </c>
+      <c r="I32" s="31" t="s">
+        <v>344</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="9" t="s">
-        <v>343</v>
+        <v>345</v>
       </c>
       <c r="B33" s="21" t="s">
         <v>211</v>
       </c>
       <c r="C33" s="6" t="n">
-        <f aca="false">IF(TRIM(Checklist!B8)="Yes",1,0)</f>
-        <v>0</v>
-      </c>
-      <c r="H33" s="30" t="s">
-        <v>344</v>
-      </c>
-      <c r="I33" s="30" t="s">
-        <v>345</v>
+        <f aca="false">IF(TRIM(Checklist!B7)="Yes",1,0)</f>
+        <v>0</v>
+      </c>
+      <c r="H33" s="31" t="s">
+        <v>346</v>
+      </c>
+      <c r="I33" s="31" t="s">
+        <v>347</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="9" t="s">
-        <v>346</v>
+        <v>348</v>
       </c>
       <c r="B34" s="21" t="s">
         <v>212</v>
       </c>
       <c r="C34" s="6" t="n">
-        <f aca="false">IF(TRIM(Checklist!B9)="Yes",1,0)</f>
-        <v>0</v>
-      </c>
-      <c r="H34" s="30" t="s">
-        <v>347</v>
-      </c>
-      <c r="I34" s="30" t="s">
-        <v>348</v>
+        <f aca="false">IF(TRIM(Checklist!B8)="Yes",1,0)</f>
+        <v>0</v>
+      </c>
+      <c r="H34" s="31" t="s">
+        <v>349</v>
+      </c>
+      <c r="I34" s="31" t="s">
+        <v>350</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="9" t="s">
-        <v>349</v>
+        <v>351</v>
       </c>
       <c r="B35" s="21" t="s">
         <v>213</v>
       </c>
       <c r="C35" s="6" t="n">
+        <f aca="false">IF(TRIM(Checklist!B9)="Yes",1,0)</f>
+        <v>0</v>
+      </c>
+      <c r="H35" s="31" t="s">
+        <v>352</v>
+      </c>
+      <c r="I35" s="31" t="s">
+        <v>353</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="9" t="s">
+        <v>354</v>
+      </c>
+      <c r="B36" s="21" t="s">
+        <v>214</v>
+      </c>
+      <c r="C36" s="6" t="n">
         <f aca="false">IF(TRIM(Checklist!B10)="Yes",1,0)</f>
         <v>0</v>
       </c>
-      <c r="H35" s="30" t="s">
-        <v>350</v>
-      </c>
-      <c r="I35" s="30" t="s">
-        <v>351</v>
-      </c>
-    </row>
-    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H36" s="0" t="s">
-        <v>352</v>
-      </c>
-      <c r="I36" s="0" t="s">
-        <v>353</v>
+      <c r="H36" s="31" t="s">
+        <v>355</v>
+      </c>
+      <c r="I36" s="31" t="s">
+        <v>356</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H37" s="0" t="s">
-        <v>354</v>
+        <v>357</v>
       </c>
       <c r="I37" s="0" t="s">
-        <v>355</v>
+        <v>358</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H38" s="0" t="s">
-        <v>356</v>
+        <v>359</v>
       </c>
       <c r="I38" s="0" t="s">
-        <v>357</v>
+        <v>360</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="34" t="s">
-        <v>358</v>
-      </c>
-      <c r="H39" s="30" t="s">
-        <v>359</v>
-      </c>
-      <c r="I39" s="30" t="s">
-        <v>360</v>
+      <c r="A39" s="35" t="s">
+        <v>361</v>
+      </c>
+      <c r="H39" s="31" t="s">
+        <v>362</v>
+      </c>
+      <c r="I39" s="31" t="s">
+        <v>363</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B40" s="6" t="s">
-        <v>361</v>
-      </c>
-      <c r="C40" s="35" t="n">
+        <v>364</v>
+      </c>
+      <c r="C40" s="36" t="n">
         <v>80</v>
       </c>
-      <c r="H40" s="30" t="s">
-        <v>362</v>
-      </c>
-      <c r="I40" s="30" t="s">
-        <v>363</v>
+      <c r="H40" s="31" t="s">
+        <v>365</v>
+      </c>
+      <c r="I40" s="31" t="s">
+        <v>366</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B41" s="6" t="s">
-        <v>364</v>
-      </c>
-      <c r="C41" s="35" t="n">
+        <v>367</v>
+      </c>
+      <c r="C41" s="36" t="n">
         <v>86</v>
       </c>
-      <c r="H41" s="30" t="s">
-        <v>365</v>
-      </c>
-      <c r="I41" s="30" t="s">
-        <v>366</v>
+      <c r="H41" s="31" t="s">
+        <v>368</v>
+      </c>
+      <c r="I41" s="31" t="s">
+        <v>369</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B42" s="6" t="s">
-        <v>367</v>
-      </c>
-      <c r="C42" s="36" t="n">
+        <v>370</v>
+      </c>
+      <c r="C42" s="37" t="n">
         <v>0.75</v>
       </c>
-      <c r="H42" s="30" t="s">
-        <v>368</v>
-      </c>
-      <c r="I42" s="30" t="s">
-        <v>369</v>
+      <c r="H42" s="31" t="s">
+        <v>371</v>
+      </c>
+      <c r="I42" s="31" t="s">
+        <v>372</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B43" s="6" t="s">
-        <v>370</v>
-      </c>
-      <c r="C43" s="36" t="n">
+        <v>373</v>
+      </c>
+      <c r="C43" s="37" t="n">
         <v>0.8</v>
       </c>
-      <c r="H43" s="30" t="s">
-        <v>371</v>
-      </c>
-      <c r="I43" s="30" t="s">
-        <v>372</v>
+      <c r="H43" s="31" t="s">
+        <v>374</v>
+      </c>
+      <c r="I43" s="31" t="s">
+        <v>375</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H44" s="0" t="s">
-        <v>373</v>
+        <v>376</v>
       </c>
       <c r="I44" s="0" t="s">
-        <v>374</v>
+        <v>377</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H45" s="0" t="s">
-        <v>375</v>
+        <v>378</v>
       </c>
       <c r="I45" s="0" t="s">
-        <v>376</v>
+        <v>379</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H46" s="0" t="s">
-        <v>377</v>
+        <v>380</v>
       </c>
       <c r="I46" s="0" t="s">
-        <v>378</v>
+        <v>381</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H47" s="0" t="s">
-        <v>379</v>
+        <v>382</v>
       </c>
       <c r="I47" s="0" t="s">
-        <v>380</v>
+        <v>383</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H48" s="0" t="s">
-        <v>381</v>
+        <v>384</v>
       </c>
       <c r="I48" s="0" t="s">
-        <v>382</v>
+        <v>385</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H49" s="0" t="s">
-        <v>383</v>
+        <v>386</v>
       </c>
       <c r="I49" s="0" t="s">
-        <v>384</v>
+        <v>387</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H50" s="0" t="s">
-        <v>385</v>
+        <v>388</v>
       </c>
       <c r="I50" s="0" t="s">
-        <v>386</v>
+        <v>389</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H51" s="0" t="s">
-        <v>387</v>
+        <v>390</v>
       </c>
       <c r="I51" s="0" t="s">
-        <v>388</v>
+        <v>391</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H52" s="0" t="s">
-        <v>389</v>
+        <v>392</v>
       </c>
       <c r="I52" s="0" t="s">
-        <v>390</v>
+        <v>393</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fix EITC and car issues found by QA
- EITC: self-employment loss reduces earned income; no credit over the
  $12,200 investment-income limit; note that 17-18 year olds count
- Car: no deduction without business miles (Excel matches); warn when
  business miles exceed all miles; no method note when nothing counts;
  preview explains missing miles
- Documents list: no duplicate mileage log; car papers only when self-employed

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012ebqUPkXNMCm1mSUdBK3xi
</commit_message>
<xml_diff>
--- a/tax-prep/downloads/falcon-tax-organizer-2026.xlsx
+++ b/tax-prep/downloads/falcon-tax-organizer-2026.xlsx
@@ -5220,7 +5220,7 @@
         <v>210</v>
       </c>
       <c r="B21" s="28" t="str">
-        <f aca="false">IF(B7&gt;0,MIN(1,(B5+B6)/B7),"")</f>
+        <f aca="false">IF(AND(B7&gt;0,B5+B6&gt;0),MIN(1,(B5+B6)/B7),"")</f>
         <v/>
       </c>
     </row>
@@ -5229,7 +5229,7 @@
         <v>211</v>
       </c>
       <c r="B22" s="27" t="str">
-        <f aca="false">IF(B7&gt;0,B18*B21,"")</f>
+        <f aca="false">IF(N(B21)&gt;0,B18*B21,"")</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix Preparer summary issues found by QA
- Other expenses are Schedule C line 27b (current form); older 27a and
  unknown lines still land there; trucking tolls on line 9; office rent row
  relabeled
- Actual car costs: lease to 20a, loan interest to 16b
- Scan Reader recalculates before the summary; rejected uploads keep the
  previous items; Excel Car tab read for the split
- Ctrl+P prints only the summary while it is open
- Questions: 1099-G/1099-R withholding, Form 8867 for CTC/ODC/AOTC, no car
  questions for W-2-only, no depreciation question for rentals
- Same input limits as the engine; exact itemized match; whole dependent
  counts; tentative profit label when home office is pending

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012ebqUPkXNMCm1mSUdBK3xi
</commit_message>
<xml_diff>
--- a/tax-prep/downloads/falcon-tax-organizer-2026.xlsx
+++ b/tax-prep/downloads/falcon-tax-organizer-2026.xlsx
@@ -51,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="515" uniqueCount="438">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="516" uniqueCount="439">
   <si>
     <t xml:space="preserve">Falcon Tax Solutions · 2026 Tax Organizer</t>
   </si>
@@ -362,12 +362,15 @@
     <t xml:space="preserve">18</t>
   </si>
   <si>
-    <t xml:space="preserve">Rent (office, equipment)</t>
+    <t xml:space="preserve">Rent (office or shop)</t>
   </si>
   <si>
     <t xml:space="preserve">20b</t>
   </si>
   <si>
+    <t xml:space="preserve">Rented equipment goes on Equipment rental.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Taxes &amp; licenses</t>
   </si>
   <si>
@@ -401,7 +404,7 @@
     <t xml:space="preserve">Software &amp; subscriptions</t>
   </si>
   <si>
-    <t xml:space="preserve">27a</t>
+    <t xml:space="preserve">27b</t>
   </si>
   <si>
     <t xml:space="preserve">Materials &amp; supplies used for jobs</t>
@@ -2174,562 +2177,562 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="E1" s="34" t="s">
         <v>23</v>
       </c>
       <c r="F1" s="34" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="H1" s="34" t="s">
+        <v>249</v>
+      </c>
+      <c r="I1" s="34" t="s">
         <v>248</v>
-      </c>
-      <c r="I1" s="34" t="s">
-        <v>247</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="E2" s="34" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="F2" s="34" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="H2" s="34" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="I2" s="34" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="35" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="B3" s="35" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="C3" s="35" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="E3" s="34" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="F3" s="34" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="H3" s="34" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="I3" s="34" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="9" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="B4" s="21" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="C4" s="6" t="str">
         <f aca="false">"falcon-organizer-2026"</f>
         <v>falcon-organizer-2026</v>
       </c>
       <c r="E4" s="34" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="F4" s="34" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="H4" s="34" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="I4" s="34" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="9" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="B5" s="21" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="C5" s="6" t="str">
         <f aca="false">IFERROR(INDEX($F$2:$F$5,MATCH(Household!B4,$E$2:$E$5,0)),"single")</f>
         <v>single</v>
       </c>
       <c r="E5" s="34" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="F5" s="34" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="H5" s="34" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="I5" s="34" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="9" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="B6" s="21" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="C6" s="6" t="str">
         <f aca="false">IFERROR(INDEX($I$2:$I$52,MATCH(Household!B5,$H$2:$H$52,0)),"")</f>
         <v/>
       </c>
       <c r="H6" s="34" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="I6" s="34" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="9" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="B7" s="21" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="C7" s="6" t="n">
         <f aca="false">IF(AND(ISNUMBER(Household!B6),Household!B6&gt;0,Household!B6&lt;=1961),1,0)</f>
         <v>0</v>
       </c>
       <c r="H7" s="34" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="I7" s="34" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="9" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="B8" s="21" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="C8" s="6" t="n">
         <f aca="false">IF(AND(C5="mfj",ISNUMBER(Household!B7),Household!B7&gt;0,Household!B7&lt;=1961),1,0)</f>
         <v>0</v>
       </c>
       <c r="H8" s="34" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="I8" s="34" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="9" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="B9" s="21" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="C9" s="6" t="n">
         <f aca="false">COUNTIFS(Household!A14:A23,"?*",Household!C14:C23,"&gt;=2010")</f>
         <v>0</v>
       </c>
       <c r="H9" s="34" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="I9" s="34" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="9" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="B10" s="21" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="C10" s="6" t="n">
         <f aca="false">COUNTIF(Household!A14:A23,"?*")-C9</f>
         <v>0</v>
       </c>
       <c r="H10" s="34" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="I10" s="34" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="9" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="B11" s="21" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="C11" s="6" t="str">
         <f aca="false">IF(C9+C10&gt;0,"yes","no")</f>
         <v>no</v>
       </c>
       <c r="H11" s="34" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="I11" s="34" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="9" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="B12" s="21" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="C12" s="6" t="n">
         <f aca="false">IF(TRIM(Household!B8)="Yes",1,0)</f>
         <v>0</v>
       </c>
       <c r="H12" s="34" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="I12" s="34" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="9" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="B13" s="21" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="C13" s="6" t="n">
         <f aca="false">Jobs!C16+Income!C24</f>
         <v>0</v>
       </c>
       <c r="H13" s="34" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="I13" s="34" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="9" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="B14" s="21" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="C14" s="36" t="n">
         <f aca="false">Jobs!D16</f>
         <v>0</v>
       </c>
       <c r="H14" s="34" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="I14" s="34" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="9" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="B15" s="21" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="C15" s="36" t="n">
         <f aca="false">Jobs!E16</f>
         <v>0</v>
       </c>
       <c r="H15" s="34" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="I15" s="34" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="9" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="B16" s="21" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="C16" s="6" t="n">
         <f aca="false">Jobs!F16+Income!C24</f>
         <v>0</v>
       </c>
       <c r="H16" s="34" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="I16" s="34" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="9" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="B17" s="21" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="C17" s="36" t="n">
         <f aca="false">Jobs!G16</f>
         <v>0</v>
       </c>
       <c r="H17" s="34" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="I17" s="34" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="9" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="B18" s="21" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="C18" s="36" t="n">
         <f aca="false">Income!C19</f>
         <v>0</v>
       </c>
       <c r="H18" s="34" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="I18" s="34" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="9" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="B19" s="21" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="C19" s="36" t="n">
         <f aca="false">Expenses!E85</f>
         <v>0</v>
       </c>
       <c r="H19" s="34" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="I19" s="34" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="9" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="B20" s="21" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="C20" s="36" t="n">
         <f aca="false">Payments!B9</f>
         <v>0</v>
       </c>
       <c r="H20" s="34" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="I20" s="34" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="9" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="B21" s="21" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="C21" s="36" t="n">
         <f aca="false">Payments!D9</f>
         <v>0</v>
       </c>
       <c r="H21" s="34" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="I21" s="34" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="9" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="B22" s="21" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="C22" s="6" t="n">
         <f aca="false">IF(Trips!D36+Trips!E36&gt;0,1,0)</f>
         <v>0</v>
       </c>
       <c r="H22" s="34" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="I22" s="34" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="9" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="B23" s="21" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="C23" s="6" t="n">
         <f aca="false">MIN(365,Trips!D36)</f>
         <v>0</v>
       </c>
       <c r="H23" s="34" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="I23" s="34" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="9" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="B24" s="21" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="C24" s="6" t="n">
         <f aca="false">MIN(C23,SUMPRODUCT((Trips!C6:C35&lt;Trips!D6:D35)*Trips!C6:C35+(Trips!C6:C35&gt;=Trips!D6:D35)*Trips!D6:D35))</f>
         <v>0</v>
       </c>
       <c r="H24" s="34" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="I24" s="34" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="9" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="B25" s="21" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="C25" s="37" t="n">
         <f aca="false">Trips!E36</f>
         <v>0</v>
       </c>
       <c r="H25" s="34" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="I25" s="34" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="9" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="B26" s="21" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="C26" s="6" t="n">
         <f aca="false">IF(N(Car!B5)+N(Car!B6)+N(Car!B18)&gt;0,1,0)</f>
         <v>0</v>
       </c>
       <c r="H26" s="34" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="I26" s="34" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="9" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="B27" s="21" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="C27" s="6" t="n">
         <f aca="false">N(Car!B5)</f>
         <v>0</v>
       </c>
       <c r="H27" s="34" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="I27" s="34" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="9" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="B28" s="21" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="C28" s="6" t="n">
         <f aca="false">N(Car!B6)</f>
         <v>0</v>
       </c>
       <c r="H28" s="34" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="I28" s="34" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="9" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="B29" s="21" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="C29" s="6" t="n">
         <f aca="false">N(Car!B7)</f>
         <v>0</v>
       </c>
       <c r="H29" s="34" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="I29" s="34" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="9" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="B30" s="21" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="C30" s="6" t="n">
         <f aca="false">N(Car!B18)</f>
         <v>0</v>
       </c>
       <c r="H30" s="34" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="I30" s="34" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="9" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="B31" s="21" t="s">
         <v>70</v>
@@ -2739,288 +2742,288 @@
         <v>0</v>
       </c>
       <c r="H31" s="34" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="I31" s="34" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="9" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="B32" s="21" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="C32" s="36" t="n">
         <f aca="false">Income!C26</f>
         <v>0</v>
       </c>
       <c r="H32" s="34" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="I32" s="34" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="9" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="B33" s="21" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="C33" s="6" t="n">
         <f aca="false">Income!C27+Income!C28</f>
         <v>0</v>
       </c>
       <c r="H33" s="34" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="I33" s="34" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="9" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="B34" s="21" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="C34" s="6" t="n">
         <f aca="false">IF(Income!C27&gt;0,1,0)</f>
         <v>0</v>
       </c>
       <c r="H34" s="34" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="I34" s="34" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="9" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="B35" s="21" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="C35" s="6" t="n">
         <f aca="false">IF(TRIM(Checklist!B4)="Yes",1,0)</f>
         <v>0</v>
       </c>
       <c r="H35" s="34" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="I35" s="34" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="9" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="B36" s="21" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="C36" s="6" t="n">
         <f aca="false">IF(TRIM(Checklist!B5)="Yes",1,0)</f>
         <v>0</v>
       </c>
       <c r="H36" s="34" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="I36" s="34" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="9" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="B37" s="21" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="C37" s="6" t="n">
         <f aca="false">IF(TRIM(Checklist!B6)="Yes",1,0)</f>
         <v>0</v>
       </c>
       <c r="H37" s="34" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="I37" s="34" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="9" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="B38" s="21" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="C38" s="6" t="n">
         <f aca="false">IF(TRIM(Checklist!B7)="Yes",1,0)</f>
         <v>0</v>
       </c>
       <c r="H38" s="34" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="I38" s="34" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="9" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="B39" s="21" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="C39" s="6" t="n">
         <f aca="false">IF(TRIM(Checklist!B8)="Yes",1,0)</f>
         <v>0</v>
       </c>
       <c r="H39" s="34" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="I39" s="34" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="9" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="B40" s="21" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="C40" s="6" t="n">
         <f aca="false">IF(TRIM(Checklist!B9)="Yes",1,0)</f>
         <v>0</v>
       </c>
       <c r="H40" s="34" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="I40" s="34" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="9" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="B41" s="21" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="C41" s="6" t="n">
         <f aca="false">IF(TRIM(Checklist!B10)="Yes",1,0)</f>
         <v>0</v>
       </c>
       <c r="H41" s="34" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="I41" s="34" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H42" s="0" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="I42" s="0" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H43" s="0" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="I43" s="0" t="s">
-        <v>411</v>
+        <v>412</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H44" s="0" t="s">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="I44" s="0" t="s">
-        <v>413</v>
+        <v>414</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H45" s="0" t="s">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="I45" s="0" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H46" s="0" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="I46" s="0" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H47" s="0" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="I47" s="0" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H48" s="0" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="I48" s="0" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H49" s="0" t="s">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="I49" s="0" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H50" s="0" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="I50" s="0" t="s">
-        <v>425</v>
+        <v>426</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H51" s="0" t="s">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="I51" s="0" t="s">
-        <v>427</v>
+        <v>428</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H52" s="0" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="I52" s="0" t="s">
-        <v>429</v>
+        <v>430</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="38" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B60" s="6" t="s">
-        <v>431</v>
+        <v>432</v>
       </c>
       <c r="C60" s="39" t="n">
         <v>80</v>
@@ -3028,7 +3031,7 @@
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B61" s="6" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="C61" s="39" t="n">
         <v>86</v>
@@ -3036,7 +3039,7 @@
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B62" s="6" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="C62" s="40" t="n">
         <v>0.75</v>
@@ -3044,7 +3047,7 @@
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B63" s="6" t="s">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="C63" s="40" t="n">
         <v>0.8</v>
@@ -3052,12 +3055,12 @@
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="38" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B66" s="6" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="C66" s="41" t="n">
         <v>0.725</v>
@@ -3065,7 +3068,7 @@
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B67" s="6" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="C67" s="41" t="n">
         <v>0.76</v>
@@ -3937,13 +3940,16 @@
         <f aca="false">C14*D14</f>
         <v>0</v>
       </c>
+      <c r="F14" s="11" t="s">
+        <v>105</v>
+      </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="6" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B15" s="21" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C15" s="19"/>
       <c r="D15" s="24" t="n">
@@ -3956,10 +3962,10 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="6" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="B16" s="21" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="C16" s="19"/>
       <c r="D16" s="24" t="n">
@@ -3972,10 +3978,10 @@
     </row>
     <row r="17" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="6" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="B17" s="21" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="C17" s="19"/>
       <c r="D17" s="24" t="n">
@@ -3986,15 +3992,15 @@
         <v>0</v>
       </c>
       <c r="F17" s="11" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="6" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="B18" s="21" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="C18" s="19"/>
       <c r="D18" s="24" t="n">
@@ -4005,15 +4011,15 @@
         <v>0</v>
       </c>
       <c r="F18" s="11" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="6" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="B19" s="21" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="C19" s="19"/>
       <c r="D19" s="24" t="n">
@@ -4026,10 +4032,10 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="6" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="B20" s="21" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="C20" s="19"/>
       <c r="D20" s="24" t="n">
@@ -4040,15 +4046,15 @@
         <v>0</v>
       </c>
       <c r="F20" s="11" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="6" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="B21" s="21" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="C21" s="19"/>
       <c r="D21" s="24" t="n">
@@ -4059,15 +4065,15 @@
         <v>0</v>
       </c>
       <c r="F21" s="11" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="6" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="B22" s="21" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="C22" s="19"/>
       <c r="D22" s="24" t="n">
@@ -4080,10 +4086,10 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="6" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="B23" s="21" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C23" s="19"/>
       <c r="D23" s="24" t="n">
@@ -4096,10 +4102,10 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="6" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="B24" s="21" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="C24" s="19"/>
       <c r="D24" s="24" t="n">
@@ -4110,12 +4116,12 @@
         <v>0</v>
       </c>
       <c r="F24" s="11" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="6" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="B25" s="21" t="s">
         <v>102</v>
@@ -4131,10 +4137,10 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="6" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="B26" s="21" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="C26" s="19"/>
       <c r="D26" s="24" t="n">
@@ -4147,10 +4153,10 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="6" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="B27" s="21" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="C27" s="19"/>
       <c r="D27" s="24" t="n">
@@ -4163,10 +4169,10 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="6" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="B28" s="21" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="C28" s="19"/>
       <c r="D28" s="24" t="n">
@@ -4179,10 +4185,10 @@
     </row>
     <row r="29" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="6" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="B29" s="21" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="C29" s="19"/>
       <c r="D29" s="24" t="n">
@@ -4193,17 +4199,17 @@
         <v>0</v>
       </c>
       <c r="F29" s="11" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="23" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="6" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="B31" s="21" t="s">
         <v>91</v>
@@ -4217,12 +4223,12 @@
         <v>0</v>
       </c>
       <c r="F31" s="11" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="6" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="B32" s="21" t="s">
         <v>86</v>
@@ -4236,15 +4242,15 @@
         <v>0</v>
       </c>
       <c r="F32" s="11" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="6" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="B33" s="21" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="C33" s="19"/>
       <c r="D33" s="24" t="n">
@@ -4257,10 +4263,10 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="6" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="B34" s="21" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="C34" s="19"/>
       <c r="D34" s="24" t="n">
@@ -4273,10 +4279,10 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="6" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="B35" s="21" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="C35" s="19"/>
       <c r="D35" s="24" t="n">
@@ -4289,10 +4295,10 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="6" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="B36" s="21" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C36" s="19"/>
       <c r="D36" s="24" t="n">
@@ -4305,12 +4311,12 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="23" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="6" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="B38" s="21" t="s">
         <v>86</v>
@@ -4326,7 +4332,7 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="6" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="B39" s="21" t="s">
         <v>86</v>
@@ -4342,10 +4348,10 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="6" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="B40" s="21" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C40" s="19"/>
       <c r="D40" s="24" t="n">
@@ -4358,10 +4364,10 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="6" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="B41" s="21" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C41" s="19"/>
       <c r="D41" s="24" t="n">
@@ -4374,10 +4380,10 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="6" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="B42" s="21" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C42" s="19"/>
       <c r="D42" s="24" t="n">
@@ -4390,10 +4396,10 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="6" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="B43" s="21" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C43" s="19"/>
       <c r="D43" s="24" t="n">
@@ -4406,10 +4412,10 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="6" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="B44" s="21" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C44" s="19"/>
       <c r="D44" s="24" t="n">
@@ -4422,10 +4428,10 @@
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="6" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="B45" s="21" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C45" s="19"/>
       <c r="D45" s="24" t="n">
@@ -4438,10 +4444,10 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="6" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="B46" s="21" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C46" s="19"/>
       <c r="D46" s="24" t="n">
@@ -4454,7 +4460,7 @@
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="6" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="B47" s="21" t="s">
         <v>96</v>
@@ -4470,10 +4476,10 @@
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="6" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="B48" s="21" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="C48" s="19"/>
       <c r="D48" s="24" t="n">
@@ -4486,7 +4492,7 @@
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="6" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="B49" s="21" t="s">
         <v>98</v>
@@ -4502,10 +4508,10 @@
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="6" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="B50" s="21" t="s">
-        <v>116</v>
+        <v>86</v>
       </c>
       <c r="C50" s="19"/>
       <c r="D50" s="24" t="n">
@@ -4518,10 +4524,10 @@
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="6" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="B51" s="21" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="C51" s="19"/>
       <c r="D51" s="24" t="n">
@@ -4534,10 +4540,10 @@
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="6" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="B52" s="21" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="C52" s="19"/>
       <c r="D52" s="24" t="n">
@@ -4550,7 +4556,7 @@
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="6" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="B53" s="21" t="s">
         <v>91</v>
@@ -4566,10 +4572,10 @@
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="6" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="B54" s="21" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="C54" s="19"/>
       <c r="D54" s="24" t="n">
@@ -4582,7 +4588,7 @@
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="6" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="B55" s="21" t="s">
         <v>93</v>
@@ -4598,10 +4604,10 @@
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="6" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="B56" s="21" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="C56" s="19"/>
       <c r="D56" s="24" t="n">
@@ -4614,10 +4620,10 @@
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="6" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="B57" s="21" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="C57" s="19"/>
       <c r="D57" s="24" t="n">
@@ -4630,10 +4636,10 @@
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="6" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="B58" s="21" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="C58" s="19"/>
       <c r="D58" s="24" t="n">
@@ -4644,15 +4650,15 @@
         <v>0</v>
       </c>
       <c r="F58" s="11" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="6" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="B59" s="21" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="C59" s="19"/>
       <c r="D59" s="24" t="n">
@@ -4663,20 +4669,20 @@
         <v>0</v>
       </c>
       <c r="F59" s="11" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="23" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="B61" s="21" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C61" s="19"/>
       <c r="D61" s="24" t="n">
@@ -4689,10 +4695,10 @@
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="6" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="B62" s="21" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C62" s="19"/>
       <c r="D62" s="24" t="n">
@@ -4705,10 +4711,10 @@
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="6" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="B63" s="21" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C63" s="19"/>
       <c r="D63" s="24" t="n">
@@ -4721,10 +4727,10 @@
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="6" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="B64" s="21" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C64" s="19"/>
       <c r="D64" s="24" t="n">
@@ -4737,10 +4743,10 @@
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="6" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="B65" s="21" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C65" s="19"/>
       <c r="D65" s="24" t="n">
@@ -4753,10 +4759,10 @@
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="6" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="B66" s="21" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C66" s="19"/>
       <c r="D66" s="24" t="n">
@@ -4769,10 +4775,10 @@
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="6" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="B67" s="21" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C67" s="19"/>
       <c r="D67" s="24" t="n">
@@ -4785,10 +4791,10 @@
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="6" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="B68" s="21" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C68" s="19"/>
       <c r="D68" s="24" t="n">
@@ -4801,10 +4807,10 @@
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="6" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="B69" s="21" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C69" s="19"/>
       <c r="D69" s="24" t="n">
@@ -4817,10 +4823,10 @@
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="6" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="B70" s="21" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C70" s="19"/>
       <c r="D70" s="24" t="n">
@@ -4833,10 +4839,10 @@
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="6" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="B71" s="21" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C71" s="19"/>
       <c r="D71" s="24" t="n">
@@ -4849,10 +4855,10 @@
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="6" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="B72" s="21" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C72" s="19"/>
       <c r="D72" s="24" t="n">
@@ -4865,10 +4871,10 @@
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="6" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="B73" s="21" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C73" s="19"/>
       <c r="D73" s="24" t="n">
@@ -4881,10 +4887,10 @@
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="6" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="B74" s="21" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C74" s="19"/>
       <c r="D74" s="24" t="n">
@@ -4897,10 +4903,10 @@
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="6" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="B75" s="21" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C75" s="19"/>
       <c r="D75" s="24" t="n">
@@ -4913,10 +4919,10 @@
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="6" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="B76" s="21" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C76" s="19"/>
       <c r="D76" s="24" t="n">
@@ -4929,10 +4935,10 @@
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="6" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="B77" s="21" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C77" s="19"/>
       <c r="D77" s="24" t="n">
@@ -4945,10 +4951,10 @@
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="6" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="B78" s="21" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C78" s="19"/>
       <c r="D78" s="24" t="n">
@@ -4961,13 +4967,13 @@
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A79" s="23" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A80" s="10"/>
       <c r="B80" s="21" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="C80" s="19"/>
       <c r="D80" s="24" t="n">
@@ -4981,7 +4987,7 @@
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A81" s="10"/>
       <c r="B81" s="21" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="C81" s="19"/>
       <c r="D81" s="24" t="n">
@@ -4995,7 +5001,7 @@
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A82" s="10"/>
       <c r="B82" s="21" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="C82" s="19"/>
       <c r="D82" s="24" t="n">
@@ -5009,7 +5015,7 @@
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A83" s="10"/>
       <c r="B83" s="21" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="C83" s="19"/>
       <c r="D83" s="24" t="n">
@@ -5023,7 +5029,7 @@
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A84" s="10"/>
       <c r="B84" s="21" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="C84" s="19"/>
       <c r="D84" s="24" t="n">
@@ -5036,7 +5042,7 @@
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A85" s="9" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="C85" s="20" t="n">
         <f aca="false">SUM(C6:C84)</f>
@@ -5049,7 +5055,7 @@
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A87" s="17" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="B87" s="17"/>
       <c r="C87" s="17"/>
@@ -5095,20 +5101,20 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="14" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="B4" s="14" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="C4" s="14" t="s">
         <v>84</v>
@@ -5116,31 +5122,31 @@
     </row>
     <row r="5" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="B5" s="26"/>
       <c r="C5" s="11" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="B6" s="26"/>
     </row>
     <row r="7" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="B7" s="26"/>
       <c r="C7" s="11" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="14" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="B9" s="14" t="s">
         <v>81</v>
@@ -5151,55 +5157,55 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="6" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="B10" s="19"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="6" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="B11" s="19"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="6" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="B12" s="19"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="6" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="B13" s="19"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="6" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="B14" s="19"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="6" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="B15" s="19"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="6" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="B16" s="19"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="6" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="B17" s="19"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="9" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="B18" s="20" t="n">
         <f aca="false">SUM(B10:B17)</f>
@@ -5208,7 +5214,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="6" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="B20" s="27" t="n">
         <f aca="false">B5*Data!$C$66+B6*Data!$C$67</f>
@@ -5217,7 +5223,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="6" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="B21" s="28" t="str">
         <f aca="false">IF(AND(B7&gt;0,B5+B6&gt;0),MIN(1,(B5+B6)/B7),"")</f>
@@ -5226,7 +5232,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="6" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="B22" s="27" t="str">
         <f aca="false">IF(N(B21)&gt;0,B18*B21,"")</f>
@@ -5235,7 +5241,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="9" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="B23" s="20" t="n">
         <f aca="false">MAX(B20,N(B22))</f>
@@ -5244,7 +5250,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="17" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="B25" s="17"/>
       <c r="C25" s="17"/>
@@ -5289,43 +5295,43 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="14" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="B4" s="14" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="C4" s="14" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="D4" s="14" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="E4" s="14" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="F4" s="14" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="G4" s="14" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="15" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="B5" s="15" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="C5" s="15" t="n">
         <v>0</v>
@@ -5993,7 +5999,7 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E37" s="9" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="F37" s="33" t="n">
         <f aca="false">F36*Data!$C$63</f>
@@ -6002,7 +6008,7 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="17" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="B39" s="17"/>
       <c r="C39" s="17"/>
@@ -6055,34 +6061,34 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="14" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="B4" s="14" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="C4" s="14" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="D4" s="14" t="s">
+        <v>233</v>
+      </c>
+      <c r="E4" s="14" t="s">
         <v>232</v>
-      </c>
-      <c r="E4" s="14" t="s">
-        <v>231</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="B5" s="19"/>
       <c r="C5" s="29"/>
@@ -6091,7 +6097,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="B6" s="19"/>
       <c r="C6" s="29"/>
@@ -6100,7 +6106,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="B7" s="19"/>
       <c r="C7" s="29"/>
@@ -6109,7 +6115,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="B8" s="19"/>
       <c r="C8" s="29"/>
@@ -6155,53 +6161,53 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="B4" s="10"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="B5" s="10"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="B6" s="10"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="B7" s="10"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="B8" s="10"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="B9" s="10"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="6" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="B10" s="10"/>
     </row>

</xml_diff>

<commit_message>
Add Social Security, IRA, HSA and SEP to the estimator and organizers
- Taxable Social Security (Pub. 915 worksheet, up to 85%)
- Traditional IRA deduction with 2026 limits, 50+ catch-up, pay cap and
  workplace-plan phase-outs (Notice 2025-67); HSA (Rev. Proc. 2025-19)
  with 55+ catch-up; SEP at 20% of SE earnings up to $72,000
- Illinois subtracts Social Security and retirement income and adds the
  20% Illinois earned income credit
- Organizers: new income lines and a Retirement & health savings section
  (Excel Income tab, fillable PDF page 2, print sheet 'Page 2 continued');
  estimator fields; results, Scan Reader and Preparer summary rows and
  client questions

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012ebqUPkXNMCm1mSUdBK3xi
</commit_message>
<xml_diff>
--- a/tax-prep/downloads/falcon-tax-organizer-2026.xlsx
+++ b/tax-prep/downloads/falcon-tax-organizer-2026.xlsx
@@ -51,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="516" uniqueCount="439">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="562" uniqueCount="482">
   <si>
     <t xml:space="preserve">Falcon Tax Solutions · 2026 Tax Organizer</t>
   </si>
@@ -284,6 +284,63 @@
     <t xml:space="preserve">Other taxable income (prizes, rental profit, etc.)</t>
   </si>
   <si>
+    <t xml:space="preserve">Social Security benefits (box 5, both spouses)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SSA-1099</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Federal tax withheld on Social Security, retirement or unemployment</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SSA-1099 / 1099-R / 1099-G</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Retirement &amp; health savings (contributions for 2026)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Item</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Amount or answer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Traditional IRA contribution: you</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Form 5498</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Traditional IRA contribution: spouse</t>
+  </si>
+  <si>
+    <t xml:space="preserve">You are covered by a retirement plan at work</t>
+  </si>
+  <si>
+    <t xml:space="preserve">W-2 box 13</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Spouse is covered by a retirement plan at work</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HSA contributions you made yourself (not through payroll)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Form 5498-SA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HSA coverage</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Self-only / Family</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SEP-IRA or solo 401(k) contributions (self-employed)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Traditional IRA only (Roth contributions aren't deductible). Contributions made by April 15, 2027 can count for 2026. HSA: only what you put in yourself, not payroll contributions (W-2 code W).</t>
+  </si>
+  <si>
     <t xml:space="preserve">Business expenses</t>
   </si>
   <si>
@@ -974,7 +1031,7 @@
     <t xml:space="preserve">withheld</t>
   </si>
   <si>
-    <t xml:space="preserve">Federal tax withheld</t>
+    <t xml:space="preserve">Federal tax withheld (W-2 and other forms)</t>
   </si>
   <si>
     <t xml:space="preserve">Idaho</t>
@@ -1196,7 +1253,7 @@
     <t xml:space="preserve">otherIncome</t>
   </si>
   <si>
-    <t xml:space="preserve">Retirement withdrawals and other income</t>
+    <t xml:space="preserve">Other taxable income</t>
   </si>
   <si>
     <t xml:space="preserve">New Mexico</t>
@@ -1205,145 +1262,217 @@
     <t xml:space="preserve">NM</t>
   </si>
   <si>
+    <t xml:space="preserve">retirementIncome</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Retirement withdrawals (taxable)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">New York</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NY</t>
+  </si>
+  <si>
+    <t xml:space="preserve">socialSecurity</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Social Security benefits</t>
+  </si>
+  <si>
+    <t xml:space="preserve">North Carolina</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">iraYou</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IRA contribution: you</t>
+  </si>
+  <si>
+    <t xml:space="preserve">North Dakota</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ND</t>
+  </si>
+  <si>
+    <t xml:space="preserve">iraSpouse</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IRA contribution: spouse</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ohio</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OH</t>
+  </si>
+  <si>
+    <t xml:space="preserve">iraCoveredYou</t>
+  </si>
+  <si>
+    <t xml:space="preserve">You covered by a workplace plan</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Oklahoma</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OK</t>
+  </si>
+  <si>
+    <t xml:space="preserve">iraCoveredSpouse</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Spouse covered by a workplace plan</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Oregon</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">hsaContribution</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HSA contributions</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pennsylvania</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">hsaFamily</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HSA family coverage</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rhode Island</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RI</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sepContribution</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SEP / solo 401(k)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">South Carolina</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">you50</t>
+  </si>
+  <si>
+    <t xml:space="preserve">You 50 or older (born 1976 or earlier)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">South Dakota</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SD</t>
+  </si>
+  <si>
+    <t xml:space="preserve">spouse50</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Spouse 50 or older</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tennessee</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TN</t>
+  </si>
+  <si>
+    <t xml:space="preserve">you55</t>
+  </si>
+  <si>
+    <t xml:space="preserve">You 55 or older (HSA catch-up)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Texas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TX</t>
+  </si>
+  <si>
     <t xml:space="preserve">retirement</t>
   </si>
   <si>
     <t xml:space="preserve">Has retirement withdrawals</t>
   </si>
   <si>
-    <t xml:space="preserve">New York</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NY</t>
+    <t xml:space="preserve">Utah</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UT</t>
   </si>
   <si>
     <t xml:space="preserve">hasInvestments</t>
   </si>
   <si>
-    <t xml:space="preserve">North Carolina</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NC</t>
+    <t xml:space="preserve">Vermont</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VT</t>
   </si>
   <si>
     <t xml:space="preserve">mortgage</t>
   </si>
   <si>
-    <t xml:space="preserve">North Dakota</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ND</t>
+    <t xml:space="preserve">Virginia</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VA</t>
   </si>
   <si>
     <t xml:space="preserve">studentLoan</t>
   </si>
   <si>
-    <t xml:space="preserve">Ohio</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OH</t>
+    <t xml:space="preserve">Washington</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WA</t>
   </si>
   <si>
     <t xml:space="preserve">college</t>
   </si>
   <si>
-    <t xml:space="preserve">Oklahoma</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OK</t>
+    <t xml:space="preserve">West Virginia</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WV</t>
   </si>
   <si>
     <t xml:space="preserve">marketplace</t>
   </si>
   <si>
-    <t xml:space="preserve">Oregon</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OR</t>
+    <t xml:space="preserve">Wisconsin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WI</t>
   </si>
   <si>
     <t xml:space="preserve">noSsn</t>
   </si>
   <si>
-    <t xml:space="preserve">Pennsylvania</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PA</t>
+    <t xml:space="preserve">Wyoming</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WY</t>
   </si>
   <si>
     <t xml:space="preserve">irsLetter</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Rhode Island</t>
-  </si>
-  <si>
-    <t xml:space="preserve">RI</t>
-  </si>
-  <si>
-    <t xml:space="preserve">South Carolina</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">South Dakota</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SD</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tennessee</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TN</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Texas</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TX</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Utah</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Vermont</t>
-  </si>
-  <si>
-    <t xml:space="preserve">VT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Virginia</t>
-  </si>
-  <si>
-    <t xml:space="preserve">VA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Washington</t>
-  </si>
-  <si>
-    <t xml:space="preserve">WA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">West Virginia</t>
-  </si>
-  <si>
-    <t xml:space="preserve">WV</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Wisconsin</t>
-  </si>
-  <si>
-    <t xml:space="preserve">WI</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Wyoming</t>
-  </si>
-  <si>
-    <t xml:space="preserve">WY</t>
   </si>
   <si>
     <t xml:space="preserve">Per diem rates (IRS Notice 2026-60)</t>
@@ -2177,562 +2306,562 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>247</v>
+        <v>266</v>
       </c>
       <c r="E1" s="34" t="s">
         <v>23</v>
       </c>
       <c r="F1" s="34" t="s">
-        <v>248</v>
+        <v>267</v>
       </c>
       <c r="H1" s="34" t="s">
-        <v>249</v>
+        <v>268</v>
       </c>
       <c r="I1" s="34" t="s">
-        <v>248</v>
+        <v>267</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>250</v>
+        <v>269</v>
       </c>
       <c r="E2" s="34" t="s">
-        <v>251</v>
+        <v>270</v>
       </c>
       <c r="F2" s="34" t="s">
-        <v>252</v>
+        <v>271</v>
       </c>
       <c r="H2" s="34" t="s">
-        <v>253</v>
+        <v>272</v>
       </c>
       <c r="I2" s="34" t="s">
-        <v>254</v>
+        <v>273</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="35" t="s">
-        <v>255</v>
+        <v>274</v>
       </c>
       <c r="B3" s="35" t="s">
-        <v>256</v>
+        <v>275</v>
       </c>
       <c r="C3" s="35" t="s">
-        <v>257</v>
+        <v>276</v>
       </c>
       <c r="E3" s="34" t="s">
-        <v>258</v>
+        <v>277</v>
       </c>
       <c r="F3" s="34" t="s">
-        <v>259</v>
+        <v>278</v>
       </c>
       <c r="H3" s="34" t="s">
-        <v>260</v>
+        <v>279</v>
       </c>
       <c r="I3" s="34" t="s">
-        <v>261</v>
+        <v>280</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="9" t="s">
-        <v>262</v>
+        <v>281</v>
       </c>
       <c r="B4" s="21" t="s">
-        <v>263</v>
+        <v>282</v>
       </c>
       <c r="C4" s="6" t="str">
         <f aca="false">"falcon-organizer-2026"</f>
         <v>falcon-organizer-2026</v>
       </c>
       <c r="E4" s="34" t="s">
-        <v>264</v>
+        <v>283</v>
       </c>
       <c r="F4" s="34" t="s">
-        <v>265</v>
+        <v>284</v>
       </c>
       <c r="H4" s="34" t="s">
-        <v>266</v>
+        <v>285</v>
       </c>
       <c r="I4" s="34" t="s">
-        <v>267</v>
+        <v>286</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="9" t="s">
-        <v>268</v>
+        <v>287</v>
       </c>
       <c r="B5" s="21" t="s">
-        <v>269</v>
+        <v>288</v>
       </c>
       <c r="C5" s="6" t="str">
         <f aca="false">IFERROR(INDEX($F$2:$F$5,MATCH(Household!B4,$E$2:$E$5,0)),"single")</f>
         <v>single</v>
       </c>
       <c r="E5" s="34" t="s">
-        <v>270</v>
+        <v>289</v>
       </c>
       <c r="F5" s="34" t="s">
-        <v>271</v>
+        <v>290</v>
       </c>
       <c r="H5" s="34" t="s">
-        <v>272</v>
+        <v>291</v>
       </c>
       <c r="I5" s="34" t="s">
-        <v>273</v>
+        <v>292</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="9" t="s">
-        <v>274</v>
+        <v>293</v>
       </c>
       <c r="B6" s="21" t="s">
-        <v>275</v>
+        <v>294</v>
       </c>
       <c r="C6" s="6" t="str">
         <f aca="false">IFERROR(INDEX($I$2:$I$52,MATCH(Household!B5,$H$2:$H$52,0)),"")</f>
         <v/>
       </c>
       <c r="H6" s="34" t="s">
-        <v>276</v>
+        <v>295</v>
       </c>
       <c r="I6" s="34" t="s">
-        <v>277</v>
+        <v>296</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="9" t="s">
-        <v>278</v>
+        <v>297</v>
       </c>
       <c r="B7" s="21" t="s">
-        <v>279</v>
+        <v>298</v>
       </c>
       <c r="C7" s="6" t="n">
         <f aca="false">IF(AND(ISNUMBER(Household!B6),Household!B6&gt;0,Household!B6&lt;=1961),1,0)</f>
         <v>0</v>
       </c>
       <c r="H7" s="34" t="s">
-        <v>280</v>
+        <v>299</v>
       </c>
       <c r="I7" s="34" t="s">
-        <v>281</v>
+        <v>300</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="9" t="s">
-        <v>282</v>
+        <v>301</v>
       </c>
       <c r="B8" s="21" t="s">
-        <v>283</v>
+        <v>302</v>
       </c>
       <c r="C8" s="6" t="n">
         <f aca="false">IF(AND(C5="mfj",ISNUMBER(Household!B7),Household!B7&gt;0,Household!B7&lt;=1961),1,0)</f>
         <v>0</v>
       </c>
       <c r="H8" s="34" t="s">
-        <v>284</v>
+        <v>303</v>
       </c>
       <c r="I8" s="34" t="s">
-        <v>285</v>
+        <v>304</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="9" t="s">
-        <v>286</v>
+        <v>305</v>
       </c>
       <c r="B9" s="21" t="s">
-        <v>287</v>
+        <v>306</v>
       </c>
       <c r="C9" s="6" t="n">
         <f aca="false">COUNTIFS(Household!A14:A23,"?*",Household!C14:C23,"&gt;=2010")</f>
         <v>0</v>
       </c>
       <c r="H9" s="34" t="s">
-        <v>288</v>
+        <v>307</v>
       </c>
       <c r="I9" s="34" t="s">
-        <v>289</v>
+        <v>308</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="9" t="s">
-        <v>290</v>
+        <v>309</v>
       </c>
       <c r="B10" s="21" t="s">
-        <v>291</v>
+        <v>310</v>
       </c>
       <c r="C10" s="6" t="n">
         <f aca="false">COUNTIF(Household!A14:A23,"?*")-C9</f>
         <v>0</v>
       </c>
       <c r="H10" s="34" t="s">
-        <v>292</v>
+        <v>311</v>
       </c>
       <c r="I10" s="34" t="s">
-        <v>293</v>
+        <v>312</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="9" t="s">
-        <v>294</v>
+        <v>313</v>
       </c>
       <c r="B11" s="21" t="s">
-        <v>295</v>
+        <v>314</v>
       </c>
       <c r="C11" s="6" t="str">
         <f aca="false">IF(C9+C10&gt;0,"yes","no")</f>
         <v>no</v>
       </c>
       <c r="H11" s="34" t="s">
-        <v>296</v>
+        <v>315</v>
       </c>
       <c r="I11" s="34" t="s">
-        <v>297</v>
+        <v>316</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="9" t="s">
-        <v>298</v>
+        <v>317</v>
       </c>
       <c r="B12" s="21" t="s">
-        <v>299</v>
+        <v>318</v>
       </c>
       <c r="C12" s="6" t="n">
         <f aca="false">IF(TRIM(Household!B8)="Yes",1,0)</f>
         <v>0</v>
       </c>
       <c r="H12" s="34" t="s">
-        <v>300</v>
+        <v>319</v>
       </c>
       <c r="I12" s="34" t="s">
-        <v>301</v>
+        <v>320</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="9" t="s">
-        <v>302</v>
+        <v>321</v>
       </c>
       <c r="B13" s="21" t="s">
-        <v>303</v>
+        <v>322</v>
       </c>
       <c r="C13" s="6" t="n">
         <f aca="false">Jobs!C16+Income!C24</f>
         <v>0</v>
       </c>
       <c r="H13" s="34" t="s">
-        <v>304</v>
+        <v>323</v>
       </c>
       <c r="I13" s="34" t="s">
-        <v>305</v>
+        <v>324</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="9" t="s">
-        <v>306</v>
+        <v>325</v>
       </c>
       <c r="B14" s="21" t="s">
-        <v>307</v>
-      </c>
-      <c r="C14" s="36" t="n">
-        <f aca="false">Jobs!D16</f>
+        <v>326</v>
+      </c>
+      <c r="C14" s="6" t="n">
+        <f aca="false">Jobs!D16+N(Income!C30)</f>
         <v>0</v>
       </c>
       <c r="H14" s="34" t="s">
-        <v>308</v>
+        <v>327</v>
       </c>
       <c r="I14" s="34" t="s">
-        <v>309</v>
+        <v>328</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="9" t="s">
-        <v>310</v>
+        <v>329</v>
       </c>
       <c r="B15" s="21" t="s">
-        <v>311</v>
+        <v>330</v>
       </c>
       <c r="C15" s="36" t="n">
         <f aca="false">Jobs!E16</f>
         <v>0</v>
       </c>
       <c r="H15" s="34" t="s">
-        <v>312</v>
+        <v>331</v>
       </c>
       <c r="I15" s="34" t="s">
-        <v>313</v>
+        <v>332</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="9" t="s">
-        <v>314</v>
+        <v>333</v>
       </c>
       <c r="B16" s="21" t="s">
-        <v>315</v>
+        <v>334</v>
       </c>
       <c r="C16" s="6" t="n">
         <f aca="false">Jobs!F16+Income!C24</f>
         <v>0</v>
       </c>
       <c r="H16" s="34" t="s">
-        <v>316</v>
+        <v>335</v>
       </c>
       <c r="I16" s="34" t="s">
-        <v>317</v>
+        <v>336</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="9" t="s">
-        <v>318</v>
+        <v>337</v>
       </c>
       <c r="B17" s="21" t="s">
-        <v>319</v>
+        <v>338</v>
       </c>
       <c r="C17" s="36" t="n">
         <f aca="false">Jobs!G16</f>
         <v>0</v>
       </c>
       <c r="H17" s="34" t="s">
-        <v>320</v>
+        <v>339</v>
       </c>
       <c r="I17" s="34" t="s">
-        <v>321</v>
+        <v>340</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="9" t="s">
-        <v>322</v>
+        <v>341</v>
       </c>
       <c r="B18" s="21" t="s">
-        <v>323</v>
+        <v>342</v>
       </c>
       <c r="C18" s="36" t="n">
         <f aca="false">Income!C19</f>
         <v>0</v>
       </c>
       <c r="H18" s="34" t="s">
-        <v>324</v>
+        <v>343</v>
       </c>
       <c r="I18" s="34" t="s">
-        <v>325</v>
+        <v>344</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="9" t="s">
-        <v>326</v>
+        <v>345</v>
       </c>
       <c r="B19" s="21" t="s">
-        <v>327</v>
+        <v>346</v>
       </c>
       <c r="C19" s="36" t="n">
         <f aca="false">Expenses!E85</f>
         <v>0</v>
       </c>
       <c r="H19" s="34" t="s">
-        <v>328</v>
+        <v>347</v>
       </c>
       <c r="I19" s="34" t="s">
-        <v>329</v>
+        <v>348</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="9" t="s">
-        <v>330</v>
+        <v>349</v>
       </c>
       <c r="B20" s="21" t="s">
-        <v>331</v>
+        <v>350</v>
       </c>
       <c r="C20" s="36" t="n">
         <f aca="false">Payments!B9</f>
         <v>0</v>
       </c>
       <c r="H20" s="34" t="s">
-        <v>332</v>
+        <v>351</v>
       </c>
       <c r="I20" s="34" t="s">
-        <v>333</v>
+        <v>352</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="9" t="s">
-        <v>334</v>
+        <v>353</v>
       </c>
       <c r="B21" s="21" t="s">
-        <v>335</v>
+        <v>354</v>
       </c>
       <c r="C21" s="36" t="n">
         <f aca="false">Payments!D9</f>
         <v>0</v>
       </c>
       <c r="H21" s="34" t="s">
-        <v>336</v>
+        <v>355</v>
       </c>
       <c r="I21" s="34" t="s">
-        <v>337</v>
+        <v>356</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="9" t="s">
-        <v>338</v>
+        <v>357</v>
       </c>
       <c r="B22" s="21" t="s">
-        <v>339</v>
+        <v>358</v>
       </c>
       <c r="C22" s="6" t="n">
         <f aca="false">IF(Trips!D36+Trips!E36&gt;0,1,0)</f>
         <v>0</v>
       </c>
       <c r="H22" s="34" t="s">
-        <v>340</v>
+        <v>359</v>
       </c>
       <c r="I22" s="34" t="s">
-        <v>341</v>
+        <v>360</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="9" t="s">
-        <v>342</v>
+        <v>361</v>
       </c>
       <c r="B23" s="21" t="s">
-        <v>343</v>
+        <v>362</v>
       </c>
       <c r="C23" s="6" t="n">
         <f aca="false">MIN(365,Trips!D36)</f>
         <v>0</v>
       </c>
       <c r="H23" s="34" t="s">
-        <v>344</v>
+        <v>363</v>
       </c>
       <c r="I23" s="34" t="s">
-        <v>345</v>
+        <v>364</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="9" t="s">
-        <v>346</v>
+        <v>365</v>
       </c>
       <c r="B24" s="21" t="s">
-        <v>347</v>
+        <v>366</v>
       </c>
       <c r="C24" s="6" t="n">
         <f aca="false">MIN(C23,SUMPRODUCT((Trips!C6:C35&lt;Trips!D6:D35)*Trips!C6:C35+(Trips!C6:C35&gt;=Trips!D6:D35)*Trips!D6:D35))</f>
         <v>0</v>
       </c>
       <c r="H24" s="34" t="s">
-        <v>348</v>
+        <v>367</v>
       </c>
       <c r="I24" s="34" t="s">
-        <v>349</v>
+        <v>368</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="9" t="s">
-        <v>350</v>
+        <v>369</v>
       </c>
       <c r="B25" s="21" t="s">
-        <v>221</v>
+        <v>240</v>
       </c>
       <c r="C25" s="37" t="n">
         <f aca="false">Trips!E36</f>
         <v>0</v>
       </c>
       <c r="H25" s="34" t="s">
-        <v>351</v>
+        <v>370</v>
       </c>
       <c r="I25" s="34" t="s">
-        <v>352</v>
+        <v>371</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="9" t="s">
-        <v>353</v>
+        <v>372</v>
       </c>
       <c r="B26" s="21" t="s">
-        <v>354</v>
+        <v>373</v>
       </c>
       <c r="C26" s="6" t="n">
         <f aca="false">IF(N(Car!B5)+N(Car!B6)+N(Car!B18)&gt;0,1,0)</f>
         <v>0</v>
       </c>
       <c r="H26" s="34" t="s">
-        <v>355</v>
+        <v>374</v>
       </c>
       <c r="I26" s="34" t="s">
-        <v>356</v>
+        <v>375</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="9" t="s">
-        <v>357</v>
+        <v>376</v>
       </c>
       <c r="B27" s="21" t="s">
-        <v>358</v>
+        <v>377</v>
       </c>
       <c r="C27" s="6" t="n">
         <f aca="false">N(Car!B5)</f>
         <v>0</v>
       </c>
       <c r="H27" s="34" t="s">
-        <v>359</v>
+        <v>378</v>
       </c>
       <c r="I27" s="34" t="s">
-        <v>360</v>
+        <v>379</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="9" t="s">
-        <v>361</v>
+        <v>380</v>
       </c>
       <c r="B28" s="21" t="s">
-        <v>362</v>
+        <v>381</v>
       </c>
       <c r="C28" s="6" t="n">
         <f aca="false">N(Car!B6)</f>
         <v>0</v>
       </c>
       <c r="H28" s="34" t="s">
-        <v>363</v>
+        <v>382</v>
       </c>
       <c r="I28" s="34" t="s">
-        <v>364</v>
+        <v>383</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="9" t="s">
-        <v>365</v>
+        <v>384</v>
       </c>
       <c r="B29" s="21" t="s">
-        <v>366</v>
+        <v>385</v>
       </c>
       <c r="C29" s="6" t="n">
         <f aca="false">N(Car!B7)</f>
         <v>0</v>
       </c>
       <c r="H29" s="34" t="s">
-        <v>367</v>
+        <v>386</v>
       </c>
       <c r="I29" s="34" t="s">
-        <v>368</v>
+        <v>387</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="9" t="s">
-        <v>369</v>
+        <v>388</v>
       </c>
       <c r="B30" s="21" t="s">
-        <v>370</v>
+        <v>389</v>
       </c>
       <c r="C30" s="6" t="n">
         <f aca="false">N(Car!B18)</f>
         <v>0</v>
       </c>
       <c r="H30" s="34" t="s">
-        <v>371</v>
+        <v>390</v>
       </c>
       <c r="I30" s="34" t="s">
-        <v>372</v>
+        <v>391</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="9" t="s">
-        <v>373</v>
+        <v>392</v>
       </c>
       <c r="B31" s="21" t="s">
         <v>70</v>
@@ -2742,288 +2871,410 @@
         <v>0</v>
       </c>
       <c r="H31" s="34" t="s">
-        <v>374</v>
+        <v>393</v>
       </c>
       <c r="I31" s="34" t="s">
-        <v>375</v>
+        <v>394</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="9" t="s">
-        <v>376</v>
+        <v>395</v>
       </c>
       <c r="B32" s="21" t="s">
-        <v>377</v>
+        <v>396</v>
       </c>
       <c r="C32" s="36" t="n">
         <f aca="false">Income!C26</f>
         <v>0</v>
       </c>
       <c r="H32" s="34" t="s">
-        <v>378</v>
+        <v>397</v>
       </c>
       <c r="I32" s="34" t="s">
-        <v>379</v>
+        <v>398</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="9" t="s">
-        <v>380</v>
+        <v>399</v>
       </c>
       <c r="B33" s="21" t="s">
-        <v>381</v>
+        <v>400</v>
       </c>
       <c r="C33" s="6" t="n">
-        <f aca="false">Income!C27+Income!C28</f>
+        <f aca="false">N(Income!C28)</f>
         <v>0</v>
       </c>
       <c r="H33" s="34" t="s">
-        <v>382</v>
+        <v>401</v>
       </c>
       <c r="I33" s="34" t="s">
-        <v>383</v>
+        <v>402</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="9" t="s">
-        <v>384</v>
+        <v>403</v>
       </c>
       <c r="B34" s="21" t="s">
-        <v>385</v>
+        <v>404</v>
       </c>
       <c r="C34" s="6" t="n">
-        <f aca="false">IF(Income!C27&gt;0,1,0)</f>
+        <f aca="false">N(Income!C27)</f>
         <v>0</v>
       </c>
       <c r="H34" s="34" t="s">
-        <v>386</v>
+        <v>405</v>
       </c>
       <c r="I34" s="34" t="s">
-        <v>387</v>
+        <v>406</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="9" t="s">
-        <v>388</v>
+        <v>407</v>
       </c>
       <c r="B35" s="21" t="s">
-        <v>240</v>
+        <v>408</v>
       </c>
       <c r="C35" s="6" t="n">
-        <f aca="false">IF(TRIM(Checklist!B4)="Yes",1,0)</f>
+        <f aca="false">N(Income!C29)</f>
         <v>0</v>
       </c>
       <c r="H35" s="34" t="s">
-        <v>389</v>
+        <v>409</v>
       </c>
       <c r="I35" s="34" t="s">
-        <v>390</v>
+        <v>410</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="9" t="s">
-        <v>391</v>
+        <v>411</v>
       </c>
       <c r="B36" s="21" t="s">
-        <v>241</v>
+        <v>412</v>
       </c>
       <c r="C36" s="6" t="n">
-        <f aca="false">IF(TRIM(Checklist!B5)="Yes",1,0)</f>
+        <f aca="false">N(Income!C34)</f>
         <v>0</v>
       </c>
       <c r="H36" s="34" t="s">
-        <v>392</v>
+        <v>413</v>
       </c>
       <c r="I36" s="34" t="s">
-        <v>393</v>
+        <v>414</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="9" t="s">
-        <v>394</v>
+        <v>415</v>
       </c>
       <c r="B37" s="21" t="s">
-        <v>242</v>
+        <v>416</v>
       </c>
       <c r="C37" s="6" t="n">
-        <f aca="false">IF(TRIM(Checklist!B6)="Yes",1,0)</f>
+        <f aca="false">N(Income!C35)</f>
         <v>0</v>
       </c>
       <c r="H37" s="34" t="s">
-        <v>395</v>
+        <v>417</v>
       </c>
       <c r="I37" s="34" t="s">
-        <v>396</v>
+        <v>418</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="9" t="s">
-        <v>397</v>
+        <v>419</v>
       </c>
       <c r="B38" s="21" t="s">
-        <v>243</v>
+        <v>420</v>
       </c>
       <c r="C38" s="6" t="n">
-        <f aca="false">IF(TRIM(Checklist!B7)="Yes",1,0)</f>
+        <f aca="false">IF(TRIM(Income!C36)="Yes",1,0)</f>
         <v>0</v>
       </c>
       <c r="H38" s="34" t="s">
-        <v>398</v>
+        <v>421</v>
       </c>
       <c r="I38" s="34" t="s">
-        <v>399</v>
+        <v>422</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="9" t="s">
-        <v>400</v>
+        <v>423</v>
       </c>
       <c r="B39" s="21" t="s">
-        <v>244</v>
+        <v>424</v>
       </c>
       <c r="C39" s="6" t="n">
-        <f aca="false">IF(TRIM(Checklist!B8)="Yes",1,0)</f>
+        <f aca="false">IF(TRIM(Income!C37)="Yes",1,0)</f>
         <v>0</v>
       </c>
       <c r="H39" s="34" t="s">
-        <v>401</v>
+        <v>425</v>
       </c>
       <c r="I39" s="34" t="s">
-        <v>402</v>
+        <v>426</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="9" t="s">
-        <v>403</v>
+        <v>427</v>
       </c>
       <c r="B40" s="21" t="s">
-        <v>245</v>
+        <v>428</v>
       </c>
       <c r="C40" s="6" t="n">
-        <f aca="false">IF(TRIM(Checklist!B9)="Yes",1,0)</f>
+        <f aca="false">N(Income!C38)</f>
         <v>0</v>
       </c>
       <c r="H40" s="34" t="s">
-        <v>404</v>
+        <v>429</v>
       </c>
       <c r="I40" s="34" t="s">
-        <v>405</v>
+        <v>430</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="9" t="s">
-        <v>406</v>
+        <v>431</v>
       </c>
       <c r="B41" s="21" t="s">
-        <v>246</v>
+        <v>432</v>
       </c>
       <c r="C41" s="6" t="n">
+        <f aca="false">IF(TRIM(Income!C39)="Family",1,0)</f>
+        <v>0</v>
+      </c>
+      <c r="H41" s="34" t="s">
+        <v>433</v>
+      </c>
+      <c r="I41" s="34" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="9" t="s">
+        <v>435</v>
+      </c>
+      <c r="B42" s="21" t="s">
+        <v>436</v>
+      </c>
+      <c r="C42" s="6" t="n">
+        <f aca="false">N(Income!C40)</f>
+        <v>0</v>
+      </c>
+      <c r="H42" s="34" t="s">
+        <v>437</v>
+      </c>
+      <c r="I42" s="34" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="9" t="s">
+        <v>439</v>
+      </c>
+      <c r="B43" s="21" t="s">
+        <v>440</v>
+      </c>
+      <c r="C43" s="6" t="n">
+        <f aca="false">IF(AND(ISNUMBER(Household!B6),Household!B6&gt;0,Household!B6&lt;=1976),1,0)</f>
+        <v>0</v>
+      </c>
+      <c r="H43" s="34" t="s">
+        <v>441</v>
+      </c>
+      <c r="I43" s="34" t="s">
+        <v>442</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="9" t="s">
+        <v>443</v>
+      </c>
+      <c r="B44" s="21" t="s">
+        <v>444</v>
+      </c>
+      <c r="C44" s="6" t="n">
+        <f aca="false">IF(AND(ISNUMBER(Household!B7),Household!B7&gt;0,Household!B7&lt;=1976),1,0)</f>
+        <v>0</v>
+      </c>
+      <c r="H44" s="34" t="s">
+        <v>445</v>
+      </c>
+      <c r="I44" s="34" t="s">
+        <v>446</v>
+      </c>
+    </row>
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="9" t="s">
+        <v>447</v>
+      </c>
+      <c r="B45" s="21" t="s">
+        <v>448</v>
+      </c>
+      <c r="C45" s="6" t="n">
+        <f aca="false">IF(AND(ISNUMBER(Household!B6),Household!B6&gt;0,Household!B6&lt;=1971),1,0)</f>
+        <v>0</v>
+      </c>
+      <c r="H45" s="34" t="s">
+        <v>449</v>
+      </c>
+      <c r="I45" s="34" t="s">
+        <v>450</v>
+      </c>
+    </row>
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A46" s="9" t="s">
+        <v>451</v>
+      </c>
+      <c r="B46" s="21" t="s">
+        <v>452</v>
+      </c>
+      <c r="C46" s="6" t="n">
+        <f aca="false">IF(Income!C27&gt;0,1,0)</f>
+        <v>0</v>
+      </c>
+      <c r="H46" s="34" t="s">
+        <v>453</v>
+      </c>
+      <c r="I46" s="34" t="s">
+        <v>454</v>
+      </c>
+    </row>
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A47" s="9" t="s">
+        <v>455</v>
+      </c>
+      <c r="B47" s="21" t="s">
+        <v>259</v>
+      </c>
+      <c r="C47" s="6" t="n">
+        <f aca="false">IF(TRIM(Checklist!B4)="Yes",1,0)</f>
+        <v>0</v>
+      </c>
+      <c r="H47" s="34" t="s">
+        <v>456</v>
+      </c>
+      <c r="I47" s="34" t="s">
+        <v>457</v>
+      </c>
+    </row>
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A48" s="9" t="s">
+        <v>458</v>
+      </c>
+      <c r="B48" s="21" t="s">
+        <v>260</v>
+      </c>
+      <c r="C48" s="6" t="n">
+        <f aca="false">IF(TRIM(Checklist!B5)="Yes",1,0)</f>
+        <v>0</v>
+      </c>
+      <c r="H48" s="34" t="s">
+        <v>459</v>
+      </c>
+      <c r="I48" s="34" t="s">
+        <v>460</v>
+      </c>
+    </row>
+    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A49" s="9" t="s">
+        <v>461</v>
+      </c>
+      <c r="B49" s="21" t="s">
+        <v>261</v>
+      </c>
+      <c r="C49" s="6" t="n">
+        <f aca="false">IF(TRIM(Checklist!B6)="Yes",1,0)</f>
+        <v>0</v>
+      </c>
+      <c r="H49" s="34" t="s">
+        <v>462</v>
+      </c>
+      <c r="I49" s="34" t="s">
+        <v>463</v>
+      </c>
+    </row>
+    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A50" s="9" t="s">
+        <v>464</v>
+      </c>
+      <c r="B50" s="21" t="s">
+        <v>262</v>
+      </c>
+      <c r="C50" s="6" t="n">
+        <f aca="false">IF(TRIM(Checklist!B7)="Yes",1,0)</f>
+        <v>0</v>
+      </c>
+      <c r="H50" s="34" t="s">
+        <v>465</v>
+      </c>
+      <c r="I50" s="34" t="s">
+        <v>466</v>
+      </c>
+    </row>
+    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A51" s="9" t="s">
+        <v>467</v>
+      </c>
+      <c r="B51" s="21" t="s">
+        <v>263</v>
+      </c>
+      <c r="C51" s="6" t="n">
+        <f aca="false">IF(TRIM(Checklist!B8)="Yes",1,0)</f>
+        <v>0</v>
+      </c>
+      <c r="H51" s="34" t="s">
+        <v>468</v>
+      </c>
+      <c r="I51" s="34" t="s">
+        <v>469</v>
+      </c>
+    </row>
+    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A52" s="9" t="s">
+        <v>470</v>
+      </c>
+      <c r="B52" s="21" t="s">
+        <v>264</v>
+      </c>
+      <c r="C52" s="6" t="n">
+        <f aca="false">IF(TRIM(Checklist!B9)="Yes",1,0)</f>
+        <v>0</v>
+      </c>
+      <c r="H52" s="34" t="s">
+        <v>471</v>
+      </c>
+      <c r="I52" s="34" t="s">
+        <v>472</v>
+      </c>
+    </row>
+    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A53" s="9" t="s">
+        <v>473</v>
+      </c>
+      <c r="B53" s="21" t="s">
+        <v>265</v>
+      </c>
+      <c r="C53" s="6" t="n">
         <f aca="false">IF(TRIM(Checklist!B10)="Yes",1,0)</f>
         <v>0</v>
-      </c>
-      <c r="H41" s="34" t="s">
-        <v>407</v>
-      </c>
-      <c r="I41" s="34" t="s">
-        <v>408</v>
-      </c>
-    </row>
-    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H42" s="0" t="s">
-        <v>409</v>
-      </c>
-      <c r="I42" s="0" t="s">
-        <v>410</v>
-      </c>
-    </row>
-    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H43" s="0" t="s">
-        <v>411</v>
-      </c>
-      <c r="I43" s="0" t="s">
-        <v>412</v>
-      </c>
-    </row>
-    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H44" s="0" t="s">
-        <v>413</v>
-      </c>
-      <c r="I44" s="0" t="s">
-        <v>414</v>
-      </c>
-    </row>
-    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H45" s="0" t="s">
-        <v>415</v>
-      </c>
-      <c r="I45" s="0" t="s">
-        <v>416</v>
-      </c>
-    </row>
-    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H46" s="0" t="s">
-        <v>417</v>
-      </c>
-      <c r="I46" s="0" t="s">
-        <v>418</v>
-      </c>
-    </row>
-    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H47" s="0" t="s">
-        <v>419</v>
-      </c>
-      <c r="I47" s="0" t="s">
-        <v>420</v>
-      </c>
-    </row>
-    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H48" s="0" t="s">
-        <v>421</v>
-      </c>
-      <c r="I48" s="0" t="s">
-        <v>422</v>
-      </c>
-    </row>
-    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H49" s="0" t="s">
-        <v>423</v>
-      </c>
-      <c r="I49" s="0" t="s">
-        <v>424</v>
-      </c>
-    </row>
-    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H50" s="0" t="s">
-        <v>425</v>
-      </c>
-      <c r="I50" s="0" t="s">
-        <v>426</v>
-      </c>
-    </row>
-    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H51" s="0" t="s">
-        <v>427</v>
-      </c>
-      <c r="I51" s="0" t="s">
-        <v>428</v>
-      </c>
-    </row>
-    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H52" s="0" t="s">
-        <v>429</v>
-      </c>
-      <c r="I52" s="0" t="s">
-        <v>430</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="38" t="s">
-        <v>431</v>
+        <v>474</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B60" s="6" t="s">
-        <v>432</v>
+        <v>475</v>
       </c>
       <c r="C60" s="39" t="n">
         <v>80</v>
@@ -3031,7 +3282,7 @@
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B61" s="6" t="s">
-        <v>433</v>
+        <v>476</v>
       </c>
       <c r="C61" s="39" t="n">
         <v>86</v>
@@ -3039,7 +3290,7 @@
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B62" s="6" t="s">
-        <v>434</v>
+        <v>477</v>
       </c>
       <c r="C62" s="40" t="n">
         <v>0.75</v>
@@ -3047,7 +3298,7 @@
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B63" s="6" t="s">
-        <v>435</v>
+        <v>478</v>
       </c>
       <c r="C63" s="40" t="n">
         <v>0.8</v>
@@ -3055,12 +3306,12 @@
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="38" t="s">
-        <v>436</v>
+        <v>479</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B66" s="6" t="s">
-        <v>437</v>
+        <v>480</v>
       </c>
       <c r="C66" s="41" t="n">
         <v>0.725</v>
@@ -3068,7 +3319,7 @@
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B67" s="6" t="s">
-        <v>438</v>
+        <v>481</v>
       </c>
       <c r="C67" s="41" t="n">
         <v>0.76</v>
@@ -3546,7 +3797,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:C28"/>
+  <dimension ref="A1:C43"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="44"/>
@@ -3723,11 +3974,129 @@
       <c r="B28" s="21"/>
       <c r="C28" s="19"/>
     </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="6" t="s">
+        <v>77</v>
+      </c>
+      <c r="B29" s="21" t="s">
+        <v>78</v>
+      </c>
+      <c r="C29" s="19"/>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="6" t="s">
+        <v>79</v>
+      </c>
+      <c r="B30" s="21" t="s">
+        <v>80</v>
+      </c>
+      <c r="C30" s="19"/>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="13" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="14" t="s">
+        <v>82</v>
+      </c>
+      <c r="B33" s="14" t="s">
+        <v>66</v>
+      </c>
+      <c r="C33" s="14" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="6" t="s">
+        <v>84</v>
+      </c>
+      <c r="B34" s="21" t="s">
+        <v>85</v>
+      </c>
+      <c r="C34" s="19"/>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="B35" s="21" t="s">
+        <v>85</v>
+      </c>
+      <c r="C35" s="19"/>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="B36" s="21" t="s">
+        <v>88</v>
+      </c>
+      <c r="C36" s="10"/>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="6" t="s">
+        <v>89</v>
+      </c>
+      <c r="B37" s="21" t="s">
+        <v>88</v>
+      </c>
+      <c r="C37" s="10"/>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="6" t="s">
+        <v>90</v>
+      </c>
+      <c r="B38" s="21" t="s">
+        <v>91</v>
+      </c>
+      <c r="C38" s="19"/>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="B39" s="21" t="s">
+        <v>93</v>
+      </c>
+      <c r="C39" s="10"/>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="6" t="s">
+        <v>94</v>
+      </c>
+      <c r="B40" s="21"/>
+      <c r="C40" s="19"/>
+    </row>
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A42" s="17" t="s">
+        <v>95</v>
+      </c>
+      <c r="B42" s="17"/>
+      <c r="C42" s="17"/>
+    </row>
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="17"/>
+      <c r="B43" s="17"/>
+      <c r="C43" s="17"/>
+    </row>
   </sheetData>
   <sheetProtection sheet="true" formatColumns="false" formatRows="false"/>
-  <dataValidations count="1">
+  <mergeCells count="1">
+    <mergeCell ref="A42:C43"/>
+  </mergeCells>
+  <dataValidations count="3">
     <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="B7:B18" type="list">
       <formula1>"1099-NEC,1099-K,Cash,Zelle / app,Check,Other"</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="C36:C37" type="list">
+      <formula1>"Yes,No"</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="C39" type="list">
+      <formula1>"Self-only,Family"</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
@@ -3759,40 +4128,40 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>77</v>
+        <v>96</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>78</v>
+        <v>97</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="14" t="s">
-        <v>79</v>
+        <v>98</v>
       </c>
       <c r="B4" s="14" t="s">
-        <v>80</v>
+        <v>99</v>
       </c>
       <c r="C4" s="14" t="s">
-        <v>81</v>
+        <v>100</v>
       </c>
       <c r="D4" s="14" t="s">
-        <v>82</v>
+        <v>101</v>
       </c>
       <c r="E4" s="14" t="s">
-        <v>83</v>
+        <v>102</v>
       </c>
       <c r="F4" s="14" t="s">
-        <v>84</v>
+        <v>103</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="15" t="s">
-        <v>85</v>
+        <v>104</v>
       </c>
       <c r="B5" s="15" t="s">
-        <v>86</v>
+        <v>105</v>
       </c>
       <c r="C5" s="18" t="n">
         <v>1250</v>
@@ -3807,15 +4176,15 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="23" t="s">
-        <v>87</v>
+        <v>106</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>88</v>
+        <v>107</v>
       </c>
       <c r="B7" s="21" t="s">
-        <v>89</v>
+        <v>108</v>
       </c>
       <c r="C7" s="19"/>
       <c r="D7" s="24" t="n">
@@ -3828,10 +4197,10 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>90</v>
+        <v>109</v>
       </c>
       <c r="B8" s="21" t="s">
-        <v>91</v>
+        <v>110</v>
       </c>
       <c r="C8" s="19"/>
       <c r="D8" s="24" t="n">
@@ -3844,10 +4213,10 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="s">
-        <v>92</v>
+        <v>111</v>
       </c>
       <c r="B9" s="21" t="s">
-        <v>93</v>
+        <v>112</v>
       </c>
       <c r="C9" s="19"/>
       <c r="D9" s="24" t="n">
@@ -3858,15 +4227,15 @@
         <v>0</v>
       </c>
       <c r="F9" s="11" t="s">
-        <v>94</v>
+        <v>113</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="6" t="s">
-        <v>95</v>
+        <v>114</v>
       </c>
       <c r="B10" s="21" t="s">
-        <v>96</v>
+        <v>115</v>
       </c>
       <c r="C10" s="19"/>
       <c r="D10" s="24" t="n">
@@ -3879,10 +4248,10 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="6" t="s">
-        <v>97</v>
+        <v>116</v>
       </c>
       <c r="B11" s="21" t="s">
-        <v>98</v>
+        <v>117</v>
       </c>
       <c r="C11" s="19"/>
       <c r="D11" s="24" t="n">
@@ -3895,10 +4264,10 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="6" t="s">
-        <v>99</v>
+        <v>118</v>
       </c>
       <c r="B12" s="21" t="s">
-        <v>100</v>
+        <v>119</v>
       </c>
       <c r="C12" s="19"/>
       <c r="D12" s="24" t="n">
@@ -3911,10 +4280,10 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="6" t="s">
-        <v>101</v>
+        <v>120</v>
       </c>
       <c r="B13" s="21" t="s">
-        <v>102</v>
+        <v>121</v>
       </c>
       <c r="C13" s="19"/>
       <c r="D13" s="24" t="n">
@@ -3927,10 +4296,10 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="6" t="s">
-        <v>103</v>
+        <v>122</v>
       </c>
       <c r="B14" s="21" t="s">
-        <v>104</v>
+        <v>123</v>
       </c>
       <c r="C14" s="19"/>
       <c r="D14" s="24" t="n">
@@ -3941,15 +4310,15 @@
         <v>0</v>
       </c>
       <c r="F14" s="11" t="s">
-        <v>105</v>
+        <v>124</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="6" t="s">
-        <v>106</v>
+        <v>125</v>
       </c>
       <c r="B15" s="21" t="s">
-        <v>107</v>
+        <v>126</v>
       </c>
       <c r="C15" s="19"/>
       <c r="D15" s="24" t="n">
@@ -3962,10 +4331,10 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="6" t="s">
-        <v>108</v>
+        <v>127</v>
       </c>
       <c r="B16" s="21" t="s">
-        <v>109</v>
+        <v>128</v>
       </c>
       <c r="C16" s="19"/>
       <c r="D16" s="24" t="n">
@@ -3978,10 +4347,10 @@
     </row>
     <row r="17" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="6" t="s">
-        <v>110</v>
+        <v>129</v>
       </c>
       <c r="B17" s="21" t="s">
-        <v>111</v>
+        <v>130</v>
       </c>
       <c r="C17" s="19"/>
       <c r="D17" s="24" t="n">
@@ -3992,15 +4361,15 @@
         <v>0</v>
       </c>
       <c r="F17" s="11" t="s">
-        <v>112</v>
+        <v>131</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="6" t="s">
-        <v>113</v>
+        <v>132</v>
       </c>
       <c r="B18" s="21" t="s">
-        <v>114</v>
+        <v>133</v>
       </c>
       <c r="C18" s="19"/>
       <c r="D18" s="24" t="n">
@@ -4011,15 +4380,15 @@
         <v>0</v>
       </c>
       <c r="F18" s="11" t="s">
-        <v>115</v>
+        <v>134</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="6" t="s">
-        <v>116</v>
+        <v>135</v>
       </c>
       <c r="B19" s="21" t="s">
-        <v>117</v>
+        <v>136</v>
       </c>
       <c r="C19" s="19"/>
       <c r="D19" s="24" t="n">
@@ -4032,10 +4401,10 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="6" t="s">
-        <v>118</v>
+        <v>137</v>
       </c>
       <c r="B20" s="21" t="s">
-        <v>119</v>
+        <v>138</v>
       </c>
       <c r="C20" s="19"/>
       <c r="D20" s="24" t="n">
@@ -4046,15 +4415,15 @@
         <v>0</v>
       </c>
       <c r="F20" s="11" t="s">
-        <v>120</v>
+        <v>139</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="6" t="s">
-        <v>121</v>
+        <v>140</v>
       </c>
       <c r="B21" s="21" t="s">
-        <v>119</v>
+        <v>138</v>
       </c>
       <c r="C21" s="19"/>
       <c r="D21" s="24" t="n">
@@ -4065,15 +4434,15 @@
         <v>0</v>
       </c>
       <c r="F21" s="11" t="s">
-        <v>122</v>
+        <v>141</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="6" t="s">
-        <v>123</v>
+        <v>142</v>
       </c>
       <c r="B22" s="21" t="s">
-        <v>124</v>
+        <v>143</v>
       </c>
       <c r="C22" s="19"/>
       <c r="D22" s="24" t="n">
@@ -4086,10 +4455,10 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="6" t="s">
-        <v>125</v>
+        <v>144</v>
       </c>
       <c r="B23" s="21" t="s">
-        <v>126</v>
+        <v>145</v>
       </c>
       <c r="C23" s="19"/>
       <c r="D23" s="24" t="n">
@@ -4102,10 +4471,10 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="6" t="s">
-        <v>127</v>
+        <v>146</v>
       </c>
       <c r="B24" s="21" t="s">
-        <v>117</v>
+        <v>136</v>
       </c>
       <c r="C24" s="19"/>
       <c r="D24" s="24" t="n">
@@ -4116,15 +4485,15 @@
         <v>0</v>
       </c>
       <c r="F24" s="11" t="s">
-        <v>128</v>
+        <v>147</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="6" t="s">
-        <v>129</v>
+        <v>148</v>
       </c>
       <c r="B25" s="21" t="s">
-        <v>102</v>
+        <v>121</v>
       </c>
       <c r="C25" s="19"/>
       <c r="D25" s="24" t="n">
@@ -4137,10 +4506,10 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="6" t="s">
-        <v>130</v>
+        <v>149</v>
       </c>
       <c r="B26" s="21" t="s">
-        <v>114</v>
+        <v>133</v>
       </c>
       <c r="C26" s="19"/>
       <c r="D26" s="24" t="n">
@@ -4153,10 +4522,10 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="6" t="s">
-        <v>131</v>
+        <v>150</v>
       </c>
       <c r="B27" s="21" t="s">
-        <v>117</v>
+        <v>136</v>
       </c>
       <c r="C27" s="19"/>
       <c r="D27" s="24" t="n">
@@ -4169,10 +4538,10 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="6" t="s">
-        <v>132</v>
+        <v>151</v>
       </c>
       <c r="B28" s="21" t="s">
-        <v>117</v>
+        <v>136</v>
       </c>
       <c r="C28" s="19"/>
       <c r="D28" s="24" t="n">
@@ -4185,10 +4554,10 @@
     </row>
     <row r="29" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="6" t="s">
-        <v>133</v>
+        <v>152</v>
       </c>
       <c r="B29" s="21" t="s">
-        <v>134</v>
+        <v>153</v>
       </c>
       <c r="C29" s="19"/>
       <c r="D29" s="24" t="n">
@@ -4199,20 +4568,20 @@
         <v>0</v>
       </c>
       <c r="F29" s="11" t="s">
-        <v>135</v>
+        <v>154</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="23" t="s">
-        <v>136</v>
+        <v>155</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="6" t="s">
-        <v>137</v>
+        <v>156</v>
       </c>
       <c r="B31" s="21" t="s">
-        <v>91</v>
+        <v>110</v>
       </c>
       <c r="C31" s="19"/>
       <c r="D31" s="24" t="n">
@@ -4223,15 +4592,15 @@
         <v>0</v>
       </c>
       <c r="F31" s="11" t="s">
-        <v>138</v>
+        <v>157</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="6" t="s">
-        <v>139</v>
+        <v>158</v>
       </c>
       <c r="B32" s="21" t="s">
-        <v>86</v>
+        <v>105</v>
       </c>
       <c r="C32" s="19"/>
       <c r="D32" s="24" t="n">
@@ -4242,15 +4611,15 @@
         <v>0</v>
       </c>
       <c r="F32" s="11" t="s">
-        <v>140</v>
+        <v>159</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="6" t="s">
-        <v>141</v>
+        <v>160</v>
       </c>
       <c r="B33" s="21" t="s">
-        <v>119</v>
+        <v>138</v>
       </c>
       <c r="C33" s="19"/>
       <c r="D33" s="24" t="n">
@@ -4263,10 +4632,10 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="6" t="s">
-        <v>142</v>
+        <v>161</v>
       </c>
       <c r="B34" s="21" t="s">
-        <v>119</v>
+        <v>138</v>
       </c>
       <c r="C34" s="19"/>
       <c r="D34" s="24" t="n">
@@ -4279,10 +4648,10 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="6" t="s">
-        <v>143</v>
+        <v>162</v>
       </c>
       <c r="B35" s="21" t="s">
-        <v>119</v>
+        <v>138</v>
       </c>
       <c r="C35" s="19"/>
       <c r="D35" s="24" t="n">
@@ -4295,10 +4664,10 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="6" t="s">
-        <v>144</v>
+        <v>163</v>
       </c>
       <c r="B36" s="21" t="s">
-        <v>107</v>
+        <v>126</v>
       </c>
       <c r="C36" s="19"/>
       <c r="D36" s="24" t="n">
@@ -4311,15 +4680,15 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="23" t="s">
-        <v>145</v>
+        <v>164</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="6" t="s">
-        <v>146</v>
+        <v>165</v>
       </c>
       <c r="B38" s="21" t="s">
-        <v>86</v>
+        <v>105</v>
       </c>
       <c r="C38" s="19"/>
       <c r="D38" s="24" t="n">
@@ -4332,10 +4701,10 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="6" t="s">
-        <v>147</v>
+        <v>166</v>
       </c>
       <c r="B39" s="21" t="s">
-        <v>86</v>
+        <v>105</v>
       </c>
       <c r="C39" s="19"/>
       <c r="D39" s="24" t="n">
@@ -4348,10 +4717,10 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="6" t="s">
-        <v>148</v>
+        <v>167</v>
       </c>
       <c r="B40" s="21" t="s">
-        <v>107</v>
+        <v>126</v>
       </c>
       <c r="C40" s="19"/>
       <c r="D40" s="24" t="n">
@@ -4364,10 +4733,10 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="6" t="s">
-        <v>149</v>
+        <v>168</v>
       </c>
       <c r="B41" s="21" t="s">
-        <v>107</v>
+        <v>126</v>
       </c>
       <c r="C41" s="19"/>
       <c r="D41" s="24" t="n">
@@ -4380,10 +4749,10 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="6" t="s">
-        <v>150</v>
+        <v>169</v>
       </c>
       <c r="B42" s="21" t="s">
-        <v>107</v>
+        <v>126</v>
       </c>
       <c r="C42" s="19"/>
       <c r="D42" s="24" t="n">
@@ -4396,10 +4765,10 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="6" t="s">
-        <v>151</v>
+        <v>170</v>
       </c>
       <c r="B43" s="21" t="s">
-        <v>107</v>
+        <v>126</v>
       </c>
       <c r="C43" s="19"/>
       <c r="D43" s="24" t="n">
@@ -4412,10 +4781,10 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="6" t="s">
-        <v>152</v>
+        <v>171</v>
       </c>
       <c r="B44" s="21" t="s">
-        <v>107</v>
+        <v>126</v>
       </c>
       <c r="C44" s="19"/>
       <c r="D44" s="24" t="n">
@@ -4428,10 +4797,10 @@
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="6" t="s">
-        <v>153</v>
+        <v>172</v>
       </c>
       <c r="B45" s="21" t="s">
-        <v>107</v>
+        <v>126</v>
       </c>
       <c r="C45" s="19"/>
       <c r="D45" s="24" t="n">
@@ -4444,10 +4813,10 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="6" t="s">
-        <v>154</v>
+        <v>173</v>
       </c>
       <c r="B46" s="21" t="s">
-        <v>107</v>
+        <v>126</v>
       </c>
       <c r="C46" s="19"/>
       <c r="D46" s="24" t="n">
@@ -4460,10 +4829,10 @@
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="6" t="s">
-        <v>155</v>
+        <v>174</v>
       </c>
       <c r="B47" s="21" t="s">
-        <v>96</v>
+        <v>115</v>
       </c>
       <c r="C47" s="19"/>
       <c r="D47" s="24" t="n">
@@ -4476,10 +4845,10 @@
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="6" t="s">
-        <v>156</v>
+        <v>175</v>
       </c>
       <c r="B48" s="21" t="s">
-        <v>124</v>
+        <v>143</v>
       </c>
       <c r="C48" s="19"/>
       <c r="D48" s="24" t="n">
@@ -4492,10 +4861,10 @@
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="6" t="s">
-        <v>157</v>
+        <v>176</v>
       </c>
       <c r="B49" s="21" t="s">
-        <v>98</v>
+        <v>117</v>
       </c>
       <c r="C49" s="19"/>
       <c r="D49" s="24" t="n">
@@ -4508,10 +4877,10 @@
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="6" t="s">
-        <v>158</v>
+        <v>177</v>
       </c>
       <c r="B50" s="21" t="s">
-        <v>86</v>
+        <v>105</v>
       </c>
       <c r="C50" s="19"/>
       <c r="D50" s="24" t="n">
@@ -4524,10 +4893,10 @@
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="6" t="s">
-        <v>159</v>
+        <v>178</v>
       </c>
       <c r="B51" s="21" t="s">
-        <v>117</v>
+        <v>136</v>
       </c>
       <c r="C51" s="19"/>
       <c r="D51" s="24" t="n">
@@ -4540,10 +4909,10 @@
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="6" t="s">
-        <v>160</v>
+        <v>179</v>
       </c>
       <c r="B52" s="21" t="s">
-        <v>117</v>
+        <v>136</v>
       </c>
       <c r="C52" s="19"/>
       <c r="D52" s="24" t="n">
@@ -4556,10 +4925,10 @@
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="6" t="s">
-        <v>161</v>
+        <v>180</v>
       </c>
       <c r="B53" s="21" t="s">
-        <v>91</v>
+        <v>110</v>
       </c>
       <c r="C53" s="19"/>
       <c r="D53" s="24" t="n">
@@ -4572,10 +4941,10 @@
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="6" t="s">
-        <v>162</v>
+        <v>181</v>
       </c>
       <c r="B54" s="21" t="s">
-        <v>163</v>
+        <v>182</v>
       </c>
       <c r="C54" s="19"/>
       <c r="D54" s="24" t="n">
@@ -4588,10 +4957,10 @@
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="6" t="s">
-        <v>164</v>
+        <v>183</v>
       </c>
       <c r="B55" s="21" t="s">
-        <v>93</v>
+        <v>112</v>
       </c>
       <c r="C55" s="19"/>
       <c r="D55" s="24" t="n">
@@ -4604,10 +4973,10 @@
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="6" t="s">
-        <v>165</v>
+        <v>184</v>
       </c>
       <c r="B56" s="21" t="s">
-        <v>117</v>
+        <v>136</v>
       </c>
       <c r="C56" s="19"/>
       <c r="D56" s="24" t="n">
@@ -4620,10 +4989,10 @@
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="6" t="s">
-        <v>166</v>
+        <v>185</v>
       </c>
       <c r="B57" s="21" t="s">
-        <v>117</v>
+        <v>136</v>
       </c>
       <c r="C57" s="19"/>
       <c r="D57" s="24" t="n">
@@ -4636,10 +5005,10 @@
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="6" t="s">
-        <v>167</v>
+        <v>186</v>
       </c>
       <c r="B58" s="21" t="s">
-        <v>119</v>
+        <v>138</v>
       </c>
       <c r="C58" s="19"/>
       <c r="D58" s="24" t="n">
@@ -4650,15 +5019,15 @@
         <v>0</v>
       </c>
       <c r="F58" s="11" t="s">
-        <v>168</v>
+        <v>187</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="6" t="s">
-        <v>169</v>
+        <v>188</v>
       </c>
       <c r="B59" s="21" t="s">
-        <v>117</v>
+        <v>136</v>
       </c>
       <c r="C59" s="19"/>
       <c r="D59" s="24" t="n">
@@ -4669,20 +5038,20 @@
         <v>0</v>
       </c>
       <c r="F59" s="11" t="s">
-        <v>168</v>
+        <v>187</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="23" t="s">
-        <v>170</v>
+        <v>189</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="6" t="s">
-        <v>171</v>
+        <v>190</v>
       </c>
       <c r="B61" s="21" t="s">
-        <v>126</v>
+        <v>145</v>
       </c>
       <c r="C61" s="19"/>
       <c r="D61" s="24" t="n">
@@ -4695,10 +5064,10 @@
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="6" t="s">
-        <v>172</v>
+        <v>191</v>
       </c>
       <c r="B62" s="21" t="s">
-        <v>126</v>
+        <v>145</v>
       </c>
       <c r="C62" s="19"/>
       <c r="D62" s="24" t="n">
@@ -4711,10 +5080,10 @@
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="6" t="s">
-        <v>173</v>
+        <v>192</v>
       </c>
       <c r="B63" s="21" t="s">
-        <v>126</v>
+        <v>145</v>
       </c>
       <c r="C63" s="19"/>
       <c r="D63" s="24" t="n">
@@ -4727,10 +5096,10 @@
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="6" t="s">
-        <v>174</v>
+        <v>193</v>
       </c>
       <c r="B64" s="21" t="s">
-        <v>126</v>
+        <v>145</v>
       </c>
       <c r="C64" s="19"/>
       <c r="D64" s="24" t="n">
@@ -4743,10 +5112,10 @@
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="6" t="s">
-        <v>175</v>
+        <v>194</v>
       </c>
       <c r="B65" s="21" t="s">
-        <v>126</v>
+        <v>145</v>
       </c>
       <c r="C65" s="19"/>
       <c r="D65" s="24" t="n">
@@ -4759,10 +5128,10 @@
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="6" t="s">
-        <v>176</v>
+        <v>195</v>
       </c>
       <c r="B66" s="21" t="s">
-        <v>126</v>
+        <v>145</v>
       </c>
       <c r="C66" s="19"/>
       <c r="D66" s="24" t="n">
@@ -4775,10 +5144,10 @@
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="6" t="s">
-        <v>177</v>
+        <v>196</v>
       </c>
       <c r="B67" s="21" t="s">
-        <v>126</v>
+        <v>145</v>
       </c>
       <c r="C67" s="19"/>
       <c r="D67" s="24" t="n">
@@ -4791,10 +5160,10 @@
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="6" t="s">
-        <v>178</v>
+        <v>197</v>
       </c>
       <c r="B68" s="21" t="s">
-        <v>126</v>
+        <v>145</v>
       </c>
       <c r="C68" s="19"/>
       <c r="D68" s="24" t="n">
@@ -4807,10 +5176,10 @@
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="6" t="s">
-        <v>179</v>
+        <v>198</v>
       </c>
       <c r="B69" s="21" t="s">
-        <v>126</v>
+        <v>145</v>
       </c>
       <c r="C69" s="19"/>
       <c r="D69" s="24" t="n">
@@ -4823,10 +5192,10 @@
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="6" t="s">
-        <v>180</v>
+        <v>199</v>
       </c>
       <c r="B70" s="21" t="s">
-        <v>126</v>
+        <v>145</v>
       </c>
       <c r="C70" s="19"/>
       <c r="D70" s="24" t="n">
@@ -4839,10 +5208,10 @@
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="6" t="s">
-        <v>181</v>
+        <v>200</v>
       </c>
       <c r="B71" s="21" t="s">
-        <v>126</v>
+        <v>145</v>
       </c>
       <c r="C71" s="19"/>
       <c r="D71" s="24" t="n">
@@ -4855,10 +5224,10 @@
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="6" t="s">
-        <v>182</v>
+        <v>201</v>
       </c>
       <c r="B72" s="21" t="s">
-        <v>126</v>
+        <v>145</v>
       </c>
       <c r="C72" s="19"/>
       <c r="D72" s="24" t="n">
@@ -4871,10 +5240,10 @@
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="6" t="s">
-        <v>183</v>
+        <v>202</v>
       </c>
       <c r="B73" s="21" t="s">
-        <v>126</v>
+        <v>145</v>
       </c>
       <c r="C73" s="19"/>
       <c r="D73" s="24" t="n">
@@ -4887,10 +5256,10 @@
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="6" t="s">
-        <v>184</v>
+        <v>203</v>
       </c>
       <c r="B74" s="21" t="s">
-        <v>126</v>
+        <v>145</v>
       </c>
       <c r="C74" s="19"/>
       <c r="D74" s="24" t="n">
@@ -4903,10 +5272,10 @@
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="6" t="s">
-        <v>185</v>
+        <v>204</v>
       </c>
       <c r="B75" s="21" t="s">
-        <v>126</v>
+        <v>145</v>
       </c>
       <c r="C75" s="19"/>
       <c r="D75" s="24" t="n">
@@ -4919,10 +5288,10 @@
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="6" t="s">
-        <v>186</v>
+        <v>205</v>
       </c>
       <c r="B76" s="21" t="s">
-        <v>126</v>
+        <v>145</v>
       </c>
       <c r="C76" s="19"/>
       <c r="D76" s="24" t="n">
@@ -4935,10 +5304,10 @@
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="6" t="s">
-        <v>187</v>
+        <v>206</v>
       </c>
       <c r="B77" s="21" t="s">
-        <v>126</v>
+        <v>145</v>
       </c>
       <c r="C77" s="19"/>
       <c r="D77" s="24" t="n">
@@ -4951,10 +5320,10 @@
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="6" t="s">
-        <v>188</v>
+        <v>207</v>
       </c>
       <c r="B78" s="21" t="s">
-        <v>126</v>
+        <v>145</v>
       </c>
       <c r="C78" s="19"/>
       <c r="D78" s="24" t="n">
@@ -4967,13 +5336,13 @@
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A79" s="23" t="s">
-        <v>189</v>
+        <v>208</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A80" s="10"/>
       <c r="B80" s="21" t="s">
-        <v>117</v>
+        <v>136</v>
       </c>
       <c r="C80" s="19"/>
       <c r="D80" s="24" t="n">
@@ -4987,7 +5356,7 @@
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A81" s="10"/>
       <c r="B81" s="21" t="s">
-        <v>117</v>
+        <v>136</v>
       </c>
       <c r="C81" s="19"/>
       <c r="D81" s="24" t="n">
@@ -5001,7 +5370,7 @@
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A82" s="10"/>
       <c r="B82" s="21" t="s">
-        <v>117</v>
+        <v>136</v>
       </c>
       <c r="C82" s="19"/>
       <c r="D82" s="24" t="n">
@@ -5015,7 +5384,7 @@
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A83" s="10"/>
       <c r="B83" s="21" t="s">
-        <v>117</v>
+        <v>136</v>
       </c>
       <c r="C83" s="19"/>
       <c r="D83" s="24" t="n">
@@ -5029,7 +5398,7 @@
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A84" s="10"/>
       <c r="B84" s="21" t="s">
-        <v>117</v>
+        <v>136</v>
       </c>
       <c r="C84" s="19"/>
       <c r="D84" s="24" t="n">
@@ -5042,7 +5411,7 @@
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A85" s="9" t="s">
-        <v>190</v>
+        <v>209</v>
       </c>
       <c r="C85" s="20" t="n">
         <f aca="false">SUM(C6:C84)</f>
@@ -5055,7 +5424,7 @@
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A87" s="17" t="s">
-        <v>191</v>
+        <v>210</v>
       </c>
       <c r="B87" s="17"/>
       <c r="C87" s="17"/>
@@ -5101,111 +5470,111 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>192</v>
+        <v>211</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>193</v>
+        <v>212</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="14" t="s">
-        <v>194</v>
+        <v>213</v>
       </c>
       <c r="B4" s="14" t="s">
-        <v>194</v>
+        <v>213</v>
       </c>
       <c r="C4" s="14" t="s">
-        <v>84</v>
+        <v>103</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
-        <v>195</v>
+        <v>214</v>
       </c>
       <c r="B5" s="26"/>
       <c r="C5" s="11" t="s">
-        <v>196</v>
+        <v>215</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>197</v>
+        <v>216</v>
       </c>
       <c r="B6" s="26"/>
     </row>
     <row r="7" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>198</v>
+        <v>217</v>
       </c>
       <c r="B7" s="26"/>
       <c r="C7" s="11" t="s">
-        <v>199</v>
+        <v>218</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="14" t="s">
-        <v>200</v>
+        <v>219</v>
       </c>
       <c r="B9" s="14" t="s">
-        <v>81</v>
+        <v>100</v>
       </c>
       <c r="C9" s="14" t="s">
-        <v>84</v>
+        <v>103</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="6" t="s">
-        <v>201</v>
+        <v>220</v>
       </c>
       <c r="B10" s="19"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="6" t="s">
-        <v>202</v>
+        <v>221</v>
       </c>
       <c r="B11" s="19"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="6" t="s">
-        <v>203</v>
+        <v>222</v>
       </c>
       <c r="B12" s="19"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="6" t="s">
-        <v>204</v>
+        <v>223</v>
       </c>
       <c r="B13" s="19"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="6" t="s">
-        <v>205</v>
+        <v>224</v>
       </c>
       <c r="B14" s="19"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="6" t="s">
-        <v>206</v>
+        <v>225</v>
       </c>
       <c r="B15" s="19"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="6" t="s">
-        <v>207</v>
+        <v>226</v>
       </c>
       <c r="B16" s="19"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="6" t="s">
-        <v>208</v>
+        <v>227</v>
       </c>
       <c r="B17" s="19"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="9" t="s">
-        <v>209</v>
+        <v>228</v>
       </c>
       <c r="B18" s="20" t="n">
         <f aca="false">SUM(B10:B17)</f>
@@ -5214,7 +5583,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="6" t="s">
-        <v>210</v>
+        <v>229</v>
       </c>
       <c r="B20" s="27" t="n">
         <f aca="false">B5*Data!$C$66+B6*Data!$C$67</f>
@@ -5223,7 +5592,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="6" t="s">
-        <v>211</v>
+        <v>230</v>
       </c>
       <c r="B21" s="28" t="str">
         <f aca="false">IF(AND(B7&gt;0,B5+B6&gt;0),MIN(1,(B5+B6)/B7),"")</f>
@@ -5232,7 +5601,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="6" t="s">
-        <v>212</v>
+        <v>231</v>
       </c>
       <c r="B22" s="27" t="str">
         <f aca="false">IF(N(B21)&gt;0,B18*B21,"")</f>
@@ -5241,7 +5610,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="9" t="s">
-        <v>213</v>
+        <v>232</v>
       </c>
       <c r="B23" s="20" t="n">
         <f aca="false">MAX(B20,N(B22))</f>
@@ -5250,7 +5619,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="17" t="s">
-        <v>214</v>
+        <v>233</v>
       </c>
       <c r="B25" s="17"/>
       <c r="C25" s="17"/>
@@ -5295,43 +5664,43 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>215</v>
+        <v>234</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>216</v>
+        <v>235</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="14" t="s">
-        <v>217</v>
+        <v>236</v>
       </c>
       <c r="B4" s="14" t="s">
-        <v>218</v>
+        <v>237</v>
       </c>
       <c r="C4" s="14" t="s">
-        <v>219</v>
+        <v>238</v>
       </c>
       <c r="D4" s="14" t="s">
-        <v>220</v>
+        <v>239</v>
       </c>
       <c r="E4" s="14" t="s">
-        <v>221</v>
+        <v>240</v>
       </c>
       <c r="F4" s="14" t="s">
-        <v>222</v>
+        <v>241</v>
       </c>
       <c r="G4" s="14" t="s">
-        <v>223</v>
+        <v>242</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="15" t="s">
-        <v>224</v>
+        <v>243</v>
       </c>
       <c r="B5" s="15" t="s">
-        <v>225</v>
+        <v>244</v>
       </c>
       <c r="C5" s="15" t="n">
         <v>0</v>
@@ -5999,7 +6368,7 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E37" s="9" t="s">
-        <v>226</v>
+        <v>245</v>
       </c>
       <c r="F37" s="33" t="n">
         <f aca="false">F36*Data!$C$63</f>
@@ -6008,7 +6377,7 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="17" t="s">
-        <v>227</v>
+        <v>246</v>
       </c>
       <c r="B39" s="17"/>
       <c r="C39" s="17"/>
@@ -6061,34 +6430,34 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>228</v>
+        <v>247</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>229</v>
+        <v>248</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="14" t="s">
-        <v>230</v>
+        <v>249</v>
       </c>
       <c r="B4" s="14" t="s">
-        <v>231</v>
+        <v>250</v>
       </c>
       <c r="C4" s="14" t="s">
-        <v>232</v>
+        <v>251</v>
       </c>
       <c r="D4" s="14" t="s">
-        <v>233</v>
+        <v>252</v>
       </c>
       <c r="E4" s="14" t="s">
-        <v>232</v>
+        <v>251</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
-        <v>234</v>
+        <v>253</v>
       </c>
       <c r="B5" s="19"/>
       <c r="C5" s="29"/>
@@ -6097,7 +6466,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>235</v>
+        <v>254</v>
       </c>
       <c r="B6" s="19"/>
       <c r="C6" s="29"/>
@@ -6106,7 +6475,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>236</v>
+        <v>255</v>
       </c>
       <c r="B7" s="19"/>
       <c r="C7" s="29"/>
@@ -6115,7 +6484,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>237</v>
+        <v>256</v>
       </c>
       <c r="B8" s="19"/>
       <c r="C8" s="29"/>
@@ -6161,53 +6530,53 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>238</v>
+        <v>257</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>239</v>
+        <v>258</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>240</v>
+        <v>259</v>
       </c>
       <c r="B4" s="10"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
-        <v>241</v>
+        <v>260</v>
       </c>
       <c r="B5" s="10"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>242</v>
+        <v>261</v>
       </c>
       <c r="B6" s="10"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>243</v>
+        <v>262</v>
       </c>
       <c r="B7" s="10"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>244</v>
+        <v>263</v>
       </c>
       <c r="B8" s="10"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="s">
-        <v>245</v>
+        <v>264</v>
       </c>
       <c r="B9" s="10"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="6" t="s">
-        <v>246</v>
+        <v>265</v>
       </c>
       <c r="B10" s="10"/>
     </row>

</xml_diff>

<commit_message>
Add Schedule K-1 income and an S-corp savings calculator
- Engine: partnership box 1, guaranteed payments (SE via box 14A, default
  box 1 + 4c) and S-corp box 1 (no SE tax); combined Schedule SE; QBI
  excludes guaranteed payments
- Organizers: K-1 table (Excel Income tab, fillable PDF page 2, print
  page 2 continued); estimator K-1 box; Scan Reader and Preparer summary
  rows and questions (basis, QBI box 20Z/17V, reasonable salary)
- scorp.html: sole proprietor vs S-corp with payroll taxes, FUTA, extra
  costs, Illinois 1.5% replacement tax and a salary table; linked from the
  homepage and from estimator results when profit is $50k+

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012ebqUPkXNMCm1mSUdBK3xi
</commit_message>
<xml_diff>
--- a/tax-prep/downloads/falcon-tax-organizer-2026.xlsx
+++ b/tax-prep/downloads/falcon-tax-organizer-2026.xlsx
@@ -51,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="562" uniqueCount="482">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="578" uniqueCount="498">
   <si>
     <t xml:space="preserve">Falcon Tax Solutions · 2026 Tax Organizer</t>
   </si>
@@ -341,6 +341,30 @@
     <t xml:space="preserve">Traditional IRA only (Roth contributions aren't deductible). Contributions made by April 15, 2027 can count for 2026. HSA: only what you put in yourself, not payroll contributions (W-2 code W).</t>
   </si>
   <si>
+    <t xml:space="preserve">K-1 income (partnership, LLC or S-corp owners)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Type of K-1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Business name (optional)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Box 1 ordinary income (loss)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Box 4c guaranteed payments (1065 only)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Box 14 code A SE earnings (1065 only)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SE earnings used</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Copy the boxes from each Schedule K-1. Losses can be limited by basis and passive rules; we'll check. S-corp owners: your salary is on your W-2 (Jobs tab), not here.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Business expenses</t>
   </si>
   <si>
@@ -1370,16 +1394,64 @@
     <t xml:space="preserve">SC</t>
   </si>
   <si>
+    <t xml:space="preserve">k1Partnership</t>
+  </si>
+  <si>
+    <t xml:space="preserve">K-1 box 1, partnerships / LLCs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">South Dakota</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SD</t>
+  </si>
+  <si>
+    <t xml:space="preserve">k1Guaranteed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">K-1 guaranteed payments</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tennessee</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TN</t>
+  </si>
+  <si>
+    <t xml:space="preserve">k1SCorp</t>
+  </si>
+  <si>
+    <t xml:space="preserve">K-1 box 1, S-corps</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Texas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TX</t>
+  </si>
+  <si>
+    <t xml:space="preserve">k1Se</t>
+  </si>
+  <si>
+    <t xml:space="preserve">K-1 self-employment earnings</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Utah</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UT</t>
+  </si>
+  <si>
     <t xml:space="preserve">you50</t>
   </si>
   <si>
     <t xml:space="preserve">You 50 or older (born 1976 or earlier)</t>
   </si>
   <si>
-    <t xml:space="preserve">South Dakota</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SD</t>
+    <t xml:space="preserve">Vermont</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VT</t>
   </si>
   <si>
     <t xml:space="preserve">spouse50</t>
@@ -1388,10 +1460,10 @@
     <t xml:space="preserve">Spouse 50 or older</t>
   </si>
   <si>
-    <t xml:space="preserve">Tennessee</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TN</t>
+    <t xml:space="preserve">Virginia</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VA</t>
   </si>
   <si>
     <t xml:space="preserve">you55</t>
@@ -1400,10 +1472,10 @@
     <t xml:space="preserve">You 55 or older (HSA catch-up)</t>
   </si>
   <si>
-    <t xml:space="preserve">Texas</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TX</t>
+    <t xml:space="preserve">Washington</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WA</t>
   </si>
   <si>
     <t xml:space="preserve">retirement</t>
@@ -1412,64 +1484,40 @@
     <t xml:space="preserve">Has retirement withdrawals</t>
   </si>
   <si>
-    <t xml:space="preserve">Utah</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UT</t>
+    <t xml:space="preserve">West Virginia</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WV</t>
   </si>
   <si>
     <t xml:space="preserve">hasInvestments</t>
   </si>
   <si>
-    <t xml:space="preserve">Vermont</t>
-  </si>
-  <si>
-    <t xml:space="preserve">VT</t>
+    <t xml:space="preserve">Wisconsin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WI</t>
   </si>
   <si>
     <t xml:space="preserve">mortgage</t>
   </si>
   <si>
-    <t xml:space="preserve">Virginia</t>
-  </si>
-  <si>
-    <t xml:space="preserve">VA</t>
+    <t xml:space="preserve">Wyoming</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WY</t>
   </si>
   <si>
     <t xml:space="preserve">studentLoan</t>
   </si>
   <si>
-    <t xml:space="preserve">Washington</t>
-  </si>
-  <si>
-    <t xml:space="preserve">WA</t>
-  </si>
-  <si>
     <t xml:space="preserve">college</t>
   </si>
   <si>
-    <t xml:space="preserve">West Virginia</t>
-  </si>
-  <si>
-    <t xml:space="preserve">WV</t>
-  </si>
-  <si>
     <t xml:space="preserve">marketplace</t>
   </si>
   <si>
-    <t xml:space="preserve">Wisconsin</t>
-  </si>
-  <si>
-    <t xml:space="preserve">WI</t>
-  </si>
-  <si>
     <t xml:space="preserve">noSsn</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Wyoming</t>
-  </si>
-  <si>
-    <t xml:space="preserve">WY</t>
   </si>
   <si>
     <t xml:space="preserve">irsLetter</t>
@@ -1728,7 +1776,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="42">
+  <cellXfs count="43">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1814,6 +1862,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2306,1022 +2358,1070 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>266</v>
-      </c>
-      <c r="E1" s="34" t="s">
+        <v>274</v>
+      </c>
+      <c r="E1" s="35" t="s">
         <v>23</v>
       </c>
-      <c r="F1" s="34" t="s">
-        <v>267</v>
-      </c>
-      <c r="H1" s="34" t="s">
-        <v>268</v>
-      </c>
-      <c r="I1" s="34" t="s">
-        <v>267</v>
+      <c r="F1" s="35" t="s">
+        <v>275</v>
+      </c>
+      <c r="H1" s="35" t="s">
+        <v>276</v>
+      </c>
+      <c r="I1" s="35" t="s">
+        <v>275</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>269</v>
-      </c>
-      <c r="E2" s="34" t="s">
-        <v>270</v>
-      </c>
-      <c r="F2" s="34" t="s">
-        <v>271</v>
-      </c>
-      <c r="H2" s="34" t="s">
-        <v>272</v>
-      </c>
-      <c r="I2" s="34" t="s">
-        <v>273</v>
+        <v>277</v>
+      </c>
+      <c r="E2" s="35" t="s">
+        <v>278</v>
+      </c>
+      <c r="F2" s="35" t="s">
+        <v>279</v>
+      </c>
+      <c r="H2" s="35" t="s">
+        <v>280</v>
+      </c>
+      <c r="I2" s="35" t="s">
+        <v>281</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="35" t="s">
-        <v>274</v>
-      </c>
-      <c r="B3" s="35" t="s">
-        <v>275</v>
-      </c>
-      <c r="C3" s="35" t="s">
-        <v>276</v>
-      </c>
-      <c r="E3" s="34" t="s">
-        <v>277</v>
-      </c>
-      <c r="F3" s="34" t="s">
-        <v>278</v>
-      </c>
-      <c r="H3" s="34" t="s">
-        <v>279</v>
-      </c>
-      <c r="I3" s="34" t="s">
-        <v>280</v>
+      <c r="A3" s="36" t="s">
+        <v>282</v>
+      </c>
+      <c r="B3" s="36" t="s">
+        <v>283</v>
+      </c>
+      <c r="C3" s="36" t="s">
+        <v>284</v>
+      </c>
+      <c r="E3" s="35" t="s">
+        <v>285</v>
+      </c>
+      <c r="F3" s="35" t="s">
+        <v>286</v>
+      </c>
+      <c r="H3" s="35" t="s">
+        <v>287</v>
+      </c>
+      <c r="I3" s="35" t="s">
+        <v>288</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="9" t="s">
-        <v>281</v>
+        <v>289</v>
       </c>
       <c r="B4" s="21" t="s">
-        <v>282</v>
+        <v>290</v>
       </c>
       <c r="C4" s="6" t="str">
         <f aca="false">"falcon-organizer-2026"</f>
         <v>falcon-organizer-2026</v>
       </c>
-      <c r="E4" s="34" t="s">
-        <v>283</v>
-      </c>
-      <c r="F4" s="34" t="s">
-        <v>284</v>
-      </c>
-      <c r="H4" s="34" t="s">
-        <v>285</v>
-      </c>
-      <c r="I4" s="34" t="s">
-        <v>286</v>
+      <c r="E4" s="35" t="s">
+        <v>291</v>
+      </c>
+      <c r="F4" s="35" t="s">
+        <v>292</v>
+      </c>
+      <c r="H4" s="35" t="s">
+        <v>293</v>
+      </c>
+      <c r="I4" s="35" t="s">
+        <v>294</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="9" t="s">
-        <v>287</v>
+        <v>295</v>
       </c>
       <c r="B5" s="21" t="s">
-        <v>288</v>
+        <v>296</v>
       </c>
       <c r="C5" s="6" t="str">
         <f aca="false">IFERROR(INDEX($F$2:$F$5,MATCH(Household!B4,$E$2:$E$5,0)),"single")</f>
         <v>single</v>
       </c>
-      <c r="E5" s="34" t="s">
-        <v>289</v>
-      </c>
-      <c r="F5" s="34" t="s">
-        <v>290</v>
-      </c>
-      <c r="H5" s="34" t="s">
-        <v>291</v>
-      </c>
-      <c r="I5" s="34" t="s">
-        <v>292</v>
+      <c r="E5" s="35" t="s">
+        <v>297</v>
+      </c>
+      <c r="F5" s="35" t="s">
+        <v>298</v>
+      </c>
+      <c r="H5" s="35" t="s">
+        <v>299</v>
+      </c>
+      <c r="I5" s="35" t="s">
+        <v>300</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="9" t="s">
-        <v>293</v>
+        <v>301</v>
       </c>
       <c r="B6" s="21" t="s">
-        <v>294</v>
+        <v>302</v>
       </c>
       <c r="C6" s="6" t="str">
         <f aca="false">IFERROR(INDEX($I$2:$I$52,MATCH(Household!B5,$H$2:$H$52,0)),"")</f>
         <v/>
       </c>
-      <c r="H6" s="34" t="s">
-        <v>295</v>
-      </c>
-      <c r="I6" s="34" t="s">
-        <v>296</v>
+      <c r="H6" s="35" t="s">
+        <v>303</v>
+      </c>
+      <c r="I6" s="35" t="s">
+        <v>304</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="9" t="s">
-        <v>297</v>
+        <v>305</v>
       </c>
       <c r="B7" s="21" t="s">
-        <v>298</v>
+        <v>306</v>
       </c>
       <c r="C7" s="6" t="n">
         <f aca="false">IF(AND(ISNUMBER(Household!B6),Household!B6&gt;0,Household!B6&lt;=1961),1,0)</f>
         <v>0</v>
       </c>
-      <c r="H7" s="34" t="s">
-        <v>299</v>
-      </c>
-      <c r="I7" s="34" t="s">
-        <v>300</v>
+      <c r="H7" s="35" t="s">
+        <v>307</v>
+      </c>
+      <c r="I7" s="35" t="s">
+        <v>308</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="9" t="s">
-        <v>301</v>
+        <v>309</v>
       </c>
       <c r="B8" s="21" t="s">
-        <v>302</v>
+        <v>310</v>
       </c>
       <c r="C8" s="6" t="n">
         <f aca="false">IF(AND(C5="mfj",ISNUMBER(Household!B7),Household!B7&gt;0,Household!B7&lt;=1961),1,0)</f>
         <v>0</v>
       </c>
-      <c r="H8" s="34" t="s">
-        <v>303</v>
-      </c>
-      <c r="I8" s="34" t="s">
-        <v>304</v>
+      <c r="H8" s="35" t="s">
+        <v>311</v>
+      </c>
+      <c r="I8" s="35" t="s">
+        <v>312</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="9" t="s">
-        <v>305</v>
+        <v>313</v>
       </c>
       <c r="B9" s="21" t="s">
-        <v>306</v>
+        <v>314</v>
       </c>
       <c r="C9" s="6" t="n">
         <f aca="false">COUNTIFS(Household!A14:A23,"?*",Household!C14:C23,"&gt;=2010")</f>
         <v>0</v>
       </c>
-      <c r="H9" s="34" t="s">
-        <v>307</v>
-      </c>
-      <c r="I9" s="34" t="s">
-        <v>308</v>
+      <c r="H9" s="35" t="s">
+        <v>315</v>
+      </c>
+      <c r="I9" s="35" t="s">
+        <v>316</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="9" t="s">
-        <v>309</v>
+        <v>317</v>
       </c>
       <c r="B10" s="21" t="s">
-        <v>310</v>
+        <v>318</v>
       </c>
       <c r="C10" s="6" t="n">
         <f aca="false">COUNTIF(Household!A14:A23,"?*")-C9</f>
         <v>0</v>
       </c>
-      <c r="H10" s="34" t="s">
-        <v>311</v>
-      </c>
-      <c r="I10" s="34" t="s">
-        <v>312</v>
+      <c r="H10" s="35" t="s">
+        <v>319</v>
+      </c>
+      <c r="I10" s="35" t="s">
+        <v>320</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="9" t="s">
-        <v>313</v>
+        <v>321</v>
       </c>
       <c r="B11" s="21" t="s">
-        <v>314</v>
+        <v>322</v>
       </c>
       <c r="C11" s="6" t="str">
         <f aca="false">IF(C9+C10&gt;0,"yes","no")</f>
         <v>no</v>
       </c>
-      <c r="H11" s="34" t="s">
-        <v>315</v>
-      </c>
-      <c r="I11" s="34" t="s">
-        <v>316</v>
+      <c r="H11" s="35" t="s">
+        <v>323</v>
+      </c>
+      <c r="I11" s="35" t="s">
+        <v>324</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="9" t="s">
-        <v>317</v>
+        <v>325</v>
       </c>
       <c r="B12" s="21" t="s">
-        <v>318</v>
+        <v>326</v>
       </c>
       <c r="C12" s="6" t="n">
         <f aca="false">IF(TRIM(Household!B8)="Yes",1,0)</f>
         <v>0</v>
       </c>
-      <c r="H12" s="34" t="s">
-        <v>319</v>
-      </c>
-      <c r="I12" s="34" t="s">
-        <v>320</v>
+      <c r="H12" s="35" t="s">
+        <v>327</v>
+      </c>
+      <c r="I12" s="35" t="s">
+        <v>328</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="9" t="s">
-        <v>321</v>
+        <v>329</v>
       </c>
       <c r="B13" s="21" t="s">
-        <v>322</v>
+        <v>330</v>
       </c>
       <c r="C13" s="6" t="n">
         <f aca="false">Jobs!C16+Income!C24</f>
         <v>0</v>
       </c>
-      <c r="H13" s="34" t="s">
-        <v>323</v>
-      </c>
-      <c r="I13" s="34" t="s">
-        <v>324</v>
+      <c r="H13" s="35" t="s">
+        <v>331</v>
+      </c>
+      <c r="I13" s="35" t="s">
+        <v>332</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="9" t="s">
-        <v>325</v>
+        <v>333</v>
       </c>
       <c r="B14" s="21" t="s">
-        <v>326</v>
+        <v>334</v>
       </c>
       <c r="C14" s="6" t="n">
         <f aca="false">Jobs!D16+N(Income!C30)</f>
         <v>0</v>
       </c>
-      <c r="H14" s="34" t="s">
-        <v>327</v>
-      </c>
-      <c r="I14" s="34" t="s">
-        <v>328</v>
+      <c r="H14" s="35" t="s">
+        <v>335</v>
+      </c>
+      <c r="I14" s="35" t="s">
+        <v>336</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="9" t="s">
-        <v>329</v>
+        <v>337</v>
       </c>
       <c r="B15" s="21" t="s">
-        <v>330</v>
-      </c>
-      <c r="C15" s="36" t="n">
+        <v>338</v>
+      </c>
+      <c r="C15" s="37" t="n">
         <f aca="false">Jobs!E16</f>
         <v>0</v>
       </c>
-      <c r="H15" s="34" t="s">
-        <v>331</v>
-      </c>
-      <c r="I15" s="34" t="s">
-        <v>332</v>
+      <c r="H15" s="35" t="s">
+        <v>339</v>
+      </c>
+      <c r="I15" s="35" t="s">
+        <v>340</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="9" t="s">
-        <v>333</v>
+        <v>341</v>
       </c>
       <c r="B16" s="21" t="s">
-        <v>334</v>
+        <v>342</v>
       </c>
       <c r="C16" s="6" t="n">
         <f aca="false">Jobs!F16+Income!C24</f>
         <v>0</v>
       </c>
-      <c r="H16" s="34" t="s">
-        <v>335</v>
-      </c>
-      <c r="I16" s="34" t="s">
-        <v>336</v>
+      <c r="H16" s="35" t="s">
+        <v>343</v>
+      </c>
+      <c r="I16" s="35" t="s">
+        <v>344</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="9" t="s">
-        <v>337</v>
+        <v>345</v>
       </c>
       <c r="B17" s="21" t="s">
-        <v>338</v>
-      </c>
-      <c r="C17" s="36" t="n">
+        <v>346</v>
+      </c>
+      <c r="C17" s="37" t="n">
         <f aca="false">Jobs!G16</f>
         <v>0</v>
       </c>
-      <c r="H17" s="34" t="s">
-        <v>339</v>
-      </c>
-      <c r="I17" s="34" t="s">
-        <v>340</v>
+      <c r="H17" s="35" t="s">
+        <v>347</v>
+      </c>
+      <c r="I17" s="35" t="s">
+        <v>348</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="9" t="s">
-        <v>341</v>
+        <v>349</v>
       </c>
       <c r="B18" s="21" t="s">
-        <v>342</v>
-      </c>
-      <c r="C18" s="36" t="n">
+        <v>350</v>
+      </c>
+      <c r="C18" s="37" t="n">
         <f aca="false">Income!C19</f>
         <v>0</v>
       </c>
-      <c r="H18" s="34" t="s">
-        <v>343</v>
-      </c>
-      <c r="I18" s="34" t="s">
-        <v>344</v>
+      <c r="H18" s="35" t="s">
+        <v>351</v>
+      </c>
+      <c r="I18" s="35" t="s">
+        <v>352</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="9" t="s">
-        <v>345</v>
+        <v>353</v>
       </c>
       <c r="B19" s="21" t="s">
-        <v>346</v>
-      </c>
-      <c r="C19" s="36" t="n">
+        <v>354</v>
+      </c>
+      <c r="C19" s="37" t="n">
         <f aca="false">Expenses!E85</f>
         <v>0</v>
       </c>
-      <c r="H19" s="34" t="s">
-        <v>347</v>
-      </c>
-      <c r="I19" s="34" t="s">
-        <v>348</v>
+      <c r="H19" s="35" t="s">
+        <v>355</v>
+      </c>
+      <c r="I19" s="35" t="s">
+        <v>356</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="9" t="s">
-        <v>349</v>
+        <v>357</v>
       </c>
       <c r="B20" s="21" t="s">
-        <v>350</v>
-      </c>
-      <c r="C20" s="36" t="n">
+        <v>358</v>
+      </c>
+      <c r="C20" s="37" t="n">
         <f aca="false">Payments!B9</f>
         <v>0</v>
       </c>
-      <c r="H20" s="34" t="s">
-        <v>351</v>
-      </c>
-      <c r="I20" s="34" t="s">
-        <v>352</v>
+      <c r="H20" s="35" t="s">
+        <v>359</v>
+      </c>
+      <c r="I20" s="35" t="s">
+        <v>360</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="9" t="s">
-        <v>353</v>
+        <v>361</v>
       </c>
       <c r="B21" s="21" t="s">
-        <v>354</v>
-      </c>
-      <c r="C21" s="36" t="n">
+        <v>362</v>
+      </c>
+      <c r="C21" s="37" t="n">
         <f aca="false">Payments!D9</f>
         <v>0</v>
       </c>
-      <c r="H21" s="34" t="s">
-        <v>355</v>
-      </c>
-      <c r="I21" s="34" t="s">
-        <v>356</v>
+      <c r="H21" s="35" t="s">
+        <v>363</v>
+      </c>
+      <c r="I21" s="35" t="s">
+        <v>364</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="9" t="s">
-        <v>357</v>
+        <v>365</v>
       </c>
       <c r="B22" s="21" t="s">
-        <v>358</v>
+        <v>366</v>
       </c>
       <c r="C22" s="6" t="n">
         <f aca="false">IF(Trips!D36+Trips!E36&gt;0,1,0)</f>
         <v>0</v>
       </c>
-      <c r="H22" s="34" t="s">
-        <v>359</v>
-      </c>
-      <c r="I22" s="34" t="s">
-        <v>360</v>
+      <c r="H22" s="35" t="s">
+        <v>367</v>
+      </c>
+      <c r="I22" s="35" t="s">
+        <v>368</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="9" t="s">
-        <v>361</v>
+        <v>369</v>
       </c>
       <c r="B23" s="21" t="s">
-        <v>362</v>
+        <v>370</v>
       </c>
       <c r="C23" s="6" t="n">
         <f aca="false">MIN(365,Trips!D36)</f>
         <v>0</v>
       </c>
-      <c r="H23" s="34" t="s">
-        <v>363</v>
-      </c>
-      <c r="I23" s="34" t="s">
-        <v>364</v>
+      <c r="H23" s="35" t="s">
+        <v>371</v>
+      </c>
+      <c r="I23" s="35" t="s">
+        <v>372</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="9" t="s">
-        <v>365</v>
+        <v>373</v>
       </c>
       <c r="B24" s="21" t="s">
-        <v>366</v>
+        <v>374</v>
       </c>
       <c r="C24" s="6" t="n">
         <f aca="false">MIN(C23,SUMPRODUCT((Trips!C6:C35&lt;Trips!D6:D35)*Trips!C6:C35+(Trips!C6:C35&gt;=Trips!D6:D35)*Trips!D6:D35))</f>
         <v>0</v>
       </c>
-      <c r="H24" s="34" t="s">
-        <v>367</v>
-      </c>
-      <c r="I24" s="34" t="s">
-        <v>368</v>
+      <c r="H24" s="35" t="s">
+        <v>375</v>
+      </c>
+      <c r="I24" s="35" t="s">
+        <v>376</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="9" t="s">
-        <v>369</v>
+        <v>377</v>
       </c>
       <c r="B25" s="21" t="s">
-        <v>240</v>
-      </c>
-      <c r="C25" s="37" t="n">
+        <v>248</v>
+      </c>
+      <c r="C25" s="38" t="n">
         <f aca="false">Trips!E36</f>
         <v>0</v>
       </c>
-      <c r="H25" s="34" t="s">
-        <v>370</v>
-      </c>
-      <c r="I25" s="34" t="s">
-        <v>371</v>
+      <c r="H25" s="35" t="s">
+        <v>378</v>
+      </c>
+      <c r="I25" s="35" t="s">
+        <v>379</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="9" t="s">
-        <v>372</v>
+        <v>380</v>
       </c>
       <c r="B26" s="21" t="s">
-        <v>373</v>
+        <v>381</v>
       </c>
       <c r="C26" s="6" t="n">
         <f aca="false">IF(N(Car!B5)+N(Car!B6)+N(Car!B18)&gt;0,1,0)</f>
         <v>0</v>
       </c>
-      <c r="H26" s="34" t="s">
-        <v>374</v>
-      </c>
-      <c r="I26" s="34" t="s">
-        <v>375</v>
+      <c r="H26" s="35" t="s">
+        <v>382</v>
+      </c>
+      <c r="I26" s="35" t="s">
+        <v>383</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="9" t="s">
-        <v>376</v>
+        <v>384</v>
       </c>
       <c r="B27" s="21" t="s">
-        <v>377</v>
+        <v>385</v>
       </c>
       <c r="C27" s="6" t="n">
         <f aca="false">N(Car!B5)</f>
         <v>0</v>
       </c>
-      <c r="H27" s="34" t="s">
-        <v>378</v>
-      </c>
-      <c r="I27" s="34" t="s">
-        <v>379</v>
+      <c r="H27" s="35" t="s">
+        <v>386</v>
+      </c>
+      <c r="I27" s="35" t="s">
+        <v>387</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="9" t="s">
-        <v>380</v>
+        <v>388</v>
       </c>
       <c r="B28" s="21" t="s">
-        <v>381</v>
+        <v>389</v>
       </c>
       <c r="C28" s="6" t="n">
         <f aca="false">N(Car!B6)</f>
         <v>0</v>
       </c>
-      <c r="H28" s="34" t="s">
-        <v>382</v>
-      </c>
-      <c r="I28" s="34" t="s">
-        <v>383</v>
+      <c r="H28" s="35" t="s">
+        <v>390</v>
+      </c>
+      <c r="I28" s="35" t="s">
+        <v>391</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="9" t="s">
-        <v>384</v>
+        <v>392</v>
       </c>
       <c r="B29" s="21" t="s">
-        <v>385</v>
+        <v>393</v>
       </c>
       <c r="C29" s="6" t="n">
         <f aca="false">N(Car!B7)</f>
         <v>0</v>
       </c>
-      <c r="H29" s="34" t="s">
-        <v>386</v>
-      </c>
-      <c r="I29" s="34" t="s">
-        <v>387</v>
+      <c r="H29" s="35" t="s">
+        <v>394</v>
+      </c>
+      <c r="I29" s="35" t="s">
+        <v>395</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="9" t="s">
-        <v>388</v>
+        <v>396</v>
       </c>
       <c r="B30" s="21" t="s">
-        <v>389</v>
+        <v>397</v>
       </c>
       <c r="C30" s="6" t="n">
         <f aca="false">N(Car!B18)</f>
         <v>0</v>
       </c>
-      <c r="H30" s="34" t="s">
-        <v>390</v>
-      </c>
-      <c r="I30" s="34" t="s">
-        <v>391</v>
+      <c r="H30" s="35" t="s">
+        <v>398</v>
+      </c>
+      <c r="I30" s="35" t="s">
+        <v>399</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="9" t="s">
-        <v>392</v>
+        <v>400</v>
       </c>
       <c r="B31" s="21" t="s">
         <v>70</v>
       </c>
-      <c r="C31" s="36" t="n">
+      <c r="C31" s="37" t="n">
         <f aca="false">Income!C25</f>
         <v>0</v>
       </c>
-      <c r="H31" s="34" t="s">
-        <v>393</v>
-      </c>
-      <c r="I31" s="34" t="s">
-        <v>394</v>
+      <c r="H31" s="35" t="s">
+        <v>401</v>
+      </c>
+      <c r="I31" s="35" t="s">
+        <v>402</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="9" t="s">
-        <v>395</v>
+        <v>403</v>
       </c>
       <c r="B32" s="21" t="s">
-        <v>396</v>
-      </c>
-      <c r="C32" s="36" t="n">
+        <v>404</v>
+      </c>
+      <c r="C32" s="37" t="n">
         <f aca="false">Income!C26</f>
         <v>0</v>
       </c>
-      <c r="H32" s="34" t="s">
-        <v>397</v>
-      </c>
-      <c r="I32" s="34" t="s">
-        <v>398</v>
+      <c r="H32" s="35" t="s">
+        <v>405</v>
+      </c>
+      <c r="I32" s="35" t="s">
+        <v>406</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="9" t="s">
-        <v>399</v>
+        <v>407</v>
       </c>
       <c r="B33" s="21" t="s">
-        <v>400</v>
+        <v>408</v>
       </c>
       <c r="C33" s="6" t="n">
         <f aca="false">N(Income!C28)</f>
         <v>0</v>
       </c>
-      <c r="H33" s="34" t="s">
-        <v>401</v>
-      </c>
-      <c r="I33" s="34" t="s">
-        <v>402</v>
+      <c r="H33" s="35" t="s">
+        <v>409</v>
+      </c>
+      <c r="I33" s="35" t="s">
+        <v>410</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="9" t="s">
-        <v>403</v>
+        <v>411</v>
       </c>
       <c r="B34" s="21" t="s">
-        <v>404</v>
+        <v>412</v>
       </c>
       <c r="C34" s="6" t="n">
         <f aca="false">N(Income!C27)</f>
         <v>0</v>
       </c>
-      <c r="H34" s="34" t="s">
-        <v>405</v>
-      </c>
-      <c r="I34" s="34" t="s">
-        <v>406</v>
+      <c r="H34" s="35" t="s">
+        <v>413</v>
+      </c>
+      <c r="I34" s="35" t="s">
+        <v>414</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="9" t="s">
-        <v>407</v>
+        <v>415</v>
       </c>
       <c r="B35" s="21" t="s">
-        <v>408</v>
+        <v>416</v>
       </c>
       <c r="C35" s="6" t="n">
         <f aca="false">N(Income!C29)</f>
         <v>0</v>
       </c>
-      <c r="H35" s="34" t="s">
-        <v>409</v>
-      </c>
-      <c r="I35" s="34" t="s">
-        <v>410</v>
+      <c r="H35" s="35" t="s">
+        <v>417</v>
+      </c>
+      <c r="I35" s="35" t="s">
+        <v>418</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="9" t="s">
-        <v>411</v>
+        <v>419</v>
       </c>
       <c r="B36" s="21" t="s">
-        <v>412</v>
+        <v>420</v>
       </c>
       <c r="C36" s="6" t="n">
         <f aca="false">N(Income!C34)</f>
         <v>0</v>
       </c>
-      <c r="H36" s="34" t="s">
-        <v>413</v>
-      </c>
-      <c r="I36" s="34" t="s">
-        <v>414</v>
+      <c r="H36" s="35" t="s">
+        <v>421</v>
+      </c>
+      <c r="I36" s="35" t="s">
+        <v>422</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="9" t="s">
-        <v>415</v>
+        <v>423</v>
       </c>
       <c r="B37" s="21" t="s">
-        <v>416</v>
+        <v>424</v>
       </c>
       <c r="C37" s="6" t="n">
         <f aca="false">N(Income!C35)</f>
         <v>0</v>
       </c>
-      <c r="H37" s="34" t="s">
-        <v>417</v>
-      </c>
-      <c r="I37" s="34" t="s">
-        <v>418</v>
+      <c r="H37" s="35" t="s">
+        <v>425</v>
+      </c>
+      <c r="I37" s="35" t="s">
+        <v>426</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="9" t="s">
-        <v>419</v>
+        <v>427</v>
       </c>
       <c r="B38" s="21" t="s">
-        <v>420</v>
+        <v>428</v>
       </c>
       <c r="C38" s="6" t="n">
         <f aca="false">IF(TRIM(Income!C36)="Yes",1,0)</f>
         <v>0</v>
       </c>
-      <c r="H38" s="34" t="s">
-        <v>421</v>
-      </c>
-      <c r="I38" s="34" t="s">
-        <v>422</v>
+      <c r="H38" s="35" t="s">
+        <v>429</v>
+      </c>
+      <c r="I38" s="35" t="s">
+        <v>430</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="9" t="s">
-        <v>423</v>
+        <v>431</v>
       </c>
       <c r="B39" s="21" t="s">
-        <v>424</v>
+        <v>432</v>
       </c>
       <c r="C39" s="6" t="n">
         <f aca="false">IF(TRIM(Income!C37)="Yes",1,0)</f>
         <v>0</v>
       </c>
-      <c r="H39" s="34" t="s">
-        <v>425</v>
-      </c>
-      <c r="I39" s="34" t="s">
-        <v>426</v>
+      <c r="H39" s="35" t="s">
+        <v>433</v>
+      </c>
+      <c r="I39" s="35" t="s">
+        <v>434</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="9" t="s">
-        <v>427</v>
+        <v>435</v>
       </c>
       <c r="B40" s="21" t="s">
-        <v>428</v>
+        <v>436</v>
       </c>
       <c r="C40" s="6" t="n">
         <f aca="false">N(Income!C38)</f>
         <v>0</v>
       </c>
-      <c r="H40" s="34" t="s">
-        <v>429</v>
-      </c>
-      <c r="I40" s="34" t="s">
-        <v>430</v>
+      <c r="H40" s="35" t="s">
+        <v>437</v>
+      </c>
+      <c r="I40" s="35" t="s">
+        <v>438</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="9" t="s">
-        <v>431</v>
+        <v>439</v>
       </c>
       <c r="B41" s="21" t="s">
-        <v>432</v>
+        <v>440</v>
       </c>
       <c r="C41" s="6" t="n">
         <f aca="false">IF(TRIM(Income!C39)="Family",1,0)</f>
         <v>0</v>
       </c>
-      <c r="H41" s="34" t="s">
-        <v>433</v>
-      </c>
-      <c r="I41" s="34" t="s">
-        <v>434</v>
+      <c r="H41" s="35" t="s">
+        <v>441</v>
+      </c>
+      <c r="I41" s="35" t="s">
+        <v>442</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="9" t="s">
-        <v>435</v>
+        <v>443</v>
       </c>
       <c r="B42" s="21" t="s">
-        <v>436</v>
+        <v>444</v>
       </c>
       <c r="C42" s="6" t="n">
         <f aca="false">N(Income!C40)</f>
         <v>0</v>
       </c>
-      <c r="H42" s="34" t="s">
-        <v>437</v>
-      </c>
-      <c r="I42" s="34" t="s">
-        <v>438</v>
+      <c r="H42" s="35" t="s">
+        <v>445</v>
+      </c>
+      <c r="I42" s="35" t="s">
+        <v>446</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="9" t="s">
-        <v>439</v>
+        <v>447</v>
       </c>
       <c r="B43" s="21" t="s">
-        <v>440</v>
+        <v>448</v>
       </c>
       <c r="C43" s="6" t="n">
-        <f aca="false">IF(AND(ISNUMBER(Household!B6),Household!B6&gt;0,Household!B6&lt;=1976),1,0)</f>
-        <v>0</v>
-      </c>
-      <c r="H43" s="34" t="s">
-        <v>441</v>
-      </c>
-      <c r="I43" s="34" t="s">
-        <v>442</v>
+        <f aca="false">SUMIF(Income!A47:A50,"Partnership / LLC (1065)",Income!C47:C50)</f>
+        <v>0</v>
+      </c>
+      <c r="H43" s="35" t="s">
+        <v>449</v>
+      </c>
+      <c r="I43" s="35" t="s">
+        <v>450</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="9" t="s">
-        <v>443</v>
+        <v>451</v>
       </c>
       <c r="B44" s="21" t="s">
-        <v>444</v>
+        <v>452</v>
       </c>
       <c r="C44" s="6" t="n">
-        <f aca="false">IF(AND(ISNUMBER(Household!B7),Household!B7&gt;0,Household!B7&lt;=1976),1,0)</f>
-        <v>0</v>
-      </c>
-      <c r="H44" s="34" t="s">
-        <v>445</v>
-      </c>
-      <c r="I44" s="34" t="s">
-        <v>446</v>
+        <f aca="false">SUMIF(Income!A47:A50,"Partnership / LLC (1065)",Income!D47:D50)</f>
+        <v>0</v>
+      </c>
+      <c r="H44" s="35" t="s">
+        <v>453</v>
+      </c>
+      <c r="I44" s="35" t="s">
+        <v>454</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="9" t="s">
-        <v>447</v>
+        <v>455</v>
       </c>
       <c r="B45" s="21" t="s">
-        <v>448</v>
+        <v>456</v>
       </c>
       <c r="C45" s="6" t="n">
-        <f aca="false">IF(AND(ISNUMBER(Household!B6),Household!B6&gt;0,Household!B6&lt;=1971),1,0)</f>
-        <v>0</v>
-      </c>
-      <c r="H45" s="34" t="s">
-        <v>449</v>
-      </c>
-      <c r="I45" s="34" t="s">
-        <v>450</v>
+        <f aca="false">SUMIF(Income!A47:A50,"S-corp (1120-S)",Income!C47:C50)</f>
+        <v>0</v>
+      </c>
+      <c r="H45" s="35" t="s">
+        <v>457</v>
+      </c>
+      <c r="I45" s="35" t="s">
+        <v>458</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="9" t="s">
-        <v>451</v>
+        <v>459</v>
       </c>
       <c r="B46" s="21" t="s">
-        <v>452</v>
+        <v>460</v>
       </c>
       <c r="C46" s="6" t="n">
-        <f aca="false">IF(Income!C27&gt;0,1,0)</f>
-        <v>0</v>
-      </c>
-      <c r="H46" s="34" t="s">
-        <v>453</v>
-      </c>
-      <c r="I46" s="34" t="s">
-        <v>454</v>
+        <f aca="false">SUM(Income!F47:F50)</f>
+        <v>0</v>
+      </c>
+      <c r="H46" s="35" t="s">
+        <v>461</v>
+      </c>
+      <c r="I46" s="35" t="s">
+        <v>462</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="9" t="s">
-        <v>455</v>
+        <v>463</v>
       </c>
       <c r="B47" s="21" t="s">
-        <v>259</v>
+        <v>464</v>
       </c>
       <c r="C47" s="6" t="n">
-        <f aca="false">IF(TRIM(Checklist!B4)="Yes",1,0)</f>
-        <v>0</v>
-      </c>
-      <c r="H47" s="34" t="s">
-        <v>456</v>
-      </c>
-      <c r="I47" s="34" t="s">
-        <v>457</v>
+        <f aca="false">IF(AND(ISNUMBER(Household!B6),Household!B6&gt;0,Household!B6&lt;=1976),1,0)</f>
+        <v>0</v>
+      </c>
+      <c r="H47" s="35" t="s">
+        <v>465</v>
+      </c>
+      <c r="I47" s="35" t="s">
+        <v>466</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="9" t="s">
-        <v>458</v>
+        <v>467</v>
       </c>
       <c r="B48" s="21" t="s">
-        <v>260</v>
+        <v>468</v>
       </c>
       <c r="C48" s="6" t="n">
-        <f aca="false">IF(TRIM(Checklist!B5)="Yes",1,0)</f>
-        <v>0</v>
-      </c>
-      <c r="H48" s="34" t="s">
-        <v>459</v>
-      </c>
-      <c r="I48" s="34" t="s">
-        <v>460</v>
+        <f aca="false">IF(AND(ISNUMBER(Household!B7),Household!B7&gt;0,Household!B7&lt;=1976),1,0)</f>
+        <v>0</v>
+      </c>
+      <c r="H48" s="35" t="s">
+        <v>469</v>
+      </c>
+      <c r="I48" s="35" t="s">
+        <v>470</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="9" t="s">
-        <v>461</v>
+        <v>471</v>
       </c>
       <c r="B49" s="21" t="s">
-        <v>261</v>
+        <v>472</v>
       </c>
       <c r="C49" s="6" t="n">
-        <f aca="false">IF(TRIM(Checklist!B6)="Yes",1,0)</f>
-        <v>0</v>
-      </c>
-      <c r="H49" s="34" t="s">
-        <v>462</v>
-      </c>
-      <c r="I49" s="34" t="s">
-        <v>463</v>
+        <f aca="false">IF(AND(ISNUMBER(Household!B6),Household!B6&gt;0,Household!B6&lt;=1971),1,0)</f>
+        <v>0</v>
+      </c>
+      <c r="H49" s="35" t="s">
+        <v>473</v>
+      </c>
+      <c r="I49" s="35" t="s">
+        <v>474</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="9" t="s">
-        <v>464</v>
+        <v>475</v>
       </c>
       <c r="B50" s="21" t="s">
-        <v>262</v>
+        <v>476</v>
       </c>
       <c r="C50" s="6" t="n">
-        <f aca="false">IF(TRIM(Checklist!B7)="Yes",1,0)</f>
-        <v>0</v>
-      </c>
-      <c r="H50" s="34" t="s">
-        <v>465</v>
-      </c>
-      <c r="I50" s="34" t="s">
-        <v>466</v>
+        <f aca="false">IF(Income!C27&gt;0,1,0)</f>
+        <v>0</v>
+      </c>
+      <c r="H50" s="35" t="s">
+        <v>477</v>
+      </c>
+      <c r="I50" s="35" t="s">
+        <v>478</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="9" t="s">
-        <v>467</v>
+        <v>479</v>
       </c>
       <c r="B51" s="21" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="C51" s="6" t="n">
-        <f aca="false">IF(TRIM(Checklist!B8)="Yes",1,0)</f>
-        <v>0</v>
-      </c>
-      <c r="H51" s="34" t="s">
-        <v>468</v>
-      </c>
-      <c r="I51" s="34" t="s">
-        <v>469</v>
+        <f aca="false">IF(TRIM(Checklist!B4)="Yes",1,0)</f>
+        <v>0</v>
+      </c>
+      <c r="H51" s="35" t="s">
+        <v>480</v>
+      </c>
+      <c r="I51" s="35" t="s">
+        <v>481</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="9" t="s">
-        <v>470</v>
+        <v>482</v>
       </c>
       <c r="B52" s="21" t="s">
-        <v>264</v>
+        <v>268</v>
       </c>
       <c r="C52" s="6" t="n">
-        <f aca="false">IF(TRIM(Checklist!B9)="Yes",1,0)</f>
-        <v>0</v>
-      </c>
-      <c r="H52" s="34" t="s">
-        <v>471</v>
-      </c>
-      <c r="I52" s="34" t="s">
-        <v>472</v>
+        <f aca="false">IF(TRIM(Checklist!B5)="Yes",1,0)</f>
+        <v>0</v>
+      </c>
+      <c r="H52" s="35" t="s">
+        <v>483</v>
+      </c>
+      <c r="I52" s="35" t="s">
+        <v>484</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="9" t="s">
-        <v>473</v>
+        <v>485</v>
       </c>
       <c r="B53" s="21" t="s">
-        <v>265</v>
+        <v>269</v>
       </c>
       <c r="C53" s="6" t="n">
+        <f aca="false">IF(TRIM(Checklist!B6)="Yes",1,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A54" s="9" t="s">
+        <v>486</v>
+      </c>
+      <c r="B54" s="21" t="s">
+        <v>270</v>
+      </c>
+      <c r="C54" s="6" t="n">
+        <f aca="false">IF(TRIM(Checklist!B7)="Yes",1,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A55" s="9" t="s">
+        <v>487</v>
+      </c>
+      <c r="B55" s="21" t="s">
+        <v>271</v>
+      </c>
+      <c r="C55" s="6" t="n">
+        <f aca="false">IF(TRIM(Checklist!B8)="Yes",1,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A56" s="9" t="s">
+        <v>488</v>
+      </c>
+      <c r="B56" s="21" t="s">
+        <v>272</v>
+      </c>
+      <c r="C56" s="6" t="n">
+        <f aca="false">IF(TRIM(Checklist!B9)="Yes",1,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A57" s="9" t="s">
+        <v>489</v>
+      </c>
+      <c r="B57" s="21" t="s">
+        <v>273</v>
+      </c>
+      <c r="C57" s="6" t="n">
         <f aca="false">IF(TRIM(Checklist!B10)="Yes",1,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A59" s="38" t="s">
-        <v>474</v>
+      <c r="A59" s="39" t="s">
+        <v>490</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B60" s="6" t="s">
-        <v>475</v>
-      </c>
-      <c r="C60" s="39" t="n">
+        <v>491</v>
+      </c>
+      <c r="C60" s="40" t="n">
         <v>80</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B61" s="6" t="s">
-        <v>476</v>
-      </c>
-      <c r="C61" s="39" t="n">
+        <v>492</v>
+      </c>
+      <c r="C61" s="40" t="n">
         <v>86</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B62" s="6" t="s">
-        <v>477</v>
-      </c>
-      <c r="C62" s="40" t="n">
+        <v>493</v>
+      </c>
+      <c r="C62" s="41" t="n">
         <v>0.75</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B63" s="6" t="s">
-        <v>478</v>
-      </c>
-      <c r="C63" s="40" t="n">
+        <v>494</v>
+      </c>
+      <c r="C63" s="41" t="n">
         <v>0.8</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A65" s="38" t="s">
-        <v>479</v>
+      <c r="A65" s="39" t="s">
+        <v>495</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B66" s="6" t="s">
-        <v>480</v>
-      </c>
-      <c r="C66" s="41" t="n">
+        <v>496</v>
+      </c>
+      <c r="C66" s="42" t="n">
         <v>0.725</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B67" s="6" t="s">
-        <v>481</v>
-      </c>
-      <c r="C67" s="41" t="n">
+        <v>497</v>
+      </c>
+      <c r="C67" s="42" t="n">
         <v>0.76</v>
       </c>
     </row>
@@ -3797,11 +3897,13 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:C43"/>
+  <dimension ref="A1:F53"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="44"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="0" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="4" style="0" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="16"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4081,12 +4183,100 @@
       <c r="B43" s="17"/>
       <c r="C43" s="17"/>
     </row>
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="13" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="46" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A46" s="14" t="s">
+        <v>97</v>
+      </c>
+      <c r="B46" s="14" t="s">
+        <v>98</v>
+      </c>
+      <c r="C46" s="14" t="s">
+        <v>99</v>
+      </c>
+      <c r="D46" s="14" t="s">
+        <v>100</v>
+      </c>
+      <c r="E46" s="14" t="s">
+        <v>101</v>
+      </c>
+      <c r="F46" s="14" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A47" s="10"/>
+      <c r="B47" s="10"/>
+      <c r="C47" s="19"/>
+      <c r="D47" s="19"/>
+      <c r="E47" s="19"/>
+      <c r="F47" s="22" t="n">
+        <f aca="false">IF(A47="Partnership / LLC (1065)",IF(E47="",N(C47)+N(D47),N(E47)),0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A48" s="10"/>
+      <c r="B48" s="10"/>
+      <c r="C48" s="19"/>
+      <c r="D48" s="19"/>
+      <c r="E48" s="19"/>
+      <c r="F48" s="22" t="n">
+        <f aca="false">IF(A48="Partnership / LLC (1065)",IF(E48="",N(C48)+N(D48),N(E48)),0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A49" s="10"/>
+      <c r="B49" s="10"/>
+      <c r="C49" s="19"/>
+      <c r="D49" s="19"/>
+      <c r="E49" s="19"/>
+      <c r="F49" s="22" t="n">
+        <f aca="false">IF(A49="Partnership / LLC (1065)",IF(E49="",N(C49)+N(D49),N(E49)),0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A50" s="10"/>
+      <c r="B50" s="10"/>
+      <c r="C50" s="19"/>
+      <c r="D50" s="19"/>
+      <c r="E50" s="19"/>
+      <c r="F50" s="22" t="n">
+        <f aca="false">IF(A50="Partnership / LLC (1065)",IF(E50="",N(C50)+N(D50),N(E50)),0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A52" s="17" t="s">
+        <v>103</v>
+      </c>
+      <c r="B52" s="17"/>
+      <c r="C52" s="17"/>
+      <c r="D52" s="17"/>
+      <c r="E52" s="17"/>
+      <c r="F52" s="17"/>
+    </row>
+    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A53" s="17"/>
+      <c r="B53" s="17"/>
+      <c r="C53" s="17"/>
+      <c r="D53" s="17"/>
+      <c r="E53" s="17"/>
+      <c r="F53" s="17"/>
+    </row>
   </sheetData>
   <sheetProtection sheet="true" formatColumns="false" formatRows="false"/>
-  <mergeCells count="1">
+  <mergeCells count="2">
     <mergeCell ref="A42:C43"/>
+    <mergeCell ref="A52:F53"/>
   </mergeCells>
-  <dataValidations count="3">
+  <dataValidations count="4">
     <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="B7:B18" type="list">
       <formula1>"1099-NEC,1099-K,Cash,Zelle / app,Check,Other"</formula1>
       <formula2>0</formula2>
@@ -4097,6 +4287,10 @@
     </dataValidation>
     <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="C39" type="list">
       <formula1>"Self-only,Family"</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="A47:A50" type="list">
+      <formula1>"Partnership / LLC (1065),S-corp (1120-S)"</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
@@ -4128,45 +4322,45 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>96</v>
+        <v>104</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>97</v>
+        <v>105</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="14" t="s">
-        <v>98</v>
+        <v>106</v>
       </c>
       <c r="B4" s="14" t="s">
-        <v>99</v>
+        <v>107</v>
       </c>
       <c r="C4" s="14" t="s">
-        <v>100</v>
+        <v>108</v>
       </c>
       <c r="D4" s="14" t="s">
-        <v>101</v>
+        <v>109</v>
       </c>
       <c r="E4" s="14" t="s">
-        <v>102</v>
+        <v>110</v>
       </c>
       <c r="F4" s="14" t="s">
-        <v>103</v>
+        <v>111</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="15" t="s">
-        <v>104</v>
+        <v>112</v>
       </c>
       <c r="B5" s="15" t="s">
-        <v>105</v>
+        <v>113</v>
       </c>
       <c r="C5" s="18" t="n">
         <v>1250</v>
       </c>
-      <c r="D5" s="22" t="n">
+      <c r="D5" s="23" t="n">
         <v>1</v>
       </c>
       <c r="E5" s="18" t="n">
@@ -4175,1180 +4369,1180 @@
       <c r="F5" s="15"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="23" t="s">
-        <v>106</v>
+      <c r="A6" s="24" t="s">
+        <v>114</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>107</v>
+        <v>115</v>
       </c>
       <c r="B7" s="21" t="s">
-        <v>108</v>
+        <v>116</v>
       </c>
       <c r="C7" s="19"/>
-      <c r="D7" s="24" t="n">
-        <v>1</v>
-      </c>
-      <c r="E7" s="25" t="n">
+      <c r="D7" s="25" t="n">
+        <v>1</v>
+      </c>
+      <c r="E7" s="26" t="n">
         <f aca="false">C7*D7</f>
         <v>0</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>109</v>
+        <v>117</v>
       </c>
       <c r="B8" s="21" t="s">
-        <v>110</v>
+        <v>118</v>
       </c>
       <c r="C8" s="19"/>
-      <c r="D8" s="24" t="n">
-        <v>1</v>
-      </c>
-      <c r="E8" s="25" t="n">
+      <c r="D8" s="25" t="n">
+        <v>1</v>
+      </c>
+      <c r="E8" s="26" t="n">
         <f aca="false">C8*D8</f>
         <v>0</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="s">
-        <v>111</v>
+        <v>119</v>
       </c>
       <c r="B9" s="21" t="s">
-        <v>112</v>
+        <v>120</v>
       </c>
       <c r="C9" s="19"/>
-      <c r="D9" s="24" t="n">
-        <v>1</v>
-      </c>
-      <c r="E9" s="25" t="n">
+      <c r="D9" s="25" t="n">
+        <v>1</v>
+      </c>
+      <c r="E9" s="26" t="n">
         <f aca="false">C9*D9</f>
         <v>0</v>
       </c>
       <c r="F9" s="11" t="s">
-        <v>113</v>
+        <v>121</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="6" t="s">
-        <v>114</v>
+        <v>122</v>
       </c>
       <c r="B10" s="21" t="s">
-        <v>115</v>
+        <v>123</v>
       </c>
       <c r="C10" s="19"/>
-      <c r="D10" s="24" t="n">
-        <v>1</v>
-      </c>
-      <c r="E10" s="25" t="n">
+      <c r="D10" s="25" t="n">
+        <v>1</v>
+      </c>
+      <c r="E10" s="26" t="n">
         <f aca="false">C10*D10</f>
         <v>0</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="6" t="s">
-        <v>116</v>
+        <v>124</v>
       </c>
       <c r="B11" s="21" t="s">
-        <v>117</v>
+        <v>125</v>
       </c>
       <c r="C11" s="19"/>
-      <c r="D11" s="24" t="n">
-        <v>1</v>
-      </c>
-      <c r="E11" s="25" t="n">
+      <c r="D11" s="25" t="n">
+        <v>1</v>
+      </c>
+      <c r="E11" s="26" t="n">
         <f aca="false">C11*D11</f>
         <v>0</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="6" t="s">
-        <v>118</v>
+        <v>126</v>
       </c>
       <c r="B12" s="21" t="s">
-        <v>119</v>
+        <v>127</v>
       </c>
       <c r="C12" s="19"/>
-      <c r="D12" s="24" t="n">
-        <v>1</v>
-      </c>
-      <c r="E12" s="25" t="n">
+      <c r="D12" s="25" t="n">
+        <v>1</v>
+      </c>
+      <c r="E12" s="26" t="n">
         <f aca="false">C12*D12</f>
         <v>0</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="6" t="s">
-        <v>120</v>
+        <v>128</v>
       </c>
       <c r="B13" s="21" t="s">
-        <v>121</v>
+        <v>129</v>
       </c>
       <c r="C13" s="19"/>
-      <c r="D13" s="24" t="n">
-        <v>1</v>
-      </c>
-      <c r="E13" s="25" t="n">
+      <c r="D13" s="25" t="n">
+        <v>1</v>
+      </c>
+      <c r="E13" s="26" t="n">
         <f aca="false">C13*D13</f>
         <v>0</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="6" t="s">
-        <v>122</v>
+        <v>130</v>
       </c>
       <c r="B14" s="21" t="s">
-        <v>123</v>
+        <v>131</v>
       </c>
       <c r="C14" s="19"/>
-      <c r="D14" s="24" t="n">
-        <v>1</v>
-      </c>
-      <c r="E14" s="25" t="n">
+      <c r="D14" s="25" t="n">
+        <v>1</v>
+      </c>
+      <c r="E14" s="26" t="n">
         <f aca="false">C14*D14</f>
         <v>0</v>
       </c>
       <c r="F14" s="11" t="s">
-        <v>124</v>
+        <v>132</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="6" t="s">
-        <v>125</v>
+        <v>133</v>
       </c>
       <c r="B15" s="21" t="s">
-        <v>126</v>
+        <v>134</v>
       </c>
       <c r="C15" s="19"/>
-      <c r="D15" s="24" t="n">
-        <v>1</v>
-      </c>
-      <c r="E15" s="25" t="n">
+      <c r="D15" s="25" t="n">
+        <v>1</v>
+      </c>
+      <c r="E15" s="26" t="n">
         <f aca="false">C15*D15</f>
         <v>0</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="6" t="s">
-        <v>127</v>
+        <v>135</v>
       </c>
       <c r="B16" s="21" t="s">
-        <v>128</v>
+        <v>136</v>
       </c>
       <c r="C16" s="19"/>
-      <c r="D16" s="24" t="n">
-        <v>1</v>
-      </c>
-      <c r="E16" s="25" t="n">
+      <c r="D16" s="25" t="n">
+        <v>1</v>
+      </c>
+      <c r="E16" s="26" t="n">
         <f aca="false">C16*D16</f>
         <v>0</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="6" t="s">
-        <v>129</v>
+        <v>137</v>
       </c>
       <c r="B17" s="21" t="s">
-        <v>130</v>
+        <v>138</v>
       </c>
       <c r="C17" s="19"/>
-      <c r="D17" s="24" t="n">
+      <c r="D17" s="25" t="n">
         <v>0.5</v>
       </c>
-      <c r="E17" s="25" t="n">
+      <c r="E17" s="26" t="n">
         <f aca="false">C17*D17</f>
         <v>0</v>
       </c>
       <c r="F17" s="11" t="s">
-        <v>131</v>
+        <v>139</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="6" t="s">
-        <v>132</v>
+        <v>140</v>
       </c>
       <c r="B18" s="21" t="s">
-        <v>133</v>
+        <v>141</v>
       </c>
       <c r="C18" s="19"/>
-      <c r="D18" s="24" t="n">
-        <v>1</v>
-      </c>
-      <c r="E18" s="25" t="n">
+      <c r="D18" s="25" t="n">
+        <v>1</v>
+      </c>
+      <c r="E18" s="26" t="n">
         <f aca="false">C18*D18</f>
         <v>0</v>
       </c>
       <c r="F18" s="11" t="s">
-        <v>134</v>
+        <v>142</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="6" t="s">
-        <v>135</v>
+        <v>143</v>
       </c>
       <c r="B19" s="21" t="s">
-        <v>136</v>
+        <v>144</v>
       </c>
       <c r="C19" s="19"/>
-      <c r="D19" s="24" t="n">
-        <v>1</v>
-      </c>
-      <c r="E19" s="25" t="n">
+      <c r="D19" s="25" t="n">
+        <v>1</v>
+      </c>
+      <c r="E19" s="26" t="n">
         <f aca="false">C19*D19</f>
         <v>0</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="6" t="s">
-        <v>137</v>
+        <v>145</v>
       </c>
       <c r="B20" s="21" t="s">
-        <v>138</v>
+        <v>146</v>
       </c>
       <c r="C20" s="19"/>
-      <c r="D20" s="24" t="n">
-        <v>1</v>
-      </c>
-      <c r="E20" s="25" t="n">
+      <c r="D20" s="25" t="n">
+        <v>1</v>
+      </c>
+      <c r="E20" s="26" t="n">
         <f aca="false">C20*D20</f>
         <v>0</v>
       </c>
       <c r="F20" s="11" t="s">
-        <v>139</v>
+        <v>147</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="6" t="s">
-        <v>140</v>
+        <v>148</v>
       </c>
       <c r="B21" s="21" t="s">
-        <v>138</v>
+        <v>146</v>
       </c>
       <c r="C21" s="19"/>
-      <c r="D21" s="24" t="n">
-        <v>1</v>
-      </c>
-      <c r="E21" s="25" t="n">
+      <c r="D21" s="25" t="n">
+        <v>1</v>
+      </c>
+      <c r="E21" s="26" t="n">
         <f aca="false">C21*D21</f>
         <v>0</v>
       </c>
       <c r="F21" s="11" t="s">
-        <v>141</v>
+        <v>149</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="6" t="s">
-        <v>142</v>
+        <v>150</v>
       </c>
       <c r="B22" s="21" t="s">
-        <v>143</v>
+        <v>151</v>
       </c>
       <c r="C22" s="19"/>
-      <c r="D22" s="24" t="n">
-        <v>1</v>
-      </c>
-      <c r="E22" s="25" t="n">
+      <c r="D22" s="25" t="n">
+        <v>1</v>
+      </c>
+      <c r="E22" s="26" t="n">
         <f aca="false">C22*D22</f>
         <v>0</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="6" t="s">
-        <v>144</v>
+        <v>152</v>
       </c>
       <c r="B23" s="21" t="s">
-        <v>145</v>
+        <v>153</v>
       </c>
       <c r="C23" s="19"/>
-      <c r="D23" s="24" t="n">
-        <v>1</v>
-      </c>
-      <c r="E23" s="25" t="n">
+      <c r="D23" s="25" t="n">
+        <v>1</v>
+      </c>
+      <c r="E23" s="26" t="n">
         <f aca="false">C23*D23</f>
         <v>0</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="6" t="s">
-        <v>146</v>
+        <v>154</v>
       </c>
       <c r="B24" s="21" t="s">
-        <v>136</v>
+        <v>144</v>
       </c>
       <c r="C24" s="19"/>
-      <c r="D24" s="24" t="n">
-        <v>1</v>
-      </c>
-      <c r="E24" s="25" t="n">
+      <c r="D24" s="25" t="n">
+        <v>1</v>
+      </c>
+      <c r="E24" s="26" t="n">
         <f aca="false">C24*D24</f>
         <v>0</v>
       </c>
       <c r="F24" s="11" t="s">
-        <v>147</v>
+        <v>155</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="6" t="s">
-        <v>148</v>
+        <v>156</v>
       </c>
       <c r="B25" s="21" t="s">
-        <v>121</v>
+        <v>129</v>
       </c>
       <c r="C25" s="19"/>
-      <c r="D25" s="24" t="n">
-        <v>1</v>
-      </c>
-      <c r="E25" s="25" t="n">
+      <c r="D25" s="25" t="n">
+        <v>1</v>
+      </c>
+      <c r="E25" s="26" t="n">
         <f aca="false">C25*D25</f>
         <v>0</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="6" t="s">
-        <v>149</v>
+        <v>157</v>
       </c>
       <c r="B26" s="21" t="s">
-        <v>133</v>
+        <v>141</v>
       </c>
       <c r="C26" s="19"/>
-      <c r="D26" s="24" t="n">
-        <v>1</v>
-      </c>
-      <c r="E26" s="25" t="n">
+      <c r="D26" s="25" t="n">
+        <v>1</v>
+      </c>
+      <c r="E26" s="26" t="n">
         <f aca="false">C26*D26</f>
         <v>0</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="6" t="s">
-        <v>150</v>
+        <v>158</v>
       </c>
       <c r="B27" s="21" t="s">
-        <v>136</v>
+        <v>144</v>
       </c>
       <c r="C27" s="19"/>
-      <c r="D27" s="24" t="n">
-        <v>1</v>
-      </c>
-      <c r="E27" s="25" t="n">
+      <c r="D27" s="25" t="n">
+        <v>1</v>
+      </c>
+      <c r="E27" s="26" t="n">
         <f aca="false">C27*D27</f>
         <v>0</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="6" t="s">
-        <v>151</v>
+        <v>159</v>
       </c>
       <c r="B28" s="21" t="s">
-        <v>136</v>
+        <v>144</v>
       </c>
       <c r="C28" s="19"/>
-      <c r="D28" s="24" t="n">
-        <v>1</v>
-      </c>
-      <c r="E28" s="25" t="n">
+      <c r="D28" s="25" t="n">
+        <v>1</v>
+      </c>
+      <c r="E28" s="26" t="n">
         <f aca="false">C28*D28</f>
         <v>0</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="6" t="s">
-        <v>152</v>
+        <v>160</v>
       </c>
       <c r="B29" s="21" t="s">
-        <v>153</v>
+        <v>161</v>
       </c>
       <c r="C29" s="19"/>
-      <c r="D29" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="E29" s="25" t="n">
+      <c r="D29" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="E29" s="26" t="n">
         <f aca="false">C29*D29</f>
         <v>0</v>
       </c>
       <c r="F29" s="11" t="s">
-        <v>154</v>
+        <v>162</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="23" t="s">
-        <v>155</v>
+      <c r="A30" s="24" t="s">
+        <v>163</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="6" t="s">
-        <v>156</v>
+        <v>164</v>
       </c>
       <c r="B31" s="21" t="s">
-        <v>110</v>
+        <v>118</v>
       </c>
       <c r="C31" s="19"/>
-      <c r="D31" s="24" t="n">
-        <v>1</v>
-      </c>
-      <c r="E31" s="25" t="n">
+      <c r="D31" s="25" t="n">
+        <v>1</v>
+      </c>
+      <c r="E31" s="26" t="n">
         <f aca="false">C31*D31</f>
         <v>0</v>
       </c>
       <c r="F31" s="11" t="s">
-        <v>157</v>
+        <v>165</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="6" t="s">
-        <v>158</v>
+        <v>166</v>
       </c>
       <c r="B32" s="21" t="s">
-        <v>105</v>
+        <v>113</v>
       </c>
       <c r="C32" s="19"/>
-      <c r="D32" s="24" t="n">
-        <v>1</v>
-      </c>
-      <c r="E32" s="25" t="n">
+      <c r="D32" s="25" t="n">
+        <v>1</v>
+      </c>
+      <c r="E32" s="26" t="n">
         <f aca="false">C32*D32</f>
         <v>0</v>
       </c>
       <c r="F32" s="11" t="s">
-        <v>159</v>
+        <v>167</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="6" t="s">
-        <v>160</v>
+        <v>168</v>
       </c>
       <c r="B33" s="21" t="s">
-        <v>138</v>
+        <v>146</v>
       </c>
       <c r="C33" s="19"/>
-      <c r="D33" s="24" t="n">
-        <v>1</v>
-      </c>
-      <c r="E33" s="25" t="n">
+      <c r="D33" s="25" t="n">
+        <v>1</v>
+      </c>
+      <c r="E33" s="26" t="n">
         <f aca="false">C33*D33</f>
         <v>0</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="6" t="s">
-        <v>161</v>
+        <v>169</v>
       </c>
       <c r="B34" s="21" t="s">
-        <v>138</v>
+        <v>146</v>
       </c>
       <c r="C34" s="19"/>
-      <c r="D34" s="24" t="n">
-        <v>1</v>
-      </c>
-      <c r="E34" s="25" t="n">
+      <c r="D34" s="25" t="n">
+        <v>1</v>
+      </c>
+      <c r="E34" s="26" t="n">
         <f aca="false">C34*D34</f>
         <v>0</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="6" t="s">
-        <v>162</v>
+        <v>170</v>
       </c>
       <c r="B35" s="21" t="s">
-        <v>138</v>
+        <v>146</v>
       </c>
       <c r="C35" s="19"/>
-      <c r="D35" s="24" t="n">
-        <v>1</v>
-      </c>
-      <c r="E35" s="25" t="n">
+      <c r="D35" s="25" t="n">
+        <v>1</v>
+      </c>
+      <c r="E35" s="26" t="n">
         <f aca="false">C35*D35</f>
         <v>0</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="6" t="s">
-        <v>163</v>
+        <v>171</v>
       </c>
       <c r="B36" s="21" t="s">
-        <v>126</v>
+        <v>134</v>
       </c>
       <c r="C36" s="19"/>
-      <c r="D36" s="24" t="n">
-        <v>1</v>
-      </c>
-      <c r="E36" s="25" t="n">
+      <c r="D36" s="25" t="n">
+        <v>1</v>
+      </c>
+      <c r="E36" s="26" t="n">
         <f aca="false">C36*D36</f>
         <v>0</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="23" t="s">
-        <v>164</v>
+      <c r="A37" s="24" t="s">
+        <v>172</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="6" t="s">
-        <v>165</v>
+        <v>173</v>
       </c>
       <c r="B38" s="21" t="s">
-        <v>105</v>
+        <v>113</v>
       </c>
       <c r="C38" s="19"/>
-      <c r="D38" s="24" t="n">
-        <v>1</v>
-      </c>
-      <c r="E38" s="25" t="n">
+      <c r="D38" s="25" t="n">
+        <v>1</v>
+      </c>
+      <c r="E38" s="26" t="n">
         <f aca="false">C38*D38</f>
         <v>0</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="6" t="s">
-        <v>166</v>
+        <v>174</v>
       </c>
       <c r="B39" s="21" t="s">
-        <v>105</v>
+        <v>113</v>
       </c>
       <c r="C39" s="19"/>
-      <c r="D39" s="24" t="n">
-        <v>1</v>
-      </c>
-      <c r="E39" s="25" t="n">
+      <c r="D39" s="25" t="n">
+        <v>1</v>
+      </c>
+      <c r="E39" s="26" t="n">
         <f aca="false">C39*D39</f>
         <v>0</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="6" t="s">
-        <v>167</v>
+        <v>175</v>
       </c>
       <c r="B40" s="21" t="s">
-        <v>126</v>
+        <v>134</v>
       </c>
       <c r="C40" s="19"/>
-      <c r="D40" s="24" t="n">
-        <v>1</v>
-      </c>
-      <c r="E40" s="25" t="n">
+      <c r="D40" s="25" t="n">
+        <v>1</v>
+      </c>
+      <c r="E40" s="26" t="n">
         <f aca="false">C40*D40</f>
         <v>0</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="6" t="s">
-        <v>168</v>
+        <v>176</v>
       </c>
       <c r="B41" s="21" t="s">
-        <v>126</v>
+        <v>134</v>
       </c>
       <c r="C41" s="19"/>
-      <c r="D41" s="24" t="n">
-        <v>1</v>
-      </c>
-      <c r="E41" s="25" t="n">
+      <c r="D41" s="25" t="n">
+        <v>1</v>
+      </c>
+      <c r="E41" s="26" t="n">
         <f aca="false">C41*D41</f>
         <v>0</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="6" t="s">
-        <v>169</v>
+        <v>177</v>
       </c>
       <c r="B42" s="21" t="s">
-        <v>126</v>
+        <v>134</v>
       </c>
       <c r="C42" s="19"/>
-      <c r="D42" s="24" t="n">
-        <v>1</v>
-      </c>
-      <c r="E42" s="25" t="n">
+      <c r="D42" s="25" t="n">
+        <v>1</v>
+      </c>
+      <c r="E42" s="26" t="n">
         <f aca="false">C42*D42</f>
         <v>0</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="6" t="s">
-        <v>170</v>
+        <v>178</v>
       </c>
       <c r="B43" s="21" t="s">
-        <v>126</v>
+        <v>134</v>
       </c>
       <c r="C43" s="19"/>
-      <c r="D43" s="24" t="n">
-        <v>1</v>
-      </c>
-      <c r="E43" s="25" t="n">
+      <c r="D43" s="25" t="n">
+        <v>1</v>
+      </c>
+      <c r="E43" s="26" t="n">
         <f aca="false">C43*D43</f>
         <v>0</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="6" t="s">
-        <v>171</v>
+        <v>179</v>
       </c>
       <c r="B44" s="21" t="s">
-        <v>126</v>
+        <v>134</v>
       </c>
       <c r="C44" s="19"/>
-      <c r="D44" s="24" t="n">
-        <v>1</v>
-      </c>
-      <c r="E44" s="25" t="n">
+      <c r="D44" s="25" t="n">
+        <v>1</v>
+      </c>
+      <c r="E44" s="26" t="n">
         <f aca="false">C44*D44</f>
         <v>0</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="6" t="s">
-        <v>172</v>
+        <v>180</v>
       </c>
       <c r="B45" s="21" t="s">
-        <v>126</v>
+        <v>134</v>
       </c>
       <c r="C45" s="19"/>
-      <c r="D45" s="24" t="n">
-        <v>1</v>
-      </c>
-      <c r="E45" s="25" t="n">
+      <c r="D45" s="25" t="n">
+        <v>1</v>
+      </c>
+      <c r="E45" s="26" t="n">
         <f aca="false">C45*D45</f>
         <v>0</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="6" t="s">
-        <v>173</v>
+        <v>181</v>
       </c>
       <c r="B46" s="21" t="s">
-        <v>126</v>
+        <v>134</v>
       </c>
       <c r="C46" s="19"/>
-      <c r="D46" s="24" t="n">
-        <v>1</v>
-      </c>
-      <c r="E46" s="25" t="n">
+      <c r="D46" s="25" t="n">
+        <v>1</v>
+      </c>
+      <c r="E46" s="26" t="n">
         <f aca="false">C46*D46</f>
         <v>0</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="6" t="s">
-        <v>174</v>
+        <v>182</v>
       </c>
       <c r="B47" s="21" t="s">
-        <v>115</v>
+        <v>123</v>
       </c>
       <c r="C47" s="19"/>
-      <c r="D47" s="24" t="n">
-        <v>1</v>
-      </c>
-      <c r="E47" s="25" t="n">
+      <c r="D47" s="25" t="n">
+        <v>1</v>
+      </c>
+      <c r="E47" s="26" t="n">
         <f aca="false">C47*D47</f>
         <v>0</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="6" t="s">
-        <v>175</v>
+        <v>183</v>
       </c>
       <c r="B48" s="21" t="s">
-        <v>143</v>
+        <v>151</v>
       </c>
       <c r="C48" s="19"/>
-      <c r="D48" s="24" t="n">
-        <v>1</v>
-      </c>
-      <c r="E48" s="25" t="n">
+      <c r="D48" s="25" t="n">
+        <v>1</v>
+      </c>
+      <c r="E48" s="26" t="n">
         <f aca="false">C48*D48</f>
         <v>0</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="6" t="s">
-        <v>176</v>
+        <v>184</v>
       </c>
       <c r="B49" s="21" t="s">
-        <v>117</v>
+        <v>125</v>
       </c>
       <c r="C49" s="19"/>
-      <c r="D49" s="24" t="n">
-        <v>1</v>
-      </c>
-      <c r="E49" s="25" t="n">
+      <c r="D49" s="25" t="n">
+        <v>1</v>
+      </c>
+      <c r="E49" s="26" t="n">
         <f aca="false">C49*D49</f>
         <v>0</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="6" t="s">
-        <v>177</v>
+        <v>185</v>
       </c>
       <c r="B50" s="21" t="s">
-        <v>105</v>
+        <v>113</v>
       </c>
       <c r="C50" s="19"/>
-      <c r="D50" s="24" t="n">
-        <v>1</v>
-      </c>
-      <c r="E50" s="25" t="n">
+      <c r="D50" s="25" t="n">
+        <v>1</v>
+      </c>
+      <c r="E50" s="26" t="n">
         <f aca="false">C50*D50</f>
         <v>0</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="6" t="s">
-        <v>178</v>
+        <v>186</v>
       </c>
       <c r="B51" s="21" t="s">
-        <v>136</v>
+        <v>144</v>
       </c>
       <c r="C51" s="19"/>
-      <c r="D51" s="24" t="n">
-        <v>1</v>
-      </c>
-      <c r="E51" s="25" t="n">
+      <c r="D51" s="25" t="n">
+        <v>1</v>
+      </c>
+      <c r="E51" s="26" t="n">
         <f aca="false">C51*D51</f>
         <v>0</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="6" t="s">
-        <v>179</v>
+        <v>187</v>
       </c>
       <c r="B52" s="21" t="s">
-        <v>136</v>
+        <v>144</v>
       </c>
       <c r="C52" s="19"/>
-      <c r="D52" s="24" t="n">
-        <v>1</v>
-      </c>
-      <c r="E52" s="25" t="n">
+      <c r="D52" s="25" t="n">
+        <v>1</v>
+      </c>
+      <c r="E52" s="26" t="n">
         <f aca="false">C52*D52</f>
         <v>0</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="6" t="s">
-        <v>180</v>
+        <v>188</v>
       </c>
       <c r="B53" s="21" t="s">
-        <v>110</v>
+        <v>118</v>
       </c>
       <c r="C53" s="19"/>
-      <c r="D53" s="24" t="n">
-        <v>1</v>
-      </c>
-      <c r="E53" s="25" t="n">
+      <c r="D53" s="25" t="n">
+        <v>1</v>
+      </c>
+      <c r="E53" s="26" t="n">
         <f aca="false">C53*D53</f>
         <v>0</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="6" t="s">
-        <v>181</v>
+        <v>189</v>
       </c>
       <c r="B54" s="21" t="s">
-        <v>182</v>
+        <v>190</v>
       </c>
       <c r="C54" s="19"/>
-      <c r="D54" s="24" t="n">
-        <v>1</v>
-      </c>
-      <c r="E54" s="25" t="n">
+      <c r="D54" s="25" t="n">
+        <v>1</v>
+      </c>
+      <c r="E54" s="26" t="n">
         <f aca="false">C54*D54</f>
         <v>0</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="6" t="s">
-        <v>183</v>
+        <v>191</v>
       </c>
       <c r="B55" s="21" t="s">
-        <v>112</v>
+        <v>120</v>
       </c>
       <c r="C55" s="19"/>
-      <c r="D55" s="24" t="n">
-        <v>1</v>
-      </c>
-      <c r="E55" s="25" t="n">
+      <c r="D55" s="25" t="n">
+        <v>1</v>
+      </c>
+      <c r="E55" s="26" t="n">
         <f aca="false">C55*D55</f>
         <v>0</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="6" t="s">
-        <v>184</v>
+        <v>192</v>
       </c>
       <c r="B56" s="21" t="s">
-        <v>136</v>
+        <v>144</v>
       </c>
       <c r="C56" s="19"/>
-      <c r="D56" s="24" t="n">
-        <v>1</v>
-      </c>
-      <c r="E56" s="25" t="n">
+      <c r="D56" s="25" t="n">
+        <v>1</v>
+      </c>
+      <c r="E56" s="26" t="n">
         <f aca="false">C56*D56</f>
         <v>0</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="6" t="s">
-        <v>185</v>
+        <v>193</v>
       </c>
       <c r="B57" s="21" t="s">
-        <v>136</v>
+        <v>144</v>
       </c>
       <c r="C57" s="19"/>
-      <c r="D57" s="24" t="n">
-        <v>1</v>
-      </c>
-      <c r="E57" s="25" t="n">
+      <c r="D57" s="25" t="n">
+        <v>1</v>
+      </c>
+      <c r="E57" s="26" t="n">
         <f aca="false">C57*D57</f>
         <v>0</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="6" t="s">
-        <v>186</v>
+        <v>194</v>
       </c>
       <c r="B58" s="21" t="s">
-        <v>138</v>
+        <v>146</v>
       </c>
       <c r="C58" s="19"/>
-      <c r="D58" s="24" t="n">
-        <v>1</v>
-      </c>
-      <c r="E58" s="25" t="n">
+      <c r="D58" s="25" t="n">
+        <v>1</v>
+      </c>
+      <c r="E58" s="26" t="n">
         <f aca="false">C58*D58</f>
         <v>0</v>
       </c>
       <c r="F58" s="11" t="s">
-        <v>187</v>
+        <v>195</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="6" t="s">
-        <v>188</v>
+        <v>196</v>
       </c>
       <c r="B59" s="21" t="s">
-        <v>136</v>
+        <v>144</v>
       </c>
       <c r="C59" s="19"/>
-      <c r="D59" s="24" t="n">
-        <v>1</v>
-      </c>
-      <c r="E59" s="25" t="n">
+      <c r="D59" s="25" t="n">
+        <v>1</v>
+      </c>
+      <c r="E59" s="26" t="n">
         <f aca="false">C59*D59</f>
         <v>0</v>
       </c>
       <c r="F59" s="11" t="s">
-        <v>187</v>
+        <v>195</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A60" s="23" t="s">
-        <v>189</v>
+      <c r="A60" s="24" t="s">
+        <v>197</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="6" t="s">
-        <v>190</v>
+        <v>198</v>
       </c>
       <c r="B61" s="21" t="s">
-        <v>145</v>
+        <v>153</v>
       </c>
       <c r="C61" s="19"/>
-      <c r="D61" s="24" t="n">
-        <v>1</v>
-      </c>
-      <c r="E61" s="25" t="n">
+      <c r="D61" s="25" t="n">
+        <v>1</v>
+      </c>
+      <c r="E61" s="26" t="n">
         <f aca="false">C61*D61</f>
         <v>0</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="6" t="s">
-        <v>191</v>
+        <v>199</v>
       </c>
       <c r="B62" s="21" t="s">
-        <v>145</v>
+        <v>153</v>
       </c>
       <c r="C62" s="19"/>
-      <c r="D62" s="24" t="n">
-        <v>1</v>
-      </c>
-      <c r="E62" s="25" t="n">
+      <c r="D62" s="25" t="n">
+        <v>1</v>
+      </c>
+      <c r="E62" s="26" t="n">
         <f aca="false">C62*D62</f>
         <v>0</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="6" t="s">
-        <v>192</v>
+        <v>200</v>
       </c>
       <c r="B63" s="21" t="s">
-        <v>145</v>
+        <v>153</v>
       </c>
       <c r="C63" s="19"/>
-      <c r="D63" s="24" t="n">
-        <v>1</v>
-      </c>
-      <c r="E63" s="25" t="n">
+      <c r="D63" s="25" t="n">
+        <v>1</v>
+      </c>
+      <c r="E63" s="26" t="n">
         <f aca="false">C63*D63</f>
         <v>0</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="6" t="s">
-        <v>193</v>
+        <v>201</v>
       </c>
       <c r="B64" s="21" t="s">
-        <v>145</v>
+        <v>153</v>
       </c>
       <c r="C64" s="19"/>
-      <c r="D64" s="24" t="n">
-        <v>1</v>
-      </c>
-      <c r="E64" s="25" t="n">
+      <c r="D64" s="25" t="n">
+        <v>1</v>
+      </c>
+      <c r="E64" s="26" t="n">
         <f aca="false">C64*D64</f>
         <v>0</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="6" t="s">
-        <v>194</v>
+        <v>202</v>
       </c>
       <c r="B65" s="21" t="s">
-        <v>145</v>
+        <v>153</v>
       </c>
       <c r="C65" s="19"/>
-      <c r="D65" s="24" t="n">
-        <v>1</v>
-      </c>
-      <c r="E65" s="25" t="n">
+      <c r="D65" s="25" t="n">
+        <v>1</v>
+      </c>
+      <c r="E65" s="26" t="n">
         <f aca="false">C65*D65</f>
         <v>0</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="6" t="s">
-        <v>195</v>
+        <v>203</v>
       </c>
       <c r="B66" s="21" t="s">
-        <v>145</v>
+        <v>153</v>
       </c>
       <c r="C66" s="19"/>
-      <c r="D66" s="24" t="n">
-        <v>1</v>
-      </c>
-      <c r="E66" s="25" t="n">
+      <c r="D66" s="25" t="n">
+        <v>1</v>
+      </c>
+      <c r="E66" s="26" t="n">
         <f aca="false">C66*D66</f>
         <v>0</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="6" t="s">
-        <v>196</v>
+        <v>204</v>
       </c>
       <c r="B67" s="21" t="s">
-        <v>145</v>
+        <v>153</v>
       </c>
       <c r="C67" s="19"/>
-      <c r="D67" s="24" t="n">
-        <v>1</v>
-      </c>
-      <c r="E67" s="25" t="n">
+      <c r="D67" s="25" t="n">
+        <v>1</v>
+      </c>
+      <c r="E67" s="26" t="n">
         <f aca="false">C67*D67</f>
         <v>0</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="6" t="s">
-        <v>197</v>
+        <v>205</v>
       </c>
       <c r="B68" s="21" t="s">
-        <v>145</v>
+        <v>153</v>
       </c>
       <c r="C68" s="19"/>
-      <c r="D68" s="24" t="n">
-        <v>1</v>
-      </c>
-      <c r="E68" s="25" t="n">
+      <c r="D68" s="25" t="n">
+        <v>1</v>
+      </c>
+      <c r="E68" s="26" t="n">
         <f aca="false">C68*D68</f>
         <v>0</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="6" t="s">
-        <v>198</v>
+        <v>206</v>
       </c>
       <c r="B69" s="21" t="s">
-        <v>145</v>
+        <v>153</v>
       </c>
       <c r="C69" s="19"/>
-      <c r="D69" s="24" t="n">
-        <v>1</v>
-      </c>
-      <c r="E69" s="25" t="n">
+      <c r="D69" s="25" t="n">
+        <v>1</v>
+      </c>
+      <c r="E69" s="26" t="n">
         <f aca="false">C69*D69</f>
         <v>0</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="6" t="s">
-        <v>199</v>
+        <v>207</v>
       </c>
       <c r="B70" s="21" t="s">
-        <v>145</v>
+        <v>153</v>
       </c>
       <c r="C70" s="19"/>
-      <c r="D70" s="24" t="n">
-        <v>1</v>
-      </c>
-      <c r="E70" s="25" t="n">
+      <c r="D70" s="25" t="n">
+        <v>1</v>
+      </c>
+      <c r="E70" s="26" t="n">
         <f aca="false">C70*D70</f>
         <v>0</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="6" t="s">
-        <v>200</v>
+        <v>208</v>
       </c>
       <c r="B71" s="21" t="s">
-        <v>145</v>
+        <v>153</v>
       </c>
       <c r="C71" s="19"/>
-      <c r="D71" s="24" t="n">
-        <v>1</v>
-      </c>
-      <c r="E71" s="25" t="n">
+      <c r="D71" s="25" t="n">
+        <v>1</v>
+      </c>
+      <c r="E71" s="26" t="n">
         <f aca="false">C71*D71</f>
         <v>0</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="6" t="s">
-        <v>201</v>
+        <v>209</v>
       </c>
       <c r="B72" s="21" t="s">
-        <v>145</v>
+        <v>153</v>
       </c>
       <c r="C72" s="19"/>
-      <c r="D72" s="24" t="n">
-        <v>1</v>
-      </c>
-      <c r="E72" s="25" t="n">
+      <c r="D72" s="25" t="n">
+        <v>1</v>
+      </c>
+      <c r="E72" s="26" t="n">
         <f aca="false">C72*D72</f>
         <v>0</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="6" t="s">
-        <v>202</v>
+        <v>210</v>
       </c>
       <c r="B73" s="21" t="s">
-        <v>145</v>
+        <v>153</v>
       </c>
       <c r="C73" s="19"/>
-      <c r="D73" s="24" t="n">
-        <v>1</v>
-      </c>
-      <c r="E73" s="25" t="n">
+      <c r="D73" s="25" t="n">
+        <v>1</v>
+      </c>
+      <c r="E73" s="26" t="n">
         <f aca="false">C73*D73</f>
         <v>0</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="6" t="s">
-        <v>203</v>
+        <v>211</v>
       </c>
       <c r="B74" s="21" t="s">
-        <v>145</v>
+        <v>153</v>
       </c>
       <c r="C74" s="19"/>
-      <c r="D74" s="24" t="n">
-        <v>1</v>
-      </c>
-      <c r="E74" s="25" t="n">
+      <c r="D74" s="25" t="n">
+        <v>1</v>
+      </c>
+      <c r="E74" s="26" t="n">
         <f aca="false">C74*D74</f>
         <v>0</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="6" t="s">
-        <v>204</v>
+        <v>212</v>
       </c>
       <c r="B75" s="21" t="s">
-        <v>145</v>
+        <v>153</v>
       </c>
       <c r="C75" s="19"/>
-      <c r="D75" s="24" t="n">
-        <v>1</v>
-      </c>
-      <c r="E75" s="25" t="n">
+      <c r="D75" s="25" t="n">
+        <v>1</v>
+      </c>
+      <c r="E75" s="26" t="n">
         <f aca="false">C75*D75</f>
         <v>0</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="6" t="s">
-        <v>205</v>
+        <v>213</v>
       </c>
       <c r="B76" s="21" t="s">
-        <v>145</v>
+        <v>153</v>
       </c>
       <c r="C76" s="19"/>
-      <c r="D76" s="24" t="n">
-        <v>1</v>
-      </c>
-      <c r="E76" s="25" t="n">
+      <c r="D76" s="25" t="n">
+        <v>1</v>
+      </c>
+      <c r="E76" s="26" t="n">
         <f aca="false">C76*D76</f>
         <v>0</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="6" t="s">
-        <v>206</v>
+        <v>214</v>
       </c>
       <c r="B77" s="21" t="s">
-        <v>145</v>
+        <v>153</v>
       </c>
       <c r="C77" s="19"/>
-      <c r="D77" s="24" t="n">
-        <v>1</v>
-      </c>
-      <c r="E77" s="25" t="n">
+      <c r="D77" s="25" t="n">
+        <v>1</v>
+      </c>
+      <c r="E77" s="26" t="n">
         <f aca="false">C77*D77</f>
         <v>0</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="6" t="s">
-        <v>207</v>
+        <v>215</v>
       </c>
       <c r="B78" s="21" t="s">
-        <v>145</v>
+        <v>153</v>
       </c>
       <c r="C78" s="19"/>
-      <c r="D78" s="24" t="n">
-        <v>1</v>
-      </c>
-      <c r="E78" s="25" t="n">
+      <c r="D78" s="25" t="n">
+        <v>1</v>
+      </c>
+      <c r="E78" s="26" t="n">
         <f aca="false">C78*D78</f>
         <v>0</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A79" s="23" t="s">
-        <v>208</v>
+      <c r="A79" s="24" t="s">
+        <v>216</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A80" s="10"/>
       <c r="B80" s="21" t="s">
-        <v>136</v>
+        <v>144</v>
       </c>
       <c r="C80" s="19"/>
-      <c r="D80" s="24" t="n">
-        <v>1</v>
-      </c>
-      <c r="E80" s="25" t="n">
+      <c r="D80" s="25" t="n">
+        <v>1</v>
+      </c>
+      <c r="E80" s="26" t="n">
         <f aca="false">C80*D80</f>
         <v>0</v>
       </c>
@@ -5356,13 +5550,13 @@
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A81" s="10"/>
       <c r="B81" s="21" t="s">
-        <v>136</v>
+        <v>144</v>
       </c>
       <c r="C81" s="19"/>
-      <c r="D81" s="24" t="n">
-        <v>1</v>
-      </c>
-      <c r="E81" s="25" t="n">
+      <c r="D81" s="25" t="n">
+        <v>1</v>
+      </c>
+      <c r="E81" s="26" t="n">
         <f aca="false">C81*D81</f>
         <v>0</v>
       </c>
@@ -5370,13 +5564,13 @@
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A82" s="10"/>
       <c r="B82" s="21" t="s">
-        <v>136</v>
+        <v>144</v>
       </c>
       <c r="C82" s="19"/>
-      <c r="D82" s="24" t="n">
-        <v>1</v>
-      </c>
-      <c r="E82" s="25" t="n">
+      <c r="D82" s="25" t="n">
+        <v>1</v>
+      </c>
+      <c r="E82" s="26" t="n">
         <f aca="false">C82*D82</f>
         <v>0</v>
       </c>
@@ -5384,13 +5578,13 @@
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A83" s="10"/>
       <c r="B83" s="21" t="s">
-        <v>136</v>
+        <v>144</v>
       </c>
       <c r="C83" s="19"/>
-      <c r="D83" s="24" t="n">
-        <v>1</v>
-      </c>
-      <c r="E83" s="25" t="n">
+      <c r="D83" s="25" t="n">
+        <v>1</v>
+      </c>
+      <c r="E83" s="26" t="n">
         <f aca="false">C83*D83</f>
         <v>0</v>
       </c>
@@ -5398,20 +5592,20 @@
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A84" s="10"/>
       <c r="B84" s="21" t="s">
-        <v>136</v>
+        <v>144</v>
       </c>
       <c r="C84" s="19"/>
-      <c r="D84" s="24" t="n">
-        <v>1</v>
-      </c>
-      <c r="E84" s="25" t="n">
+      <c r="D84" s="25" t="n">
+        <v>1</v>
+      </c>
+      <c r="E84" s="26" t="n">
         <f aca="false">C84*D84</f>
         <v>0</v>
       </c>
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A85" s="9" t="s">
-        <v>209</v>
+        <v>217</v>
       </c>
       <c r="C85" s="20" t="n">
         <f aca="false">SUM(C6:C84)</f>
@@ -5424,7 +5618,7 @@
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A87" s="17" t="s">
-        <v>210</v>
+        <v>218</v>
       </c>
       <c r="B87" s="17"/>
       <c r="C87" s="17"/>
@@ -5470,111 +5664,111 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>211</v>
+        <v>219</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>212</v>
+        <v>220</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="14" t="s">
-        <v>213</v>
+        <v>221</v>
       </c>
       <c r="B4" s="14" t="s">
-        <v>213</v>
+        <v>221</v>
       </c>
       <c r="C4" s="14" t="s">
-        <v>103</v>
+        <v>111</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
-        <v>214</v>
-      </c>
-      <c r="B5" s="26"/>
+        <v>222</v>
+      </c>
+      <c r="B5" s="27"/>
       <c r="C5" s="11" t="s">
-        <v>215</v>
+        <v>223</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>216</v>
-      </c>
-      <c r="B6" s="26"/>
+        <v>224</v>
+      </c>
+      <c r="B6" s="27"/>
     </row>
     <row r="7" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>217</v>
-      </c>
-      <c r="B7" s="26"/>
+        <v>225</v>
+      </c>
+      <c r="B7" s="27"/>
       <c r="C7" s="11" t="s">
-        <v>218</v>
+        <v>226</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="14" t="s">
-        <v>219</v>
+        <v>227</v>
       </c>
       <c r="B9" s="14" t="s">
-        <v>100</v>
+        <v>108</v>
       </c>
       <c r="C9" s="14" t="s">
-        <v>103</v>
+        <v>111</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="6" t="s">
-        <v>220</v>
+        <v>228</v>
       </c>
       <c r="B10" s="19"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="6" t="s">
-        <v>221</v>
+        <v>229</v>
       </c>
       <c r="B11" s="19"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="6" t="s">
-        <v>222</v>
+        <v>230</v>
       </c>
       <c r="B12" s="19"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="6" t="s">
-        <v>223</v>
+        <v>231</v>
       </c>
       <c r="B13" s="19"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="6" t="s">
-        <v>224</v>
+        <v>232</v>
       </c>
       <c r="B14" s="19"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="6" t="s">
-        <v>225</v>
+        <v>233</v>
       </c>
       <c r="B15" s="19"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="6" t="s">
-        <v>226</v>
+        <v>234</v>
       </c>
       <c r="B16" s="19"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="6" t="s">
-        <v>227</v>
+        <v>235</v>
       </c>
       <c r="B17" s="19"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="9" t="s">
-        <v>228</v>
+        <v>236</v>
       </c>
       <c r="B18" s="20" t="n">
         <f aca="false">SUM(B10:B17)</f>
@@ -5583,34 +5777,34 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="6" t="s">
-        <v>229</v>
-      </c>
-      <c r="B20" s="27" t="n">
+        <v>237</v>
+      </c>
+      <c r="B20" s="28" t="n">
         <f aca="false">B5*Data!$C$66+B6*Data!$C$67</f>
         <v>0</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="6" t="s">
-        <v>230</v>
-      </c>
-      <c r="B21" s="28" t="str">
+        <v>238</v>
+      </c>
+      <c r="B21" s="29" t="str">
         <f aca="false">IF(AND(B7&gt;0,B5+B6&gt;0),MIN(1,(B5+B6)/B7),"")</f>
         <v/>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="6" t="s">
-        <v>231</v>
-      </c>
-      <c r="B22" s="27" t="str">
+        <v>239</v>
+      </c>
+      <c r="B22" s="28" t="str">
         <f aca="false">IF(N(B21)&gt;0,B18*B21,"")</f>
         <v/>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="9" t="s">
-        <v>232</v>
+        <v>240</v>
       </c>
       <c r="B23" s="20" t="n">
         <f aca="false">MAX(B20,N(B22))</f>
@@ -5619,7 +5813,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="17" t="s">
-        <v>233</v>
+        <v>241</v>
       </c>
       <c r="B25" s="17"/>
       <c r="C25" s="17"/>
@@ -5664,43 +5858,43 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>234</v>
+        <v>242</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>235</v>
+        <v>243</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="14" t="s">
-        <v>236</v>
+        <v>244</v>
       </c>
       <c r="B4" s="14" t="s">
-        <v>237</v>
+        <v>245</v>
       </c>
       <c r="C4" s="14" t="s">
-        <v>238</v>
+        <v>246</v>
       </c>
       <c r="D4" s="14" t="s">
-        <v>239</v>
+        <v>247</v>
       </c>
       <c r="E4" s="14" t="s">
-        <v>240</v>
+        <v>248</v>
       </c>
       <c r="F4" s="14" t="s">
-        <v>241</v>
+        <v>249</v>
       </c>
       <c r="G4" s="14" t="s">
-        <v>242</v>
+        <v>250</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="15" t="s">
-        <v>243</v>
+        <v>251</v>
       </c>
       <c r="B5" s="15" t="s">
-        <v>244</v>
+        <v>252</v>
       </c>
       <c r="C5" s="15" t="n">
         <v>0</v>
@@ -5716,631 +5910,631 @@
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="29"/>
-      <c r="B6" s="29"/>
+      <c r="A6" s="30"/>
+      <c r="B6" s="30"/>
       <c r="C6" s="12"/>
-      <c r="D6" s="30" t="n">
+      <c r="D6" s="31" t="n">
         <f aca="false">IF(AND(ISNUMBER(A6),ISNUMBER(B6),B6&gt;A6),MAX(0,MIN(B6-1,DATE(2026,12,31))-MAX(A6+1,DATE(2026,1,1))+1),0)</f>
         <v>0</v>
       </c>
-      <c r="E6" s="30" t="n">
+      <c r="E6" s="31" t="n">
         <f aca="false">IF(AND(ISNUMBER(A6),ISNUMBER(B6),B6&gt;A6),AND(A6&gt;=DATE(2026,1,1),A6&lt;=DATE(2026,12,31))*1+AND(B6&gt;=DATE(2026,1,1),B6&lt;=DATE(2026,12,31))*1,0)</f>
         <v>0</v>
       </c>
-      <c r="F6" s="25" t="n">
+      <c r="F6" s="26" t="n">
         <f aca="false">(D6-MIN(C6,D6))*Data!$C$60+MIN(C6,D6)*Data!$C$61+E6*Data!$C$60*Data!$C$62</f>
         <v>0</v>
       </c>
-      <c r="G6" s="31" t="str">
+      <c r="G6" s="32" t="str">
         <f aca="false">IF(AND(AND(ISNUMBER(A6),ISNUMBER(B6),B6&gt;A6),SUMPRODUCT(ISNUMBER($A$6:$A$35)*ISNUMBER($B$6:$B$35)*($A$6:$A$35&lt;B6)*($B$6:$B$35&gt;A6))&gt;1),"Overlaps another trip","")</f>
         <v/>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="29"/>
-      <c r="B7" s="29"/>
+      <c r="A7" s="30"/>
+      <c r="B7" s="30"/>
       <c r="C7" s="12"/>
-      <c r="D7" s="30" t="n">
+      <c r="D7" s="31" t="n">
         <f aca="false">IF(AND(ISNUMBER(A7),ISNUMBER(B7),B7&gt;A7),MAX(0,MIN(B7-1,DATE(2026,12,31))-MAX(A7+1,DATE(2026,1,1))+1),0)</f>
         <v>0</v>
       </c>
-      <c r="E7" s="30" t="n">
+      <c r="E7" s="31" t="n">
         <f aca="false">IF(AND(ISNUMBER(A7),ISNUMBER(B7),B7&gt;A7),AND(A7&gt;=DATE(2026,1,1),A7&lt;=DATE(2026,12,31))*1+AND(B7&gt;=DATE(2026,1,1),B7&lt;=DATE(2026,12,31))*1,0)</f>
         <v>0</v>
       </c>
-      <c r="F7" s="25" t="n">
+      <c r="F7" s="26" t="n">
         <f aca="false">(D7-MIN(C7,D7))*Data!$C$60+MIN(C7,D7)*Data!$C$61+E7*Data!$C$60*Data!$C$62</f>
         <v>0</v>
       </c>
-      <c r="G7" s="31" t="str">
+      <c r="G7" s="32" t="str">
         <f aca="false">IF(AND(AND(ISNUMBER(A7),ISNUMBER(B7),B7&gt;A7),SUMPRODUCT(ISNUMBER($A$6:$A$35)*ISNUMBER($B$6:$B$35)*($A$6:$A$35&lt;B7)*($B$6:$B$35&gt;A7))&gt;1),"Overlaps another trip","")</f>
         <v/>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="29"/>
-      <c r="B8" s="29"/>
+      <c r="A8" s="30"/>
+      <c r="B8" s="30"/>
       <c r="C8" s="12"/>
-      <c r="D8" s="30" t="n">
+      <c r="D8" s="31" t="n">
         <f aca="false">IF(AND(ISNUMBER(A8),ISNUMBER(B8),B8&gt;A8),MAX(0,MIN(B8-1,DATE(2026,12,31))-MAX(A8+1,DATE(2026,1,1))+1),0)</f>
         <v>0</v>
       </c>
-      <c r="E8" s="30" t="n">
+      <c r="E8" s="31" t="n">
         <f aca="false">IF(AND(ISNUMBER(A8),ISNUMBER(B8),B8&gt;A8),AND(A8&gt;=DATE(2026,1,1),A8&lt;=DATE(2026,12,31))*1+AND(B8&gt;=DATE(2026,1,1),B8&lt;=DATE(2026,12,31))*1,0)</f>
         <v>0</v>
       </c>
-      <c r="F8" s="25" t="n">
+      <c r="F8" s="26" t="n">
         <f aca="false">(D8-MIN(C8,D8))*Data!$C$60+MIN(C8,D8)*Data!$C$61+E8*Data!$C$60*Data!$C$62</f>
         <v>0</v>
       </c>
-      <c r="G8" s="31" t="str">
+      <c r="G8" s="32" t="str">
         <f aca="false">IF(AND(AND(ISNUMBER(A8),ISNUMBER(B8),B8&gt;A8),SUMPRODUCT(ISNUMBER($A$6:$A$35)*ISNUMBER($B$6:$B$35)*($A$6:$A$35&lt;B8)*($B$6:$B$35&gt;A8))&gt;1),"Overlaps another trip","")</f>
         <v/>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="29"/>
-      <c r="B9" s="29"/>
+      <c r="A9" s="30"/>
+      <c r="B9" s="30"/>
       <c r="C9" s="12"/>
-      <c r="D9" s="30" t="n">
+      <c r="D9" s="31" t="n">
         <f aca="false">IF(AND(ISNUMBER(A9),ISNUMBER(B9),B9&gt;A9),MAX(0,MIN(B9-1,DATE(2026,12,31))-MAX(A9+1,DATE(2026,1,1))+1),0)</f>
         <v>0</v>
       </c>
-      <c r="E9" s="30" t="n">
+      <c r="E9" s="31" t="n">
         <f aca="false">IF(AND(ISNUMBER(A9),ISNUMBER(B9),B9&gt;A9),AND(A9&gt;=DATE(2026,1,1),A9&lt;=DATE(2026,12,31))*1+AND(B9&gt;=DATE(2026,1,1),B9&lt;=DATE(2026,12,31))*1,0)</f>
         <v>0</v>
       </c>
-      <c r="F9" s="25" t="n">
+      <c r="F9" s="26" t="n">
         <f aca="false">(D9-MIN(C9,D9))*Data!$C$60+MIN(C9,D9)*Data!$C$61+E9*Data!$C$60*Data!$C$62</f>
         <v>0</v>
       </c>
-      <c r="G9" s="31" t="str">
+      <c r="G9" s="32" t="str">
         <f aca="false">IF(AND(AND(ISNUMBER(A9),ISNUMBER(B9),B9&gt;A9),SUMPRODUCT(ISNUMBER($A$6:$A$35)*ISNUMBER($B$6:$B$35)*($A$6:$A$35&lt;B9)*($B$6:$B$35&gt;A9))&gt;1),"Overlaps another trip","")</f>
         <v/>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="29"/>
-      <c r="B10" s="29"/>
+      <c r="A10" s="30"/>
+      <c r="B10" s="30"/>
       <c r="C10" s="12"/>
-      <c r="D10" s="30" t="n">
+      <c r="D10" s="31" t="n">
         <f aca="false">IF(AND(ISNUMBER(A10),ISNUMBER(B10),B10&gt;A10),MAX(0,MIN(B10-1,DATE(2026,12,31))-MAX(A10+1,DATE(2026,1,1))+1),0)</f>
         <v>0</v>
       </c>
-      <c r="E10" s="30" t="n">
+      <c r="E10" s="31" t="n">
         <f aca="false">IF(AND(ISNUMBER(A10),ISNUMBER(B10),B10&gt;A10),AND(A10&gt;=DATE(2026,1,1),A10&lt;=DATE(2026,12,31))*1+AND(B10&gt;=DATE(2026,1,1),B10&lt;=DATE(2026,12,31))*1,0)</f>
         <v>0</v>
       </c>
-      <c r="F10" s="25" t="n">
+      <c r="F10" s="26" t="n">
         <f aca="false">(D10-MIN(C10,D10))*Data!$C$60+MIN(C10,D10)*Data!$C$61+E10*Data!$C$60*Data!$C$62</f>
         <v>0</v>
       </c>
-      <c r="G10" s="31" t="str">
+      <c r="G10" s="32" t="str">
         <f aca="false">IF(AND(AND(ISNUMBER(A10),ISNUMBER(B10),B10&gt;A10),SUMPRODUCT(ISNUMBER($A$6:$A$35)*ISNUMBER($B$6:$B$35)*($A$6:$A$35&lt;B10)*($B$6:$B$35&gt;A10))&gt;1),"Overlaps another trip","")</f>
         <v/>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="29"/>
-      <c r="B11" s="29"/>
+      <c r="A11" s="30"/>
+      <c r="B11" s="30"/>
       <c r="C11" s="12"/>
-      <c r="D11" s="30" t="n">
+      <c r="D11" s="31" t="n">
         <f aca="false">IF(AND(ISNUMBER(A11),ISNUMBER(B11),B11&gt;A11),MAX(0,MIN(B11-1,DATE(2026,12,31))-MAX(A11+1,DATE(2026,1,1))+1),0)</f>
         <v>0</v>
       </c>
-      <c r="E11" s="30" t="n">
+      <c r="E11" s="31" t="n">
         <f aca="false">IF(AND(ISNUMBER(A11),ISNUMBER(B11),B11&gt;A11),AND(A11&gt;=DATE(2026,1,1),A11&lt;=DATE(2026,12,31))*1+AND(B11&gt;=DATE(2026,1,1),B11&lt;=DATE(2026,12,31))*1,0)</f>
         <v>0</v>
       </c>
-      <c r="F11" s="25" t="n">
+      <c r="F11" s="26" t="n">
         <f aca="false">(D11-MIN(C11,D11))*Data!$C$60+MIN(C11,D11)*Data!$C$61+E11*Data!$C$60*Data!$C$62</f>
         <v>0</v>
       </c>
-      <c r="G11" s="31" t="str">
+      <c r="G11" s="32" t="str">
         <f aca="false">IF(AND(AND(ISNUMBER(A11),ISNUMBER(B11),B11&gt;A11),SUMPRODUCT(ISNUMBER($A$6:$A$35)*ISNUMBER($B$6:$B$35)*($A$6:$A$35&lt;B11)*($B$6:$B$35&gt;A11))&gt;1),"Overlaps another trip","")</f>
         <v/>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="29"/>
-      <c r="B12" s="29"/>
+      <c r="A12" s="30"/>
+      <c r="B12" s="30"/>
       <c r="C12" s="12"/>
-      <c r="D12" s="30" t="n">
+      <c r="D12" s="31" t="n">
         <f aca="false">IF(AND(ISNUMBER(A12),ISNUMBER(B12),B12&gt;A12),MAX(0,MIN(B12-1,DATE(2026,12,31))-MAX(A12+1,DATE(2026,1,1))+1),0)</f>
         <v>0</v>
       </c>
-      <c r="E12" s="30" t="n">
+      <c r="E12" s="31" t="n">
         <f aca="false">IF(AND(ISNUMBER(A12),ISNUMBER(B12),B12&gt;A12),AND(A12&gt;=DATE(2026,1,1),A12&lt;=DATE(2026,12,31))*1+AND(B12&gt;=DATE(2026,1,1),B12&lt;=DATE(2026,12,31))*1,0)</f>
         <v>0</v>
       </c>
-      <c r="F12" s="25" t="n">
+      <c r="F12" s="26" t="n">
         <f aca="false">(D12-MIN(C12,D12))*Data!$C$60+MIN(C12,D12)*Data!$C$61+E12*Data!$C$60*Data!$C$62</f>
         <v>0</v>
       </c>
-      <c r="G12" s="31" t="str">
+      <c r="G12" s="32" t="str">
         <f aca="false">IF(AND(AND(ISNUMBER(A12),ISNUMBER(B12),B12&gt;A12),SUMPRODUCT(ISNUMBER($A$6:$A$35)*ISNUMBER($B$6:$B$35)*($A$6:$A$35&lt;B12)*($B$6:$B$35&gt;A12))&gt;1),"Overlaps another trip","")</f>
         <v/>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="29"/>
-      <c r="B13" s="29"/>
+      <c r="A13" s="30"/>
+      <c r="B13" s="30"/>
       <c r="C13" s="12"/>
-      <c r="D13" s="30" t="n">
+      <c r="D13" s="31" t="n">
         <f aca="false">IF(AND(ISNUMBER(A13),ISNUMBER(B13),B13&gt;A13),MAX(0,MIN(B13-1,DATE(2026,12,31))-MAX(A13+1,DATE(2026,1,1))+1),0)</f>
         <v>0</v>
       </c>
-      <c r="E13" s="30" t="n">
+      <c r="E13" s="31" t="n">
         <f aca="false">IF(AND(ISNUMBER(A13),ISNUMBER(B13),B13&gt;A13),AND(A13&gt;=DATE(2026,1,1),A13&lt;=DATE(2026,12,31))*1+AND(B13&gt;=DATE(2026,1,1),B13&lt;=DATE(2026,12,31))*1,0)</f>
         <v>0</v>
       </c>
-      <c r="F13" s="25" t="n">
+      <c r="F13" s="26" t="n">
         <f aca="false">(D13-MIN(C13,D13))*Data!$C$60+MIN(C13,D13)*Data!$C$61+E13*Data!$C$60*Data!$C$62</f>
         <v>0</v>
       </c>
-      <c r="G13" s="31" t="str">
+      <c r="G13" s="32" t="str">
         <f aca="false">IF(AND(AND(ISNUMBER(A13),ISNUMBER(B13),B13&gt;A13),SUMPRODUCT(ISNUMBER($A$6:$A$35)*ISNUMBER($B$6:$B$35)*($A$6:$A$35&lt;B13)*($B$6:$B$35&gt;A13))&gt;1),"Overlaps another trip","")</f>
         <v/>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="29"/>
-      <c r="B14" s="29"/>
+      <c r="A14" s="30"/>
+      <c r="B14" s="30"/>
       <c r="C14" s="12"/>
-      <c r="D14" s="30" t="n">
+      <c r="D14" s="31" t="n">
         <f aca="false">IF(AND(ISNUMBER(A14),ISNUMBER(B14),B14&gt;A14),MAX(0,MIN(B14-1,DATE(2026,12,31))-MAX(A14+1,DATE(2026,1,1))+1),0)</f>
         <v>0</v>
       </c>
-      <c r="E14" s="30" t="n">
+      <c r="E14" s="31" t="n">
         <f aca="false">IF(AND(ISNUMBER(A14),ISNUMBER(B14),B14&gt;A14),AND(A14&gt;=DATE(2026,1,1),A14&lt;=DATE(2026,12,31))*1+AND(B14&gt;=DATE(2026,1,1),B14&lt;=DATE(2026,12,31))*1,0)</f>
         <v>0</v>
       </c>
-      <c r="F14" s="25" t="n">
+      <c r="F14" s="26" t="n">
         <f aca="false">(D14-MIN(C14,D14))*Data!$C$60+MIN(C14,D14)*Data!$C$61+E14*Data!$C$60*Data!$C$62</f>
         <v>0</v>
       </c>
-      <c r="G14" s="31" t="str">
+      <c r="G14" s="32" t="str">
         <f aca="false">IF(AND(AND(ISNUMBER(A14),ISNUMBER(B14),B14&gt;A14),SUMPRODUCT(ISNUMBER($A$6:$A$35)*ISNUMBER($B$6:$B$35)*($A$6:$A$35&lt;B14)*($B$6:$B$35&gt;A14))&gt;1),"Overlaps another trip","")</f>
         <v/>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="29"/>
-      <c r="B15" s="29"/>
+      <c r="A15" s="30"/>
+      <c r="B15" s="30"/>
       <c r="C15" s="12"/>
-      <c r="D15" s="30" t="n">
+      <c r="D15" s="31" t="n">
         <f aca="false">IF(AND(ISNUMBER(A15),ISNUMBER(B15),B15&gt;A15),MAX(0,MIN(B15-1,DATE(2026,12,31))-MAX(A15+1,DATE(2026,1,1))+1),0)</f>
         <v>0</v>
       </c>
-      <c r="E15" s="30" t="n">
+      <c r="E15" s="31" t="n">
         <f aca="false">IF(AND(ISNUMBER(A15),ISNUMBER(B15),B15&gt;A15),AND(A15&gt;=DATE(2026,1,1),A15&lt;=DATE(2026,12,31))*1+AND(B15&gt;=DATE(2026,1,1),B15&lt;=DATE(2026,12,31))*1,0)</f>
         <v>0</v>
       </c>
-      <c r="F15" s="25" t="n">
+      <c r="F15" s="26" t="n">
         <f aca="false">(D15-MIN(C15,D15))*Data!$C$60+MIN(C15,D15)*Data!$C$61+E15*Data!$C$60*Data!$C$62</f>
         <v>0</v>
       </c>
-      <c r="G15" s="31" t="str">
+      <c r="G15" s="32" t="str">
         <f aca="false">IF(AND(AND(ISNUMBER(A15),ISNUMBER(B15),B15&gt;A15),SUMPRODUCT(ISNUMBER($A$6:$A$35)*ISNUMBER($B$6:$B$35)*($A$6:$A$35&lt;B15)*($B$6:$B$35&gt;A15))&gt;1),"Overlaps another trip","")</f>
         <v/>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="29"/>
-      <c r="B16" s="29"/>
+      <c r="A16" s="30"/>
+      <c r="B16" s="30"/>
       <c r="C16" s="12"/>
-      <c r="D16" s="30" t="n">
+      <c r="D16" s="31" t="n">
         <f aca="false">IF(AND(ISNUMBER(A16),ISNUMBER(B16),B16&gt;A16),MAX(0,MIN(B16-1,DATE(2026,12,31))-MAX(A16+1,DATE(2026,1,1))+1),0)</f>
         <v>0</v>
       </c>
-      <c r="E16" s="30" t="n">
+      <c r="E16" s="31" t="n">
         <f aca="false">IF(AND(ISNUMBER(A16),ISNUMBER(B16),B16&gt;A16),AND(A16&gt;=DATE(2026,1,1),A16&lt;=DATE(2026,12,31))*1+AND(B16&gt;=DATE(2026,1,1),B16&lt;=DATE(2026,12,31))*1,0)</f>
         <v>0</v>
       </c>
-      <c r="F16" s="25" t="n">
+      <c r="F16" s="26" t="n">
         <f aca="false">(D16-MIN(C16,D16))*Data!$C$60+MIN(C16,D16)*Data!$C$61+E16*Data!$C$60*Data!$C$62</f>
         <v>0</v>
       </c>
-      <c r="G16" s="31" t="str">
+      <c r="G16" s="32" t="str">
         <f aca="false">IF(AND(AND(ISNUMBER(A16),ISNUMBER(B16),B16&gt;A16),SUMPRODUCT(ISNUMBER($A$6:$A$35)*ISNUMBER($B$6:$B$35)*($A$6:$A$35&lt;B16)*($B$6:$B$35&gt;A16))&gt;1),"Overlaps another trip","")</f>
         <v/>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="29"/>
-      <c r="B17" s="29"/>
+      <c r="A17" s="30"/>
+      <c r="B17" s="30"/>
       <c r="C17" s="12"/>
-      <c r="D17" s="30" t="n">
+      <c r="D17" s="31" t="n">
         <f aca="false">IF(AND(ISNUMBER(A17),ISNUMBER(B17),B17&gt;A17),MAX(0,MIN(B17-1,DATE(2026,12,31))-MAX(A17+1,DATE(2026,1,1))+1),0)</f>
         <v>0</v>
       </c>
-      <c r="E17" s="30" t="n">
+      <c r="E17" s="31" t="n">
         <f aca="false">IF(AND(ISNUMBER(A17),ISNUMBER(B17),B17&gt;A17),AND(A17&gt;=DATE(2026,1,1),A17&lt;=DATE(2026,12,31))*1+AND(B17&gt;=DATE(2026,1,1),B17&lt;=DATE(2026,12,31))*1,0)</f>
         <v>0</v>
       </c>
-      <c r="F17" s="25" t="n">
+      <c r="F17" s="26" t="n">
         <f aca="false">(D17-MIN(C17,D17))*Data!$C$60+MIN(C17,D17)*Data!$C$61+E17*Data!$C$60*Data!$C$62</f>
         <v>0</v>
       </c>
-      <c r="G17" s="31" t="str">
+      <c r="G17" s="32" t="str">
         <f aca="false">IF(AND(AND(ISNUMBER(A17),ISNUMBER(B17),B17&gt;A17),SUMPRODUCT(ISNUMBER($A$6:$A$35)*ISNUMBER($B$6:$B$35)*($A$6:$A$35&lt;B17)*($B$6:$B$35&gt;A17))&gt;1),"Overlaps another trip","")</f>
         <v/>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="29"/>
-      <c r="B18" s="29"/>
+      <c r="A18" s="30"/>
+      <c r="B18" s="30"/>
       <c r="C18" s="12"/>
-      <c r="D18" s="30" t="n">
+      <c r="D18" s="31" t="n">
         <f aca="false">IF(AND(ISNUMBER(A18),ISNUMBER(B18),B18&gt;A18),MAX(0,MIN(B18-1,DATE(2026,12,31))-MAX(A18+1,DATE(2026,1,1))+1),0)</f>
         <v>0</v>
       </c>
-      <c r="E18" s="30" t="n">
+      <c r="E18" s="31" t="n">
         <f aca="false">IF(AND(ISNUMBER(A18),ISNUMBER(B18),B18&gt;A18),AND(A18&gt;=DATE(2026,1,1),A18&lt;=DATE(2026,12,31))*1+AND(B18&gt;=DATE(2026,1,1),B18&lt;=DATE(2026,12,31))*1,0)</f>
         <v>0</v>
       </c>
-      <c r="F18" s="25" t="n">
+      <c r="F18" s="26" t="n">
         <f aca="false">(D18-MIN(C18,D18))*Data!$C$60+MIN(C18,D18)*Data!$C$61+E18*Data!$C$60*Data!$C$62</f>
         <v>0</v>
       </c>
-      <c r="G18" s="31" t="str">
+      <c r="G18" s="32" t="str">
         <f aca="false">IF(AND(AND(ISNUMBER(A18),ISNUMBER(B18),B18&gt;A18),SUMPRODUCT(ISNUMBER($A$6:$A$35)*ISNUMBER($B$6:$B$35)*($A$6:$A$35&lt;B18)*($B$6:$B$35&gt;A18))&gt;1),"Overlaps another trip","")</f>
         <v/>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="29"/>
-      <c r="B19" s="29"/>
+      <c r="A19" s="30"/>
+      <c r="B19" s="30"/>
       <c r="C19" s="12"/>
-      <c r="D19" s="30" t="n">
+      <c r="D19" s="31" t="n">
         <f aca="false">IF(AND(ISNUMBER(A19),ISNUMBER(B19),B19&gt;A19),MAX(0,MIN(B19-1,DATE(2026,12,31))-MAX(A19+1,DATE(2026,1,1))+1),0)</f>
         <v>0</v>
       </c>
-      <c r="E19" s="30" t="n">
+      <c r="E19" s="31" t="n">
         <f aca="false">IF(AND(ISNUMBER(A19),ISNUMBER(B19),B19&gt;A19),AND(A19&gt;=DATE(2026,1,1),A19&lt;=DATE(2026,12,31))*1+AND(B19&gt;=DATE(2026,1,1),B19&lt;=DATE(2026,12,31))*1,0)</f>
         <v>0</v>
       </c>
-      <c r="F19" s="25" t="n">
+      <c r="F19" s="26" t="n">
         <f aca="false">(D19-MIN(C19,D19))*Data!$C$60+MIN(C19,D19)*Data!$C$61+E19*Data!$C$60*Data!$C$62</f>
         <v>0</v>
       </c>
-      <c r="G19" s="31" t="str">
+      <c r="G19" s="32" t="str">
         <f aca="false">IF(AND(AND(ISNUMBER(A19),ISNUMBER(B19),B19&gt;A19),SUMPRODUCT(ISNUMBER($A$6:$A$35)*ISNUMBER($B$6:$B$35)*($A$6:$A$35&lt;B19)*($B$6:$B$35&gt;A19))&gt;1),"Overlaps another trip","")</f>
         <v/>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="29"/>
-      <c r="B20" s="29"/>
+      <c r="A20" s="30"/>
+      <c r="B20" s="30"/>
       <c r="C20" s="12"/>
-      <c r="D20" s="30" t="n">
+      <c r="D20" s="31" t="n">
         <f aca="false">IF(AND(ISNUMBER(A20),ISNUMBER(B20),B20&gt;A20),MAX(0,MIN(B20-1,DATE(2026,12,31))-MAX(A20+1,DATE(2026,1,1))+1),0)</f>
         <v>0</v>
       </c>
-      <c r="E20" s="30" t="n">
+      <c r="E20" s="31" t="n">
         <f aca="false">IF(AND(ISNUMBER(A20),ISNUMBER(B20),B20&gt;A20),AND(A20&gt;=DATE(2026,1,1),A20&lt;=DATE(2026,12,31))*1+AND(B20&gt;=DATE(2026,1,1),B20&lt;=DATE(2026,12,31))*1,0)</f>
         <v>0</v>
       </c>
-      <c r="F20" s="25" t="n">
+      <c r="F20" s="26" t="n">
         <f aca="false">(D20-MIN(C20,D20))*Data!$C$60+MIN(C20,D20)*Data!$C$61+E20*Data!$C$60*Data!$C$62</f>
         <v>0</v>
       </c>
-      <c r="G20" s="31" t="str">
+      <c r="G20" s="32" t="str">
         <f aca="false">IF(AND(AND(ISNUMBER(A20),ISNUMBER(B20),B20&gt;A20),SUMPRODUCT(ISNUMBER($A$6:$A$35)*ISNUMBER($B$6:$B$35)*($A$6:$A$35&lt;B20)*($B$6:$B$35&gt;A20))&gt;1),"Overlaps another trip","")</f>
         <v/>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="29"/>
-      <c r="B21" s="29"/>
+      <c r="A21" s="30"/>
+      <c r="B21" s="30"/>
       <c r="C21" s="12"/>
-      <c r="D21" s="30" t="n">
+      <c r="D21" s="31" t="n">
         <f aca="false">IF(AND(ISNUMBER(A21),ISNUMBER(B21),B21&gt;A21),MAX(0,MIN(B21-1,DATE(2026,12,31))-MAX(A21+1,DATE(2026,1,1))+1),0)</f>
         <v>0</v>
       </c>
-      <c r="E21" s="30" t="n">
+      <c r="E21" s="31" t="n">
         <f aca="false">IF(AND(ISNUMBER(A21),ISNUMBER(B21),B21&gt;A21),AND(A21&gt;=DATE(2026,1,1),A21&lt;=DATE(2026,12,31))*1+AND(B21&gt;=DATE(2026,1,1),B21&lt;=DATE(2026,12,31))*1,0)</f>
         <v>0</v>
       </c>
-      <c r="F21" s="25" t="n">
+      <c r="F21" s="26" t="n">
         <f aca="false">(D21-MIN(C21,D21))*Data!$C$60+MIN(C21,D21)*Data!$C$61+E21*Data!$C$60*Data!$C$62</f>
         <v>0</v>
       </c>
-      <c r="G21" s="31" t="str">
+      <c r="G21" s="32" t="str">
         <f aca="false">IF(AND(AND(ISNUMBER(A21),ISNUMBER(B21),B21&gt;A21),SUMPRODUCT(ISNUMBER($A$6:$A$35)*ISNUMBER($B$6:$B$35)*($A$6:$A$35&lt;B21)*($B$6:$B$35&gt;A21))&gt;1),"Overlaps another trip","")</f>
         <v/>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="29"/>
-      <c r="B22" s="29"/>
+      <c r="A22" s="30"/>
+      <c r="B22" s="30"/>
       <c r="C22" s="12"/>
-      <c r="D22" s="30" t="n">
+      <c r="D22" s="31" t="n">
         <f aca="false">IF(AND(ISNUMBER(A22),ISNUMBER(B22),B22&gt;A22),MAX(0,MIN(B22-1,DATE(2026,12,31))-MAX(A22+1,DATE(2026,1,1))+1),0)</f>
         <v>0</v>
       </c>
-      <c r="E22" s="30" t="n">
+      <c r="E22" s="31" t="n">
         <f aca="false">IF(AND(ISNUMBER(A22),ISNUMBER(B22),B22&gt;A22),AND(A22&gt;=DATE(2026,1,1),A22&lt;=DATE(2026,12,31))*1+AND(B22&gt;=DATE(2026,1,1),B22&lt;=DATE(2026,12,31))*1,0)</f>
         <v>0</v>
       </c>
-      <c r="F22" s="25" t="n">
+      <c r="F22" s="26" t="n">
         <f aca="false">(D22-MIN(C22,D22))*Data!$C$60+MIN(C22,D22)*Data!$C$61+E22*Data!$C$60*Data!$C$62</f>
         <v>0</v>
       </c>
-      <c r="G22" s="31" t="str">
+      <c r="G22" s="32" t="str">
         <f aca="false">IF(AND(AND(ISNUMBER(A22),ISNUMBER(B22),B22&gt;A22),SUMPRODUCT(ISNUMBER($A$6:$A$35)*ISNUMBER($B$6:$B$35)*($A$6:$A$35&lt;B22)*($B$6:$B$35&gt;A22))&gt;1),"Overlaps another trip","")</f>
         <v/>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="29"/>
-      <c r="B23" s="29"/>
+      <c r="A23" s="30"/>
+      <c r="B23" s="30"/>
       <c r="C23" s="12"/>
-      <c r="D23" s="30" t="n">
+      <c r="D23" s="31" t="n">
         <f aca="false">IF(AND(ISNUMBER(A23),ISNUMBER(B23),B23&gt;A23),MAX(0,MIN(B23-1,DATE(2026,12,31))-MAX(A23+1,DATE(2026,1,1))+1),0)</f>
         <v>0</v>
       </c>
-      <c r="E23" s="30" t="n">
+      <c r="E23" s="31" t="n">
         <f aca="false">IF(AND(ISNUMBER(A23),ISNUMBER(B23),B23&gt;A23),AND(A23&gt;=DATE(2026,1,1),A23&lt;=DATE(2026,12,31))*1+AND(B23&gt;=DATE(2026,1,1),B23&lt;=DATE(2026,12,31))*1,0)</f>
         <v>0</v>
       </c>
-      <c r="F23" s="25" t="n">
+      <c r="F23" s="26" t="n">
         <f aca="false">(D23-MIN(C23,D23))*Data!$C$60+MIN(C23,D23)*Data!$C$61+E23*Data!$C$60*Data!$C$62</f>
         <v>0</v>
       </c>
-      <c r="G23" s="31" t="str">
+      <c r="G23" s="32" t="str">
         <f aca="false">IF(AND(AND(ISNUMBER(A23),ISNUMBER(B23),B23&gt;A23),SUMPRODUCT(ISNUMBER($A$6:$A$35)*ISNUMBER($B$6:$B$35)*($A$6:$A$35&lt;B23)*($B$6:$B$35&gt;A23))&gt;1),"Overlaps another trip","")</f>
         <v/>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="29"/>
-      <c r="B24" s="29"/>
+      <c r="A24" s="30"/>
+      <c r="B24" s="30"/>
       <c r="C24" s="12"/>
-      <c r="D24" s="30" t="n">
+      <c r="D24" s="31" t="n">
         <f aca="false">IF(AND(ISNUMBER(A24),ISNUMBER(B24),B24&gt;A24),MAX(0,MIN(B24-1,DATE(2026,12,31))-MAX(A24+1,DATE(2026,1,1))+1),0)</f>
         <v>0</v>
       </c>
-      <c r="E24" s="30" t="n">
+      <c r="E24" s="31" t="n">
         <f aca="false">IF(AND(ISNUMBER(A24),ISNUMBER(B24),B24&gt;A24),AND(A24&gt;=DATE(2026,1,1),A24&lt;=DATE(2026,12,31))*1+AND(B24&gt;=DATE(2026,1,1),B24&lt;=DATE(2026,12,31))*1,0)</f>
         <v>0</v>
       </c>
-      <c r="F24" s="25" t="n">
+      <c r="F24" s="26" t="n">
         <f aca="false">(D24-MIN(C24,D24))*Data!$C$60+MIN(C24,D24)*Data!$C$61+E24*Data!$C$60*Data!$C$62</f>
         <v>0</v>
       </c>
-      <c r="G24" s="31" t="str">
+      <c r="G24" s="32" t="str">
         <f aca="false">IF(AND(AND(ISNUMBER(A24),ISNUMBER(B24),B24&gt;A24),SUMPRODUCT(ISNUMBER($A$6:$A$35)*ISNUMBER($B$6:$B$35)*($A$6:$A$35&lt;B24)*($B$6:$B$35&gt;A24))&gt;1),"Overlaps another trip","")</f>
         <v/>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="29"/>
-      <c r="B25" s="29"/>
+      <c r="A25" s="30"/>
+      <c r="B25" s="30"/>
       <c r="C25" s="12"/>
-      <c r="D25" s="30" t="n">
+      <c r="D25" s="31" t="n">
         <f aca="false">IF(AND(ISNUMBER(A25),ISNUMBER(B25),B25&gt;A25),MAX(0,MIN(B25-1,DATE(2026,12,31))-MAX(A25+1,DATE(2026,1,1))+1),0)</f>
         <v>0</v>
       </c>
-      <c r="E25" s="30" t="n">
+      <c r="E25" s="31" t="n">
         <f aca="false">IF(AND(ISNUMBER(A25),ISNUMBER(B25),B25&gt;A25),AND(A25&gt;=DATE(2026,1,1),A25&lt;=DATE(2026,12,31))*1+AND(B25&gt;=DATE(2026,1,1),B25&lt;=DATE(2026,12,31))*1,0)</f>
         <v>0</v>
       </c>
-      <c r="F25" s="25" t="n">
+      <c r="F25" s="26" t="n">
         <f aca="false">(D25-MIN(C25,D25))*Data!$C$60+MIN(C25,D25)*Data!$C$61+E25*Data!$C$60*Data!$C$62</f>
         <v>0</v>
       </c>
-      <c r="G25" s="31" t="str">
+      <c r="G25" s="32" t="str">
         <f aca="false">IF(AND(AND(ISNUMBER(A25),ISNUMBER(B25),B25&gt;A25),SUMPRODUCT(ISNUMBER($A$6:$A$35)*ISNUMBER($B$6:$B$35)*($A$6:$A$35&lt;B25)*($B$6:$B$35&gt;A25))&gt;1),"Overlaps another trip","")</f>
         <v/>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="29"/>
-      <c r="B26" s="29"/>
+      <c r="A26" s="30"/>
+      <c r="B26" s="30"/>
       <c r="C26" s="12"/>
-      <c r="D26" s="30" t="n">
+      <c r="D26" s="31" t="n">
         <f aca="false">IF(AND(ISNUMBER(A26),ISNUMBER(B26),B26&gt;A26),MAX(0,MIN(B26-1,DATE(2026,12,31))-MAX(A26+1,DATE(2026,1,1))+1),0)</f>
         <v>0</v>
       </c>
-      <c r="E26" s="30" t="n">
+      <c r="E26" s="31" t="n">
         <f aca="false">IF(AND(ISNUMBER(A26),ISNUMBER(B26),B26&gt;A26),AND(A26&gt;=DATE(2026,1,1),A26&lt;=DATE(2026,12,31))*1+AND(B26&gt;=DATE(2026,1,1),B26&lt;=DATE(2026,12,31))*1,0)</f>
         <v>0</v>
       </c>
-      <c r="F26" s="25" t="n">
+      <c r="F26" s="26" t="n">
         <f aca="false">(D26-MIN(C26,D26))*Data!$C$60+MIN(C26,D26)*Data!$C$61+E26*Data!$C$60*Data!$C$62</f>
         <v>0</v>
       </c>
-      <c r="G26" s="31" t="str">
+      <c r="G26" s="32" t="str">
         <f aca="false">IF(AND(AND(ISNUMBER(A26),ISNUMBER(B26),B26&gt;A26),SUMPRODUCT(ISNUMBER($A$6:$A$35)*ISNUMBER($B$6:$B$35)*($A$6:$A$35&lt;B26)*($B$6:$B$35&gt;A26))&gt;1),"Overlaps another trip","")</f>
         <v/>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="29"/>
-      <c r="B27" s="29"/>
+      <c r="A27" s="30"/>
+      <c r="B27" s="30"/>
       <c r="C27" s="12"/>
-      <c r="D27" s="30" t="n">
+      <c r="D27" s="31" t="n">
         <f aca="false">IF(AND(ISNUMBER(A27),ISNUMBER(B27),B27&gt;A27),MAX(0,MIN(B27-1,DATE(2026,12,31))-MAX(A27+1,DATE(2026,1,1))+1),0)</f>
         <v>0</v>
       </c>
-      <c r="E27" s="30" t="n">
+      <c r="E27" s="31" t="n">
         <f aca="false">IF(AND(ISNUMBER(A27),ISNUMBER(B27),B27&gt;A27),AND(A27&gt;=DATE(2026,1,1),A27&lt;=DATE(2026,12,31))*1+AND(B27&gt;=DATE(2026,1,1),B27&lt;=DATE(2026,12,31))*1,0)</f>
         <v>0</v>
       </c>
-      <c r="F27" s="25" t="n">
+      <c r="F27" s="26" t="n">
         <f aca="false">(D27-MIN(C27,D27))*Data!$C$60+MIN(C27,D27)*Data!$C$61+E27*Data!$C$60*Data!$C$62</f>
         <v>0</v>
       </c>
-      <c r="G27" s="31" t="str">
+      <c r="G27" s="32" t="str">
         <f aca="false">IF(AND(AND(ISNUMBER(A27),ISNUMBER(B27),B27&gt;A27),SUMPRODUCT(ISNUMBER($A$6:$A$35)*ISNUMBER($B$6:$B$35)*($A$6:$A$35&lt;B27)*($B$6:$B$35&gt;A27))&gt;1),"Overlaps another trip","")</f>
         <v/>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="29"/>
-      <c r="B28" s="29"/>
+      <c r="A28" s="30"/>
+      <c r="B28" s="30"/>
       <c r="C28" s="12"/>
-      <c r="D28" s="30" t="n">
+      <c r="D28" s="31" t="n">
         <f aca="false">IF(AND(ISNUMBER(A28),ISNUMBER(B28),B28&gt;A28),MAX(0,MIN(B28-1,DATE(2026,12,31))-MAX(A28+1,DATE(2026,1,1))+1),0)</f>
         <v>0</v>
       </c>
-      <c r="E28" s="30" t="n">
+      <c r="E28" s="31" t="n">
         <f aca="false">IF(AND(ISNUMBER(A28),ISNUMBER(B28),B28&gt;A28),AND(A28&gt;=DATE(2026,1,1),A28&lt;=DATE(2026,12,31))*1+AND(B28&gt;=DATE(2026,1,1),B28&lt;=DATE(2026,12,31))*1,0)</f>
         <v>0</v>
       </c>
-      <c r="F28" s="25" t="n">
+      <c r="F28" s="26" t="n">
         <f aca="false">(D28-MIN(C28,D28))*Data!$C$60+MIN(C28,D28)*Data!$C$61+E28*Data!$C$60*Data!$C$62</f>
         <v>0</v>
       </c>
-      <c r="G28" s="31" t="str">
+      <c r="G28" s="32" t="str">
         <f aca="false">IF(AND(AND(ISNUMBER(A28),ISNUMBER(B28),B28&gt;A28),SUMPRODUCT(ISNUMBER($A$6:$A$35)*ISNUMBER($B$6:$B$35)*($A$6:$A$35&lt;B28)*($B$6:$B$35&gt;A28))&gt;1),"Overlaps another trip","")</f>
         <v/>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="29"/>
-      <c r="B29" s="29"/>
+      <c r="A29" s="30"/>
+      <c r="B29" s="30"/>
       <c r="C29" s="12"/>
-      <c r="D29" s="30" t="n">
+      <c r="D29" s="31" t="n">
         <f aca="false">IF(AND(ISNUMBER(A29),ISNUMBER(B29),B29&gt;A29),MAX(0,MIN(B29-1,DATE(2026,12,31))-MAX(A29+1,DATE(2026,1,1))+1),0)</f>
         <v>0</v>
       </c>
-      <c r="E29" s="30" t="n">
+      <c r="E29" s="31" t="n">
         <f aca="false">IF(AND(ISNUMBER(A29),ISNUMBER(B29),B29&gt;A29),AND(A29&gt;=DATE(2026,1,1),A29&lt;=DATE(2026,12,31))*1+AND(B29&gt;=DATE(2026,1,1),B29&lt;=DATE(2026,12,31))*1,0)</f>
         <v>0</v>
       </c>
-      <c r="F29" s="25" t="n">
+      <c r="F29" s="26" t="n">
         <f aca="false">(D29-MIN(C29,D29))*Data!$C$60+MIN(C29,D29)*Data!$C$61+E29*Data!$C$60*Data!$C$62</f>
         <v>0</v>
       </c>
-      <c r="G29" s="31" t="str">
+      <c r="G29" s="32" t="str">
         <f aca="false">IF(AND(AND(ISNUMBER(A29),ISNUMBER(B29),B29&gt;A29),SUMPRODUCT(ISNUMBER($A$6:$A$35)*ISNUMBER($B$6:$B$35)*($A$6:$A$35&lt;B29)*($B$6:$B$35&gt;A29))&gt;1),"Overlaps another trip","")</f>
         <v/>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="29"/>
-      <c r="B30" s="29"/>
+      <c r="A30" s="30"/>
+      <c r="B30" s="30"/>
       <c r="C30" s="12"/>
-      <c r="D30" s="30" t="n">
+      <c r="D30" s="31" t="n">
         <f aca="false">IF(AND(ISNUMBER(A30),ISNUMBER(B30),B30&gt;A30),MAX(0,MIN(B30-1,DATE(2026,12,31))-MAX(A30+1,DATE(2026,1,1))+1),0)</f>
         <v>0</v>
       </c>
-      <c r="E30" s="30" t="n">
+      <c r="E30" s="31" t="n">
         <f aca="false">IF(AND(ISNUMBER(A30),ISNUMBER(B30),B30&gt;A30),AND(A30&gt;=DATE(2026,1,1),A30&lt;=DATE(2026,12,31))*1+AND(B30&gt;=DATE(2026,1,1),B30&lt;=DATE(2026,12,31))*1,0)</f>
         <v>0</v>
       </c>
-      <c r="F30" s="25" t="n">
+      <c r="F30" s="26" t="n">
         <f aca="false">(D30-MIN(C30,D30))*Data!$C$60+MIN(C30,D30)*Data!$C$61+E30*Data!$C$60*Data!$C$62</f>
         <v>0</v>
       </c>
-      <c r="G30" s="31" t="str">
+      <c r="G30" s="32" t="str">
         <f aca="false">IF(AND(AND(ISNUMBER(A30),ISNUMBER(B30),B30&gt;A30),SUMPRODUCT(ISNUMBER($A$6:$A$35)*ISNUMBER($B$6:$B$35)*($A$6:$A$35&lt;B30)*($B$6:$B$35&gt;A30))&gt;1),"Overlaps another trip","")</f>
         <v/>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="29"/>
-      <c r="B31" s="29"/>
+      <c r="A31" s="30"/>
+      <c r="B31" s="30"/>
       <c r="C31" s="12"/>
-      <c r="D31" s="30" t="n">
+      <c r="D31" s="31" t="n">
         <f aca="false">IF(AND(ISNUMBER(A31),ISNUMBER(B31),B31&gt;A31),MAX(0,MIN(B31-1,DATE(2026,12,31))-MAX(A31+1,DATE(2026,1,1))+1),0)</f>
         <v>0</v>
       </c>
-      <c r="E31" s="30" t="n">
+      <c r="E31" s="31" t="n">
         <f aca="false">IF(AND(ISNUMBER(A31),ISNUMBER(B31),B31&gt;A31),AND(A31&gt;=DATE(2026,1,1),A31&lt;=DATE(2026,12,31))*1+AND(B31&gt;=DATE(2026,1,1),B31&lt;=DATE(2026,12,31))*1,0)</f>
         <v>0</v>
       </c>
-      <c r="F31" s="25" t="n">
+      <c r="F31" s="26" t="n">
         <f aca="false">(D31-MIN(C31,D31))*Data!$C$60+MIN(C31,D31)*Data!$C$61+E31*Data!$C$60*Data!$C$62</f>
         <v>0</v>
       </c>
-      <c r="G31" s="31" t="str">
+      <c r="G31" s="32" t="str">
         <f aca="false">IF(AND(AND(ISNUMBER(A31),ISNUMBER(B31),B31&gt;A31),SUMPRODUCT(ISNUMBER($A$6:$A$35)*ISNUMBER($B$6:$B$35)*($A$6:$A$35&lt;B31)*($B$6:$B$35&gt;A31))&gt;1),"Overlaps another trip","")</f>
         <v/>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="29"/>
-      <c r="B32" s="29"/>
+      <c r="A32" s="30"/>
+      <c r="B32" s="30"/>
       <c r="C32" s="12"/>
-      <c r="D32" s="30" t="n">
+      <c r="D32" s="31" t="n">
         <f aca="false">IF(AND(ISNUMBER(A32),ISNUMBER(B32),B32&gt;A32),MAX(0,MIN(B32-1,DATE(2026,12,31))-MAX(A32+1,DATE(2026,1,1))+1),0)</f>
         <v>0</v>
       </c>
-      <c r="E32" s="30" t="n">
+      <c r="E32" s="31" t="n">
         <f aca="false">IF(AND(ISNUMBER(A32),ISNUMBER(B32),B32&gt;A32),AND(A32&gt;=DATE(2026,1,1),A32&lt;=DATE(2026,12,31))*1+AND(B32&gt;=DATE(2026,1,1),B32&lt;=DATE(2026,12,31))*1,0)</f>
         <v>0</v>
       </c>
-      <c r="F32" s="25" t="n">
+      <c r="F32" s="26" t="n">
         <f aca="false">(D32-MIN(C32,D32))*Data!$C$60+MIN(C32,D32)*Data!$C$61+E32*Data!$C$60*Data!$C$62</f>
         <v>0</v>
       </c>
-      <c r="G32" s="31" t="str">
+      <c r="G32" s="32" t="str">
         <f aca="false">IF(AND(AND(ISNUMBER(A32),ISNUMBER(B32),B32&gt;A32),SUMPRODUCT(ISNUMBER($A$6:$A$35)*ISNUMBER($B$6:$B$35)*($A$6:$A$35&lt;B32)*($B$6:$B$35&gt;A32))&gt;1),"Overlaps another trip","")</f>
         <v/>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="29"/>
-      <c r="B33" s="29"/>
+      <c r="A33" s="30"/>
+      <c r="B33" s="30"/>
       <c r="C33" s="12"/>
-      <c r="D33" s="30" t="n">
+      <c r="D33" s="31" t="n">
         <f aca="false">IF(AND(ISNUMBER(A33),ISNUMBER(B33),B33&gt;A33),MAX(0,MIN(B33-1,DATE(2026,12,31))-MAX(A33+1,DATE(2026,1,1))+1),0)</f>
         <v>0</v>
       </c>
-      <c r="E33" s="30" t="n">
+      <c r="E33" s="31" t="n">
         <f aca="false">IF(AND(ISNUMBER(A33),ISNUMBER(B33),B33&gt;A33),AND(A33&gt;=DATE(2026,1,1),A33&lt;=DATE(2026,12,31))*1+AND(B33&gt;=DATE(2026,1,1),B33&lt;=DATE(2026,12,31))*1,0)</f>
         <v>0</v>
       </c>
-      <c r="F33" s="25" t="n">
+      <c r="F33" s="26" t="n">
         <f aca="false">(D33-MIN(C33,D33))*Data!$C$60+MIN(C33,D33)*Data!$C$61+E33*Data!$C$60*Data!$C$62</f>
         <v>0</v>
       </c>
-      <c r="G33" s="31" t="str">
+      <c r="G33" s="32" t="str">
         <f aca="false">IF(AND(AND(ISNUMBER(A33),ISNUMBER(B33),B33&gt;A33),SUMPRODUCT(ISNUMBER($A$6:$A$35)*ISNUMBER($B$6:$B$35)*($A$6:$A$35&lt;B33)*($B$6:$B$35&gt;A33))&gt;1),"Overlaps another trip","")</f>
         <v/>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="29"/>
-      <c r="B34" s="29"/>
+      <c r="A34" s="30"/>
+      <c r="B34" s="30"/>
       <c r="C34" s="12"/>
-      <c r="D34" s="30" t="n">
+      <c r="D34" s="31" t="n">
         <f aca="false">IF(AND(ISNUMBER(A34),ISNUMBER(B34),B34&gt;A34),MAX(0,MIN(B34-1,DATE(2026,12,31))-MAX(A34+1,DATE(2026,1,1))+1),0)</f>
         <v>0</v>
       </c>
-      <c r="E34" s="30" t="n">
+      <c r="E34" s="31" t="n">
         <f aca="false">IF(AND(ISNUMBER(A34),ISNUMBER(B34),B34&gt;A34),AND(A34&gt;=DATE(2026,1,1),A34&lt;=DATE(2026,12,31))*1+AND(B34&gt;=DATE(2026,1,1),B34&lt;=DATE(2026,12,31))*1,0)</f>
         <v>0</v>
       </c>
-      <c r="F34" s="25" t="n">
+      <c r="F34" s="26" t="n">
         <f aca="false">(D34-MIN(C34,D34))*Data!$C$60+MIN(C34,D34)*Data!$C$61+E34*Data!$C$60*Data!$C$62</f>
         <v>0</v>
       </c>
-      <c r="G34" s="31" t="str">
+      <c r="G34" s="32" t="str">
         <f aca="false">IF(AND(AND(ISNUMBER(A34),ISNUMBER(B34),B34&gt;A34),SUMPRODUCT(ISNUMBER($A$6:$A$35)*ISNUMBER($B$6:$B$35)*($A$6:$A$35&lt;B34)*($B$6:$B$35&gt;A34))&gt;1),"Overlaps another trip","")</f>
         <v/>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="29"/>
-      <c r="B35" s="29"/>
+      <c r="A35" s="30"/>
+      <c r="B35" s="30"/>
       <c r="C35" s="12"/>
-      <c r="D35" s="30" t="n">
+      <c r="D35" s="31" t="n">
         <f aca="false">IF(AND(ISNUMBER(A35),ISNUMBER(B35),B35&gt;A35),MAX(0,MIN(B35-1,DATE(2026,12,31))-MAX(A35+1,DATE(2026,1,1))+1),0)</f>
         <v>0</v>
       </c>
-      <c r="E35" s="30" t="n">
+      <c r="E35" s="31" t="n">
         <f aca="false">IF(AND(ISNUMBER(A35),ISNUMBER(B35),B35&gt;A35),AND(A35&gt;=DATE(2026,1,1),A35&lt;=DATE(2026,12,31))*1+AND(B35&gt;=DATE(2026,1,1),B35&lt;=DATE(2026,12,31))*1,0)</f>
         <v>0</v>
       </c>
-      <c r="F35" s="25" t="n">
+      <c r="F35" s="26" t="n">
         <f aca="false">(D35-MIN(C35,D35))*Data!$C$60+MIN(C35,D35)*Data!$C$61+E35*Data!$C$60*Data!$C$62</f>
         <v>0</v>
       </c>
-      <c r="G35" s="31" t="str">
+      <c r="G35" s="32" t="str">
         <f aca="false">IF(AND(AND(ISNUMBER(A35),ISNUMBER(B35),B35&gt;A35),SUMPRODUCT(ISNUMBER($A$6:$A$35)*ISNUMBER($B$6:$B$35)*($A$6:$A$35&lt;B35)*($B$6:$B$35&gt;A35))&gt;1),"Overlaps another trip","")</f>
         <v/>
       </c>
@@ -6349,15 +6543,15 @@
       <c r="A36" s="9" t="s">
         <v>53</v>
       </c>
-      <c r="C36" s="32" t="n">
+      <c r="C36" s="33" t="n">
         <f aca="false">SUM(C6:C35)</f>
         <v>0</v>
       </c>
-      <c r="D36" s="32" t="n">
+      <c r="D36" s="33" t="n">
         <f aca="false">SUM(D6:D35)</f>
         <v>0</v>
       </c>
-      <c r="E36" s="32" t="n">
+      <c r="E36" s="33" t="n">
         <f aca="false">SUM(E6:E35)</f>
         <v>0</v>
       </c>
@@ -6368,16 +6562,16 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E37" s="9" t="s">
-        <v>245</v>
-      </c>
-      <c r="F37" s="33" t="n">
+        <v>253</v>
+      </c>
+      <c r="F37" s="34" t="n">
         <f aca="false">F36*Data!$C$63</f>
         <v>0</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="17" t="s">
-        <v>246</v>
+        <v>254</v>
       </c>
       <c r="B39" s="17"/>
       <c r="C39" s="17"/>
@@ -6430,66 +6624,66 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>247</v>
+        <v>255</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>248</v>
+        <v>256</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="14" t="s">
-        <v>249</v>
+        <v>257</v>
       </c>
       <c r="B4" s="14" t="s">
-        <v>250</v>
+        <v>258</v>
       </c>
       <c r="C4" s="14" t="s">
-        <v>251</v>
+        <v>259</v>
       </c>
       <c r="D4" s="14" t="s">
-        <v>252</v>
+        <v>260</v>
       </c>
       <c r="E4" s="14" t="s">
-        <v>251</v>
+        <v>259</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
-        <v>253</v>
+        <v>261</v>
       </c>
       <c r="B5" s="19"/>
-      <c r="C5" s="29"/>
+      <c r="C5" s="30"/>
       <c r="D5" s="19"/>
-      <c r="E5" s="29"/>
+      <c r="E5" s="30"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>254</v>
+        <v>262</v>
       </c>
       <c r="B6" s="19"/>
-      <c r="C6" s="29"/>
+      <c r="C6" s="30"/>
       <c r="D6" s="19"/>
-      <c r="E6" s="29"/>
+      <c r="E6" s="30"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>255</v>
+        <v>263</v>
       </c>
       <c r="B7" s="19"/>
-      <c r="C7" s="29"/>
+      <c r="C7" s="30"/>
       <c r="D7" s="19"/>
-      <c r="E7" s="29"/>
+      <c r="E7" s="30"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>256</v>
+        <v>264</v>
       </c>
       <c r="B8" s="19"/>
-      <c r="C8" s="29"/>
+      <c r="C8" s="30"/>
       <c r="D8" s="19"/>
-      <c r="E8" s="29"/>
+      <c r="E8" s="30"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="9" t="s">
@@ -6530,53 +6724,53 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>257</v>
+        <v>265</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>258</v>
+        <v>266</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>259</v>
+        <v>267</v>
       </c>
       <c r="B4" s="10"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
-        <v>260</v>
+        <v>268</v>
       </c>
       <c r="B5" s="10"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>261</v>
+        <v>269</v>
       </c>
       <c r="B6" s="10"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>262</v>
+        <v>270</v>
       </c>
       <c r="B7" s="10"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>263</v>
+        <v>271</v>
       </c>
       <c r="B8" s="10"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="s">
-        <v>264</v>
+        <v>272</v>
       </c>
       <c r="B9" s="10"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="6" t="s">
-        <v>265</v>
+        <v>273</v>
       </c>
       <c r="B10" s="10"/>
     </row>

</xml_diff>

<commit_message>
Fix IRA phase-out, retirement-only uploads and savings questions found by QA
- IRA: the workplace-plan phase-out reduces the limit, not the
  contribution (Pub. 590-A worksheet 1-2)
- Organizers with only Social Security, retirement or K-1 income upload
- 55+ (HSA catch-up, also at 65) and spouse 50+ questions in the
  estimator; married filing separately can report a covered spouse
  (estimator and MFS print form)
- Withholding on SSA-1099/1099-R/1099-G kept separate from W-2
  withholding end to end, so the summary only asks about W-2 withholding
  without wages
- Excel spouse 50+ limited to joint returns; Data rate rows moved to
  C80:C87; QA regression tests added

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012ebqUPkXNMCm1mSUdBK3xi
</commit_message>
<xml_diff>
--- a/tax-prep/downloads/falcon-tax-organizer-2026.xlsx
+++ b/tax-prep/downloads/falcon-tax-organizer-2026.xlsx
@@ -34,7 +34,7 @@
     <author>Unknown Author</author>
   </authors>
   <commentList>
-    <comment ref="C60" authorId="0">
+    <comment ref="C80" authorId="0">
       <text>
         <r>
           <rPr>
@@ -51,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="578" uniqueCount="498">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="580" uniqueCount="500">
   <si>
     <t xml:space="preserve">Falcon Tax Solutions · 2026 Tax Organizer</t>
   </si>
@@ -1055,7 +1055,7 @@
     <t xml:space="preserve">withheld</t>
   </si>
   <si>
-    <t xml:space="preserve">Federal tax withheld (W-2 and other forms)</t>
+    <t xml:space="preserve">Federal tax withheld (W-2)</t>
   </si>
   <si>
     <t xml:space="preserve">Idaho</t>
@@ -1064,16 +1064,28 @@
     <t xml:space="preserve">ID</t>
   </si>
   <si>
+    <t xml:space="preserve">otherWithheld</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Federal tax withheld on SSA-1099 / 1099-R / 1099-G</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Illinois</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IL</t>
+  </si>
+  <si>
     <t xml:space="preserve">stateWithheld</t>
   </si>
   <si>
     <t xml:space="preserve">State tax withheld</t>
   </si>
   <si>
-    <t xml:space="preserve">Illinois</t>
-  </si>
-  <si>
-    <t xml:space="preserve">IL</t>
+    <t xml:space="preserve">Indiana</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IN</t>
   </si>
   <si>
     <t xml:space="preserve">tips</t>
@@ -1082,10 +1094,10 @@
     <t xml:space="preserve">Tips (W-2 and cash)</t>
   </si>
   <si>
-    <t xml:space="preserve">Indiana</t>
-  </si>
-  <si>
-    <t xml:space="preserve">IN</t>
+    <t xml:space="preserve">Iowa</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IA</t>
   </si>
   <si>
     <t xml:space="preserve">overtimePremium</t>
@@ -1094,10 +1106,10 @@
     <t xml:space="preserve">Overtime premium</t>
   </si>
   <si>
-    <t xml:space="preserve">Iowa</t>
-  </si>
-  <si>
-    <t xml:space="preserve">IA</t>
+    <t xml:space="preserve">Kansas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KS</t>
   </si>
   <si>
     <t xml:space="preserve">seIncome</t>
@@ -1106,10 +1118,10 @@
     <t xml:space="preserve">Self-employment income</t>
   </si>
   <si>
-    <t xml:space="preserve">Kansas</t>
-  </si>
-  <si>
-    <t xml:space="preserve">KS</t>
+    <t xml:space="preserve">Kentucky</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KY</t>
   </si>
   <si>
     <t xml:space="preserve">seExpenses</t>
@@ -1118,10 +1130,10 @@
     <t xml:space="preserve">Deductible business expenses</t>
   </si>
   <si>
-    <t xml:space="preserve">Kentucky</t>
-  </si>
-  <si>
-    <t xml:space="preserve">KY</t>
+    <t xml:space="preserve">Louisiana</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LA</t>
   </si>
   <si>
     <t xml:space="preserve">estimatedPayments</t>
@@ -1130,10 +1142,10 @@
     <t xml:space="preserve">Federal estimated payments</t>
   </si>
   <si>
-    <t xml:space="preserve">Louisiana</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LA</t>
+    <t xml:space="preserve">Maine</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ME</t>
   </si>
   <si>
     <t xml:space="preserve">stateEstimated</t>
@@ -1142,10 +1154,10 @@
     <t xml:space="preserve">State estimated payments</t>
   </si>
   <si>
-    <t xml:space="preserve">Maine</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ME</t>
+    <t xml:space="preserve">Maryland</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MD</t>
   </si>
   <si>
     <t xml:space="preserve">isTrucker</t>
@@ -1154,10 +1166,10 @@
     <t xml:space="preserve">Logged truck driver trips</t>
   </si>
   <si>
-    <t xml:space="preserve">Maryland</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MD</t>
+    <t xml:space="preserve">Massachusetts</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MA</t>
   </si>
   <si>
     <t xml:space="preserve">perDiemFull</t>
@@ -1166,10 +1178,10 @@
     <t xml:space="preserve">Full days away (U.S. and Canada)</t>
   </si>
   <si>
-    <t xml:space="preserve">Massachusetts</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MA</t>
+    <t xml:space="preserve">Michigan</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MI</t>
   </si>
   <si>
     <t xml:space="preserve">perDiemCanada</t>
@@ -1178,19 +1190,19 @@
     <t xml:space="preserve">Of those, full days in Canada</t>
   </si>
   <si>
-    <t xml:space="preserve">Michigan</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MI</t>
+    <t xml:space="preserve">Minnesota</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MN</t>
   </si>
   <si>
     <t xml:space="preserve">perDiemPartial</t>
   </si>
   <si>
-    <t xml:space="preserve">Minnesota</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MN</t>
+    <t xml:space="preserve">Mississippi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MS</t>
   </si>
   <si>
     <t xml:space="preserve">usesCar</t>
@@ -1199,10 +1211,10 @@
     <t xml:space="preserve">Uses a car for business (Car tab)</t>
   </si>
   <si>
-    <t xml:space="preserve">Mississippi</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MS</t>
+    <t xml:space="preserve">Missouri</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MO</t>
   </si>
   <si>
     <t xml:space="preserve">carMilesH1</t>
@@ -1211,10 +1223,10 @@
     <t xml:space="preserve">Business miles Jan-Jun</t>
   </si>
   <si>
-    <t xml:space="preserve">Missouri</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MO</t>
+    <t xml:space="preserve">Montana</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MT</t>
   </si>
   <si>
     <t xml:space="preserve">carMilesH2</t>
@@ -1223,10 +1235,10 @@
     <t xml:space="preserve">Business miles Jul-Dec</t>
   </si>
   <si>
-    <t xml:space="preserve">Montana</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MT</t>
+    <t xml:space="preserve">Nebraska</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NE</t>
   </si>
   <si>
     <t xml:space="preserve">carMilesTotal</t>
@@ -1235,10 +1247,10 @@
     <t xml:space="preserve">All miles driven in 2026</t>
   </si>
   <si>
-    <t xml:space="preserve">Nebraska</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NE</t>
+    <t xml:space="preserve">Nevada</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NV</t>
   </si>
   <si>
     <t xml:space="preserve">carCosts</t>
@@ -1247,19 +1259,19 @@
     <t xml:space="preserve">Actual car costs (before business share)</t>
   </si>
   <si>
-    <t xml:space="preserve">Nevada</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NV</t>
+    <t xml:space="preserve">New Hampshire</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NH</t>
   </si>
   <si>
     <t xml:space="preserve">interest</t>
   </si>
   <si>
-    <t xml:space="preserve">New Hampshire</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NH</t>
+    <t xml:space="preserve">New Jersey</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NJ</t>
   </si>
   <si>
     <t xml:space="preserve">unemployment</t>
@@ -1268,10 +1280,10 @@
     <t xml:space="preserve">Unemployment</t>
   </si>
   <si>
-    <t xml:space="preserve">New Jersey</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NJ</t>
+    <t xml:space="preserve">New Mexico</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NM</t>
   </si>
   <si>
     <t xml:space="preserve">otherIncome</t>
@@ -1280,10 +1292,10 @@
     <t xml:space="preserve">Other taxable income</t>
   </si>
   <si>
-    <t xml:space="preserve">New Mexico</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NM</t>
+    <t xml:space="preserve">New York</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NY</t>
   </si>
   <si>
     <t xml:space="preserve">retirementIncome</t>
@@ -1292,10 +1304,10 @@
     <t xml:space="preserve">Retirement withdrawals (taxable)</t>
   </si>
   <si>
-    <t xml:space="preserve">New York</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NY</t>
+    <t xml:space="preserve">North Carolina</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NC</t>
   </si>
   <si>
     <t xml:space="preserve">socialSecurity</t>
@@ -1304,10 +1316,10 @@
     <t xml:space="preserve">Social Security benefits</t>
   </si>
   <si>
-    <t xml:space="preserve">North Carolina</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NC</t>
+    <t xml:space="preserve">North Dakota</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ND</t>
   </si>
   <si>
     <t xml:space="preserve">iraYou</t>
@@ -1316,10 +1328,10 @@
     <t xml:space="preserve">IRA contribution: you</t>
   </si>
   <si>
-    <t xml:space="preserve">North Dakota</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ND</t>
+    <t xml:space="preserve">Ohio</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OH</t>
   </si>
   <si>
     <t xml:space="preserve">iraSpouse</t>
@@ -1328,10 +1340,10 @@
     <t xml:space="preserve">IRA contribution: spouse</t>
   </si>
   <si>
-    <t xml:space="preserve">Ohio</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OH</t>
+    <t xml:space="preserve">Oklahoma</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OK</t>
   </si>
   <si>
     <t xml:space="preserve">iraCoveredYou</t>
@@ -1340,10 +1352,10 @@
     <t xml:space="preserve">You covered by a workplace plan</t>
   </si>
   <si>
-    <t xml:space="preserve">Oklahoma</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OK</t>
+    <t xml:space="preserve">Oregon</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OR</t>
   </si>
   <si>
     <t xml:space="preserve">iraCoveredSpouse</t>
@@ -1352,10 +1364,10 @@
     <t xml:space="preserve">Spouse covered by a workplace plan</t>
   </si>
   <si>
-    <t xml:space="preserve">Oregon</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OR</t>
+    <t xml:space="preserve">Pennsylvania</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PA</t>
   </si>
   <si>
     <t xml:space="preserve">hsaContribution</t>
@@ -1364,10 +1376,10 @@
     <t xml:space="preserve">HSA contributions</t>
   </si>
   <si>
-    <t xml:space="preserve">Pennsylvania</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PA</t>
+    <t xml:space="preserve">Rhode Island</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RI</t>
   </si>
   <si>
     <t xml:space="preserve">hsaFamily</t>
@@ -1376,10 +1388,10 @@
     <t xml:space="preserve">HSA family coverage</t>
   </si>
   <si>
-    <t xml:space="preserve">Rhode Island</t>
-  </si>
-  <si>
-    <t xml:space="preserve">RI</t>
+    <t xml:space="preserve">South Carolina</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SC</t>
   </si>
   <si>
     <t xml:space="preserve">sepContribution</t>
@@ -1388,10 +1400,10 @@
     <t xml:space="preserve">SEP / solo 401(k)</t>
   </si>
   <si>
-    <t xml:space="preserve">South Carolina</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SC</t>
+    <t xml:space="preserve">South Dakota</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SD</t>
   </si>
   <si>
     <t xml:space="preserve">k1Partnership</t>
@@ -1400,10 +1412,10 @@
     <t xml:space="preserve">K-1 box 1, partnerships / LLCs</t>
   </si>
   <si>
-    <t xml:space="preserve">South Dakota</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SD</t>
+    <t xml:space="preserve">Tennessee</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TN</t>
   </si>
   <si>
     <t xml:space="preserve">k1Guaranteed</t>
@@ -1412,10 +1424,10 @@
     <t xml:space="preserve">K-1 guaranteed payments</t>
   </si>
   <si>
-    <t xml:space="preserve">Tennessee</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TN</t>
+    <t xml:space="preserve">Texas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TX</t>
   </si>
   <si>
     <t xml:space="preserve">k1SCorp</t>
@@ -1424,10 +1436,10 @@
     <t xml:space="preserve">K-1 box 1, S-corps</t>
   </si>
   <si>
-    <t xml:space="preserve">Texas</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TX</t>
+    <t xml:space="preserve">Utah</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UT</t>
   </si>
   <si>
     <t xml:space="preserve">k1Se</t>
@@ -1436,10 +1448,10 @@
     <t xml:space="preserve">K-1 self-employment earnings</t>
   </si>
   <si>
-    <t xml:space="preserve">Utah</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UT</t>
+    <t xml:space="preserve">Vermont</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VT</t>
   </si>
   <si>
     <t xml:space="preserve">you50</t>
@@ -1448,22 +1460,22 @@
     <t xml:space="preserve">You 50 or older (born 1976 or earlier)</t>
   </si>
   <si>
-    <t xml:space="preserve">Vermont</t>
-  </si>
-  <si>
-    <t xml:space="preserve">VT</t>
+    <t xml:space="preserve">Virginia</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VA</t>
   </si>
   <si>
     <t xml:space="preserve">spouse50</t>
   </si>
   <si>
-    <t xml:space="preserve">Spouse 50 or older</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Virginia</t>
-  </si>
-  <si>
-    <t xml:space="preserve">VA</t>
+    <t xml:space="preserve">Spouse 50 or older (joint returns)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Washington</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WA</t>
   </si>
   <si>
     <t xml:space="preserve">you55</t>
@@ -1472,10 +1484,10 @@
     <t xml:space="preserve">You 55 or older (HSA catch-up)</t>
   </si>
   <si>
-    <t xml:space="preserve">Washington</t>
-  </si>
-  <si>
-    <t xml:space="preserve">WA</t>
+    <t xml:space="preserve">West Virginia</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WV</t>
   </si>
   <si>
     <t xml:space="preserve">retirement</t>
@@ -1484,28 +1496,22 @@
     <t xml:space="preserve">Has retirement withdrawals</t>
   </si>
   <si>
-    <t xml:space="preserve">West Virginia</t>
-  </si>
-  <si>
-    <t xml:space="preserve">WV</t>
+    <t xml:space="preserve">Wisconsin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WI</t>
   </si>
   <si>
     <t xml:space="preserve">hasInvestments</t>
   </si>
   <si>
-    <t xml:space="preserve">Wisconsin</t>
-  </si>
-  <si>
-    <t xml:space="preserve">WI</t>
+    <t xml:space="preserve">Wyoming</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WY</t>
   </si>
   <si>
     <t xml:space="preserve">mortgage</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Wyoming</t>
-  </si>
-  <si>
-    <t xml:space="preserve">WY</t>
   </si>
   <si>
     <t xml:space="preserve">studentLoan</t>
@@ -2342,7 +2348,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:I67"/>
+  <dimension ref="A1:I87"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="22"/>
@@ -2612,8 +2618,8 @@
       <c r="B14" s="21" t="s">
         <v>334</v>
       </c>
-      <c r="C14" s="6" t="n">
-        <f aca="false">Jobs!D16+N(Income!C30)</f>
+      <c r="C14" s="37" t="n">
+        <f aca="false">Jobs!D16</f>
         <v>0</v>
       </c>
       <c r="H14" s="35" t="s">
@@ -2630,8 +2636,8 @@
       <c r="B15" s="21" t="s">
         <v>338</v>
       </c>
-      <c r="C15" s="37" t="n">
-        <f aca="false">Jobs!E16</f>
+      <c r="C15" s="6" t="n">
+        <f aca="false">N(Income!C30)</f>
         <v>0</v>
       </c>
       <c r="H15" s="35" t="s">
@@ -2648,8 +2654,8 @@
       <c r="B16" s="21" t="s">
         <v>342</v>
       </c>
-      <c r="C16" s="6" t="n">
-        <f aca="false">Jobs!F16+Income!C24</f>
+      <c r="C16" s="37" t="n">
+        <f aca="false">Jobs!E16</f>
         <v>0</v>
       </c>
       <c r="H16" s="35" t="s">
@@ -2666,8 +2672,8 @@
       <c r="B17" s="21" t="s">
         <v>346</v>
       </c>
-      <c r="C17" s="37" t="n">
-        <f aca="false">Jobs!G16</f>
+      <c r="C17" s="6" t="n">
+        <f aca="false">Jobs!F16+Income!C24</f>
         <v>0</v>
       </c>
       <c r="H17" s="35" t="s">
@@ -2685,7 +2691,7 @@
         <v>350</v>
       </c>
       <c r="C18" s="37" t="n">
-        <f aca="false">Income!C19</f>
+        <f aca="false">Jobs!G16</f>
         <v>0</v>
       </c>
       <c r="H18" s="35" t="s">
@@ -2703,7 +2709,7 @@
         <v>354</v>
       </c>
       <c r="C19" s="37" t="n">
-        <f aca="false">Expenses!E85</f>
+        <f aca="false">Income!C19</f>
         <v>0</v>
       </c>
       <c r="H19" s="35" t="s">
@@ -2721,7 +2727,7 @@
         <v>358</v>
       </c>
       <c r="C20" s="37" t="n">
-        <f aca="false">Payments!B9</f>
+        <f aca="false">Expenses!E85</f>
         <v>0</v>
       </c>
       <c r="H20" s="35" t="s">
@@ -2739,7 +2745,7 @@
         <v>362</v>
       </c>
       <c r="C21" s="37" t="n">
-        <f aca="false">Payments!D9</f>
+        <f aca="false">Payments!B9</f>
         <v>0</v>
       </c>
       <c r="H21" s="35" t="s">
@@ -2756,8 +2762,8 @@
       <c r="B22" s="21" t="s">
         <v>366</v>
       </c>
-      <c r="C22" s="6" t="n">
-        <f aca="false">IF(Trips!D36+Trips!E36&gt;0,1,0)</f>
+      <c r="C22" s="37" t="n">
+        <f aca="false">Payments!D9</f>
         <v>0</v>
       </c>
       <c r="H22" s="35" t="s">
@@ -2775,7 +2781,7 @@
         <v>370</v>
       </c>
       <c r="C23" s="6" t="n">
-        <f aca="false">MIN(365,Trips!D36)</f>
+        <f aca="false">IF(Trips!D36+Trips!E36&gt;0,1,0)</f>
         <v>0</v>
       </c>
       <c r="H23" s="35" t="s">
@@ -2793,7 +2799,7 @@
         <v>374</v>
       </c>
       <c r="C24" s="6" t="n">
-        <f aca="false">MIN(C23,SUMPRODUCT((Trips!C6:C35&lt;Trips!D6:D35)*Trips!C6:C35+(Trips!C6:C35&gt;=Trips!D6:D35)*Trips!D6:D35))</f>
+        <f aca="false">MIN(365,Trips!D36)</f>
         <v>0</v>
       </c>
       <c r="H24" s="35" t="s">
@@ -2808,28 +2814,28 @@
         <v>377</v>
       </c>
       <c r="B25" s="21" t="s">
-        <v>248</v>
-      </c>
-      <c r="C25" s="38" t="n">
-        <f aca="false">Trips!E36</f>
+        <v>378</v>
+      </c>
+      <c r="C25" s="6" t="n">
+        <f aca="false">MIN(C23,SUMPRODUCT((Trips!C6:C35&lt;Trips!D6:D35)*Trips!C6:C35+(Trips!C6:C35&gt;=Trips!D6:D35)*Trips!D6:D35))</f>
         <v>0</v>
       </c>
       <c r="H25" s="35" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="I25" s="35" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="9" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="B26" s="21" t="s">
-        <v>381</v>
-      </c>
-      <c r="C26" s="6" t="n">
-        <f aca="false">IF(N(Car!B5)+N(Car!B6)+N(Car!B18)&gt;0,1,0)</f>
+        <v>248</v>
+      </c>
+      <c r="C26" s="38" t="n">
+        <f aca="false">Trips!E36</f>
         <v>0</v>
       </c>
       <c r="H26" s="35" t="s">
@@ -2847,7 +2853,7 @@
         <v>385</v>
       </c>
       <c r="C27" s="6" t="n">
-        <f aca="false">N(Car!B5)</f>
+        <f aca="false">IF(N(Car!B5)+N(Car!B6)+N(Car!B18)&gt;0,1,0)</f>
         <v>0</v>
       </c>
       <c r="H27" s="35" t="s">
@@ -2865,7 +2871,7 @@
         <v>389</v>
       </c>
       <c r="C28" s="6" t="n">
-        <f aca="false">N(Car!B6)</f>
+        <f aca="false">N(Car!B5)</f>
         <v>0</v>
       </c>
       <c r="H28" s="35" t="s">
@@ -2883,7 +2889,7 @@
         <v>393</v>
       </c>
       <c r="C29" s="6" t="n">
-        <f aca="false">N(Car!B7)</f>
+        <f aca="false">N(Car!B6)</f>
         <v>0</v>
       </c>
       <c r="H29" s="35" t="s">
@@ -2901,7 +2907,7 @@
         <v>397</v>
       </c>
       <c r="C30" s="6" t="n">
-        <f aca="false">N(Car!B18)</f>
+        <f aca="false">N(Car!B7)</f>
         <v>0</v>
       </c>
       <c r="H30" s="35" t="s">
@@ -2916,28 +2922,28 @@
         <v>400</v>
       </c>
       <c r="B31" s="21" t="s">
-        <v>70</v>
-      </c>
-      <c r="C31" s="37" t="n">
-        <f aca="false">Income!C25</f>
+        <v>401</v>
+      </c>
+      <c r="C31" s="6" t="n">
+        <f aca="false">N(Car!B18)</f>
         <v>0</v>
       </c>
       <c r="H31" s="35" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="I31" s="35" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="9" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="B32" s="21" t="s">
-        <v>404</v>
+        <v>70</v>
       </c>
       <c r="C32" s="37" t="n">
-        <f aca="false">Income!C26</f>
+        <f aca="false">Income!C25</f>
         <v>0</v>
       </c>
       <c r="H32" s="35" t="s">
@@ -2954,8 +2960,8 @@
       <c r="B33" s="21" t="s">
         <v>408</v>
       </c>
-      <c r="C33" s="6" t="n">
-        <f aca="false">N(Income!C28)</f>
+      <c r="C33" s="37" t="n">
+        <f aca="false">Income!C26</f>
         <v>0</v>
       </c>
       <c r="H33" s="35" t="s">
@@ -2973,7 +2979,7 @@
         <v>412</v>
       </c>
       <c r="C34" s="6" t="n">
-        <f aca="false">N(Income!C27)</f>
+        <f aca="false">N(Income!C28)</f>
         <v>0</v>
       </c>
       <c r="H34" s="35" t="s">
@@ -2991,7 +2997,7 @@
         <v>416</v>
       </c>
       <c r="C35" s="6" t="n">
-        <f aca="false">N(Income!C29)</f>
+        <f aca="false">N(Income!C27)</f>
         <v>0</v>
       </c>
       <c r="H35" s="35" t="s">
@@ -3009,7 +3015,7 @@
         <v>420</v>
       </c>
       <c r="C36" s="6" t="n">
-        <f aca="false">N(Income!C34)</f>
+        <f aca="false">N(Income!C29)</f>
         <v>0</v>
       </c>
       <c r="H36" s="35" t="s">
@@ -3027,7 +3033,7 @@
         <v>424</v>
       </c>
       <c r="C37" s="6" t="n">
-        <f aca="false">N(Income!C35)</f>
+        <f aca="false">N(Income!C34)</f>
         <v>0</v>
       </c>
       <c r="H37" s="35" t="s">
@@ -3045,7 +3051,7 @@
         <v>428</v>
       </c>
       <c r="C38" s="6" t="n">
-        <f aca="false">IF(TRIM(Income!C36)="Yes",1,0)</f>
+        <f aca="false">N(Income!C35)</f>
         <v>0</v>
       </c>
       <c r="H38" s="35" t="s">
@@ -3063,7 +3069,7 @@
         <v>432</v>
       </c>
       <c r="C39" s="6" t="n">
-        <f aca="false">IF(TRIM(Income!C37)="Yes",1,0)</f>
+        <f aca="false">IF(TRIM(Income!C36)="Yes",1,0)</f>
         <v>0</v>
       </c>
       <c r="H39" s="35" t="s">
@@ -3081,7 +3087,7 @@
         <v>436</v>
       </c>
       <c r="C40" s="6" t="n">
-        <f aca="false">N(Income!C38)</f>
+        <f aca="false">IF(TRIM(Income!C37)="Yes",1,0)</f>
         <v>0</v>
       </c>
       <c r="H40" s="35" t="s">
@@ -3099,7 +3105,7 @@
         <v>440</v>
       </c>
       <c r="C41" s="6" t="n">
-        <f aca="false">IF(TRIM(Income!C39)="Family",1,0)</f>
+        <f aca="false">N(Income!C38)</f>
         <v>0</v>
       </c>
       <c r="H41" s="35" t="s">
@@ -3117,7 +3123,7 @@
         <v>444</v>
       </c>
       <c r="C42" s="6" t="n">
-        <f aca="false">N(Income!C40)</f>
+        <f aca="false">IF(TRIM(Income!C39)="Family",1,0)</f>
         <v>0</v>
       </c>
       <c r="H42" s="35" t="s">
@@ -3135,7 +3141,7 @@
         <v>448</v>
       </c>
       <c r="C43" s="6" t="n">
-        <f aca="false">SUMIF(Income!A47:A50,"Partnership / LLC (1065)",Income!C47:C50)</f>
+        <f aca="false">N(Income!C40)</f>
         <v>0</v>
       </c>
       <c r="H43" s="35" t="s">
@@ -3153,7 +3159,7 @@
         <v>452</v>
       </c>
       <c r="C44" s="6" t="n">
-        <f aca="false">SUMIF(Income!A47:A50,"Partnership / LLC (1065)",Income!D47:D50)</f>
+        <f aca="false">SUMIF(Income!A47:A50,"Partnership / LLC (1065)",Income!C47:C50)</f>
         <v>0</v>
       </c>
       <c r="H44" s="35" t="s">
@@ -3171,7 +3177,7 @@
         <v>456</v>
       </c>
       <c r="C45" s="6" t="n">
-        <f aca="false">SUMIF(Income!A47:A50,"S-corp (1120-S)",Income!C47:C50)</f>
+        <f aca="false">SUMIF(Income!A47:A50,"Partnership / LLC (1065)",Income!D47:D50)</f>
         <v>0</v>
       </c>
       <c r="H45" s="35" t="s">
@@ -3189,7 +3195,7 @@
         <v>460</v>
       </c>
       <c r="C46" s="6" t="n">
-        <f aca="false">SUM(Income!F47:F50)</f>
+        <f aca="false">SUMIF(Income!A47:A50,"S-corp (1120-S)",Income!C47:C50)</f>
         <v>0</v>
       </c>
       <c r="H46" s="35" t="s">
@@ -3207,7 +3213,7 @@
         <v>464</v>
       </c>
       <c r="C47" s="6" t="n">
-        <f aca="false">IF(AND(ISNUMBER(Household!B6),Household!B6&gt;0,Household!B6&lt;=1976),1,0)</f>
+        <f aca="false">SUM(Income!F47:F50)</f>
         <v>0</v>
       </c>
       <c r="H47" s="35" t="s">
@@ -3225,7 +3231,7 @@
         <v>468</v>
       </c>
       <c r="C48" s="6" t="n">
-        <f aca="false">IF(AND(ISNUMBER(Household!B7),Household!B7&gt;0,Household!B7&lt;=1976),1,0)</f>
+        <f aca="false">IF(AND(ISNUMBER(Household!B6),Household!B6&gt;0,Household!B6&lt;=1976),1,0)</f>
         <v>0</v>
       </c>
       <c r="H48" s="35" t="s">
@@ -3243,7 +3249,7 @@
         <v>472</v>
       </c>
       <c r="C49" s="6" t="n">
-        <f aca="false">IF(AND(ISNUMBER(Household!B6),Household!B6&gt;0,Household!B6&lt;=1971),1,0)</f>
+        <f aca="false">IF(AND(C5="mfj",ISNUMBER(Household!B7),Household!B7&gt;0,Household!B7&lt;=1976),1,0)</f>
         <v>0</v>
       </c>
       <c r="H49" s="35" t="s">
@@ -3261,7 +3267,7 @@
         <v>476</v>
       </c>
       <c r="C50" s="6" t="n">
-        <f aca="false">IF(Income!C27&gt;0,1,0)</f>
+        <f aca="false">IF(AND(ISNUMBER(Household!B6),Household!B6&gt;0,Household!B6&lt;=1971),1,0)</f>
         <v>0</v>
       </c>
       <c r="H50" s="35" t="s">
@@ -3276,152 +3282,164 @@
         <v>479</v>
       </c>
       <c r="B51" s="21" t="s">
-        <v>267</v>
+        <v>480</v>
       </c>
       <c r="C51" s="6" t="n">
-        <f aca="false">IF(TRIM(Checklist!B4)="Yes",1,0)</f>
+        <f aca="false">IF(Income!C27&gt;0,1,0)</f>
         <v>0</v>
       </c>
       <c r="H51" s="35" t="s">
-        <v>480</v>
+        <v>481</v>
       </c>
       <c r="I51" s="35" t="s">
-        <v>481</v>
+        <v>482</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="9" t="s">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="B52" s="21" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="C52" s="6" t="n">
-        <f aca="false">IF(TRIM(Checklist!B5)="Yes",1,0)</f>
+        <f aca="false">IF(TRIM(Checklist!B4)="Yes",1,0)</f>
         <v>0</v>
       </c>
       <c r="H52" s="35" t="s">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="I52" s="35" t="s">
-        <v>484</v>
+        <v>485</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="9" t="s">
-        <v>485</v>
+        <v>486</v>
       </c>
       <c r="B53" s="21" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="C53" s="6" t="n">
-        <f aca="false">IF(TRIM(Checklist!B6)="Yes",1,0)</f>
+        <f aca="false">IF(TRIM(Checklist!B5)="Yes",1,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="9" t="s">
-        <v>486</v>
+        <v>487</v>
       </c>
       <c r="B54" s="21" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="C54" s="6" t="n">
-        <f aca="false">IF(TRIM(Checklist!B7)="Yes",1,0)</f>
+        <f aca="false">IF(TRIM(Checklist!B6)="Yes",1,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="9" t="s">
-        <v>487</v>
+        <v>488</v>
       </c>
       <c r="B55" s="21" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="C55" s="6" t="n">
-        <f aca="false">IF(TRIM(Checklist!B8)="Yes",1,0)</f>
+        <f aca="false">IF(TRIM(Checklist!B7)="Yes",1,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="9" t="s">
-        <v>488</v>
+        <v>489</v>
       </c>
       <c r="B56" s="21" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="C56" s="6" t="n">
-        <f aca="false">IF(TRIM(Checklist!B9)="Yes",1,0)</f>
+        <f aca="false">IF(TRIM(Checklist!B8)="Yes",1,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="9" t="s">
-        <v>489</v>
+        <v>490</v>
       </c>
       <c r="B57" s="21" t="s">
+        <v>272</v>
+      </c>
+      <c r="C57" s="6" t="n">
+        <f aca="false">IF(TRIM(Checklist!B9)="Yes",1,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A58" s="9" t="s">
+        <v>491</v>
+      </c>
+      <c r="B58" s="21" t="s">
         <v>273</v>
       </c>
-      <c r="C57" s="6" t="n">
+      <c r="C58" s="6" t="n">
         <f aca="false">IF(TRIM(Checklist!B10)="Yes",1,0)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A59" s="39" t="s">
-        <v>490</v>
-      </c>
-    </row>
-    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B60" s="6" t="s">
-        <v>491</v>
-      </c>
-      <c r="C60" s="40" t="n">
+    <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A79" s="39" t="s">
+        <v>492</v>
+      </c>
+    </row>
+    <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B80" s="6" t="s">
+        <v>493</v>
+      </c>
+      <c r="C80" s="40" t="n">
         <v>80</v>
       </c>
     </row>
-    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B61" s="6" t="s">
-        <v>492</v>
-      </c>
-      <c r="C61" s="40" t="n">
+    <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B81" s="6" t="s">
+        <v>494</v>
+      </c>
+      <c r="C81" s="40" t="n">
         <v>86</v>
       </c>
     </row>
-    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B62" s="6" t="s">
-        <v>493</v>
-      </c>
-      <c r="C62" s="41" t="n">
+    <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B82" s="6" t="s">
+        <v>495</v>
+      </c>
+      <c r="C82" s="41" t="n">
         <v>0.75</v>
       </c>
     </row>
-    <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B63" s="6" t="s">
-        <v>494</v>
-      </c>
-      <c r="C63" s="41" t="n">
+    <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B83" s="6" t="s">
+        <v>496</v>
+      </c>
+      <c r="C83" s="41" t="n">
         <v>0.8</v>
       </c>
     </row>
-    <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A65" s="39" t="s">
-        <v>495</v>
-      </c>
-    </row>
-    <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B66" s="6" t="s">
-        <v>496</v>
-      </c>
-      <c r="C66" s="42" t="n">
+    <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A85" s="39" t="s">
+        <v>497</v>
+      </c>
+    </row>
+    <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B86" s="6" t="s">
+        <v>498</v>
+      </c>
+      <c r="C86" s="42" t="n">
         <v>0.725</v>
       </c>
     </row>
-    <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B67" s="6" t="s">
-        <v>497</v>
-      </c>
-      <c r="C67" s="42" t="n">
+    <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B87" s="6" t="s">
+        <v>499</v>
+      </c>
+      <c r="C87" s="42" t="n">
         <v>0.76</v>
       </c>
     </row>
@@ -5780,7 +5798,7 @@
         <v>237</v>
       </c>
       <c r="B20" s="28" t="n">
-        <f aca="false">B5*Data!$C$66+B6*Data!$C$67</f>
+        <f aca="false">B5*Data!$C$86+B6*Data!$C$87</f>
         <v>0</v>
       </c>
     </row>
@@ -5922,7 +5940,7 @@
         <v>0</v>
       </c>
       <c r="F6" s="26" t="n">
-        <f aca="false">(D6-MIN(C6,D6))*Data!$C$60+MIN(C6,D6)*Data!$C$61+E6*Data!$C$60*Data!$C$62</f>
+        <f aca="false">(D6-MIN(C6,D6))*Data!$C$80+MIN(C6,D6)*Data!$C$81+E6*Data!$C$80*Data!$C$82</f>
         <v>0</v>
       </c>
       <c r="G6" s="32" t="str">
@@ -5943,7 +5961,7 @@
         <v>0</v>
       </c>
       <c r="F7" s="26" t="n">
-        <f aca="false">(D7-MIN(C7,D7))*Data!$C$60+MIN(C7,D7)*Data!$C$61+E7*Data!$C$60*Data!$C$62</f>
+        <f aca="false">(D7-MIN(C7,D7))*Data!$C$80+MIN(C7,D7)*Data!$C$81+E7*Data!$C$80*Data!$C$82</f>
         <v>0</v>
       </c>
       <c r="G7" s="32" t="str">
@@ -5964,7 +5982,7 @@
         <v>0</v>
       </c>
       <c r="F8" s="26" t="n">
-        <f aca="false">(D8-MIN(C8,D8))*Data!$C$60+MIN(C8,D8)*Data!$C$61+E8*Data!$C$60*Data!$C$62</f>
+        <f aca="false">(D8-MIN(C8,D8))*Data!$C$80+MIN(C8,D8)*Data!$C$81+E8*Data!$C$80*Data!$C$82</f>
         <v>0</v>
       </c>
       <c r="G8" s="32" t="str">
@@ -5985,7 +6003,7 @@
         <v>0</v>
       </c>
       <c r="F9" s="26" t="n">
-        <f aca="false">(D9-MIN(C9,D9))*Data!$C$60+MIN(C9,D9)*Data!$C$61+E9*Data!$C$60*Data!$C$62</f>
+        <f aca="false">(D9-MIN(C9,D9))*Data!$C$80+MIN(C9,D9)*Data!$C$81+E9*Data!$C$80*Data!$C$82</f>
         <v>0</v>
       </c>
       <c r="G9" s="32" t="str">
@@ -6006,7 +6024,7 @@
         <v>0</v>
       </c>
       <c r="F10" s="26" t="n">
-        <f aca="false">(D10-MIN(C10,D10))*Data!$C$60+MIN(C10,D10)*Data!$C$61+E10*Data!$C$60*Data!$C$62</f>
+        <f aca="false">(D10-MIN(C10,D10))*Data!$C$80+MIN(C10,D10)*Data!$C$81+E10*Data!$C$80*Data!$C$82</f>
         <v>0</v>
       </c>
       <c r="G10" s="32" t="str">
@@ -6027,7 +6045,7 @@
         <v>0</v>
       </c>
       <c r="F11" s="26" t="n">
-        <f aca="false">(D11-MIN(C11,D11))*Data!$C$60+MIN(C11,D11)*Data!$C$61+E11*Data!$C$60*Data!$C$62</f>
+        <f aca="false">(D11-MIN(C11,D11))*Data!$C$80+MIN(C11,D11)*Data!$C$81+E11*Data!$C$80*Data!$C$82</f>
         <v>0</v>
       </c>
       <c r="G11" s="32" t="str">
@@ -6048,7 +6066,7 @@
         <v>0</v>
       </c>
       <c r="F12" s="26" t="n">
-        <f aca="false">(D12-MIN(C12,D12))*Data!$C$60+MIN(C12,D12)*Data!$C$61+E12*Data!$C$60*Data!$C$62</f>
+        <f aca="false">(D12-MIN(C12,D12))*Data!$C$80+MIN(C12,D12)*Data!$C$81+E12*Data!$C$80*Data!$C$82</f>
         <v>0</v>
       </c>
       <c r="G12" s="32" t="str">
@@ -6069,7 +6087,7 @@
         <v>0</v>
       </c>
       <c r="F13" s="26" t="n">
-        <f aca="false">(D13-MIN(C13,D13))*Data!$C$60+MIN(C13,D13)*Data!$C$61+E13*Data!$C$60*Data!$C$62</f>
+        <f aca="false">(D13-MIN(C13,D13))*Data!$C$80+MIN(C13,D13)*Data!$C$81+E13*Data!$C$80*Data!$C$82</f>
         <v>0</v>
       </c>
       <c r="G13" s="32" t="str">
@@ -6090,7 +6108,7 @@
         <v>0</v>
       </c>
       <c r="F14" s="26" t="n">
-        <f aca="false">(D14-MIN(C14,D14))*Data!$C$60+MIN(C14,D14)*Data!$C$61+E14*Data!$C$60*Data!$C$62</f>
+        <f aca="false">(D14-MIN(C14,D14))*Data!$C$80+MIN(C14,D14)*Data!$C$81+E14*Data!$C$80*Data!$C$82</f>
         <v>0</v>
       </c>
       <c r="G14" s="32" t="str">
@@ -6111,7 +6129,7 @@
         <v>0</v>
       </c>
       <c r="F15" s="26" t="n">
-        <f aca="false">(D15-MIN(C15,D15))*Data!$C$60+MIN(C15,D15)*Data!$C$61+E15*Data!$C$60*Data!$C$62</f>
+        <f aca="false">(D15-MIN(C15,D15))*Data!$C$80+MIN(C15,D15)*Data!$C$81+E15*Data!$C$80*Data!$C$82</f>
         <v>0</v>
       </c>
       <c r="G15" s="32" t="str">
@@ -6132,7 +6150,7 @@
         <v>0</v>
       </c>
       <c r="F16" s="26" t="n">
-        <f aca="false">(D16-MIN(C16,D16))*Data!$C$60+MIN(C16,D16)*Data!$C$61+E16*Data!$C$60*Data!$C$62</f>
+        <f aca="false">(D16-MIN(C16,D16))*Data!$C$80+MIN(C16,D16)*Data!$C$81+E16*Data!$C$80*Data!$C$82</f>
         <v>0</v>
       </c>
       <c r="G16" s="32" t="str">
@@ -6153,7 +6171,7 @@
         <v>0</v>
       </c>
       <c r="F17" s="26" t="n">
-        <f aca="false">(D17-MIN(C17,D17))*Data!$C$60+MIN(C17,D17)*Data!$C$61+E17*Data!$C$60*Data!$C$62</f>
+        <f aca="false">(D17-MIN(C17,D17))*Data!$C$80+MIN(C17,D17)*Data!$C$81+E17*Data!$C$80*Data!$C$82</f>
         <v>0</v>
       </c>
       <c r="G17" s="32" t="str">
@@ -6174,7 +6192,7 @@
         <v>0</v>
       </c>
       <c r="F18" s="26" t="n">
-        <f aca="false">(D18-MIN(C18,D18))*Data!$C$60+MIN(C18,D18)*Data!$C$61+E18*Data!$C$60*Data!$C$62</f>
+        <f aca="false">(D18-MIN(C18,D18))*Data!$C$80+MIN(C18,D18)*Data!$C$81+E18*Data!$C$80*Data!$C$82</f>
         <v>0</v>
       </c>
       <c r="G18" s="32" t="str">
@@ -6195,7 +6213,7 @@
         <v>0</v>
       </c>
       <c r="F19" s="26" t="n">
-        <f aca="false">(D19-MIN(C19,D19))*Data!$C$60+MIN(C19,D19)*Data!$C$61+E19*Data!$C$60*Data!$C$62</f>
+        <f aca="false">(D19-MIN(C19,D19))*Data!$C$80+MIN(C19,D19)*Data!$C$81+E19*Data!$C$80*Data!$C$82</f>
         <v>0</v>
       </c>
       <c r="G19" s="32" t="str">
@@ -6216,7 +6234,7 @@
         <v>0</v>
       </c>
       <c r="F20" s="26" t="n">
-        <f aca="false">(D20-MIN(C20,D20))*Data!$C$60+MIN(C20,D20)*Data!$C$61+E20*Data!$C$60*Data!$C$62</f>
+        <f aca="false">(D20-MIN(C20,D20))*Data!$C$80+MIN(C20,D20)*Data!$C$81+E20*Data!$C$80*Data!$C$82</f>
         <v>0</v>
       </c>
       <c r="G20" s="32" t="str">
@@ -6237,7 +6255,7 @@
         <v>0</v>
       </c>
       <c r="F21" s="26" t="n">
-        <f aca="false">(D21-MIN(C21,D21))*Data!$C$60+MIN(C21,D21)*Data!$C$61+E21*Data!$C$60*Data!$C$62</f>
+        <f aca="false">(D21-MIN(C21,D21))*Data!$C$80+MIN(C21,D21)*Data!$C$81+E21*Data!$C$80*Data!$C$82</f>
         <v>0</v>
       </c>
       <c r="G21" s="32" t="str">
@@ -6258,7 +6276,7 @@
         <v>0</v>
       </c>
       <c r="F22" s="26" t="n">
-        <f aca="false">(D22-MIN(C22,D22))*Data!$C$60+MIN(C22,D22)*Data!$C$61+E22*Data!$C$60*Data!$C$62</f>
+        <f aca="false">(D22-MIN(C22,D22))*Data!$C$80+MIN(C22,D22)*Data!$C$81+E22*Data!$C$80*Data!$C$82</f>
         <v>0</v>
       </c>
       <c r="G22" s="32" t="str">
@@ -6279,7 +6297,7 @@
         <v>0</v>
       </c>
       <c r="F23" s="26" t="n">
-        <f aca="false">(D23-MIN(C23,D23))*Data!$C$60+MIN(C23,D23)*Data!$C$61+E23*Data!$C$60*Data!$C$62</f>
+        <f aca="false">(D23-MIN(C23,D23))*Data!$C$80+MIN(C23,D23)*Data!$C$81+E23*Data!$C$80*Data!$C$82</f>
         <v>0</v>
       </c>
       <c r="G23" s="32" t="str">
@@ -6300,7 +6318,7 @@
         <v>0</v>
       </c>
       <c r="F24" s="26" t="n">
-        <f aca="false">(D24-MIN(C24,D24))*Data!$C$60+MIN(C24,D24)*Data!$C$61+E24*Data!$C$60*Data!$C$62</f>
+        <f aca="false">(D24-MIN(C24,D24))*Data!$C$80+MIN(C24,D24)*Data!$C$81+E24*Data!$C$80*Data!$C$82</f>
         <v>0</v>
       </c>
       <c r="G24" s="32" t="str">
@@ -6321,7 +6339,7 @@
         <v>0</v>
       </c>
       <c r="F25" s="26" t="n">
-        <f aca="false">(D25-MIN(C25,D25))*Data!$C$60+MIN(C25,D25)*Data!$C$61+E25*Data!$C$60*Data!$C$62</f>
+        <f aca="false">(D25-MIN(C25,D25))*Data!$C$80+MIN(C25,D25)*Data!$C$81+E25*Data!$C$80*Data!$C$82</f>
         <v>0</v>
       </c>
       <c r="G25" s="32" t="str">
@@ -6342,7 +6360,7 @@
         <v>0</v>
       </c>
       <c r="F26" s="26" t="n">
-        <f aca="false">(D26-MIN(C26,D26))*Data!$C$60+MIN(C26,D26)*Data!$C$61+E26*Data!$C$60*Data!$C$62</f>
+        <f aca="false">(D26-MIN(C26,D26))*Data!$C$80+MIN(C26,D26)*Data!$C$81+E26*Data!$C$80*Data!$C$82</f>
         <v>0</v>
       </c>
       <c r="G26" s="32" t="str">
@@ -6363,7 +6381,7 @@
         <v>0</v>
       </c>
       <c r="F27" s="26" t="n">
-        <f aca="false">(D27-MIN(C27,D27))*Data!$C$60+MIN(C27,D27)*Data!$C$61+E27*Data!$C$60*Data!$C$62</f>
+        <f aca="false">(D27-MIN(C27,D27))*Data!$C$80+MIN(C27,D27)*Data!$C$81+E27*Data!$C$80*Data!$C$82</f>
         <v>0</v>
       </c>
       <c r="G27" s="32" t="str">
@@ -6384,7 +6402,7 @@
         <v>0</v>
       </c>
       <c r="F28" s="26" t="n">
-        <f aca="false">(D28-MIN(C28,D28))*Data!$C$60+MIN(C28,D28)*Data!$C$61+E28*Data!$C$60*Data!$C$62</f>
+        <f aca="false">(D28-MIN(C28,D28))*Data!$C$80+MIN(C28,D28)*Data!$C$81+E28*Data!$C$80*Data!$C$82</f>
         <v>0</v>
       </c>
       <c r="G28" s="32" t="str">
@@ -6405,7 +6423,7 @@
         <v>0</v>
       </c>
       <c r="F29" s="26" t="n">
-        <f aca="false">(D29-MIN(C29,D29))*Data!$C$60+MIN(C29,D29)*Data!$C$61+E29*Data!$C$60*Data!$C$62</f>
+        <f aca="false">(D29-MIN(C29,D29))*Data!$C$80+MIN(C29,D29)*Data!$C$81+E29*Data!$C$80*Data!$C$82</f>
         <v>0</v>
       </c>
       <c r="G29" s="32" t="str">
@@ -6426,7 +6444,7 @@
         <v>0</v>
       </c>
       <c r="F30" s="26" t="n">
-        <f aca="false">(D30-MIN(C30,D30))*Data!$C$60+MIN(C30,D30)*Data!$C$61+E30*Data!$C$60*Data!$C$62</f>
+        <f aca="false">(D30-MIN(C30,D30))*Data!$C$80+MIN(C30,D30)*Data!$C$81+E30*Data!$C$80*Data!$C$82</f>
         <v>0</v>
       </c>
       <c r="G30" s="32" t="str">
@@ -6447,7 +6465,7 @@
         <v>0</v>
       </c>
       <c r="F31" s="26" t="n">
-        <f aca="false">(D31-MIN(C31,D31))*Data!$C$60+MIN(C31,D31)*Data!$C$61+E31*Data!$C$60*Data!$C$62</f>
+        <f aca="false">(D31-MIN(C31,D31))*Data!$C$80+MIN(C31,D31)*Data!$C$81+E31*Data!$C$80*Data!$C$82</f>
         <v>0</v>
       </c>
       <c r="G31" s="32" t="str">
@@ -6468,7 +6486,7 @@
         <v>0</v>
       </c>
       <c r="F32" s="26" t="n">
-        <f aca="false">(D32-MIN(C32,D32))*Data!$C$60+MIN(C32,D32)*Data!$C$61+E32*Data!$C$60*Data!$C$62</f>
+        <f aca="false">(D32-MIN(C32,D32))*Data!$C$80+MIN(C32,D32)*Data!$C$81+E32*Data!$C$80*Data!$C$82</f>
         <v>0</v>
       </c>
       <c r="G32" s="32" t="str">
@@ -6489,7 +6507,7 @@
         <v>0</v>
       </c>
       <c r="F33" s="26" t="n">
-        <f aca="false">(D33-MIN(C33,D33))*Data!$C$60+MIN(C33,D33)*Data!$C$61+E33*Data!$C$60*Data!$C$62</f>
+        <f aca="false">(D33-MIN(C33,D33))*Data!$C$80+MIN(C33,D33)*Data!$C$81+E33*Data!$C$80*Data!$C$82</f>
         <v>0</v>
       </c>
       <c r="G33" s="32" t="str">
@@ -6510,7 +6528,7 @@
         <v>0</v>
       </c>
       <c r="F34" s="26" t="n">
-        <f aca="false">(D34-MIN(C34,D34))*Data!$C$60+MIN(C34,D34)*Data!$C$61+E34*Data!$C$60*Data!$C$62</f>
+        <f aca="false">(D34-MIN(C34,D34))*Data!$C$80+MIN(C34,D34)*Data!$C$81+E34*Data!$C$80*Data!$C$82</f>
         <v>0</v>
       </c>
       <c r="G34" s="32" t="str">
@@ -6531,7 +6549,7 @@
         <v>0</v>
       </c>
       <c r="F35" s="26" t="n">
-        <f aca="false">(D35-MIN(C35,D35))*Data!$C$60+MIN(C35,D35)*Data!$C$61+E35*Data!$C$60*Data!$C$62</f>
+        <f aca="false">(D35-MIN(C35,D35))*Data!$C$80+MIN(C35,D35)*Data!$C$81+E35*Data!$C$80*Data!$C$82</f>
         <v>0</v>
       </c>
       <c r="G35" s="32" t="str">
@@ -6565,7 +6583,7 @@
         <v>253</v>
       </c>
       <c r="F37" s="34" t="n">
-        <f aca="false">F36*Data!$C$63</f>
+        <f aca="false">F36*Data!$C$83</f>
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix K-1 and S-corp issues found by QA
- Engine: a spouse's W-2 no longer uses the business owner's Social
  Security wage base (seOwnerWages); QBI 50% W-2 wage limit above the
  threshold (qbiW2Wages); 0.9% additional Medicare tax
- S-corp calculator: salary counts as W-2 wages for QBI, excess Social
  Security credit with another job, Illinois replacement tax deducted
  before the K-1, other-state entity tax note, input validation,
  fieldset/legend, smaller live region, corrected copy
- K-1: visible box 14A field in the estimator; Start over clears K-1
  state; blank K-1 type counts as partnership in Excel like the PDF;
  assumed-SE flag reaches the Preparer summary; QA regression tests

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012ebqUPkXNMCm1mSUdBK3xi
</commit_message>
<xml_diff>
--- a/tax-prep/downloads/falcon-tax-organizer-2026.xlsx
+++ b/tax-prep/downloads/falcon-tax-organizer-2026.xlsx
@@ -51,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="580" uniqueCount="500">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="582" uniqueCount="502">
   <si>
     <t xml:space="preserve">Falcon Tax Solutions · 2026 Tax Organizer</t>
   </si>
@@ -1454,16 +1454,28 @@
     <t xml:space="preserve">VT</t>
   </si>
   <si>
+    <t xml:space="preserve">k1SeAssumed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Box 14A left blank on a partnership K-1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Virginia</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VA</t>
+  </si>
+  <si>
     <t xml:space="preserve">you50</t>
   </si>
   <si>
     <t xml:space="preserve">You 50 or older (born 1976 or earlier)</t>
   </si>
   <si>
-    <t xml:space="preserve">Virginia</t>
-  </si>
-  <si>
-    <t xml:space="preserve">VA</t>
+    <t xml:space="preserve">Washington</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WA</t>
   </si>
   <si>
     <t xml:space="preserve">spouse50</t>
@@ -1472,10 +1484,10 @@
     <t xml:space="preserve">Spouse 50 or older (joint returns)</t>
   </si>
   <si>
-    <t xml:space="preserve">Washington</t>
-  </si>
-  <si>
-    <t xml:space="preserve">WA</t>
+    <t xml:space="preserve">West Virginia</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WV</t>
   </si>
   <si>
     <t xml:space="preserve">you55</t>
@@ -1484,10 +1496,10 @@
     <t xml:space="preserve">You 55 or older (HSA catch-up)</t>
   </si>
   <si>
-    <t xml:space="preserve">West Virginia</t>
-  </si>
-  <si>
-    <t xml:space="preserve">WV</t>
+    <t xml:space="preserve">Wisconsin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WI</t>
   </si>
   <si>
     <t xml:space="preserve">retirement</t>
@@ -1496,19 +1508,13 @@
     <t xml:space="preserve">Has retirement withdrawals</t>
   </si>
   <si>
-    <t xml:space="preserve">Wisconsin</t>
-  </si>
-  <si>
-    <t xml:space="preserve">WI</t>
+    <t xml:space="preserve">Wyoming</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WY</t>
   </si>
   <si>
     <t xml:space="preserve">hasInvestments</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Wyoming</t>
-  </si>
-  <si>
-    <t xml:space="preserve">WY</t>
   </si>
   <si>
     <t xml:space="preserve">mortgage</t>
@@ -3159,7 +3165,7 @@
         <v>452</v>
       </c>
       <c r="C44" s="6" t="n">
-        <f aca="false">SUMIF(Income!A47:A50,"Partnership / LLC (1065)",Income!C47:C50)</f>
+        <f aca="false">SUM(Income!C47:C50)-SUMIF(Income!A47:A50,"S-corp (1120-S)",Income!C47:C50)</f>
         <v>0</v>
       </c>
       <c r="H44" s="35" t="s">
@@ -3177,7 +3183,7 @@
         <v>456</v>
       </c>
       <c r="C45" s="6" t="n">
-        <f aca="false">SUMIF(Income!A47:A50,"Partnership / LLC (1065)",Income!D47:D50)</f>
+        <f aca="false">SUM(Income!D47:D50)-SUMIF(Income!A47:A50,"S-corp (1120-S)",Income!D47:D50)</f>
         <v>0</v>
       </c>
       <c r="H45" s="35" t="s">
@@ -3231,7 +3237,7 @@
         <v>468</v>
       </c>
       <c r="C48" s="6" t="n">
-        <f aca="false">IF(AND(ISNUMBER(Household!B6),Household!B6&gt;0,Household!B6&lt;=1976),1,0)</f>
+        <f aca="false">IF(SUMPRODUCT((Income!A47:A50&lt;&gt;"S-corp (1120-S)")*((Income!C47:C50&lt;&gt;"")+(Income!D47:D50&lt;&gt;"")&gt;0)*(Income!E47:E50=""))&gt;0,1,0)</f>
         <v>0</v>
       </c>
       <c r="H48" s="35" t="s">
@@ -3249,7 +3255,7 @@
         <v>472</v>
       </c>
       <c r="C49" s="6" t="n">
-        <f aca="false">IF(AND(C5="mfj",ISNUMBER(Household!B7),Household!B7&gt;0,Household!B7&lt;=1976),1,0)</f>
+        <f aca="false">IF(AND(ISNUMBER(Household!B6),Household!B6&gt;0,Household!B6&lt;=1976),1,0)</f>
         <v>0</v>
       </c>
       <c r="H49" s="35" t="s">
@@ -3267,7 +3273,7 @@
         <v>476</v>
       </c>
       <c r="C50" s="6" t="n">
-        <f aca="false">IF(AND(ISNUMBER(Household!B6),Household!B6&gt;0,Household!B6&lt;=1971),1,0)</f>
+        <f aca="false">IF(AND(C5="mfj",ISNUMBER(Household!B7),Household!B7&gt;0,Household!B7&lt;=1976),1,0)</f>
         <v>0</v>
       </c>
       <c r="H50" s="35" t="s">
@@ -3285,7 +3291,7 @@
         <v>480</v>
       </c>
       <c r="C51" s="6" t="n">
-        <f aca="false">IF(Income!C27&gt;0,1,0)</f>
+        <f aca="false">IF(AND(ISNUMBER(Household!B6),Household!B6&gt;0,Household!B6&lt;=1971),1,0)</f>
         <v>0</v>
       </c>
       <c r="H51" s="35" t="s">
@@ -3300,99 +3306,111 @@
         <v>483</v>
       </c>
       <c r="B52" s="21" t="s">
-        <v>267</v>
+        <v>484</v>
       </c>
       <c r="C52" s="6" t="n">
-        <f aca="false">IF(TRIM(Checklist!B4)="Yes",1,0)</f>
+        <f aca="false">IF(Income!C27&gt;0,1,0)</f>
         <v>0</v>
       </c>
       <c r="H52" s="35" t="s">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="I52" s="35" t="s">
-        <v>485</v>
+        <v>486</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="9" t="s">
-        <v>486</v>
+        <v>487</v>
       </c>
       <c r="B53" s="21" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="C53" s="6" t="n">
-        <f aca="false">IF(TRIM(Checklist!B5)="Yes",1,0)</f>
+        <f aca="false">IF(TRIM(Checklist!B4)="Yes",1,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="9" t="s">
-        <v>487</v>
+        <v>488</v>
       </c>
       <c r="B54" s="21" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="C54" s="6" t="n">
-        <f aca="false">IF(TRIM(Checklist!B6)="Yes",1,0)</f>
+        <f aca="false">IF(TRIM(Checklist!B5)="Yes",1,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="9" t="s">
-        <v>488</v>
+        <v>489</v>
       </c>
       <c r="B55" s="21" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="C55" s="6" t="n">
-        <f aca="false">IF(TRIM(Checklist!B7)="Yes",1,0)</f>
+        <f aca="false">IF(TRIM(Checklist!B6)="Yes",1,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="9" t="s">
-        <v>489</v>
+        <v>490</v>
       </c>
       <c r="B56" s="21" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="C56" s="6" t="n">
-        <f aca="false">IF(TRIM(Checklist!B8)="Yes",1,0)</f>
+        <f aca="false">IF(TRIM(Checklist!B7)="Yes",1,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="9" t="s">
-        <v>490</v>
+        <v>491</v>
       </c>
       <c r="B57" s="21" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="C57" s="6" t="n">
-        <f aca="false">IF(TRIM(Checklist!B9)="Yes",1,0)</f>
+        <f aca="false">IF(TRIM(Checklist!B8)="Yes",1,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="9" t="s">
-        <v>491</v>
+        <v>492</v>
       </c>
       <c r="B58" s="21" t="s">
+        <v>272</v>
+      </c>
+      <c r="C58" s="6" t="n">
+        <f aca="false">IF(TRIM(Checklist!B9)="Yes",1,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A59" s="9" t="s">
+        <v>493</v>
+      </c>
+      <c r="B59" s="21" t="s">
         <v>273</v>
       </c>
-      <c r="C58" s="6" t="n">
+      <c r="C59" s="6" t="n">
         <f aca="false">IF(TRIM(Checklist!B10)="Yes",1,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A79" s="39" t="s">
-        <v>492</v>
+        <v>494</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B80" s="6" t="s">
-        <v>493</v>
+        <v>495</v>
       </c>
       <c r="C80" s="40" t="n">
         <v>80</v>
@@ -3400,7 +3418,7 @@
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B81" s="6" t="s">
-        <v>494</v>
+        <v>496</v>
       </c>
       <c r="C81" s="40" t="n">
         <v>86</v>
@@ -3408,7 +3426,7 @@
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B82" s="6" t="s">
-        <v>495</v>
+        <v>497</v>
       </c>
       <c r="C82" s="41" t="n">
         <v>0.75</v>
@@ -3416,7 +3434,7 @@
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B83" s="6" t="s">
-        <v>496</v>
+        <v>498</v>
       </c>
       <c r="C83" s="41" t="n">
         <v>0.8</v>
@@ -3424,12 +3442,12 @@
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A85" s="39" t="s">
-        <v>497</v>
+        <v>499</v>
       </c>
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B86" s="6" t="s">
-        <v>498</v>
+        <v>500</v>
       </c>
       <c r="C86" s="42" t="n">
         <v>0.725</v>
@@ -3437,7 +3455,7 @@
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B87" s="6" t="s">
-        <v>499</v>
+        <v>501</v>
       </c>
       <c r="C87" s="42" t="n">
         <v>0.76</v>
@@ -4233,7 +4251,7 @@
       <c r="D47" s="19"/>
       <c r="E47" s="19"/>
       <c r="F47" s="22" t="n">
-        <f aca="false">IF(A47="Partnership / LLC (1065)",IF(E47="",N(C47)+N(D47),N(E47)),0)</f>
+        <f aca="false">IF(A47="S-corp (1120-S)",0,IF(E47="",N(C47)+N(D47),N(E47)))</f>
         <v>0</v>
       </c>
     </row>
@@ -4244,7 +4262,7 @@
       <c r="D48" s="19"/>
       <c r="E48" s="19"/>
       <c r="F48" s="22" t="n">
-        <f aca="false">IF(A48="Partnership / LLC (1065)",IF(E48="",N(C48)+N(D48),N(E48)),0)</f>
+        <f aca="false">IF(A48="S-corp (1120-S)",0,IF(E48="",N(C48)+N(D48),N(E48)))</f>
         <v>0</v>
       </c>
     </row>
@@ -4255,7 +4273,7 @@
       <c r="D49" s="19"/>
       <c r="E49" s="19"/>
       <c r="F49" s="22" t="n">
-        <f aca="false">IF(A49="Partnership / LLC (1065)",IF(E49="",N(C49)+N(D49),N(E49)),0)</f>
+        <f aca="false">IF(A49="S-corp (1120-S)",0,IF(E49="",N(C49)+N(D49),N(E49)))</f>
         <v>0</v>
       </c>
     </row>
@@ -4266,7 +4284,7 @@
       <c r="D50" s="19"/>
       <c r="E50" s="19"/>
       <c r="F50" s="22" t="n">
-        <f aca="false">IF(A50="Partnership / LLC (1065)",IF(E50="",N(C50)+N(D50),N(E50)),0)</f>
+        <f aca="false">IF(A50="S-corp (1120-S)",0,IF(E50="",N(C50)+N(D50),N(E50)))</f>
         <v>0</v>
       </c>
     </row>

</xml_diff>